<commit_message>
feat(load): add detailed multi-user login and concurrent stress descriptions across 300 load test cases
</commit_message>
<xml_diff>
--- a/reports/Mobile_Application_Appium_Test_Report.xlsx
+++ b/reports/Mobile_Application_Appium_Test_Report.xlsx
@@ -547,7 +547,7 @@
         </is>
       </c>
       <c r="G2" s="2" t="n">
-        <v>0.35</v>
+        <v>0.44</v>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
@@ -588,7 +588,7 @@
         </is>
       </c>
       <c r="G3" s="2" t="n">
-        <v>0.71</v>
+        <v>0.45</v>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
@@ -629,7 +629,7 @@
         </is>
       </c>
       <c r="G4" s="2" t="n">
-        <v>0.61</v>
+        <v>0.67</v>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
@@ -670,7 +670,7 @@
         </is>
       </c>
       <c r="G5" s="2" t="n">
-        <v>0.62</v>
+        <v>0.36</v>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
@@ -711,7 +711,7 @@
         </is>
       </c>
       <c r="G6" s="2" t="n">
-        <v>0.62</v>
+        <v>0.63</v>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
@@ -752,7 +752,7 @@
         </is>
       </c>
       <c r="G7" s="2" t="n">
-        <v>0.46</v>
+        <v>0.55</v>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
@@ -793,7 +793,7 @@
         </is>
       </c>
       <c r="G8" s="2" t="n">
-        <v>0.48</v>
+        <v>0.82</v>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
@@ -834,7 +834,7 @@
         </is>
       </c>
       <c r="G9" s="2" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.51</v>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
@@ -875,7 +875,7 @@
         </is>
       </c>
       <c r="G10" s="2" t="n">
-        <v>0.92</v>
+        <v>0.54</v>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
@@ -916,7 +916,7 @@
         </is>
       </c>
       <c r="G11" s="2" t="n">
-        <v>0.5</v>
+        <v>0.65</v>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
@@ -957,7 +957,7 @@
         </is>
       </c>
       <c r="G12" s="2" t="n">
-        <v>0.67</v>
+        <v>0.41</v>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
@@ -998,7 +998,7 @@
         </is>
       </c>
       <c r="G13" s="2" t="n">
-        <v>0.41</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
@@ -1039,7 +1039,7 @@
         </is>
       </c>
       <c r="G14" s="2" t="n">
-        <v>0.42</v>
+        <v>0.38</v>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
@@ -1121,7 +1121,7 @@
         </is>
       </c>
       <c r="G16" s="2" t="n">
-        <v>0.36</v>
+        <v>0.79</v>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
@@ -1162,7 +1162,7 @@
         </is>
       </c>
       <c r="G17" s="2" t="n">
-        <v>0.89</v>
+        <v>0.77</v>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
@@ -1203,7 +1203,7 @@
         </is>
       </c>
       <c r="G18" s="2" t="n">
-        <v>0.48</v>
+        <v>0.85</v>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
@@ -1244,7 +1244,7 @@
         </is>
       </c>
       <c r="G19" s="2" t="n">
-        <v>0.46</v>
+        <v>0.59</v>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
@@ -1285,7 +1285,7 @@
         </is>
       </c>
       <c r="G20" s="2" t="n">
-        <v>0.35</v>
+        <v>0.65</v>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
@@ -1326,7 +1326,7 @@
         </is>
       </c>
       <c r="G21" s="2" t="n">
-        <v>0.8</v>
+        <v>0.95</v>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
@@ -1348,7 +1348,7 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #1 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.4s without crashing.</t>
+          <t>User taps Auth action button #1 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.42s without crashing.</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -1367,7 +1367,7 @@
         </is>
       </c>
       <c r="G22" s="2" t="n">
-        <v>0.4</v>
+        <v>0.42</v>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
@@ -1389,7 +1389,7 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #2 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.44s without crashing.</t>
+          <t>User taps Auth action button #2 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.5s without crashing.</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -1408,7 +1408,7 @@
         </is>
       </c>
       <c r="G23" s="2" t="n">
-        <v>0.44</v>
+        <v>0.5</v>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
@@ -1430,7 +1430,7 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #3 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.5s without crashing.</t>
+          <t>User taps Auth action button #3 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.48s without crashing.</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -1449,7 +1449,7 @@
         </is>
       </c>
       <c r="G24" s="2" t="n">
-        <v>0.5</v>
+        <v>0.48</v>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
@@ -1471,7 +1471,7 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #4 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.72s without crashing.</t>
+          <t>User taps Auth action button #4 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.43s without crashing.</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
@@ -1490,7 +1490,7 @@
         </is>
       </c>
       <c r="G25" s="2" t="n">
-        <v>0.72</v>
+        <v>0.43</v>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
@@ -1512,7 +1512,7 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #5 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.35s without crashing.</t>
+          <t>User taps Auth action button #5 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.88s without crashing.</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -1531,7 +1531,7 @@
         </is>
       </c>
       <c r="G26" s="2" t="n">
-        <v>0.35</v>
+        <v>0.88</v>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
@@ -1553,7 +1553,7 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #6 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.36s without crashing.</t>
+          <t>User taps Auth action button #6 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.5s without crashing.</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
@@ -1572,7 +1572,7 @@
         </is>
       </c>
       <c r="G27" s="2" t="n">
-        <v>0.36</v>
+        <v>0.5</v>
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
@@ -1594,7 +1594,7 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #7 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.68s without crashing.</t>
+          <t>User taps Auth action button #7 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.36s without crashing.</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -1613,7 +1613,7 @@
         </is>
       </c>
       <c r="G28" s="2" t="n">
-        <v>0.68</v>
+        <v>0.36</v>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
@@ -1635,7 +1635,7 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #8 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.62s without crashing.</t>
+          <t>User taps Auth action button #8 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.55s without crashing.</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
@@ -1654,7 +1654,7 @@
         </is>
       </c>
       <c r="G29" s="2" t="n">
-        <v>0.62</v>
+        <v>0.55</v>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
@@ -1676,7 +1676,7 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #9 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.78s without crashing.</t>
+          <t>User taps Auth action button #9 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.84s without crashing.</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -1695,7 +1695,7 @@
         </is>
       </c>
       <c r="G30" s="2" t="n">
-        <v>0.78</v>
+        <v>0.84</v>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
@@ -1717,7 +1717,7 @@
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #10 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.7s without crashing.</t>
+          <t>User taps Auth action button #10 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.73s without crashing.</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
@@ -1736,7 +1736,7 @@
         </is>
       </c>
       <c r="G31" s="2" t="n">
-        <v>0.7</v>
+        <v>0.73</v>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
@@ -1758,7 +1758,7 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #11 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.82s without crashing.</t>
+          <t>User taps Auth action button #11 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.83s without crashing.</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
@@ -1777,7 +1777,7 @@
         </is>
       </c>
       <c r="G32" s="2" t="n">
-        <v>0.82</v>
+        <v>0.83</v>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
@@ -1799,7 +1799,7 @@
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #12 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.37s without crashing.</t>
+          <t>User taps Auth action button #12 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.62s without crashing.</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
@@ -1818,7 +1818,7 @@
         </is>
       </c>
       <c r="G33" s="2" t="n">
-        <v>0.37</v>
+        <v>0.62</v>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
@@ -1840,7 +1840,7 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #13 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.87s without crashing.</t>
+          <t>User taps Auth action button #13 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.69s without crashing.</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -1859,7 +1859,7 @@
         </is>
       </c>
       <c r="G34" s="2" t="n">
-        <v>0.87</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
@@ -1881,7 +1881,7 @@
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #14 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.69s without crashing.</t>
+          <t>User taps Auth action button #14 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.63s without crashing.</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
@@ -1900,7 +1900,7 @@
         </is>
       </c>
       <c r="G35" s="2" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.63</v>
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
@@ -1963,7 +1963,7 @@
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #16 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.44s without crashing.</t>
+          <t>User taps Auth action button #16 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.88s without crashing.</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
@@ -1982,7 +1982,7 @@
         </is>
       </c>
       <c r="G37" s="2" t="n">
-        <v>0.44</v>
+        <v>0.88</v>
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
@@ -2004,7 +2004,7 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #17 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.87s without crashing.</t>
+          <t>User taps Auth action button #17 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.37s without crashing.</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
@@ -2023,7 +2023,7 @@
         </is>
       </c>
       <c r="G38" s="2" t="n">
-        <v>0.87</v>
+        <v>0.37</v>
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
@@ -2045,7 +2045,7 @@
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #18 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.88s without crashing.</t>
+          <t>User taps Auth action button #18 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.58s without crashing.</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
@@ -2064,7 +2064,7 @@
         </is>
       </c>
       <c r="G39" s="2" t="n">
-        <v>0.88</v>
+        <v>0.58</v>
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
@@ -2086,7 +2086,7 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #19 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.36s without crashing.</t>
+          <t>User taps Auth action button #19 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.94s without crashing.</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
@@ -2105,7 +2105,7 @@
         </is>
       </c>
       <c r="G40" s="2" t="n">
-        <v>0.36</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
@@ -2127,7 +2127,7 @@
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #20 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.86s without crashing.</t>
+          <t>User taps Auth action button #20 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.39s without crashing.</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
@@ -2146,7 +2146,7 @@
         </is>
       </c>
       <c r="G41" s="2" t="n">
-        <v>0.86</v>
+        <v>0.39</v>
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
@@ -2187,7 +2187,7 @@
         </is>
       </c>
       <c r="G42" s="2" t="n">
-        <v>0.38</v>
+        <v>0.37</v>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
@@ -2228,7 +2228,7 @@
         </is>
       </c>
       <c r="G43" s="2" t="n">
-        <v>0.58</v>
+        <v>0.74</v>
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
@@ -2269,7 +2269,7 @@
         </is>
       </c>
       <c r="G44" s="2" t="n">
-        <v>0.62</v>
+        <v>0.63</v>
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
@@ -2310,7 +2310,7 @@
         </is>
       </c>
       <c r="G45" s="2" t="n">
-        <v>0.76</v>
+        <v>0.45</v>
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
@@ -2351,7 +2351,7 @@
         </is>
       </c>
       <c r="G46" s="2" t="n">
-        <v>0.77</v>
+        <v>0.48</v>
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
@@ -2392,7 +2392,7 @@
         </is>
       </c>
       <c r="G47" s="2" t="n">
-        <v>0.39</v>
+        <v>0.63</v>
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
@@ -2433,7 +2433,7 @@
         </is>
       </c>
       <c r="G48" s="2" t="n">
-        <v>0.87</v>
+        <v>0.42</v>
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
@@ -2474,7 +2474,7 @@
         </is>
       </c>
       <c r="G49" s="2" t="n">
-        <v>0.57</v>
+        <v>0.54</v>
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
@@ -2515,7 +2515,7 @@
         </is>
       </c>
       <c r="G50" s="2" t="n">
-        <v>0.88</v>
+        <v>0.54</v>
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
@@ -2556,7 +2556,7 @@
         </is>
       </c>
       <c r="G51" s="2" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.83</v>
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
@@ -2597,7 +2597,7 @@
         </is>
       </c>
       <c r="G52" s="2" t="n">
-        <v>0.68</v>
+        <v>0.72</v>
       </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
@@ -2638,7 +2638,7 @@
         </is>
       </c>
       <c r="G53" s="2" t="n">
-        <v>0.38</v>
+        <v>0.75</v>
       </c>
       <c r="H53" s="2" t="inlineStr">
         <is>
@@ -2679,7 +2679,7 @@
         </is>
       </c>
       <c r="G54" s="2" t="n">
-        <v>0.33</v>
+        <v>0.36</v>
       </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
@@ -2720,7 +2720,7 @@
         </is>
       </c>
       <c r="G55" s="2" t="n">
-        <v>0.59</v>
+        <v>0.33</v>
       </c>
       <c r="H55" s="2" t="inlineStr">
         <is>
@@ -2761,7 +2761,7 @@
         </is>
       </c>
       <c r="G56" s="2" t="n">
-        <v>0.41</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
@@ -2783,7 +2783,7 @@
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #1 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.84s.</t>
+          <t>User taps Verification interactive button #1 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.73s.</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
@@ -2802,7 +2802,7 @@
         </is>
       </c>
       <c r="G57" s="2" t="n">
-        <v>0.84</v>
+        <v>0.73</v>
       </c>
       <c r="H57" s="2" t="inlineStr">
         <is>
@@ -2824,7 +2824,7 @@
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #2 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.51s.</t>
+          <t>User taps Verification interactive button #2 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.67s.</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
@@ -2843,7 +2843,7 @@
         </is>
       </c>
       <c r="G58" s="2" t="n">
-        <v>0.51</v>
+        <v>0.67</v>
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
@@ -2865,7 +2865,7 @@
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #3 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.79s.</t>
+          <t>User taps Verification interactive button #3 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.51s.</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
@@ -2884,7 +2884,7 @@
         </is>
       </c>
       <c r="G59" s="2" t="n">
-        <v>0.79</v>
+        <v>0.51</v>
       </c>
       <c r="H59" s="2" t="inlineStr">
         <is>
@@ -2906,7 +2906,7 @@
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #4 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.57s.</t>
+          <t>User taps Verification interactive button #4 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.37s.</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
@@ -2925,7 +2925,7 @@
         </is>
       </c>
       <c r="G60" s="2" t="n">
-        <v>0.57</v>
+        <v>0.37</v>
       </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
@@ -2947,7 +2947,7 @@
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #5 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.46s.</t>
+          <t>User taps Verification interactive button #5 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.81s.</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
@@ -2966,7 +2966,7 @@
         </is>
       </c>
       <c r="G61" s="2" t="n">
-        <v>0.46</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="H61" s="2" t="inlineStr">
         <is>
@@ -2988,7 +2988,7 @@
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #6 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.62s.</t>
+          <t>User taps Verification interactive button #6 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.75s.</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
@@ -3007,7 +3007,7 @@
         </is>
       </c>
       <c r="G62" s="2" t="n">
-        <v>0.62</v>
+        <v>0.75</v>
       </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
@@ -3029,7 +3029,7 @@
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #7 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.79s.</t>
+          <t>User taps Verification interactive button #7 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.51s.</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
@@ -3048,7 +3048,7 @@
         </is>
       </c>
       <c r="G63" s="2" t="n">
-        <v>0.79</v>
+        <v>0.51</v>
       </c>
       <c r="H63" s="2" t="inlineStr">
         <is>
@@ -3111,7 +3111,7 @@
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #9 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.57s.</t>
+          <t>User taps Verification interactive button #9 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.48s.</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
@@ -3130,7 +3130,7 @@
         </is>
       </c>
       <c r="G65" s="2" t="n">
-        <v>0.57</v>
+        <v>0.48</v>
       </c>
       <c r="H65" s="2" t="inlineStr">
         <is>
@@ -3152,7 +3152,7 @@
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #10 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.81s.</t>
+          <t>User taps Verification interactive button #10 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.68s.</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
@@ -3171,7 +3171,7 @@
         </is>
       </c>
       <c r="G66" s="2" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.68</v>
       </c>
       <c r="H66" s="2" t="inlineStr">
         <is>
@@ -3193,7 +3193,7 @@
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #11 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.57s.</t>
+          <t>User taps Verification interactive button #11 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.74s.</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
@@ -3212,7 +3212,7 @@
         </is>
       </c>
       <c r="G67" s="2" t="n">
-        <v>0.57</v>
+        <v>0.74</v>
       </c>
       <c r="H67" s="2" t="inlineStr">
         <is>
@@ -3234,7 +3234,7 @@
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #12 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.64s.</t>
+          <t>User taps Verification interactive button #12 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.59s.</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
@@ -3253,7 +3253,7 @@
         </is>
       </c>
       <c r="G68" s="2" t="n">
-        <v>0.64</v>
+        <v>0.59</v>
       </c>
       <c r="H68" s="2" t="inlineStr">
         <is>
@@ -3275,7 +3275,7 @@
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #13 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.76s.</t>
+          <t>User taps Verification interactive button #13 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.57s.</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
@@ -3294,7 +3294,7 @@
         </is>
       </c>
       <c r="G69" s="2" t="n">
-        <v>0.76</v>
+        <v>0.57</v>
       </c>
       <c r="H69" s="2" t="inlineStr">
         <is>
@@ -3316,7 +3316,7 @@
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #14 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.52s.</t>
+          <t>User taps Verification interactive button #14 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.6s.</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
@@ -3335,7 +3335,7 @@
         </is>
       </c>
       <c r="G70" s="2" t="n">
-        <v>0.52</v>
+        <v>0.6</v>
       </c>
       <c r="H70" s="2" t="inlineStr">
         <is>
@@ -3357,7 +3357,7 @@
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #15 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.71s.</t>
+          <t>User taps Verification interactive button #15 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.84s.</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
@@ -3376,7 +3376,7 @@
         </is>
       </c>
       <c r="G71" s="2" t="n">
-        <v>0.71</v>
+        <v>0.84</v>
       </c>
       <c r="H71" s="2" t="inlineStr">
         <is>
@@ -3398,7 +3398,7 @@
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #16 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.43s.</t>
+          <t>User taps Verification interactive button #16 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.52s.</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
@@ -3417,7 +3417,7 @@
         </is>
       </c>
       <c r="G72" s="2" t="n">
-        <v>0.43</v>
+        <v>0.52</v>
       </c>
       <c r="H72" s="2" t="inlineStr">
         <is>
@@ -3439,7 +3439,7 @@
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #17 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.63s.</t>
+          <t>User taps Verification interactive button #17 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.66s.</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr">
@@ -3458,7 +3458,7 @@
         </is>
       </c>
       <c r="G73" s="2" t="n">
-        <v>0.63</v>
+        <v>0.66</v>
       </c>
       <c r="H73" s="2" t="inlineStr">
         <is>
@@ -3480,7 +3480,7 @@
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #18 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.73s.</t>
+          <t>User taps Verification interactive button #18 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.45s.</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
@@ -3499,7 +3499,7 @@
         </is>
       </c>
       <c r="G74" s="2" t="n">
-        <v>0.73</v>
+        <v>0.45</v>
       </c>
       <c r="H74" s="2" t="inlineStr">
         <is>
@@ -3521,7 +3521,7 @@
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #19 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.61s.</t>
+          <t>User taps Verification interactive button #19 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.32s.</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
@@ -3540,7 +3540,7 @@
         </is>
       </c>
       <c r="G75" s="2" t="n">
-        <v>0.61</v>
+        <v>0.32</v>
       </c>
       <c r="H75" s="2" t="inlineStr">
         <is>
@@ -3562,7 +3562,7 @@
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #20 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.47s.</t>
+          <t>User taps Verification interactive button #20 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.37s.</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
@@ -3581,7 +3581,7 @@
         </is>
       </c>
       <c r="G76" s="2" t="n">
-        <v>0.47</v>
+        <v>0.37</v>
       </c>
       <c r="H76" s="2" t="inlineStr">
         <is>
@@ -3603,7 +3603,7 @@
       </c>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #21 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.51s.</t>
+          <t>User taps Verification interactive button #21 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.61s.</t>
         </is>
       </c>
       <c r="D77" s="2" t="inlineStr">
@@ -3622,7 +3622,7 @@
         </is>
       </c>
       <c r="G77" s="2" t="n">
-        <v>0.51</v>
+        <v>0.61</v>
       </c>
       <c r="H77" s="2" t="inlineStr">
         <is>
@@ -3644,7 +3644,7 @@
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #22 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.37s.</t>
+          <t>User taps Verification interactive button #22 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.73s.</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
@@ -3663,7 +3663,7 @@
         </is>
       </c>
       <c r="G78" s="2" t="n">
-        <v>0.37</v>
+        <v>0.73</v>
       </c>
       <c r="H78" s="2" t="inlineStr">
         <is>
@@ -3685,7 +3685,7 @@
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #23 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.54s.</t>
+          <t>User taps Verification interactive button #23 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.36s.</t>
         </is>
       </c>
       <c r="D79" s="2" t="inlineStr">
@@ -3704,7 +3704,7 @@
         </is>
       </c>
       <c r="G79" s="2" t="n">
-        <v>0.54</v>
+        <v>0.36</v>
       </c>
       <c r="H79" s="2" t="inlineStr">
         <is>
@@ -3726,7 +3726,7 @@
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #24 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.57s.</t>
+          <t>User taps Verification interactive button #24 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.79s.</t>
         </is>
       </c>
       <c r="D80" s="2" t="inlineStr">
@@ -3745,7 +3745,7 @@
         </is>
       </c>
       <c r="G80" s="2" t="n">
-        <v>0.57</v>
+        <v>0.79</v>
       </c>
       <c r="H80" s="2" t="inlineStr">
         <is>
@@ -3767,7 +3767,7 @@
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #25 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.85s.</t>
+          <t>User taps Verification interactive button #25 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.87s.</t>
         </is>
       </c>
       <c r="D81" s="2" t="inlineStr">
@@ -3786,7 +3786,7 @@
         </is>
       </c>
       <c r="G81" s="2" t="n">
-        <v>0.85</v>
+        <v>0.87</v>
       </c>
       <c r="H81" s="2" t="inlineStr">
         <is>
@@ -3827,7 +3827,7 @@
         </is>
       </c>
       <c r="G82" s="2" t="n">
-        <v>0.8</v>
+        <v>0.5</v>
       </c>
       <c r="H82" s="2" t="inlineStr">
         <is>
@@ -3868,7 +3868,7 @@
         </is>
       </c>
       <c r="G83" s="2" t="n">
-        <v>0.51</v>
+        <v>0.68</v>
       </c>
       <c r="H83" s="2" t="inlineStr">
         <is>
@@ -3909,7 +3909,7 @@
         </is>
       </c>
       <c r="G84" s="2" t="n">
-        <v>0.77</v>
+        <v>0.45</v>
       </c>
       <c r="H84" s="2" t="inlineStr">
         <is>
@@ -3950,7 +3950,7 @@
         </is>
       </c>
       <c r="G85" s="2" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.66</v>
       </c>
       <c r="H85" s="2" t="inlineStr">
         <is>
@@ -3991,7 +3991,7 @@
         </is>
       </c>
       <c r="G86" s="2" t="n">
-        <v>0.66</v>
+        <v>0.85</v>
       </c>
       <c r="H86" s="2" t="inlineStr">
         <is>
@@ -4032,7 +4032,7 @@
         </is>
       </c>
       <c r="G87" s="2" t="n">
-        <v>0.45</v>
+        <v>0.98</v>
       </c>
       <c r="H87" s="2" t="inlineStr">
         <is>
@@ -4073,7 +4073,7 @@
         </is>
       </c>
       <c r="G88" s="2" t="n">
-        <v>0.78</v>
+        <v>1.08</v>
       </c>
       <c r="H88" s="2" t="inlineStr">
         <is>
@@ -4114,7 +4114,7 @@
         </is>
       </c>
       <c r="G89" s="2" t="n">
-        <v>0.73</v>
+        <v>0.61</v>
       </c>
       <c r="H89" s="2" t="inlineStr">
         <is>
@@ -4155,7 +4155,7 @@
         </is>
       </c>
       <c r="G90" s="2" t="n">
-        <v>1.1</v>
+        <v>0.52</v>
       </c>
       <c r="H90" s="2" t="inlineStr">
         <is>
@@ -4196,7 +4196,7 @@
         </is>
       </c>
       <c r="G91" s="2" t="n">
-        <v>0.91</v>
+        <v>0.78</v>
       </c>
       <c r="H91" s="2" t="inlineStr">
         <is>
@@ -4237,7 +4237,7 @@
         </is>
       </c>
       <c r="G92" s="2" t="n">
-        <v>0.87</v>
+        <v>1.06</v>
       </c>
       <c r="H92" s="2" t="inlineStr">
         <is>
@@ -4278,7 +4278,7 @@
         </is>
       </c>
       <c r="G93" s="2" t="n">
-        <v>0.84</v>
+        <v>0.46</v>
       </c>
       <c r="H93" s="2" t="inlineStr">
         <is>
@@ -4319,7 +4319,7 @@
         </is>
       </c>
       <c r="G94" s="2" t="n">
-        <v>0.45</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="H94" s="2" t="inlineStr">
         <is>
@@ -4360,7 +4360,7 @@
         </is>
       </c>
       <c r="G95" s="2" t="n">
-        <v>0.74</v>
+        <v>1.1</v>
       </c>
       <c r="H95" s="2" t="inlineStr">
         <is>
@@ -4401,7 +4401,7 @@
         </is>
       </c>
       <c r="G96" s="2" t="n">
-        <v>0.87</v>
+        <v>0.66</v>
       </c>
       <c r="H96" s="2" t="inlineStr">
         <is>
@@ -4423,7 +4423,7 @@
       </c>
       <c r="C97" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #1 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.82s.</t>
+          <t>User taps Issuance form action button #1 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.6s.</t>
         </is>
       </c>
       <c r="D97" s="2" t="inlineStr">
@@ -4442,7 +4442,7 @@
         </is>
       </c>
       <c r="G97" s="2" t="n">
-        <v>0.82</v>
+        <v>0.6</v>
       </c>
       <c r="H97" s="2" t="inlineStr">
         <is>
@@ -4464,7 +4464,7 @@
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #2 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.81s.</t>
+          <t>User taps Issuance form action button #2 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.5s.</t>
         </is>
       </c>
       <c r="D98" s="2" t="inlineStr">
@@ -4483,7 +4483,7 @@
         </is>
       </c>
       <c r="G98" s="2" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.5</v>
       </c>
       <c r="H98" s="2" t="inlineStr">
         <is>
@@ -4505,7 +4505,7 @@
       </c>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #3 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.71s.</t>
+          <t>User taps Issuance form action button #3 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.77s.</t>
         </is>
       </c>
       <c r="D99" s="2" t="inlineStr">
@@ -4524,7 +4524,7 @@
         </is>
       </c>
       <c r="G99" s="2" t="n">
-        <v>0.71</v>
+        <v>0.77</v>
       </c>
       <c r="H99" s="2" t="inlineStr">
         <is>
@@ -4546,7 +4546,7 @@
       </c>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #4 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.63s.</t>
+          <t>User taps Issuance form action button #4 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.68s.</t>
         </is>
       </c>
       <c r="D100" s="2" t="inlineStr">
@@ -4565,7 +4565,7 @@
         </is>
       </c>
       <c r="G100" s="2" t="n">
-        <v>0.63</v>
+        <v>0.68</v>
       </c>
       <c r="H100" s="2" t="inlineStr">
         <is>
@@ -4587,7 +4587,7 @@
       </c>
       <c r="C101" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #5 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.48s.</t>
+          <t>User taps Issuance form action button #5 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.41s.</t>
         </is>
       </c>
       <c r="D101" s="2" t="inlineStr">
@@ -4606,7 +4606,7 @@
         </is>
       </c>
       <c r="G101" s="2" t="n">
-        <v>0.48</v>
+        <v>0.41</v>
       </c>
       <c r="H101" s="2" t="inlineStr">
         <is>
@@ -4628,7 +4628,7 @@
       </c>
       <c r="C102" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #6 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.45s.</t>
+          <t>User taps Issuance form action button #6 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 1.1s.</t>
         </is>
       </c>
       <c r="D102" s="2" t="inlineStr">
@@ -4647,7 +4647,7 @@
         </is>
       </c>
       <c r="G102" s="2" t="n">
-        <v>0.45</v>
+        <v>1.1</v>
       </c>
       <c r="H102" s="2" t="inlineStr">
         <is>
@@ -4669,7 +4669,7 @@
       </c>
       <c r="C103" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #7 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.94s.</t>
+          <t>User taps Issuance form action button #7 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.99s.</t>
         </is>
       </c>
       <c r="D103" s="2" t="inlineStr">
@@ -4688,7 +4688,7 @@
         </is>
       </c>
       <c r="G103" s="2" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.99</v>
       </c>
       <c r="H103" s="2" t="inlineStr">
         <is>
@@ -4710,7 +4710,7 @@
       </c>
       <c r="C104" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #8 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.97s.</t>
+          <t>User taps Issuance form action button #8 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.75s.</t>
         </is>
       </c>
       <c r="D104" s="2" t="inlineStr">
@@ -4729,7 +4729,7 @@
         </is>
       </c>
       <c r="G104" s="2" t="n">
-        <v>0.97</v>
+        <v>0.75</v>
       </c>
       <c r="H104" s="2" t="inlineStr">
         <is>
@@ -4751,7 +4751,7 @@
       </c>
       <c r="C105" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #9 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.44s.</t>
+          <t>User taps Issuance form action button #9 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.75s.</t>
         </is>
       </c>
       <c r="D105" s="2" t="inlineStr">
@@ -4770,7 +4770,7 @@
         </is>
       </c>
       <c r="G105" s="2" t="n">
-        <v>0.44</v>
+        <v>0.75</v>
       </c>
       <c r="H105" s="2" t="inlineStr">
         <is>
@@ -4792,7 +4792,7 @@
       </c>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #10 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.52s.</t>
+          <t>User taps Issuance form action button #10 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.78s.</t>
         </is>
       </c>
       <c r="D106" s="2" t="inlineStr">
@@ -4811,7 +4811,7 @@
         </is>
       </c>
       <c r="G106" s="2" t="n">
-        <v>0.52</v>
+        <v>0.78</v>
       </c>
       <c r="H106" s="2" t="inlineStr">
         <is>
@@ -4833,7 +4833,7 @@
       </c>
       <c r="C107" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #11 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.43s.</t>
+          <t>User taps Issuance form action button #11 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.45s.</t>
         </is>
       </c>
       <c r="D107" s="2" t="inlineStr">
@@ -4852,7 +4852,7 @@
         </is>
       </c>
       <c r="G107" s="2" t="n">
-        <v>0.43</v>
+        <v>0.45</v>
       </c>
       <c r="H107" s="2" t="inlineStr">
         <is>
@@ -4874,7 +4874,7 @@
       </c>
       <c r="C108" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #12 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.93s.</t>
+          <t>User taps Issuance form action button #12 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.62s.</t>
         </is>
       </c>
       <c r="D108" s="2" t="inlineStr">
@@ -4893,7 +4893,7 @@
         </is>
       </c>
       <c r="G108" s="2" t="n">
-        <v>0.93</v>
+        <v>0.62</v>
       </c>
       <c r="H108" s="2" t="inlineStr">
         <is>
@@ -4915,7 +4915,7 @@
       </c>
       <c r="C109" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #13 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 1.09s.</t>
+          <t>User taps Issuance form action button #13 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 1.04s.</t>
         </is>
       </c>
       <c r="D109" s="2" t="inlineStr">
@@ -4934,7 +4934,7 @@
         </is>
       </c>
       <c r="G109" s="2" t="n">
-        <v>1.09</v>
+        <v>1.04</v>
       </c>
       <c r="H109" s="2" t="inlineStr">
         <is>
@@ -4956,7 +4956,7 @@
       </c>
       <c r="C110" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #14 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.83s.</t>
+          <t>User taps Issuance form action button #14 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 1.05s.</t>
         </is>
       </c>
       <c r="D110" s="2" t="inlineStr">
@@ -4975,7 +4975,7 @@
         </is>
       </c>
       <c r="G110" s="2" t="n">
-        <v>0.83</v>
+        <v>1.05</v>
       </c>
       <c r="H110" s="2" t="inlineStr">
         <is>
@@ -4997,7 +4997,7 @@
       </c>
       <c r="C111" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #15 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.84s.</t>
+          <t>User taps Issuance form action button #15 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.53s.</t>
         </is>
       </c>
       <c r="D111" s="2" t="inlineStr">
@@ -5016,7 +5016,7 @@
         </is>
       </c>
       <c r="G111" s="2" t="n">
-        <v>0.84</v>
+        <v>0.53</v>
       </c>
       <c r="H111" s="2" t="inlineStr">
         <is>
@@ -5038,7 +5038,7 @@
       </c>
       <c r="C112" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #16 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.78s.</t>
+          <t>User taps Issuance form action button #16 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.71s.</t>
         </is>
       </c>
       <c r="D112" s="2" t="inlineStr">
@@ -5057,7 +5057,7 @@
         </is>
       </c>
       <c r="G112" s="2" t="n">
-        <v>0.78</v>
+        <v>0.71</v>
       </c>
       <c r="H112" s="2" t="inlineStr">
         <is>
@@ -5079,7 +5079,7 @@
       </c>
       <c r="C113" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #17 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.7s.</t>
+          <t>User taps Issuance form action button #17 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.69s.</t>
         </is>
       </c>
       <c r="D113" s="2" t="inlineStr">
@@ -5098,7 +5098,7 @@
         </is>
       </c>
       <c r="G113" s="2" t="n">
-        <v>0.7</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="H113" s="2" t="inlineStr">
         <is>
@@ -5120,7 +5120,7 @@
       </c>
       <c r="C114" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #18 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 1.1s.</t>
+          <t>User taps Issuance form action button #18 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.45s.</t>
         </is>
       </c>
       <c r="D114" s="2" t="inlineStr">
@@ -5139,7 +5139,7 @@
         </is>
       </c>
       <c r="G114" s="2" t="n">
-        <v>1.1</v>
+        <v>0.45</v>
       </c>
       <c r="H114" s="2" t="inlineStr">
         <is>
@@ -5161,7 +5161,7 @@
       </c>
       <c r="C115" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #19 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.66s.</t>
+          <t>User taps Issuance form action button #19 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 1.11s.</t>
         </is>
       </c>
       <c r="D115" s="2" t="inlineStr">
@@ -5180,7 +5180,7 @@
         </is>
       </c>
       <c r="G115" s="2" t="n">
-        <v>0.66</v>
+        <v>1.11</v>
       </c>
       <c r="H115" s="2" t="inlineStr">
         <is>
@@ -5202,7 +5202,7 @@
       </c>
       <c r="C116" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #20 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 1.0s.</t>
+          <t>User taps Issuance form action button #20 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.87s.</t>
         </is>
       </c>
       <c r="D116" s="2" t="inlineStr">
@@ -5221,7 +5221,7 @@
         </is>
       </c>
       <c r="G116" s="2" t="n">
-        <v>1</v>
+        <v>0.87</v>
       </c>
       <c r="H116" s="2" t="inlineStr">
         <is>
@@ -5243,7 +5243,7 @@
       </c>
       <c r="C117" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #21 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 1.05s.</t>
+          <t>User taps Issuance form action button #21 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.7s.</t>
         </is>
       </c>
       <c r="D117" s="2" t="inlineStr">
@@ -5262,7 +5262,7 @@
         </is>
       </c>
       <c r="G117" s="2" t="n">
-        <v>1.05</v>
+        <v>0.7</v>
       </c>
       <c r="H117" s="2" t="inlineStr">
         <is>
@@ -5284,7 +5284,7 @@
       </c>
       <c r="C118" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #22 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.55s.</t>
+          <t>User taps Issuance form action button #22 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.6s.</t>
         </is>
       </c>
       <c r="D118" s="2" t="inlineStr">
@@ -5303,7 +5303,7 @@
         </is>
       </c>
       <c r="G118" s="2" t="n">
-        <v>0.55</v>
+        <v>0.6</v>
       </c>
       <c r="H118" s="2" t="inlineStr">
         <is>
@@ -5325,7 +5325,7 @@
       </c>
       <c r="C119" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #23 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.48s.</t>
+          <t>User taps Issuance form action button #23 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 1.06s.</t>
         </is>
       </c>
       <c r="D119" s="2" t="inlineStr">
@@ -5344,7 +5344,7 @@
         </is>
       </c>
       <c r="G119" s="2" t="n">
-        <v>0.48</v>
+        <v>1.06</v>
       </c>
       <c r="H119" s="2" t="inlineStr">
         <is>
@@ -5366,7 +5366,7 @@
       </c>
       <c r="C120" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #24 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.4s.</t>
+          <t>User taps Issuance form action button #24 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.42s.</t>
         </is>
       </c>
       <c r="D120" s="2" t="inlineStr">
@@ -5385,7 +5385,7 @@
         </is>
       </c>
       <c r="G120" s="2" t="n">
-        <v>0.4</v>
+        <v>0.42</v>
       </c>
       <c r="H120" s="2" t="inlineStr">
         <is>
@@ -5407,7 +5407,7 @@
       </c>
       <c r="C121" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #25 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 1.02s.</t>
+          <t>User taps Issuance form action button #25 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.83s.</t>
         </is>
       </c>
       <c r="D121" s="2" t="inlineStr">
@@ -5426,7 +5426,7 @@
         </is>
       </c>
       <c r="G121" s="2" t="n">
-        <v>1.02</v>
+        <v>0.83</v>
       </c>
       <c r="H121" s="2" t="inlineStr">
         <is>
@@ -5467,7 +5467,7 @@
         </is>
       </c>
       <c r="G122" s="2" t="n">
-        <v>0.75</v>
+        <v>0.59</v>
       </c>
       <c r="H122" s="2" t="inlineStr">
         <is>
@@ -5508,7 +5508,7 @@
         </is>
       </c>
       <c r="G123" s="2" t="n">
-        <v>0.61</v>
+        <v>0.85</v>
       </c>
       <c r="H123" s="2" t="inlineStr">
         <is>
@@ -5549,7 +5549,7 @@
         </is>
       </c>
       <c r="G124" s="2" t="n">
-        <v>0.37</v>
+        <v>0.4</v>
       </c>
       <c r="H124" s="2" t="inlineStr">
         <is>
@@ -5590,7 +5590,7 @@
         </is>
       </c>
       <c r="G125" s="2" t="n">
-        <v>0.44</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="H125" s="2" t="inlineStr">
         <is>
@@ -5631,7 +5631,7 @@
         </is>
       </c>
       <c r="G126" s="2" t="n">
-        <v>0.83</v>
+        <v>0.64</v>
       </c>
       <c r="H126" s="2" t="inlineStr">
         <is>
@@ -5672,7 +5672,7 @@
         </is>
       </c>
       <c r="G127" s="2" t="n">
-        <v>0.44</v>
+        <v>0.4</v>
       </c>
       <c r="H127" s="2" t="inlineStr">
         <is>
@@ -5713,7 +5713,7 @@
         </is>
       </c>
       <c r="G128" s="2" t="n">
-        <v>0.82</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="H128" s="2" t="inlineStr">
         <is>
@@ -5754,7 +5754,7 @@
         </is>
       </c>
       <c r="G129" s="2" t="n">
-        <v>0.5</v>
+        <v>0.43</v>
       </c>
       <c r="H129" s="2" t="inlineStr">
         <is>
@@ -5795,7 +5795,7 @@
         </is>
       </c>
       <c r="G130" s="2" t="n">
-        <v>0.62</v>
+        <v>0.34</v>
       </c>
       <c r="H130" s="2" t="inlineStr">
         <is>
@@ -5836,7 +5836,7 @@
         </is>
       </c>
       <c r="G131" s="2" t="n">
-        <v>0.4</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="H131" s="2" t="inlineStr">
         <is>
@@ -5858,7 +5858,7 @@
       </c>
       <c r="C132" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #1 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.48s.</t>
+          <t>User taps Registry interactive card/button #1 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.67s.</t>
         </is>
       </c>
       <c r="D132" s="2" t="inlineStr">
@@ -5877,7 +5877,7 @@
         </is>
       </c>
       <c r="G132" s="2" t="n">
-        <v>0.48</v>
+        <v>0.67</v>
       </c>
       <c r="H132" s="2" t="inlineStr">
         <is>
@@ -5899,7 +5899,7 @@
       </c>
       <c r="C133" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #2 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.76s.</t>
+          <t>User taps Registry interactive card/button #2 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.53s.</t>
         </is>
       </c>
       <c r="D133" s="2" t="inlineStr">
@@ -5918,7 +5918,7 @@
         </is>
       </c>
       <c r="G133" s="2" t="n">
-        <v>0.76</v>
+        <v>0.53</v>
       </c>
       <c r="H133" s="2" t="inlineStr">
         <is>
@@ -5940,7 +5940,7 @@
       </c>
       <c r="C134" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #3 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.56s.</t>
+          <t>User taps Registry interactive card/button #3 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.4s.</t>
         </is>
       </c>
       <c r="D134" s="2" t="inlineStr">
@@ -5959,7 +5959,7 @@
         </is>
       </c>
       <c r="G134" s="2" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.4</v>
       </c>
       <c r="H134" s="2" t="inlineStr">
         <is>
@@ -5981,7 +5981,7 @@
       </c>
       <c r="C135" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #4 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.33s.</t>
+          <t>User taps Registry interactive card/button #4 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.69s.</t>
         </is>
       </c>
       <c r="D135" s="2" t="inlineStr">
@@ -6000,7 +6000,7 @@
         </is>
       </c>
       <c r="G135" s="2" t="n">
-        <v>0.33</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="H135" s="2" t="inlineStr">
         <is>
@@ -6022,7 +6022,7 @@
       </c>
       <c r="C136" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #5 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.47s.</t>
+          <t>User taps Registry interactive card/button #5 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.42s.</t>
         </is>
       </c>
       <c r="D136" s="2" t="inlineStr">
@@ -6041,7 +6041,7 @@
         </is>
       </c>
       <c r="G136" s="2" t="n">
-        <v>0.47</v>
+        <v>0.42</v>
       </c>
       <c r="H136" s="2" t="inlineStr">
         <is>
@@ -6063,7 +6063,7 @@
       </c>
       <c r="C137" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #6 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.77s.</t>
+          <t>User taps Registry interactive card/button #6 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.66s.</t>
         </is>
       </c>
       <c r="D137" s="2" t="inlineStr">
@@ -6082,7 +6082,7 @@
         </is>
       </c>
       <c r="G137" s="2" t="n">
-        <v>0.77</v>
+        <v>0.66</v>
       </c>
       <c r="H137" s="2" t="inlineStr">
         <is>
@@ -6104,7 +6104,7 @@
       </c>
       <c r="C138" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #7 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.64s.</t>
+          <t>User taps Registry interactive card/button #7 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.58s.</t>
         </is>
       </c>
       <c r="D138" s="2" t="inlineStr">
@@ -6123,7 +6123,7 @@
         </is>
       </c>
       <c r="G138" s="2" t="n">
-        <v>0.64</v>
+        <v>0.58</v>
       </c>
       <c r="H138" s="2" t="inlineStr">
         <is>
@@ -6145,7 +6145,7 @@
       </c>
       <c r="C139" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #8 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.76s.</t>
+          <t>User taps Registry interactive card/button #8 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.36s.</t>
         </is>
       </c>
       <c r="D139" s="2" t="inlineStr">
@@ -6164,7 +6164,7 @@
         </is>
       </c>
       <c r="G139" s="2" t="n">
-        <v>0.76</v>
+        <v>0.36</v>
       </c>
       <c r="H139" s="2" t="inlineStr">
         <is>
@@ -6186,7 +6186,7 @@
       </c>
       <c r="C140" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #9 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.36s.</t>
+          <t>User taps Registry interactive card/button #9 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.6s.</t>
         </is>
       </c>
       <c r="D140" s="2" t="inlineStr">
@@ -6205,7 +6205,7 @@
         </is>
       </c>
       <c r="G140" s="2" t="n">
-        <v>0.36</v>
+        <v>0.6</v>
       </c>
       <c r="H140" s="2" t="inlineStr">
         <is>
@@ -6227,7 +6227,7 @@
       </c>
       <c r="C141" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #10 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.79s.</t>
+          <t>User taps Registry interactive card/button #10 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.6s.</t>
         </is>
       </c>
       <c r="D141" s="2" t="inlineStr">
@@ -6246,7 +6246,7 @@
         </is>
       </c>
       <c r="G141" s="2" t="n">
-        <v>0.79</v>
+        <v>0.6</v>
       </c>
       <c r="H141" s="2" t="inlineStr">
         <is>
@@ -6268,7 +6268,7 @@
       </c>
       <c r="C142" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #11 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.42s.</t>
+          <t>User taps Registry interactive card/button #11 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.53s.</t>
         </is>
       </c>
       <c r="D142" s="2" t="inlineStr">
@@ -6287,7 +6287,7 @@
         </is>
       </c>
       <c r="G142" s="2" t="n">
-        <v>0.42</v>
+        <v>0.53</v>
       </c>
       <c r="H142" s="2" t="inlineStr">
         <is>
@@ -6350,7 +6350,7 @@
       </c>
       <c r="C144" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #13 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.69s.</t>
+          <t>User taps Registry interactive card/button #13 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.51s.</t>
         </is>
       </c>
       <c r="D144" s="2" t="inlineStr">
@@ -6369,7 +6369,7 @@
         </is>
       </c>
       <c r="G144" s="2" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.51</v>
       </c>
       <c r="H144" s="2" t="inlineStr">
         <is>
@@ -6391,7 +6391,7 @@
       </c>
       <c r="C145" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #14 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.68s.</t>
+          <t>User taps Registry interactive card/button #14 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.46s.</t>
         </is>
       </c>
       <c r="D145" s="2" t="inlineStr">
@@ -6410,7 +6410,7 @@
         </is>
       </c>
       <c r="G145" s="2" t="n">
-        <v>0.68</v>
+        <v>0.46</v>
       </c>
       <c r="H145" s="2" t="inlineStr">
         <is>
@@ -6432,7 +6432,7 @@
       </c>
       <c r="C146" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #15 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.82s.</t>
+          <t>User taps Registry interactive card/button #15 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.65s.</t>
         </is>
       </c>
       <c r="D146" s="2" t="inlineStr">
@@ -6451,7 +6451,7 @@
         </is>
       </c>
       <c r="G146" s="2" t="n">
-        <v>0.82</v>
+        <v>0.65</v>
       </c>
       <c r="H146" s="2" t="inlineStr">
         <is>
@@ -6473,7 +6473,7 @@
       </c>
       <c r="C147" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #16 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.38s.</t>
+          <t>User taps Registry interactive card/button #16 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.53s.</t>
         </is>
       </c>
       <c r="D147" s="2" t="inlineStr">
@@ -6492,7 +6492,7 @@
         </is>
       </c>
       <c r="G147" s="2" t="n">
-        <v>0.38</v>
+        <v>0.53</v>
       </c>
       <c r="H147" s="2" t="inlineStr">
         <is>
@@ -6514,7 +6514,7 @@
       </c>
       <c r="C148" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #17 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.78s.</t>
+          <t>User taps Registry interactive card/button #17 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.32s.</t>
         </is>
       </c>
       <c r="D148" s="2" t="inlineStr">
@@ -6533,7 +6533,7 @@
         </is>
       </c>
       <c r="G148" s="2" t="n">
-        <v>0.78</v>
+        <v>0.32</v>
       </c>
       <c r="H148" s="2" t="inlineStr">
         <is>
@@ -6555,7 +6555,7 @@
       </c>
       <c r="C149" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #18 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.44s.</t>
+          <t>User taps Registry interactive card/button #18 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.84s.</t>
         </is>
       </c>
       <c r="D149" s="2" t="inlineStr">
@@ -6574,7 +6574,7 @@
         </is>
       </c>
       <c r="G149" s="2" t="n">
-        <v>0.44</v>
+        <v>0.84</v>
       </c>
       <c r="H149" s="2" t="inlineStr">
         <is>
@@ -6596,7 +6596,7 @@
       </c>
       <c r="C150" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #19 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.67s.</t>
+          <t>User taps Registry interactive card/button #19 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.68s.</t>
         </is>
       </c>
       <c r="D150" s="2" t="inlineStr">
@@ -6615,7 +6615,7 @@
         </is>
       </c>
       <c r="G150" s="2" t="n">
-        <v>0.67</v>
+        <v>0.68</v>
       </c>
       <c r="H150" s="2" t="inlineStr">
         <is>
@@ -6637,7 +6637,7 @@
       </c>
       <c r="C151" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #20 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.58s.</t>
+          <t>User taps Registry interactive card/button #20 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.79s.</t>
         </is>
       </c>
       <c r="D151" s="2" t="inlineStr">
@@ -6656,7 +6656,7 @@
         </is>
       </c>
       <c r="G151" s="2" t="n">
-        <v>0.58</v>
+        <v>0.79</v>
       </c>
       <c r="H151" s="2" t="inlineStr">
         <is>
@@ -6678,7 +6678,7 @@
       </c>
       <c r="C152" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #21 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.39s.</t>
+          <t>User taps Registry interactive card/button #21 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.46s.</t>
         </is>
       </c>
       <c r="D152" s="2" t="inlineStr">
@@ -6697,7 +6697,7 @@
         </is>
       </c>
       <c r="G152" s="2" t="n">
-        <v>0.39</v>
+        <v>0.46</v>
       </c>
       <c r="H152" s="2" t="inlineStr">
         <is>
@@ -6719,7 +6719,7 @@
       </c>
       <c r="C153" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #22 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.35s.</t>
+          <t>User taps Registry interactive card/button #22 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.82s.</t>
         </is>
       </c>
       <c r="D153" s="2" t="inlineStr">
@@ -6738,7 +6738,7 @@
         </is>
       </c>
       <c r="G153" s="2" t="n">
-        <v>0.35</v>
+        <v>0.82</v>
       </c>
       <c r="H153" s="2" t="inlineStr">
         <is>
@@ -6760,7 +6760,7 @@
       </c>
       <c r="C154" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #23 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.39s.</t>
+          <t>User taps Registry interactive card/button #23 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.83s.</t>
         </is>
       </c>
       <c r="D154" s="2" t="inlineStr">
@@ -6779,7 +6779,7 @@
         </is>
       </c>
       <c r="G154" s="2" t="n">
-        <v>0.39</v>
+        <v>0.83</v>
       </c>
       <c r="H154" s="2" t="inlineStr">
         <is>
@@ -6801,7 +6801,7 @@
       </c>
       <c r="C155" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #24 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.55s.</t>
+          <t>User taps Registry interactive card/button #24 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.69s.</t>
         </is>
       </c>
       <c r="D155" s="2" t="inlineStr">
@@ -6820,7 +6820,7 @@
         </is>
       </c>
       <c r="G155" s="2" t="n">
-        <v>0.55</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="H155" s="2" t="inlineStr">
         <is>
@@ -6842,7 +6842,7 @@
       </c>
       <c r="C156" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #25 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.63s.</t>
+          <t>User taps Registry interactive card/button #25 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.39s.</t>
         </is>
       </c>
       <c r="D156" s="2" t="inlineStr">
@@ -6861,7 +6861,7 @@
         </is>
       </c>
       <c r="G156" s="2" t="n">
-        <v>0.63</v>
+        <v>0.39</v>
       </c>
       <c r="H156" s="2" t="inlineStr">
         <is>
@@ -6883,7 +6883,7 @@
       </c>
       <c r="C157" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #26 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.45s.</t>
+          <t>User taps Registry interactive card/button #26 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.32s.</t>
         </is>
       </c>
       <c r="D157" s="2" t="inlineStr">
@@ -6902,7 +6902,7 @@
         </is>
       </c>
       <c r="G157" s="2" t="n">
-        <v>0.45</v>
+        <v>0.32</v>
       </c>
       <c r="H157" s="2" t="inlineStr">
         <is>
@@ -6924,7 +6924,7 @@
       </c>
       <c r="C158" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #27 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.53s.</t>
+          <t>User taps Registry interactive card/button #27 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.83s.</t>
         </is>
       </c>
       <c r="D158" s="2" t="inlineStr">
@@ -6943,7 +6943,7 @@
         </is>
       </c>
       <c r="G158" s="2" t="n">
-        <v>0.53</v>
+        <v>0.83</v>
       </c>
       <c r="H158" s="2" t="inlineStr">
         <is>
@@ -6965,7 +6965,7 @@
       </c>
       <c r="C159" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #28 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.85s.</t>
+          <t>User taps Registry interactive card/button #28 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.32s.</t>
         </is>
       </c>
       <c r="D159" s="2" t="inlineStr">
@@ -6984,7 +6984,7 @@
         </is>
       </c>
       <c r="G159" s="2" t="n">
-        <v>0.85</v>
+        <v>0.32</v>
       </c>
       <c r="H159" s="2" t="inlineStr">
         <is>
@@ -7006,7 +7006,7 @@
       </c>
       <c r="C160" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #29 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.73s.</t>
+          <t>User taps Registry interactive card/button #29 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.51s.</t>
         </is>
       </c>
       <c r="D160" s="2" t="inlineStr">
@@ -7025,7 +7025,7 @@
         </is>
       </c>
       <c r="G160" s="2" t="n">
-        <v>0.73</v>
+        <v>0.51</v>
       </c>
       <c r="H160" s="2" t="inlineStr">
         <is>
@@ -7047,7 +7047,7 @@
       </c>
       <c r="C161" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #30 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.75s.</t>
+          <t>User taps Registry interactive card/button #30 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.32s.</t>
         </is>
       </c>
       <c r="D161" s="2" t="inlineStr">
@@ -7066,7 +7066,7 @@
         </is>
       </c>
       <c r="G161" s="2" t="n">
-        <v>0.75</v>
+        <v>0.32</v>
       </c>
       <c r="H161" s="2" t="inlineStr">
         <is>
@@ -7107,7 +7107,7 @@
         </is>
       </c>
       <c r="G162" s="2" t="n">
-        <v>0.76</v>
+        <v>0.67</v>
       </c>
       <c r="H162" s="2" t="inlineStr">
         <is>
@@ -7148,7 +7148,7 @@
         </is>
       </c>
       <c r="G163" s="2" t="n">
-        <v>0.52</v>
+        <v>0.53</v>
       </c>
       <c r="H163" s="2" t="inlineStr">
         <is>
@@ -7189,7 +7189,7 @@
         </is>
       </c>
       <c r="G164" s="2" t="n">
-        <v>0.51</v>
+        <v>0.43</v>
       </c>
       <c r="H164" s="2" t="inlineStr">
         <is>
@@ -7230,7 +7230,7 @@
         </is>
       </c>
       <c r="G165" s="2" t="n">
-        <v>0.74</v>
+        <v>0.48</v>
       </c>
       <c r="H165" s="2" t="inlineStr">
         <is>
@@ -7293,7 +7293,7 @@
       </c>
       <c r="C167" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #1 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.77s.</t>
+          <t>User taps Network diagnostic button #1 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.64s.</t>
         </is>
       </c>
       <c r="D167" s="2" t="inlineStr">
@@ -7312,7 +7312,7 @@
         </is>
       </c>
       <c r="G167" s="2" t="n">
-        <v>0.77</v>
+        <v>0.64</v>
       </c>
       <c r="H167" s="2" t="inlineStr">
         <is>
@@ -7334,7 +7334,7 @@
       </c>
       <c r="C168" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #2 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.51s.</t>
+          <t>User taps Network diagnostic button #2 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.78s.</t>
         </is>
       </c>
       <c r="D168" s="2" t="inlineStr">
@@ -7353,7 +7353,7 @@
         </is>
       </c>
       <c r="G168" s="2" t="n">
-        <v>0.51</v>
+        <v>0.78</v>
       </c>
       <c r="H168" s="2" t="inlineStr">
         <is>
@@ -7375,7 +7375,7 @@
       </c>
       <c r="C169" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #3 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.48s.</t>
+          <t>User taps Network diagnostic button #3 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.66s.</t>
         </is>
       </c>
       <c r="D169" s="2" t="inlineStr">
@@ -7394,7 +7394,7 @@
         </is>
       </c>
       <c r="G169" s="2" t="n">
-        <v>0.48</v>
+        <v>0.66</v>
       </c>
       <c r="H169" s="2" t="inlineStr">
         <is>
@@ -7416,7 +7416,7 @@
       </c>
       <c r="C170" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #4 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.43s.</t>
+          <t>User taps Network diagnostic button #4 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.38s.</t>
         </is>
       </c>
       <c r="D170" s="2" t="inlineStr">
@@ -7435,7 +7435,7 @@
         </is>
       </c>
       <c r="G170" s="2" t="n">
-        <v>0.43</v>
+        <v>0.38</v>
       </c>
       <c r="H170" s="2" t="inlineStr">
         <is>
@@ -7457,7 +7457,7 @@
       </c>
       <c r="C171" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #5 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.52s.</t>
+          <t>User taps Network diagnostic button #5 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.62s.</t>
         </is>
       </c>
       <c r="D171" s="2" t="inlineStr">
@@ -7476,7 +7476,7 @@
         </is>
       </c>
       <c r="G171" s="2" t="n">
-        <v>0.52</v>
+        <v>0.62</v>
       </c>
       <c r="H171" s="2" t="inlineStr">
         <is>
@@ -7498,7 +7498,7 @@
       </c>
       <c r="C172" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #6 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.47s.</t>
+          <t>User taps Network diagnostic button #6 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.41s.</t>
         </is>
       </c>
       <c r="D172" s="2" t="inlineStr">
@@ -7517,7 +7517,7 @@
         </is>
       </c>
       <c r="G172" s="2" t="n">
-        <v>0.47</v>
+        <v>0.41</v>
       </c>
       <c r="H172" s="2" t="inlineStr">
         <is>
@@ -7539,7 +7539,7 @@
       </c>
       <c r="C173" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #7 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.42s.</t>
+          <t>User taps Network diagnostic button #7 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.73s.</t>
         </is>
       </c>
       <c r="D173" s="2" t="inlineStr">
@@ -7558,7 +7558,7 @@
         </is>
       </c>
       <c r="G173" s="2" t="n">
-        <v>0.42</v>
+        <v>0.73</v>
       </c>
       <c r="H173" s="2" t="inlineStr">
         <is>
@@ -7580,7 +7580,7 @@
       </c>
       <c r="C174" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #8 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.58s.</t>
+          <t>User taps Network diagnostic button #8 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.47s.</t>
         </is>
       </c>
       <c r="D174" s="2" t="inlineStr">
@@ -7599,7 +7599,7 @@
         </is>
       </c>
       <c r="G174" s="2" t="n">
-        <v>0.58</v>
+        <v>0.47</v>
       </c>
       <c r="H174" s="2" t="inlineStr">
         <is>
@@ -7621,7 +7621,7 @@
       </c>
       <c r="C175" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #9 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.35s.</t>
+          <t>User taps Network diagnostic button #9 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.67s.</t>
         </is>
       </c>
       <c r="D175" s="2" t="inlineStr">
@@ -7640,7 +7640,7 @@
         </is>
       </c>
       <c r="G175" s="2" t="n">
-        <v>0.35</v>
+        <v>0.67</v>
       </c>
       <c r="H175" s="2" t="inlineStr">
         <is>
@@ -7662,7 +7662,7 @@
       </c>
       <c r="C176" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #10 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.35s.</t>
+          <t>User taps Network diagnostic button #10 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.57s.</t>
         </is>
       </c>
       <c r="D176" s="2" t="inlineStr">
@@ -7681,7 +7681,7 @@
         </is>
       </c>
       <c r="G176" s="2" t="n">
-        <v>0.35</v>
+        <v>0.57</v>
       </c>
       <c r="H176" s="2" t="inlineStr">
         <is>
@@ -7744,7 +7744,7 @@
       </c>
       <c r="C178" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #12 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.41s.</t>
+          <t>User taps Network diagnostic button #12 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.56s.</t>
         </is>
       </c>
       <c r="D178" s="2" t="inlineStr">
@@ -7763,7 +7763,7 @@
         </is>
       </c>
       <c r="G178" s="2" t="n">
-        <v>0.41</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="H178" s="2" t="inlineStr">
         <is>
@@ -7785,7 +7785,7 @@
       </c>
       <c r="C179" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #13 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.47s.</t>
+          <t>User taps Network diagnostic button #13 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.38s.</t>
         </is>
       </c>
       <c r="D179" s="2" t="inlineStr">
@@ -7804,7 +7804,7 @@
         </is>
       </c>
       <c r="G179" s="2" t="n">
-        <v>0.47</v>
+        <v>0.38</v>
       </c>
       <c r="H179" s="2" t="inlineStr">
         <is>
@@ -7826,7 +7826,7 @@
       </c>
       <c r="C180" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #14 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.4s.</t>
+          <t>User taps Network diagnostic button #14 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.52s.</t>
         </is>
       </c>
       <c r="D180" s="2" t="inlineStr">
@@ -7845,7 +7845,7 @@
         </is>
       </c>
       <c r="G180" s="2" t="n">
-        <v>0.4</v>
+        <v>0.52</v>
       </c>
       <c r="H180" s="2" t="inlineStr">
         <is>
@@ -7867,7 +7867,7 @@
       </c>
       <c r="C181" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #15 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.43s.</t>
+          <t>User taps Network diagnostic button #15 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.6s.</t>
         </is>
       </c>
       <c r="D181" s="2" t="inlineStr">
@@ -7886,7 +7886,7 @@
         </is>
       </c>
       <c r="G181" s="2" t="n">
-        <v>0.43</v>
+        <v>0.6</v>
       </c>
       <c r="H181" s="2" t="inlineStr">
         <is>
@@ -7908,7 +7908,7 @@
       </c>
       <c r="C182" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #16 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.61s.</t>
+          <t>User taps Network diagnostic button #16 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.59s.</t>
         </is>
       </c>
       <c r="D182" s="2" t="inlineStr">
@@ -7927,7 +7927,7 @@
         </is>
       </c>
       <c r="G182" s="2" t="n">
-        <v>0.61</v>
+        <v>0.59</v>
       </c>
       <c r="H182" s="2" t="inlineStr">
         <is>
@@ -7949,7 +7949,7 @@
       </c>
       <c r="C183" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #17 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.39s.</t>
+          <t>User taps Network diagnostic button #17 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.71s.</t>
         </is>
       </c>
       <c r="D183" s="2" t="inlineStr">
@@ -7968,7 +7968,7 @@
         </is>
       </c>
       <c r="G183" s="2" t="n">
-        <v>0.39</v>
+        <v>0.71</v>
       </c>
       <c r="H183" s="2" t="inlineStr">
         <is>
@@ -7990,7 +7990,7 @@
       </c>
       <c r="C184" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #18 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.77s.</t>
+          <t>User taps Network diagnostic button #18 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.78s.</t>
         </is>
       </c>
       <c r="D184" s="2" t="inlineStr">
@@ -8009,7 +8009,7 @@
         </is>
       </c>
       <c r="G184" s="2" t="n">
-        <v>0.77</v>
+        <v>0.78</v>
       </c>
       <c r="H184" s="2" t="inlineStr">
         <is>
@@ -8031,7 +8031,7 @@
       </c>
       <c r="C185" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #19 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.34s.</t>
+          <t>User taps Network diagnostic button #19 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.75s.</t>
         </is>
       </c>
       <c r="D185" s="2" t="inlineStr">
@@ -8050,7 +8050,7 @@
         </is>
       </c>
       <c r="G185" s="2" t="n">
-        <v>0.34</v>
+        <v>0.75</v>
       </c>
       <c r="H185" s="2" t="inlineStr">
         <is>
@@ -8072,7 +8072,7 @@
       </c>
       <c r="C186" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #20 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.41s.</t>
+          <t>User taps Network diagnostic button #20 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.28s.</t>
         </is>
       </c>
       <c r="D186" s="2" t="inlineStr">
@@ -8091,7 +8091,7 @@
         </is>
       </c>
       <c r="G186" s="2" t="n">
-        <v>0.41</v>
+        <v>0.28</v>
       </c>
       <c r="H186" s="2" t="inlineStr">
         <is>
@@ -8113,7 +8113,7 @@
       </c>
       <c r="C187" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #21 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.43s.</t>
+          <t>User taps Network diagnostic button #21 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.42s.</t>
         </is>
       </c>
       <c r="D187" s="2" t="inlineStr">
@@ -8132,7 +8132,7 @@
         </is>
       </c>
       <c r="G187" s="2" t="n">
-        <v>0.43</v>
+        <v>0.42</v>
       </c>
       <c r="H187" s="2" t="inlineStr">
         <is>
@@ -8154,7 +8154,7 @@
       </c>
       <c r="C188" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #22 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.47s.</t>
+          <t>User taps Network diagnostic button #22 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.34s.</t>
         </is>
       </c>
       <c r="D188" s="2" t="inlineStr">
@@ -8173,7 +8173,7 @@
         </is>
       </c>
       <c r="G188" s="2" t="n">
-        <v>0.47</v>
+        <v>0.34</v>
       </c>
       <c r="H188" s="2" t="inlineStr">
         <is>
@@ -8195,7 +8195,7 @@
       </c>
       <c r="C189" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #23 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.51s.</t>
+          <t>User taps Network diagnostic button #23 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.55s.</t>
         </is>
       </c>
       <c r="D189" s="2" t="inlineStr">
@@ -8214,7 +8214,7 @@
         </is>
       </c>
       <c r="G189" s="2" t="n">
-        <v>0.51</v>
+        <v>0.55</v>
       </c>
       <c r="H189" s="2" t="inlineStr">
         <is>
@@ -8236,7 +8236,7 @@
       </c>
       <c r="C190" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #24 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.77s.</t>
+          <t>User taps Network diagnostic button #24 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.45s.</t>
         </is>
       </c>
       <c r="D190" s="2" t="inlineStr">
@@ -8255,7 +8255,7 @@
         </is>
       </c>
       <c r="G190" s="2" t="n">
-        <v>0.77</v>
+        <v>0.45</v>
       </c>
       <c r="H190" s="2" t="inlineStr">
         <is>
@@ -8277,7 +8277,7 @@
       </c>
       <c r="C191" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #25 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.39s.</t>
+          <t>User taps Network diagnostic button #25 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.73s.</t>
         </is>
       </c>
       <c r="D191" s="2" t="inlineStr">
@@ -8296,7 +8296,7 @@
         </is>
       </c>
       <c r="G191" s="2" t="n">
-        <v>0.39</v>
+        <v>0.73</v>
       </c>
       <c r="H191" s="2" t="inlineStr">
         <is>
@@ -8318,7 +8318,7 @@
       </c>
       <c r="C192" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #26 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.77s.</t>
+          <t>User taps Network diagnostic button #26 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.44s.</t>
         </is>
       </c>
       <c r="D192" s="2" t="inlineStr">
@@ -8337,7 +8337,7 @@
         </is>
       </c>
       <c r="G192" s="2" t="n">
-        <v>0.77</v>
+        <v>0.44</v>
       </c>
       <c r="H192" s="2" t="inlineStr">
         <is>
@@ -8359,7 +8359,7 @@
       </c>
       <c r="C193" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #27 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.43s.</t>
+          <t>User taps Network diagnostic button #27 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.57s.</t>
         </is>
       </c>
       <c r="D193" s="2" t="inlineStr">
@@ -8378,7 +8378,7 @@
         </is>
       </c>
       <c r="G193" s="2" t="n">
-        <v>0.43</v>
+        <v>0.57</v>
       </c>
       <c r="H193" s="2" t="inlineStr">
         <is>
@@ -8400,7 +8400,7 @@
       </c>
       <c r="C194" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #28 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.48s.</t>
+          <t>User taps Network diagnostic button #28 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.47s.</t>
         </is>
       </c>
       <c r="D194" s="2" t="inlineStr">
@@ -8419,7 +8419,7 @@
         </is>
       </c>
       <c r="G194" s="2" t="n">
-        <v>0.48</v>
+        <v>0.47</v>
       </c>
       <c r="H194" s="2" t="inlineStr">
         <is>
@@ -8441,7 +8441,7 @@
       </c>
       <c r="C195" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #29 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.78s.</t>
+          <t>User taps Network diagnostic button #29 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.52s.</t>
         </is>
       </c>
       <c r="D195" s="2" t="inlineStr">
@@ -8460,7 +8460,7 @@
         </is>
       </c>
       <c r="G195" s="2" t="n">
-        <v>0.78</v>
+        <v>0.52</v>
       </c>
       <c r="H195" s="2" t="inlineStr">
         <is>
@@ -8482,7 +8482,7 @@
       </c>
       <c r="C196" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #30 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.77s.</t>
+          <t>User taps Network diagnostic button #30 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.63s.</t>
         </is>
       </c>
       <c r="D196" s="2" t="inlineStr">
@@ -8501,7 +8501,7 @@
         </is>
       </c>
       <c r="G196" s="2" t="n">
-        <v>0.77</v>
+        <v>0.63</v>
       </c>
       <c r="H196" s="2" t="inlineStr">
         <is>
@@ -8542,7 +8542,7 @@
         </is>
       </c>
       <c r="G197" s="2" t="n">
-        <v>0.51</v>
+        <v>0.88</v>
       </c>
       <c r="H197" s="2" t="inlineStr">
         <is>
@@ -8583,7 +8583,7 @@
         </is>
       </c>
       <c r="G198" s="2" t="n">
-        <v>0.64</v>
+        <v>0.59</v>
       </c>
       <c r="H198" s="2" t="inlineStr">
         <is>
@@ -8624,7 +8624,7 @@
         </is>
       </c>
       <c r="G199" s="2" t="n">
-        <v>1.17</v>
+        <v>0.5</v>
       </c>
       <c r="H199" s="2" t="inlineStr">
         <is>
@@ -8665,7 +8665,7 @@
         </is>
       </c>
       <c r="G200" s="2" t="n">
-        <v>0.74</v>
+        <v>0.8</v>
       </c>
       <c r="H200" s="2" t="inlineStr">
         <is>
@@ -8706,7 +8706,7 @@
         </is>
       </c>
       <c r="G201" s="2" t="n">
-        <v>0.6</v>
+        <v>0.86</v>
       </c>
       <c r="H201" s="2" t="inlineStr">
         <is>
@@ -8747,7 +8747,7 @@
         </is>
       </c>
       <c r="G202" s="2" t="n">
-        <v>0.92</v>
+        <v>0.76</v>
       </c>
       <c r="H202" s="2" t="inlineStr">
         <is>
@@ -8788,7 +8788,7 @@
         </is>
       </c>
       <c r="G203" s="2" t="n">
-        <v>0.66</v>
+        <v>1.13</v>
       </c>
       <c r="H203" s="2" t="inlineStr">
         <is>
@@ -8810,7 +8810,7 @@
       </c>
       <c r="C204" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #1 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.82s.</t>
+          <t>User executes touch gesture #1 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.85s.</t>
         </is>
       </c>
       <c r="D204" s="2" t="inlineStr">
@@ -8829,7 +8829,7 @@
         </is>
       </c>
       <c r="G204" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="H204" s="2" t="inlineStr">
         <is>
@@ -8851,7 +8851,7 @@
       </c>
       <c r="C205" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #2 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.38s.</t>
+          <t>User executes touch gesture #2 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.48s.</t>
         </is>
       </c>
       <c r="D205" s="2" t="inlineStr">
@@ -8870,7 +8870,7 @@
         </is>
       </c>
       <c r="G205" s="2" t="n">
-        <v>0.38</v>
+        <v>0.48</v>
       </c>
       <c r="H205" s="2" t="inlineStr">
         <is>
@@ -8892,7 +8892,7 @@
       </c>
       <c r="C206" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #3 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.85s.</t>
+          <t>User executes touch gesture #3 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.05s.</t>
         </is>
       </c>
       <c r="D206" s="2" t="inlineStr">
@@ -8911,7 +8911,7 @@
         </is>
       </c>
       <c r="G206" s="2" t="n">
-        <v>0.85</v>
+        <v>1.05</v>
       </c>
       <c r="H206" s="2" t="inlineStr">
         <is>
@@ -8933,7 +8933,7 @@
       </c>
       <c r="C207" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #4 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.47s.</t>
+          <t>User executes touch gesture #4 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.45s.</t>
         </is>
       </c>
       <c r="D207" s="2" t="inlineStr">
@@ -8952,7 +8952,7 @@
         </is>
       </c>
       <c r="G207" s="2" t="n">
-        <v>0.47</v>
+        <v>0.45</v>
       </c>
       <c r="H207" s="2" t="inlineStr">
         <is>
@@ -8974,7 +8974,7 @@
       </c>
       <c r="C208" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #5 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.62s.</t>
+          <t>User executes touch gesture #5 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.68s.</t>
         </is>
       </c>
       <c r="D208" s="2" t="inlineStr">
@@ -8993,7 +8993,7 @@
         </is>
       </c>
       <c r="G208" s="2" t="n">
-        <v>0.62</v>
+        <v>0.68</v>
       </c>
       <c r="H208" s="2" t="inlineStr">
         <is>
@@ -9015,7 +9015,7 @@
       </c>
       <c r="C209" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #6 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.15s.</t>
+          <t>User executes touch gesture #6 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.51s.</t>
         </is>
       </c>
       <c r="D209" s="2" t="inlineStr">
@@ -9034,7 +9034,7 @@
         </is>
       </c>
       <c r="G209" s="2" t="n">
-        <v>1.15</v>
+        <v>0.51</v>
       </c>
       <c r="H209" s="2" t="inlineStr">
         <is>
@@ -9056,7 +9056,7 @@
       </c>
       <c r="C210" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #7 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.96s.</t>
+          <t>User executes touch gesture #7 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.69s.</t>
         </is>
       </c>
       <c r="D210" s="2" t="inlineStr">
@@ -9075,7 +9075,7 @@
         </is>
       </c>
       <c r="G210" s="2" t="n">
-        <v>0.96</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="H210" s="2" t="inlineStr">
         <is>
@@ -9097,7 +9097,7 @@
       </c>
       <c r="C211" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #8 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.9s.</t>
+          <t>User executes touch gesture #8 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.42s.</t>
         </is>
       </c>
       <c r="D211" s="2" t="inlineStr">
@@ -9116,7 +9116,7 @@
         </is>
       </c>
       <c r="G211" s="2" t="n">
-        <v>0.9</v>
+        <v>0.42</v>
       </c>
       <c r="H211" s="2" t="inlineStr">
         <is>
@@ -9138,7 +9138,7 @@
       </c>
       <c r="C212" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #9 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.5s.</t>
+          <t>User executes touch gesture #9 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.63s.</t>
         </is>
       </c>
       <c r="D212" s="2" t="inlineStr">
@@ -9157,7 +9157,7 @@
         </is>
       </c>
       <c r="G212" s="2" t="n">
-        <v>0.5</v>
+        <v>0.63</v>
       </c>
       <c r="H212" s="2" t="inlineStr">
         <is>
@@ -9179,7 +9179,7 @@
       </c>
       <c r="C213" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #10 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.24s.</t>
+          <t>User executes touch gesture #10 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.46s.</t>
         </is>
       </c>
       <c r="D213" s="2" t="inlineStr">
@@ -9198,7 +9198,7 @@
         </is>
       </c>
       <c r="G213" s="2" t="n">
-        <v>1.24</v>
+        <v>0.46</v>
       </c>
       <c r="H213" s="2" t="inlineStr">
         <is>
@@ -9220,7 +9220,7 @@
       </c>
       <c r="C214" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #11 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.79s.</t>
+          <t>User executes touch gesture #11 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.42s.</t>
         </is>
       </c>
       <c r="D214" s="2" t="inlineStr">
@@ -9239,7 +9239,7 @@
         </is>
       </c>
       <c r="G214" s="2" t="n">
-        <v>0.79</v>
+        <v>0.42</v>
       </c>
       <c r="H214" s="2" t="inlineStr">
         <is>
@@ -9261,7 +9261,7 @@
       </c>
       <c r="C215" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #12 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.71s.</t>
+          <t>User executes touch gesture #12 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.09s.</t>
         </is>
       </c>
       <c r="D215" s="2" t="inlineStr">
@@ -9280,7 +9280,7 @@
         </is>
       </c>
       <c r="G215" s="2" t="n">
-        <v>0.71</v>
+        <v>1.09</v>
       </c>
       <c r="H215" s="2" t="inlineStr">
         <is>
@@ -9302,7 +9302,7 @@
       </c>
       <c r="C216" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #13 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.49s.</t>
+          <t>User executes touch gesture #13 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.24s.</t>
         </is>
       </c>
       <c r="D216" s="2" t="inlineStr">
@@ -9321,7 +9321,7 @@
         </is>
       </c>
       <c r="G216" s="2" t="n">
-        <v>0.49</v>
+        <v>1.24</v>
       </c>
       <c r="H216" s="2" t="inlineStr">
         <is>
@@ -9343,7 +9343,7 @@
       </c>
       <c r="C217" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #14 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.13s.</t>
+          <t>User executes touch gesture #14 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.93s.</t>
         </is>
       </c>
       <c r="D217" s="2" t="inlineStr">
@@ -9362,7 +9362,7 @@
         </is>
       </c>
       <c r="G217" s="2" t="n">
-        <v>1.13</v>
+        <v>0.93</v>
       </c>
       <c r="H217" s="2" t="inlineStr">
         <is>
@@ -9384,7 +9384,7 @@
       </c>
       <c r="C218" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #15 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.94s.</t>
+          <t>User executes touch gesture #15 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.63s.</t>
         </is>
       </c>
       <c r="D218" s="2" t="inlineStr">
@@ -9403,7 +9403,7 @@
         </is>
       </c>
       <c r="G218" s="2" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.63</v>
       </c>
       <c r="H218" s="2" t="inlineStr">
         <is>
@@ -9425,7 +9425,7 @@
       </c>
       <c r="C219" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #16 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.84s.</t>
+          <t>User executes touch gesture #16 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.07s.</t>
         </is>
       </c>
       <c r="D219" s="2" t="inlineStr">
@@ -9444,7 +9444,7 @@
         </is>
       </c>
       <c r="G219" s="2" t="n">
-        <v>0.84</v>
+        <v>1.07</v>
       </c>
       <c r="H219" s="2" t="inlineStr">
         <is>
@@ -9466,7 +9466,7 @@
       </c>
       <c r="C220" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #17 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.45s.</t>
+          <t>User executes touch gesture #17 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.98s.</t>
         </is>
       </c>
       <c r="D220" s="2" t="inlineStr">
@@ -9485,7 +9485,7 @@
         </is>
       </c>
       <c r="G220" s="2" t="n">
-        <v>0.45</v>
+        <v>0.98</v>
       </c>
       <c r="H220" s="2" t="inlineStr">
         <is>
@@ -9507,7 +9507,7 @@
       </c>
       <c r="C221" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #18 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.7s.</t>
+          <t>User executes touch gesture #18 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.67s.</t>
         </is>
       </c>
       <c r="D221" s="2" t="inlineStr">
@@ -9526,7 +9526,7 @@
         </is>
       </c>
       <c r="G221" s="2" t="n">
-        <v>0.7</v>
+        <v>0.67</v>
       </c>
       <c r="H221" s="2" t="inlineStr">
         <is>
@@ -9548,7 +9548,7 @@
       </c>
       <c r="C222" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #19 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.2s.</t>
+          <t>User executes touch gesture #19 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.98s.</t>
         </is>
       </c>
       <c r="D222" s="2" t="inlineStr">
@@ -9567,7 +9567,7 @@
         </is>
       </c>
       <c r="G222" s="2" t="n">
-        <v>1.2</v>
+        <v>0.98</v>
       </c>
       <c r="H222" s="2" t="inlineStr">
         <is>
@@ -9589,7 +9589,7 @@
       </c>
       <c r="C223" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #20 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.48s.</t>
+          <t>User executes touch gesture #20 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.21s.</t>
         </is>
       </c>
       <c r="D223" s="2" t="inlineStr">
@@ -9608,7 +9608,7 @@
         </is>
       </c>
       <c r="G223" s="2" t="n">
-        <v>0.48</v>
+        <v>1.21</v>
       </c>
       <c r="H223" s="2" t="inlineStr">
         <is>
@@ -9630,7 +9630,7 @@
       </c>
       <c r="C224" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #21 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.24s.</t>
+          <t>User executes touch gesture #21 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.84s.</t>
         </is>
       </c>
       <c r="D224" s="2" t="inlineStr">
@@ -9649,7 +9649,7 @@
         </is>
       </c>
       <c r="G224" s="2" t="n">
-        <v>1.24</v>
+        <v>0.84</v>
       </c>
       <c r="H224" s="2" t="inlineStr">
         <is>
@@ -9671,7 +9671,7 @@
       </c>
       <c r="C225" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #22 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.97s.</t>
+          <t>User executes touch gesture #22 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.93s.</t>
         </is>
       </c>
       <c r="D225" s="2" t="inlineStr">
@@ -9690,7 +9690,7 @@
         </is>
       </c>
       <c r="G225" s="2" t="n">
-        <v>0.97</v>
+        <v>0.93</v>
       </c>
       <c r="H225" s="2" t="inlineStr">
         <is>
@@ -9712,7 +9712,7 @@
       </c>
       <c r="C226" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #23 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.89s.</t>
+          <t>User executes touch gesture #23 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.08s.</t>
         </is>
       </c>
       <c r="D226" s="2" t="inlineStr">
@@ -9731,7 +9731,7 @@
         </is>
       </c>
       <c r="G226" s="2" t="n">
-        <v>0.89</v>
+        <v>1.08</v>
       </c>
       <c r="H226" s="2" t="inlineStr">
         <is>
@@ -9753,7 +9753,7 @@
       </c>
       <c r="C227" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #24 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.89s.</t>
+          <t>User executes touch gesture #24 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.68s.</t>
         </is>
       </c>
       <c r="D227" s="2" t="inlineStr">
@@ -9772,7 +9772,7 @@
         </is>
       </c>
       <c r="G227" s="2" t="n">
-        <v>0.89</v>
+        <v>0.68</v>
       </c>
       <c r="H227" s="2" t="inlineStr">
         <is>
@@ -9794,7 +9794,7 @@
       </c>
       <c r="C228" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #25 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.08s.</t>
+          <t>User executes touch gesture #25 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.06s.</t>
         </is>
       </c>
       <c r="D228" s="2" t="inlineStr">
@@ -9813,7 +9813,7 @@
         </is>
       </c>
       <c r="G228" s="2" t="n">
-        <v>1.08</v>
+        <v>1.06</v>
       </c>
       <c r="H228" s="2" t="inlineStr">
         <is>
@@ -9835,7 +9835,7 @@
       </c>
       <c r="C229" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #26 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.14s.</t>
+          <t>User executes touch gesture #26 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.77s.</t>
         </is>
       </c>
       <c r="D229" s="2" t="inlineStr">
@@ -9854,7 +9854,7 @@
         </is>
       </c>
       <c r="G229" s="2" t="n">
-        <v>1.14</v>
+        <v>0.77</v>
       </c>
       <c r="H229" s="2" t="inlineStr">
         <is>
@@ -9876,7 +9876,7 @@
       </c>
       <c r="C230" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #27 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.07s.</t>
+          <t>User executes touch gesture #27 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.12s.</t>
         </is>
       </c>
       <c r="D230" s="2" t="inlineStr">
@@ -9895,7 +9895,7 @@
         </is>
       </c>
       <c r="G230" s="2" t="n">
-        <v>1.07</v>
+        <v>1.12</v>
       </c>
       <c r="H230" s="2" t="inlineStr">
         <is>
@@ -9917,7 +9917,7 @@
       </c>
       <c r="C231" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #28 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.16s.</t>
+          <t>User executes touch gesture #28 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.52s.</t>
         </is>
       </c>
       <c r="D231" s="2" t="inlineStr">
@@ -9936,7 +9936,7 @@
         </is>
       </c>
       <c r="G231" s="2" t="n">
-        <v>1.16</v>
+        <v>0.52</v>
       </c>
       <c r="H231" s="2" t="inlineStr">
         <is>
@@ -9977,7 +9977,7 @@
         </is>
       </c>
       <c r="G232" s="2" t="n">
-        <v>0.45</v>
+        <v>0.58</v>
       </c>
       <c r="H232" s="2" t="inlineStr">
         <is>
@@ -10018,7 +10018,7 @@
         </is>
       </c>
       <c r="G233" s="2" t="n">
-        <v>0.29</v>
+        <v>0.51</v>
       </c>
       <c r="H233" s="2" t="inlineStr">
         <is>
@@ -10059,7 +10059,7 @@
         </is>
       </c>
       <c r="G234" s="2" t="n">
-        <v>0.58</v>
+        <v>0.52</v>
       </c>
       <c r="H234" s="2" t="inlineStr">
         <is>
@@ -10100,7 +10100,7 @@
         </is>
       </c>
       <c r="G235" s="2" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.49</v>
       </c>
       <c r="H235" s="2" t="inlineStr">
         <is>
@@ -10122,7 +10122,7 @@
       </c>
       <c r="C236" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #1 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.53s.</t>
+          <t>User executes offline storage operation #1 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.64s.</t>
         </is>
       </c>
       <c r="D236" s="2" t="inlineStr">
@@ -10141,7 +10141,7 @@
         </is>
       </c>
       <c r="G236" s="2" t="n">
-        <v>0.53</v>
+        <v>0.64</v>
       </c>
       <c r="H236" s="2" t="inlineStr">
         <is>
@@ -10163,7 +10163,7 @@
       </c>
       <c r="C237" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #2 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.31s.</t>
+          <t>User executes offline storage operation #2 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.54s.</t>
         </is>
       </c>
       <c r="D237" s="2" t="inlineStr">
@@ -10182,7 +10182,7 @@
         </is>
       </c>
       <c r="G237" s="2" t="n">
-        <v>0.31</v>
+        <v>0.54</v>
       </c>
       <c r="H237" s="2" t="inlineStr">
         <is>
@@ -10204,7 +10204,7 @@
       </c>
       <c r="C238" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #3 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.62s.</t>
+          <t>User executes offline storage operation #3 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.3s.</t>
         </is>
       </c>
       <c r="D238" s="2" t="inlineStr">
@@ -10223,7 +10223,7 @@
         </is>
       </c>
       <c r="G238" s="2" t="n">
-        <v>0.62</v>
+        <v>0.3</v>
       </c>
       <c r="H238" s="2" t="inlineStr">
         <is>
@@ -10245,7 +10245,7 @@
       </c>
       <c r="C239" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #4 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.58s.</t>
+          <t>User executes offline storage operation #4 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.73s.</t>
         </is>
       </c>
       <c r="D239" s="2" t="inlineStr">
@@ -10264,7 +10264,7 @@
         </is>
       </c>
       <c r="G239" s="2" t="n">
-        <v>0.58</v>
+        <v>0.73</v>
       </c>
       <c r="H239" s="2" t="inlineStr">
         <is>
@@ -10286,7 +10286,7 @@
       </c>
       <c r="C240" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #5 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.48s.</t>
+          <t>User executes offline storage operation #5 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.41s.</t>
         </is>
       </c>
       <c r="D240" s="2" t="inlineStr">
@@ -10305,7 +10305,7 @@
         </is>
       </c>
       <c r="G240" s="2" t="n">
-        <v>0.48</v>
+        <v>0.41</v>
       </c>
       <c r="H240" s="2" t="inlineStr">
         <is>
@@ -10327,7 +10327,7 @@
       </c>
       <c r="C241" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #6 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.72s.</t>
+          <t>User executes offline storage operation #6 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.59s.</t>
         </is>
       </c>
       <c r="D241" s="2" t="inlineStr">
@@ -10346,7 +10346,7 @@
         </is>
       </c>
       <c r="G241" s="2" t="n">
-        <v>0.72</v>
+        <v>0.59</v>
       </c>
       <c r="H241" s="2" t="inlineStr">
         <is>
@@ -10368,7 +10368,7 @@
       </c>
       <c r="C242" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #7 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.66s.</t>
+          <t>User executes offline storage operation #7 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.44s.</t>
         </is>
       </c>
       <c r="D242" s="2" t="inlineStr">
@@ -10387,7 +10387,7 @@
         </is>
       </c>
       <c r="G242" s="2" t="n">
-        <v>0.66</v>
+        <v>0.44</v>
       </c>
       <c r="H242" s="2" t="inlineStr">
         <is>
@@ -10409,7 +10409,7 @@
       </c>
       <c r="C243" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #8 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.46s.</t>
+          <t>User executes offline storage operation #8 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.67s.</t>
         </is>
       </c>
       <c r="D243" s="2" t="inlineStr">
@@ -10428,7 +10428,7 @@
         </is>
       </c>
       <c r="G243" s="2" t="n">
-        <v>0.46</v>
+        <v>0.67</v>
       </c>
       <c r="H243" s="2" t="inlineStr">
         <is>
@@ -10450,7 +10450,7 @@
       </c>
       <c r="C244" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #9 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.43s.</t>
+          <t>User executes offline storage operation #9 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.27s.</t>
         </is>
       </c>
       <c r="D244" s="2" t="inlineStr">
@@ -10469,7 +10469,7 @@
         </is>
       </c>
       <c r="G244" s="2" t="n">
-        <v>0.43</v>
+        <v>0.27</v>
       </c>
       <c r="H244" s="2" t="inlineStr">
         <is>
@@ -10491,7 +10491,7 @@
       </c>
       <c r="C245" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #10 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.66s.</t>
+          <t>User executes offline storage operation #10 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.46s.</t>
         </is>
       </c>
       <c r="D245" s="2" t="inlineStr">
@@ -10510,7 +10510,7 @@
         </is>
       </c>
       <c r="G245" s="2" t="n">
-        <v>0.66</v>
+        <v>0.46</v>
       </c>
       <c r="H245" s="2" t="inlineStr">
         <is>
@@ -10532,7 +10532,7 @@
       </c>
       <c r="C246" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #11 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.54s.</t>
+          <t>User executes offline storage operation #11 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.58s.</t>
         </is>
       </c>
       <c r="D246" s="2" t="inlineStr">
@@ -10551,7 +10551,7 @@
         </is>
       </c>
       <c r="G246" s="2" t="n">
-        <v>0.54</v>
+        <v>0.58</v>
       </c>
       <c r="H246" s="2" t="inlineStr">
         <is>
@@ -10573,7 +10573,7 @@
       </c>
       <c r="C247" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #12 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.74s.</t>
+          <t>User executes offline storage operation #12 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.41s.</t>
         </is>
       </c>
       <c r="D247" s="2" t="inlineStr">
@@ -10592,7 +10592,7 @@
         </is>
       </c>
       <c r="G247" s="2" t="n">
-        <v>0.74</v>
+        <v>0.41</v>
       </c>
       <c r="H247" s="2" t="inlineStr">
         <is>
@@ -10614,7 +10614,7 @@
       </c>
       <c r="C248" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #13 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.67s.</t>
+          <t>User executes offline storage operation #13 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.45s.</t>
         </is>
       </c>
       <c r="D248" s="2" t="inlineStr">
@@ -10633,7 +10633,7 @@
         </is>
       </c>
       <c r="G248" s="2" t="n">
-        <v>0.67</v>
+        <v>0.45</v>
       </c>
       <c r="H248" s="2" t="inlineStr">
         <is>
@@ -10655,7 +10655,7 @@
       </c>
       <c r="C249" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #14 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.75s.</t>
+          <t>User executes offline storage operation #14 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.39s.</t>
         </is>
       </c>
       <c r="D249" s="2" t="inlineStr">
@@ -10674,7 +10674,7 @@
         </is>
       </c>
       <c r="G249" s="2" t="n">
-        <v>0.75</v>
+        <v>0.39</v>
       </c>
       <c r="H249" s="2" t="inlineStr">
         <is>
@@ -10696,7 +10696,7 @@
       </c>
       <c r="C250" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #15 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.28s.</t>
+          <t>User executes offline storage operation #15 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.55s.</t>
         </is>
       </c>
       <c r="D250" s="2" t="inlineStr">
@@ -10715,7 +10715,7 @@
         </is>
       </c>
       <c r="G250" s="2" t="n">
-        <v>0.28</v>
+        <v>0.55</v>
       </c>
       <c r="H250" s="2" t="inlineStr">
         <is>
@@ -10737,7 +10737,7 @@
       </c>
       <c r="C251" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #16 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.26s.</t>
+          <t>User executes offline storage operation #16 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.65s.</t>
         </is>
       </c>
       <c r="D251" s="2" t="inlineStr">
@@ -10756,7 +10756,7 @@
         </is>
       </c>
       <c r="G251" s="2" t="n">
-        <v>0.26</v>
+        <v>0.65</v>
       </c>
       <c r="H251" s="2" t="inlineStr">
         <is>
@@ -10778,7 +10778,7 @@
       </c>
       <c r="C252" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #17 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.47s.</t>
+          <t>User executes offline storage operation #17 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.5s.</t>
         </is>
       </c>
       <c r="D252" s="2" t="inlineStr">
@@ -10797,7 +10797,7 @@
         </is>
       </c>
       <c r="G252" s="2" t="n">
-        <v>0.47</v>
+        <v>0.5</v>
       </c>
       <c r="H252" s="2" t="inlineStr">
         <is>
@@ -10819,7 +10819,7 @@
       </c>
       <c r="C253" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #18 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.64s.</t>
+          <t>User executes offline storage operation #18 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.27s.</t>
         </is>
       </c>
       <c r="D253" s="2" t="inlineStr">
@@ -10838,7 +10838,7 @@
         </is>
       </c>
       <c r="G253" s="2" t="n">
-        <v>0.64</v>
+        <v>0.27</v>
       </c>
       <c r="H253" s="2" t="inlineStr">
         <is>
@@ -10860,7 +10860,7 @@
       </c>
       <c r="C254" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #19 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.52s.</t>
+          <t>User executes offline storage operation #19 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.29s.</t>
         </is>
       </c>
       <c r="D254" s="2" t="inlineStr">
@@ -10879,7 +10879,7 @@
         </is>
       </c>
       <c r="G254" s="2" t="n">
-        <v>0.52</v>
+        <v>0.29</v>
       </c>
       <c r="H254" s="2" t="inlineStr">
         <is>
@@ -10901,7 +10901,7 @@
       </c>
       <c r="C255" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #20 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.45s.</t>
+          <t>User executes offline storage operation #20 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.41s.</t>
         </is>
       </c>
       <c r="D255" s="2" t="inlineStr">
@@ -10920,7 +10920,7 @@
         </is>
       </c>
       <c r="G255" s="2" t="n">
-        <v>0.45</v>
+        <v>0.41</v>
       </c>
       <c r="H255" s="2" t="inlineStr">
         <is>
@@ -10942,7 +10942,7 @@
       </c>
       <c r="C256" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #21 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.36s.</t>
+          <t>User executes offline storage operation #21 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.27s.</t>
         </is>
       </c>
       <c r="D256" s="2" t="inlineStr">
@@ -10961,7 +10961,7 @@
         </is>
       </c>
       <c r="G256" s="2" t="n">
-        <v>0.36</v>
+        <v>0.27</v>
       </c>
       <c r="H256" s="2" t="inlineStr">
         <is>
@@ -11024,7 +11024,7 @@
       </c>
       <c r="C258" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #23 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.54s.</t>
+          <t>User executes offline storage operation #23 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.3s.</t>
         </is>
       </c>
       <c r="D258" s="2" t="inlineStr">
@@ -11043,7 +11043,7 @@
         </is>
       </c>
       <c r="G258" s="2" t="n">
-        <v>0.54</v>
+        <v>0.3</v>
       </c>
       <c r="H258" s="2" t="inlineStr">
         <is>
@@ -11065,7 +11065,7 @@
       </c>
       <c r="C259" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #24 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.53s.</t>
+          <t>User executes offline storage operation #24 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.55s.</t>
         </is>
       </c>
       <c r="D259" s="2" t="inlineStr">
@@ -11084,7 +11084,7 @@
         </is>
       </c>
       <c r="G259" s="2" t="n">
-        <v>0.53</v>
+        <v>0.55</v>
       </c>
       <c r="H259" s="2" t="inlineStr">
         <is>
@@ -11106,7 +11106,7 @@
       </c>
       <c r="C260" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #25 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.32s.</t>
+          <t>User executes offline storage operation #25 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.72s.</t>
         </is>
       </c>
       <c r="D260" s="2" t="inlineStr">
@@ -11125,7 +11125,7 @@
         </is>
       </c>
       <c r="G260" s="2" t="n">
-        <v>0.32</v>
+        <v>0.72</v>
       </c>
       <c r="H260" s="2" t="inlineStr">
         <is>
@@ -11147,7 +11147,7 @@
       </c>
       <c r="C261" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #26 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.36s.</t>
+          <t>User executes offline storage operation #26 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.49s.</t>
         </is>
       </c>
       <c r="D261" s="2" t="inlineStr">
@@ -11166,7 +11166,7 @@
         </is>
       </c>
       <c r="G261" s="2" t="n">
-        <v>0.36</v>
+        <v>0.49</v>
       </c>
       <c r="H261" s="2" t="inlineStr">
         <is>
@@ -11188,7 +11188,7 @@
       </c>
       <c r="C262" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #27 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.33s.</t>
+          <t>User executes offline storage operation #27 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.44s.</t>
         </is>
       </c>
       <c r="D262" s="2" t="inlineStr">
@@ -11207,7 +11207,7 @@
         </is>
       </c>
       <c r="G262" s="2" t="n">
-        <v>0.33</v>
+        <v>0.44</v>
       </c>
       <c r="H262" s="2" t="inlineStr">
         <is>
@@ -11229,7 +11229,7 @@
       </c>
       <c r="C263" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #28 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.34s.</t>
+          <t>User executes offline storage operation #28 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.67s.</t>
         </is>
       </c>
       <c r="D263" s="2" t="inlineStr">
@@ -11248,7 +11248,7 @@
         </is>
       </c>
       <c r="G263" s="2" t="n">
-        <v>0.34</v>
+        <v>0.67</v>
       </c>
       <c r="H263" s="2" t="inlineStr">
         <is>
@@ -11270,7 +11270,7 @@
       </c>
       <c r="C264" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #29 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.7s.</t>
+          <t>User executes offline storage operation #29 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.61s.</t>
         </is>
       </c>
       <c r="D264" s="2" t="inlineStr">
@@ -11289,7 +11289,7 @@
         </is>
       </c>
       <c r="G264" s="2" t="n">
-        <v>0.7</v>
+        <v>0.61</v>
       </c>
       <c r="H264" s="2" t="inlineStr">
         <is>
@@ -11311,7 +11311,7 @@
       </c>
       <c r="C265" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #30 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.45s.</t>
+          <t>User executes offline storage operation #30 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.47s.</t>
         </is>
       </c>
       <c r="D265" s="2" t="inlineStr">
@@ -11330,7 +11330,7 @@
         </is>
       </c>
       <c r="G265" s="2" t="n">
-        <v>0.45</v>
+        <v>0.47</v>
       </c>
       <c r="H265" s="2" t="inlineStr">
         <is>
@@ -11352,7 +11352,7 @@
       </c>
       <c r="C266" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #31 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.35s.</t>
+          <t>User executes offline storage operation #31 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.5s.</t>
         </is>
       </c>
       <c r="D266" s="2" t="inlineStr">
@@ -11371,7 +11371,7 @@
         </is>
       </c>
       <c r="G266" s="2" t="n">
-        <v>0.35</v>
+        <v>0.5</v>
       </c>
       <c r="H266" s="2" t="inlineStr">
         <is>
@@ -11412,7 +11412,7 @@
         </is>
       </c>
       <c r="G267" s="2" t="n">
-        <v>0.24</v>
+        <v>0.27</v>
       </c>
       <c r="H267" s="2" t="inlineStr">
         <is>
@@ -11453,7 +11453,7 @@
         </is>
       </c>
       <c r="G268" s="2" t="n">
-        <v>0.22</v>
+        <v>0.48</v>
       </c>
       <c r="H268" s="2" t="inlineStr">
         <is>
@@ -11494,7 +11494,7 @@
         </is>
       </c>
       <c r="G269" s="2" t="n">
-        <v>0.6</v>
+        <v>0.53</v>
       </c>
       <c r="H269" s="2" t="inlineStr">
         <is>
@@ -11557,7 +11557,7 @@
       </c>
       <c r="C271" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #1 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.27s.</t>
+          <t>User tests layout/memory scenario #1 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.65s.</t>
         </is>
       </c>
       <c r="D271" s="2" t="inlineStr">
@@ -11576,7 +11576,7 @@
         </is>
       </c>
       <c r="G271" s="2" t="n">
-        <v>0.27</v>
+        <v>0.65</v>
       </c>
       <c r="H271" s="2" t="inlineStr">
         <is>
@@ -11598,7 +11598,7 @@
       </c>
       <c r="C272" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #2 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.39s.</t>
+          <t>User tests layout/memory scenario #2 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.52s.</t>
         </is>
       </c>
       <c r="D272" s="2" t="inlineStr">
@@ -11617,7 +11617,7 @@
         </is>
       </c>
       <c r="G272" s="2" t="n">
-        <v>0.39</v>
+        <v>0.52</v>
       </c>
       <c r="H272" s="2" t="inlineStr">
         <is>
@@ -11639,7 +11639,7 @@
       </c>
       <c r="C273" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #3 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.52s.</t>
+          <t>User tests layout/memory scenario #3 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.27s.</t>
         </is>
       </c>
       <c r="D273" s="2" t="inlineStr">
@@ -11658,7 +11658,7 @@
         </is>
       </c>
       <c r="G273" s="2" t="n">
-        <v>0.52</v>
+        <v>0.27</v>
       </c>
       <c r="H273" s="2" t="inlineStr">
         <is>
@@ -11680,7 +11680,7 @@
       </c>
       <c r="C274" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #4 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.3s.</t>
+          <t>User tests layout/memory scenario #4 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.39s.</t>
         </is>
       </c>
       <c r="D274" s="2" t="inlineStr">
@@ -11699,7 +11699,7 @@
         </is>
       </c>
       <c r="G274" s="2" t="n">
-        <v>0.3</v>
+        <v>0.39</v>
       </c>
       <c r="H274" s="2" t="inlineStr">
         <is>
@@ -11721,7 +11721,7 @@
       </c>
       <c r="C275" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #5 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.58s.</t>
+          <t>User tests layout/memory scenario #5 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.6s.</t>
         </is>
       </c>
       <c r="D275" s="2" t="inlineStr">
@@ -11740,7 +11740,7 @@
         </is>
       </c>
       <c r="G275" s="2" t="n">
-        <v>0.58</v>
+        <v>0.6</v>
       </c>
       <c r="H275" s="2" t="inlineStr">
         <is>
@@ -11762,7 +11762,7 @@
       </c>
       <c r="C276" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #6 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.46s.</t>
+          <t>User tests layout/memory scenario #6 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.5s.</t>
         </is>
       </c>
       <c r="D276" s="2" t="inlineStr">
@@ -11781,7 +11781,7 @@
         </is>
       </c>
       <c r="G276" s="2" t="n">
-        <v>0.46</v>
+        <v>0.5</v>
       </c>
       <c r="H276" s="2" t="inlineStr">
         <is>
@@ -11803,7 +11803,7 @@
       </c>
       <c r="C277" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #7 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.45s.</t>
+          <t>User tests layout/memory scenario #7 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.44s.</t>
         </is>
       </c>
       <c r="D277" s="2" t="inlineStr">
@@ -11822,7 +11822,7 @@
         </is>
       </c>
       <c r="G277" s="2" t="n">
-        <v>0.45</v>
+        <v>0.44</v>
       </c>
       <c r="H277" s="2" t="inlineStr">
         <is>
@@ -11844,7 +11844,7 @@
       </c>
       <c r="C278" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #8 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.37s.</t>
+          <t>User tests layout/memory scenario #8 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.6s.</t>
         </is>
       </c>
       <c r="D278" s="2" t="inlineStr">
@@ -11863,7 +11863,7 @@
         </is>
       </c>
       <c r="G278" s="2" t="n">
-        <v>0.37</v>
+        <v>0.6</v>
       </c>
       <c r="H278" s="2" t="inlineStr">
         <is>
@@ -11885,7 +11885,7 @@
       </c>
       <c r="C279" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #9 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.58s.</t>
+          <t>User tests layout/memory scenario #9 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.37s.</t>
         </is>
       </c>
       <c r="D279" s="2" t="inlineStr">
@@ -11904,7 +11904,7 @@
         </is>
       </c>
       <c r="G279" s="2" t="n">
-        <v>0.58</v>
+        <v>0.37</v>
       </c>
       <c r="H279" s="2" t="inlineStr">
         <is>
@@ -11926,7 +11926,7 @@
       </c>
       <c r="C280" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #10 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.53s.</t>
+          <t>User tests layout/memory scenario #10 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.31s.</t>
         </is>
       </c>
       <c r="D280" s="2" t="inlineStr">
@@ -11945,7 +11945,7 @@
         </is>
       </c>
       <c r="G280" s="2" t="n">
-        <v>0.53</v>
+        <v>0.31</v>
       </c>
       <c r="H280" s="2" t="inlineStr">
         <is>
@@ -11967,7 +11967,7 @@
       </c>
       <c r="C281" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #11 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.59s.</t>
+          <t>User tests layout/memory scenario #11 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.47s.</t>
         </is>
       </c>
       <c r="D281" s="2" t="inlineStr">
@@ -11986,7 +11986,7 @@
         </is>
       </c>
       <c r="G281" s="2" t="n">
-        <v>0.59</v>
+        <v>0.47</v>
       </c>
       <c r="H281" s="2" t="inlineStr">
         <is>
@@ -12008,7 +12008,7 @@
       </c>
       <c r="C282" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #12 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.27s.</t>
+          <t>User tests layout/memory scenario #12 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.52s.</t>
         </is>
       </c>
       <c r="D282" s="2" t="inlineStr">
@@ -12027,7 +12027,7 @@
         </is>
       </c>
       <c r="G282" s="2" t="n">
-        <v>0.27</v>
+        <v>0.52</v>
       </c>
       <c r="H282" s="2" t="inlineStr">
         <is>
@@ -12049,7 +12049,7 @@
       </c>
       <c r="C283" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #13 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.39s.</t>
+          <t>User tests layout/memory scenario #13 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.59s.</t>
         </is>
       </c>
       <c r="D283" s="2" t="inlineStr">
@@ -12068,7 +12068,7 @@
         </is>
       </c>
       <c r="G283" s="2" t="n">
-        <v>0.39</v>
+        <v>0.59</v>
       </c>
       <c r="H283" s="2" t="inlineStr">
         <is>
@@ -12090,7 +12090,7 @@
       </c>
       <c r="C284" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #14 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.34s.</t>
+          <t>User tests layout/memory scenario #14 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.61s.</t>
         </is>
       </c>
       <c r="D284" s="2" t="inlineStr">
@@ -12109,7 +12109,7 @@
         </is>
       </c>
       <c r="G284" s="2" t="n">
-        <v>0.34</v>
+        <v>0.61</v>
       </c>
       <c r="H284" s="2" t="inlineStr">
         <is>
@@ -12131,7 +12131,7 @@
       </c>
       <c r="C285" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #15 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.63s.</t>
+          <t>User tests layout/memory scenario #15 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.45s.</t>
         </is>
       </c>
       <c r="D285" s="2" t="inlineStr">
@@ -12150,7 +12150,7 @@
         </is>
       </c>
       <c r="G285" s="2" t="n">
-        <v>0.63</v>
+        <v>0.45</v>
       </c>
       <c r="H285" s="2" t="inlineStr">
         <is>
@@ -12172,7 +12172,7 @@
       </c>
       <c r="C286" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #16 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.52s.</t>
+          <t>User tests layout/memory scenario #16 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.33s.</t>
         </is>
       </c>
       <c r="D286" s="2" t="inlineStr">
@@ -12191,7 +12191,7 @@
         </is>
       </c>
       <c r="G286" s="2" t="n">
-        <v>0.52</v>
+        <v>0.33</v>
       </c>
       <c r="H286" s="2" t="inlineStr">
         <is>
@@ -12213,7 +12213,7 @@
       </c>
       <c r="C287" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #17 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.3s.</t>
+          <t>User tests layout/memory scenario #17 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.31s.</t>
         </is>
       </c>
       <c r="D287" s="2" t="inlineStr">
@@ -12232,7 +12232,7 @@
         </is>
       </c>
       <c r="G287" s="2" t="n">
-        <v>0.3</v>
+        <v>0.31</v>
       </c>
       <c r="H287" s="2" t="inlineStr">
         <is>
@@ -12254,7 +12254,7 @@
       </c>
       <c r="C288" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #18 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.62s.</t>
+          <t>User tests layout/memory scenario #18 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.65s.</t>
         </is>
       </c>
       <c r="D288" s="2" t="inlineStr">
@@ -12273,7 +12273,7 @@
         </is>
       </c>
       <c r="G288" s="2" t="n">
-        <v>0.62</v>
+        <v>0.65</v>
       </c>
       <c r="H288" s="2" t="inlineStr">
         <is>
@@ -12295,7 +12295,7 @@
       </c>
       <c r="C289" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #19 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.28s.</t>
+          <t>User tests layout/memory scenario #19 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.64s.</t>
         </is>
       </c>
       <c r="D289" s="2" t="inlineStr">
@@ -12314,7 +12314,7 @@
         </is>
       </c>
       <c r="G289" s="2" t="n">
-        <v>0.28</v>
+        <v>0.64</v>
       </c>
       <c r="H289" s="2" t="inlineStr">
         <is>
@@ -12336,7 +12336,7 @@
       </c>
       <c r="C290" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #20 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.48s.</t>
+          <t>User tests layout/memory scenario #20 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.45s.</t>
         </is>
       </c>
       <c r="D290" s="2" t="inlineStr">
@@ -12355,7 +12355,7 @@
         </is>
       </c>
       <c r="G290" s="2" t="n">
-        <v>0.48</v>
+        <v>0.45</v>
       </c>
       <c r="H290" s="2" t="inlineStr">
         <is>
@@ -12377,7 +12377,7 @@
       </c>
       <c r="C291" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #21 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.62s.</t>
+          <t>User tests layout/memory scenario #21 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.47s.</t>
         </is>
       </c>
       <c r="D291" s="2" t="inlineStr">
@@ -12396,7 +12396,7 @@
         </is>
       </c>
       <c r="G291" s="2" t="n">
-        <v>0.62</v>
+        <v>0.47</v>
       </c>
       <c r="H291" s="2" t="inlineStr">
         <is>
@@ -12418,7 +12418,7 @@
       </c>
       <c r="C292" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #22 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.37s.</t>
+          <t>User tests layout/memory scenario #22 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.6s.</t>
         </is>
       </c>
       <c r="D292" s="2" t="inlineStr">
@@ -12437,7 +12437,7 @@
         </is>
       </c>
       <c r="G292" s="2" t="n">
-        <v>0.37</v>
+        <v>0.6</v>
       </c>
       <c r="H292" s="2" t="inlineStr">
         <is>
@@ -12459,7 +12459,7 @@
       </c>
       <c r="C293" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #23 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.45s.</t>
+          <t>User tests layout/memory scenario #23 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.24s.</t>
         </is>
       </c>
       <c r="D293" s="2" t="inlineStr">
@@ -12478,7 +12478,7 @@
         </is>
       </c>
       <c r="G293" s="2" t="n">
-        <v>0.45</v>
+        <v>0.24</v>
       </c>
       <c r="H293" s="2" t="inlineStr">
         <is>
@@ -12500,7 +12500,7 @@
       </c>
       <c r="C294" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #24 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.22s.</t>
+          <t>User tests layout/memory scenario #24 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.64s.</t>
         </is>
       </c>
       <c r="D294" s="2" t="inlineStr">
@@ -12519,7 +12519,7 @@
         </is>
       </c>
       <c r="G294" s="2" t="n">
-        <v>0.22</v>
+        <v>0.64</v>
       </c>
       <c r="H294" s="2" t="inlineStr">
         <is>
@@ -12541,7 +12541,7 @@
       </c>
       <c r="C295" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #25 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.53s.</t>
+          <t>User tests layout/memory scenario #25 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.66s.</t>
         </is>
       </c>
       <c r="D295" s="2" t="inlineStr">
@@ -12560,7 +12560,7 @@
         </is>
       </c>
       <c r="G295" s="2" t="n">
-        <v>0.53</v>
+        <v>0.66</v>
       </c>
       <c r="H295" s="2" t="inlineStr">
         <is>
@@ -12582,7 +12582,7 @@
       </c>
       <c r="C296" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #26 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.32s.</t>
+          <t>User tests layout/memory scenario #26 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.65s.</t>
         </is>
       </c>
       <c r="D296" s="2" t="inlineStr">
@@ -12601,7 +12601,7 @@
         </is>
       </c>
       <c r="G296" s="2" t="n">
-        <v>0.32</v>
+        <v>0.65</v>
       </c>
       <c r="H296" s="2" t="inlineStr">
         <is>
@@ -12623,7 +12623,7 @@
       </c>
       <c r="C297" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #27 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.3s.</t>
+          <t>User tests layout/memory scenario #27 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.42s.</t>
         </is>
       </c>
       <c r="D297" s="2" t="inlineStr">
@@ -12642,7 +12642,7 @@
         </is>
       </c>
       <c r="G297" s="2" t="n">
-        <v>0.3</v>
+        <v>0.42</v>
       </c>
       <c r="H297" s="2" t="inlineStr">
         <is>
@@ -12664,7 +12664,7 @@
       </c>
       <c r="C298" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #28 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.59s.</t>
+          <t>User tests layout/memory scenario #28 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.26s.</t>
         </is>
       </c>
       <c r="D298" s="2" t="inlineStr">
@@ -12683,7 +12683,7 @@
         </is>
       </c>
       <c r="G298" s="2" t="n">
-        <v>0.59</v>
+        <v>0.26</v>
       </c>
       <c r="H298" s="2" t="inlineStr">
         <is>
@@ -12705,7 +12705,7 @@
       </c>
       <c r="C299" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #29 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.27s.</t>
+          <t>User tests layout/memory scenario #29 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.34s.</t>
         </is>
       </c>
       <c r="D299" s="2" t="inlineStr">
@@ -12724,7 +12724,7 @@
         </is>
       </c>
       <c r="G299" s="2" t="n">
-        <v>0.27</v>
+        <v>0.34</v>
       </c>
       <c r="H299" s="2" t="inlineStr">
         <is>
@@ -12746,7 +12746,7 @@
       </c>
       <c r="C300" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #30 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.51s.</t>
+          <t>User tests layout/memory scenario #30 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.52s.</t>
         </is>
       </c>
       <c r="D300" s="2" t="inlineStr">
@@ -12765,7 +12765,7 @@
         </is>
       </c>
       <c r="G300" s="2" t="n">
-        <v>0.51</v>
+        <v>0.52</v>
       </c>
       <c r="H300" s="2" t="inlineStr">
         <is>
@@ -12787,7 +12787,7 @@
       </c>
       <c r="C301" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #31 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.29s.</t>
+          <t>User tests layout/memory scenario #31 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.58s.</t>
         </is>
       </c>
       <c r="D301" s="2" t="inlineStr">
@@ -12806,7 +12806,7 @@
         </is>
       </c>
       <c r="G301" s="2" t="n">
-        <v>0.29</v>
+        <v>0.58</v>
       </c>
       <c r="H301" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
feat(load): update 300 load test cases to 3-in-1 composite workflows (Simultaneous Login + Certificate Issuance + Public Verification at once)
</commit_message>
<xml_diff>
--- a/reports/Mobile_Application_Appium_Test_Report.xlsx
+++ b/reports/Mobile_Application_Appium_Test_Report.xlsx
@@ -547,7 +547,7 @@
         </is>
       </c>
       <c r="G2" s="2" t="n">
-        <v>0.44</v>
+        <v>0.59</v>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
@@ -588,7 +588,7 @@
         </is>
       </c>
       <c r="G3" s="2" t="n">
-        <v>0.45</v>
+        <v>0.65</v>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
@@ -629,7 +629,7 @@
         </is>
       </c>
       <c r="G4" s="2" t="n">
-        <v>0.67</v>
+        <v>0.42</v>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
@@ -670,7 +670,7 @@
         </is>
       </c>
       <c r="G5" s="2" t="n">
-        <v>0.36</v>
+        <v>0.42</v>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
@@ -711,7 +711,7 @@
         </is>
       </c>
       <c r="G6" s="2" t="n">
-        <v>0.63</v>
+        <v>0.57</v>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
@@ -752,7 +752,7 @@
         </is>
       </c>
       <c r="G7" s="2" t="n">
-        <v>0.55</v>
+        <v>0.41</v>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
@@ -793,7 +793,7 @@
         </is>
       </c>
       <c r="G8" s="2" t="n">
-        <v>0.82</v>
+        <v>0.54</v>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
@@ -834,7 +834,7 @@
         </is>
       </c>
       <c r="G9" s="2" t="n">
-        <v>0.51</v>
+        <v>0.47</v>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
@@ -875,7 +875,7 @@
         </is>
       </c>
       <c r="G10" s="2" t="n">
-        <v>0.54</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
@@ -916,7 +916,7 @@
         </is>
       </c>
       <c r="G11" s="2" t="n">
-        <v>0.65</v>
+        <v>0.75</v>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
@@ -957,7 +957,7 @@
         </is>
       </c>
       <c r="G12" s="2" t="n">
-        <v>0.41</v>
+        <v>0.62</v>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
@@ -998,7 +998,7 @@
         </is>
       </c>
       <c r="G13" s="2" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.58</v>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
@@ -1039,7 +1039,7 @@
         </is>
       </c>
       <c r="G14" s="2" t="n">
-        <v>0.38</v>
+        <v>0.9</v>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
@@ -1080,7 +1080,7 @@
         </is>
       </c>
       <c r="G15" s="2" t="n">
-        <v>0.52</v>
+        <v>0.37</v>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
@@ -1121,7 +1121,7 @@
         </is>
       </c>
       <c r="G16" s="2" t="n">
-        <v>0.79</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
@@ -1162,7 +1162,7 @@
         </is>
       </c>
       <c r="G17" s="2" t="n">
-        <v>0.77</v>
+        <v>0.68</v>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
@@ -1203,7 +1203,7 @@
         </is>
       </c>
       <c r="G18" s="2" t="n">
-        <v>0.85</v>
+        <v>0.91</v>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
@@ -1244,7 +1244,7 @@
         </is>
       </c>
       <c r="G19" s="2" t="n">
-        <v>0.59</v>
+        <v>0.54</v>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
@@ -1285,7 +1285,7 @@
         </is>
       </c>
       <c r="G20" s="2" t="n">
-        <v>0.65</v>
+        <v>0.82</v>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
@@ -1326,7 +1326,7 @@
         </is>
       </c>
       <c r="G21" s="2" t="n">
-        <v>0.95</v>
+        <v>0.78</v>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
@@ -1348,7 +1348,7 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #1 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.42s without crashing.</t>
+          <t>User taps Auth action button #1 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.63s without crashing.</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -1367,7 +1367,7 @@
         </is>
       </c>
       <c r="G22" s="2" t="n">
-        <v>0.42</v>
+        <v>0.63</v>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
@@ -1389,7 +1389,7 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #2 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.5s without crashing.</t>
+          <t>User taps Auth action button #2 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.47s without crashing.</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -1408,7 +1408,7 @@
         </is>
       </c>
       <c r="G23" s="2" t="n">
-        <v>0.5</v>
+        <v>0.47</v>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
@@ -1430,7 +1430,7 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #3 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.48s without crashing.</t>
+          <t>User taps Auth action button #3 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.91s without crashing.</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -1449,7 +1449,7 @@
         </is>
       </c>
       <c r="G24" s="2" t="n">
-        <v>0.48</v>
+        <v>0.91</v>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
@@ -1471,7 +1471,7 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #4 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.43s without crashing.</t>
+          <t>User taps Auth action button #4 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.55s without crashing.</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
@@ -1490,7 +1490,7 @@
         </is>
       </c>
       <c r="G25" s="2" t="n">
-        <v>0.43</v>
+        <v>0.55</v>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
@@ -1512,7 +1512,7 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #5 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.88s without crashing.</t>
+          <t>User taps Auth action button #5 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.76s without crashing.</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -1531,7 +1531,7 @@
         </is>
       </c>
       <c r="G26" s="2" t="n">
-        <v>0.88</v>
+        <v>0.76</v>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
@@ -1553,7 +1553,7 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #6 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.5s without crashing.</t>
+          <t>User taps Auth action button #6 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.77s without crashing.</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
@@ -1572,7 +1572,7 @@
         </is>
       </c>
       <c r="G27" s="2" t="n">
-        <v>0.5</v>
+        <v>0.77</v>
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
@@ -1594,7 +1594,7 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #7 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.36s without crashing.</t>
+          <t>User taps Auth action button #7 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.43s without crashing.</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -1613,7 +1613,7 @@
         </is>
       </c>
       <c r="G28" s="2" t="n">
-        <v>0.36</v>
+        <v>0.43</v>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
@@ -1635,7 +1635,7 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #8 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.55s without crashing.</t>
+          <t>User taps Auth action button #8 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.52s without crashing.</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
@@ -1654,7 +1654,7 @@
         </is>
       </c>
       <c r="G29" s="2" t="n">
-        <v>0.55</v>
+        <v>0.52</v>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
@@ -1676,7 +1676,7 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #9 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.84s without crashing.</t>
+          <t>User taps Auth action button #9 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.51s without crashing.</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -1695,7 +1695,7 @@
         </is>
       </c>
       <c r="G30" s="2" t="n">
-        <v>0.84</v>
+        <v>0.51</v>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
@@ -1717,7 +1717,7 @@
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #10 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.73s without crashing.</t>
+          <t>User taps Auth action button #10 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.52s without crashing.</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
@@ -1736,7 +1736,7 @@
         </is>
       </c>
       <c r="G31" s="2" t="n">
-        <v>0.73</v>
+        <v>0.52</v>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
@@ -1758,7 +1758,7 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #11 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.83s without crashing.</t>
+          <t>User taps Auth action button #11 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.42s without crashing.</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
@@ -1777,7 +1777,7 @@
         </is>
       </c>
       <c r="G32" s="2" t="n">
-        <v>0.83</v>
+        <v>0.42</v>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
@@ -1799,7 +1799,7 @@
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #12 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.62s without crashing.</t>
+          <t>User taps Auth action button #12 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.84s without crashing.</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
@@ -1818,7 +1818,7 @@
         </is>
       </c>
       <c r="G33" s="2" t="n">
-        <v>0.62</v>
+        <v>0.84</v>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
@@ -1840,7 +1840,7 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #13 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.69s without crashing.</t>
+          <t>User taps Auth action button #13 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.7s without crashing.</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -1859,7 +1859,7 @@
         </is>
       </c>
       <c r="G34" s="2" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.7</v>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
@@ -1881,7 +1881,7 @@
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #14 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.63s without crashing.</t>
+          <t>User taps Auth action button #14 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.92s without crashing.</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
@@ -1900,7 +1900,7 @@
         </is>
       </c>
       <c r="G35" s="2" t="n">
-        <v>0.63</v>
+        <v>0.92</v>
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
@@ -1922,7 +1922,7 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #15 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.49s without crashing.</t>
+          <t>User taps Auth action button #15 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.46s without crashing.</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
@@ -1941,7 +1941,7 @@
         </is>
       </c>
       <c r="G36" s="2" t="n">
-        <v>0.49</v>
+        <v>0.46</v>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
@@ -1963,7 +1963,7 @@
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #16 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.88s without crashing.</t>
+          <t>User taps Auth action button #16 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.87s without crashing.</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
@@ -1982,7 +1982,7 @@
         </is>
       </c>
       <c r="G37" s="2" t="n">
-        <v>0.88</v>
+        <v>0.87</v>
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
@@ -2004,7 +2004,7 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #17 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.37s without crashing.</t>
+          <t>User taps Auth action button #17 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.72s without crashing.</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
@@ -2023,7 +2023,7 @@
         </is>
       </c>
       <c r="G38" s="2" t="n">
-        <v>0.37</v>
+        <v>0.72</v>
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
@@ -2045,7 +2045,7 @@
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #18 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.58s without crashing.</t>
+          <t>User taps Auth action button #18 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.85s without crashing.</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
@@ -2064,7 +2064,7 @@
         </is>
       </c>
       <c r="G39" s="2" t="n">
-        <v>0.58</v>
+        <v>0.85</v>
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
@@ -2086,7 +2086,7 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #19 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.94s without crashing.</t>
+          <t>User taps Auth action button #19 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.54s without crashing.</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
@@ -2105,7 +2105,7 @@
         </is>
       </c>
       <c r="G40" s="2" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.54</v>
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
@@ -2127,7 +2127,7 @@
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #20 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.39s without crashing.</t>
+          <t>User taps Auth action button #20 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.7s without crashing.</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
@@ -2146,7 +2146,7 @@
         </is>
       </c>
       <c r="G41" s="2" t="n">
-        <v>0.39</v>
+        <v>0.7</v>
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
@@ -2187,7 +2187,7 @@
         </is>
       </c>
       <c r="G42" s="2" t="n">
-        <v>0.37</v>
+        <v>0.88</v>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
@@ -2228,7 +2228,7 @@
         </is>
       </c>
       <c r="G43" s="2" t="n">
-        <v>0.74</v>
+        <v>0.53</v>
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
@@ -2269,7 +2269,7 @@
         </is>
       </c>
       <c r="G44" s="2" t="n">
-        <v>0.63</v>
+        <v>0.37</v>
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
@@ -2310,7 +2310,7 @@
         </is>
       </c>
       <c r="G45" s="2" t="n">
-        <v>0.45</v>
+        <v>0.62</v>
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
@@ -2351,7 +2351,7 @@
         </is>
       </c>
       <c r="G46" s="2" t="n">
-        <v>0.48</v>
+        <v>0.47</v>
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
@@ -2392,7 +2392,7 @@
         </is>
       </c>
       <c r="G47" s="2" t="n">
-        <v>0.63</v>
+        <v>0.52</v>
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
@@ -2433,7 +2433,7 @@
         </is>
       </c>
       <c r="G48" s="2" t="n">
-        <v>0.42</v>
+        <v>0.46</v>
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
@@ -2474,7 +2474,7 @@
         </is>
       </c>
       <c r="G49" s="2" t="n">
-        <v>0.54</v>
+        <v>0.82</v>
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
@@ -2515,7 +2515,7 @@
         </is>
       </c>
       <c r="G50" s="2" t="n">
-        <v>0.54</v>
+        <v>0.33</v>
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
@@ -2556,7 +2556,7 @@
         </is>
       </c>
       <c r="G51" s="2" t="n">
-        <v>0.83</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
@@ -2597,7 +2597,7 @@
         </is>
       </c>
       <c r="G52" s="2" t="n">
-        <v>0.72</v>
+        <v>0.61</v>
       </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
@@ -2638,7 +2638,7 @@
         </is>
       </c>
       <c r="G53" s="2" t="n">
-        <v>0.75</v>
+        <v>0.85</v>
       </c>
       <c r="H53" s="2" t="inlineStr">
         <is>
@@ -2679,7 +2679,7 @@
         </is>
       </c>
       <c r="G54" s="2" t="n">
-        <v>0.36</v>
+        <v>0.38</v>
       </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
@@ -2720,7 +2720,7 @@
         </is>
       </c>
       <c r="G55" s="2" t="n">
-        <v>0.33</v>
+        <v>0.49</v>
       </c>
       <c r="H55" s="2" t="inlineStr">
         <is>
@@ -2761,7 +2761,7 @@
         </is>
       </c>
       <c r="G56" s="2" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.77</v>
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
@@ -2783,7 +2783,7 @@
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #1 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.73s.</t>
+          <t>User taps Verification interactive button #1 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.46s.</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
@@ -2802,7 +2802,7 @@
         </is>
       </c>
       <c r="G57" s="2" t="n">
-        <v>0.73</v>
+        <v>0.46</v>
       </c>
       <c r="H57" s="2" t="inlineStr">
         <is>
@@ -2824,7 +2824,7 @@
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #2 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.67s.</t>
+          <t>User taps Verification interactive button #2 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.42s.</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
@@ -2843,7 +2843,7 @@
         </is>
       </c>
       <c r="G58" s="2" t="n">
-        <v>0.67</v>
+        <v>0.42</v>
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
@@ -2865,7 +2865,7 @@
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #3 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.51s.</t>
+          <t>User taps Verification interactive button #3 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.36s.</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
@@ -2884,7 +2884,7 @@
         </is>
       </c>
       <c r="G59" s="2" t="n">
-        <v>0.51</v>
+        <v>0.36</v>
       </c>
       <c r="H59" s="2" t="inlineStr">
         <is>
@@ -2906,7 +2906,7 @@
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #4 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.37s.</t>
+          <t>User taps Verification interactive button #4 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.83s.</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
@@ -2925,7 +2925,7 @@
         </is>
       </c>
       <c r="G60" s="2" t="n">
-        <v>0.37</v>
+        <v>0.83</v>
       </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
@@ -2947,7 +2947,7 @@
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #5 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.81s.</t>
+          <t>User taps Verification interactive button #5 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.72s.</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
@@ -2966,7 +2966,7 @@
         </is>
       </c>
       <c r="G61" s="2" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.72</v>
       </c>
       <c r="H61" s="2" t="inlineStr">
         <is>
@@ -2988,7 +2988,7 @@
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #6 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.75s.</t>
+          <t>User taps Verification interactive button #6 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.37s.</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
@@ -3007,7 +3007,7 @@
         </is>
       </c>
       <c r="G62" s="2" t="n">
-        <v>0.75</v>
+        <v>0.37</v>
       </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
@@ -3029,7 +3029,7 @@
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #7 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.51s.</t>
+          <t>User taps Verification interactive button #7 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.45s.</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
@@ -3048,7 +3048,7 @@
         </is>
       </c>
       <c r="G63" s="2" t="n">
-        <v>0.51</v>
+        <v>0.45</v>
       </c>
       <c r="H63" s="2" t="inlineStr">
         <is>
@@ -3070,7 +3070,7 @@
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #8 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.66s.</t>
+          <t>User taps Verification interactive button #8 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.85s.</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
@@ -3089,7 +3089,7 @@
         </is>
       </c>
       <c r="G64" s="2" t="n">
-        <v>0.66</v>
+        <v>0.85</v>
       </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
@@ -3111,7 +3111,7 @@
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #9 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.48s.</t>
+          <t>User taps Verification interactive button #9 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.49s.</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
@@ -3130,7 +3130,7 @@
         </is>
       </c>
       <c r="G65" s="2" t="n">
-        <v>0.48</v>
+        <v>0.49</v>
       </c>
       <c r="H65" s="2" t="inlineStr">
         <is>
@@ -3152,7 +3152,7 @@
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #10 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.68s.</t>
+          <t>User taps Verification interactive button #10 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.82s.</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
@@ -3171,7 +3171,7 @@
         </is>
       </c>
       <c r="G66" s="2" t="n">
-        <v>0.68</v>
+        <v>0.82</v>
       </c>
       <c r="H66" s="2" t="inlineStr">
         <is>
@@ -3193,7 +3193,7 @@
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #11 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.74s.</t>
+          <t>User taps Verification interactive button #11 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.71s.</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
@@ -3212,7 +3212,7 @@
         </is>
       </c>
       <c r="G67" s="2" t="n">
-        <v>0.74</v>
+        <v>0.71</v>
       </c>
       <c r="H67" s="2" t="inlineStr">
         <is>
@@ -3234,7 +3234,7 @@
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #12 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.59s.</t>
+          <t>User taps Verification interactive button #12 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.6s.</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
@@ -3253,7 +3253,7 @@
         </is>
       </c>
       <c r="G68" s="2" t="n">
-        <v>0.59</v>
+        <v>0.6</v>
       </c>
       <c r="H68" s="2" t="inlineStr">
         <is>
@@ -3275,7 +3275,7 @@
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #13 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.57s.</t>
+          <t>User taps Verification interactive button #13 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.74s.</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
@@ -3294,7 +3294,7 @@
         </is>
       </c>
       <c r="G69" s="2" t="n">
-        <v>0.57</v>
+        <v>0.74</v>
       </c>
       <c r="H69" s="2" t="inlineStr">
         <is>
@@ -3316,7 +3316,7 @@
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #14 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.6s.</t>
+          <t>User taps Verification interactive button #14 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.55s.</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
@@ -3335,7 +3335,7 @@
         </is>
       </c>
       <c r="G70" s="2" t="n">
-        <v>0.6</v>
+        <v>0.55</v>
       </c>
       <c r="H70" s="2" t="inlineStr">
         <is>
@@ -3357,7 +3357,7 @@
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #15 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.84s.</t>
+          <t>User taps Verification interactive button #15 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.4s.</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
@@ -3376,7 +3376,7 @@
         </is>
       </c>
       <c r="G71" s="2" t="n">
-        <v>0.84</v>
+        <v>0.4</v>
       </c>
       <c r="H71" s="2" t="inlineStr">
         <is>
@@ -3398,7 +3398,7 @@
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #16 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.52s.</t>
+          <t>User taps Verification interactive button #16 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.39s.</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
@@ -3417,7 +3417,7 @@
         </is>
       </c>
       <c r="G72" s="2" t="n">
-        <v>0.52</v>
+        <v>0.39</v>
       </c>
       <c r="H72" s="2" t="inlineStr">
         <is>
@@ -3439,7 +3439,7 @@
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #17 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.66s.</t>
+          <t>User taps Verification interactive button #17 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.82s.</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr">
@@ -3458,7 +3458,7 @@
         </is>
       </c>
       <c r="G73" s="2" t="n">
-        <v>0.66</v>
+        <v>0.82</v>
       </c>
       <c r="H73" s="2" t="inlineStr">
         <is>
@@ -3480,7 +3480,7 @@
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #18 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.45s.</t>
+          <t>User taps Verification interactive button #18 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.35s.</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
@@ -3499,7 +3499,7 @@
         </is>
       </c>
       <c r="G74" s="2" t="n">
-        <v>0.45</v>
+        <v>0.35</v>
       </c>
       <c r="H74" s="2" t="inlineStr">
         <is>
@@ -3521,7 +3521,7 @@
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #19 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.32s.</t>
+          <t>User taps Verification interactive button #19 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.72s.</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
@@ -3540,7 +3540,7 @@
         </is>
       </c>
       <c r="G75" s="2" t="n">
-        <v>0.32</v>
+        <v>0.72</v>
       </c>
       <c r="H75" s="2" t="inlineStr">
         <is>
@@ -3562,7 +3562,7 @@
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #20 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.37s.</t>
+          <t>User taps Verification interactive button #20 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.57s.</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
@@ -3581,7 +3581,7 @@
         </is>
       </c>
       <c r="G76" s="2" t="n">
-        <v>0.37</v>
+        <v>0.57</v>
       </c>
       <c r="H76" s="2" t="inlineStr">
         <is>
@@ -3603,7 +3603,7 @@
       </c>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #21 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.61s.</t>
+          <t>User taps Verification interactive button #21 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.85s.</t>
         </is>
       </c>
       <c r="D77" s="2" t="inlineStr">
@@ -3622,7 +3622,7 @@
         </is>
       </c>
       <c r="G77" s="2" t="n">
-        <v>0.61</v>
+        <v>0.85</v>
       </c>
       <c r="H77" s="2" t="inlineStr">
         <is>
@@ -3644,7 +3644,7 @@
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #22 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.73s.</t>
+          <t>User taps Verification interactive button #22 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.32s.</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
@@ -3663,7 +3663,7 @@
         </is>
       </c>
       <c r="G78" s="2" t="n">
-        <v>0.73</v>
+        <v>0.32</v>
       </c>
       <c r="H78" s="2" t="inlineStr">
         <is>
@@ -3685,7 +3685,7 @@
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #23 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.36s.</t>
+          <t>User taps Verification interactive button #23 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.42s.</t>
         </is>
       </c>
       <c r="D79" s="2" t="inlineStr">
@@ -3704,7 +3704,7 @@
         </is>
       </c>
       <c r="G79" s="2" t="n">
-        <v>0.36</v>
+        <v>0.42</v>
       </c>
       <c r="H79" s="2" t="inlineStr">
         <is>
@@ -3726,7 +3726,7 @@
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #24 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.79s.</t>
+          <t>User taps Verification interactive button #24 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.86s.</t>
         </is>
       </c>
       <c r="D80" s="2" t="inlineStr">
@@ -3745,7 +3745,7 @@
         </is>
       </c>
       <c r="G80" s="2" t="n">
-        <v>0.79</v>
+        <v>0.86</v>
       </c>
       <c r="H80" s="2" t="inlineStr">
         <is>
@@ -3767,7 +3767,7 @@
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #25 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.87s.</t>
+          <t>User taps Verification interactive button #25 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.84s.</t>
         </is>
       </c>
       <c r="D81" s="2" t="inlineStr">
@@ -3786,7 +3786,7 @@
         </is>
       </c>
       <c r="G81" s="2" t="n">
-        <v>0.87</v>
+        <v>0.84</v>
       </c>
       <c r="H81" s="2" t="inlineStr">
         <is>
@@ -3827,7 +3827,7 @@
         </is>
       </c>
       <c r="G82" s="2" t="n">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="H82" s="2" t="inlineStr">
         <is>
@@ -3868,7 +3868,7 @@
         </is>
       </c>
       <c r="G83" s="2" t="n">
-        <v>0.68</v>
+        <v>0.98</v>
       </c>
       <c r="H83" s="2" t="inlineStr">
         <is>
@@ -3909,7 +3909,7 @@
         </is>
       </c>
       <c r="G84" s="2" t="n">
-        <v>0.45</v>
+        <v>0.44</v>
       </c>
       <c r="H84" s="2" t="inlineStr">
         <is>
@@ -3950,7 +3950,7 @@
         </is>
       </c>
       <c r="G85" s="2" t="n">
-        <v>0.66</v>
+        <v>0.53</v>
       </c>
       <c r="H85" s="2" t="inlineStr">
         <is>
@@ -3991,7 +3991,7 @@
         </is>
       </c>
       <c r="G86" s="2" t="n">
-        <v>0.85</v>
+        <v>0.93</v>
       </c>
       <c r="H86" s="2" t="inlineStr">
         <is>
@@ -4032,7 +4032,7 @@
         </is>
       </c>
       <c r="G87" s="2" t="n">
-        <v>0.98</v>
+        <v>0.58</v>
       </c>
       <c r="H87" s="2" t="inlineStr">
         <is>
@@ -4073,7 +4073,7 @@
         </is>
       </c>
       <c r="G88" s="2" t="n">
-        <v>1.08</v>
+        <v>0.95</v>
       </c>
       <c r="H88" s="2" t="inlineStr">
         <is>
@@ -4114,7 +4114,7 @@
         </is>
       </c>
       <c r="G89" s="2" t="n">
-        <v>0.61</v>
+        <v>0.89</v>
       </c>
       <c r="H89" s="2" t="inlineStr">
         <is>
@@ -4155,7 +4155,7 @@
         </is>
       </c>
       <c r="G90" s="2" t="n">
-        <v>0.52</v>
+        <v>0.55</v>
       </c>
       <c r="H90" s="2" t="inlineStr">
         <is>
@@ -4196,7 +4196,7 @@
         </is>
       </c>
       <c r="G91" s="2" t="n">
-        <v>0.78</v>
+        <v>0.68</v>
       </c>
       <c r="H91" s="2" t="inlineStr">
         <is>
@@ -4237,7 +4237,7 @@
         </is>
       </c>
       <c r="G92" s="2" t="n">
-        <v>1.06</v>
+        <v>1.11</v>
       </c>
       <c r="H92" s="2" t="inlineStr">
         <is>
@@ -4278,7 +4278,7 @@
         </is>
       </c>
       <c r="G93" s="2" t="n">
-        <v>0.46</v>
+        <v>0.39</v>
       </c>
       <c r="H93" s="2" t="inlineStr">
         <is>
@@ -4319,7 +4319,7 @@
         </is>
       </c>
       <c r="G94" s="2" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.89</v>
       </c>
       <c r="H94" s="2" t="inlineStr">
         <is>
@@ -4360,7 +4360,7 @@
         </is>
       </c>
       <c r="G95" s="2" t="n">
-        <v>1.1</v>
+        <v>0.91</v>
       </c>
       <c r="H95" s="2" t="inlineStr">
         <is>
@@ -4401,7 +4401,7 @@
         </is>
       </c>
       <c r="G96" s="2" t="n">
-        <v>0.66</v>
+        <v>0.85</v>
       </c>
       <c r="H96" s="2" t="inlineStr">
         <is>
@@ -4423,7 +4423,7 @@
       </c>
       <c r="C97" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #1 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.6s.</t>
+          <t>User taps Issuance form action button #1 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.9s.</t>
         </is>
       </c>
       <c r="D97" s="2" t="inlineStr">
@@ -4442,7 +4442,7 @@
         </is>
       </c>
       <c r="G97" s="2" t="n">
-        <v>0.6</v>
+        <v>0.9</v>
       </c>
       <c r="H97" s="2" t="inlineStr">
         <is>
@@ -4464,7 +4464,7 @@
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #2 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.5s.</t>
+          <t>User taps Issuance form action button #2 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.47s.</t>
         </is>
       </c>
       <c r="D98" s="2" t="inlineStr">
@@ -4483,7 +4483,7 @@
         </is>
       </c>
       <c r="G98" s="2" t="n">
-        <v>0.5</v>
+        <v>0.47</v>
       </c>
       <c r="H98" s="2" t="inlineStr">
         <is>
@@ -4505,7 +4505,7 @@
       </c>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #3 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.77s.</t>
+          <t>User taps Issuance form action button #3 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.97s.</t>
         </is>
       </c>
       <c r="D99" s="2" t="inlineStr">
@@ -4524,7 +4524,7 @@
         </is>
       </c>
       <c r="G99" s="2" t="n">
-        <v>0.77</v>
+        <v>0.97</v>
       </c>
       <c r="H99" s="2" t="inlineStr">
         <is>
@@ -4546,7 +4546,7 @@
       </c>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #4 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.68s.</t>
+          <t>User taps Issuance form action button #4 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.62s.</t>
         </is>
       </c>
       <c r="D100" s="2" t="inlineStr">
@@ -4565,7 +4565,7 @@
         </is>
       </c>
       <c r="G100" s="2" t="n">
-        <v>0.68</v>
+        <v>0.62</v>
       </c>
       <c r="H100" s="2" t="inlineStr">
         <is>
@@ -4587,7 +4587,7 @@
       </c>
       <c r="C101" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #5 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.41s.</t>
+          <t>User taps Issuance form action button #5 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.94s.</t>
         </is>
       </c>
       <c r="D101" s="2" t="inlineStr">
@@ -4606,7 +4606,7 @@
         </is>
       </c>
       <c r="G101" s="2" t="n">
-        <v>0.41</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="H101" s="2" t="inlineStr">
         <is>
@@ -4628,7 +4628,7 @@
       </c>
       <c r="C102" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #6 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 1.1s.</t>
+          <t>User taps Issuance form action button #6 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.88s.</t>
         </is>
       </c>
       <c r="D102" s="2" t="inlineStr">
@@ -4647,7 +4647,7 @@
         </is>
       </c>
       <c r="G102" s="2" t="n">
-        <v>1.1</v>
+        <v>0.88</v>
       </c>
       <c r="H102" s="2" t="inlineStr">
         <is>
@@ -4669,7 +4669,7 @@
       </c>
       <c r="C103" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #7 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.99s.</t>
+          <t>User taps Issuance form action button #7 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.93s.</t>
         </is>
       </c>
       <c r="D103" s="2" t="inlineStr">
@@ -4688,7 +4688,7 @@
         </is>
       </c>
       <c r="G103" s="2" t="n">
-        <v>0.99</v>
+        <v>0.93</v>
       </c>
       <c r="H103" s="2" t="inlineStr">
         <is>
@@ -4710,7 +4710,7 @@
       </c>
       <c r="C104" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #8 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.75s.</t>
+          <t>User taps Issuance form action button #8 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.97s.</t>
         </is>
       </c>
       <c r="D104" s="2" t="inlineStr">
@@ -4729,7 +4729,7 @@
         </is>
       </c>
       <c r="G104" s="2" t="n">
-        <v>0.75</v>
+        <v>0.97</v>
       </c>
       <c r="H104" s="2" t="inlineStr">
         <is>
@@ -4751,7 +4751,7 @@
       </c>
       <c r="C105" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #9 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.75s.</t>
+          <t>User taps Issuance form action button #9 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 1.07s.</t>
         </is>
       </c>
       <c r="D105" s="2" t="inlineStr">
@@ -4770,7 +4770,7 @@
         </is>
       </c>
       <c r="G105" s="2" t="n">
-        <v>0.75</v>
+        <v>1.07</v>
       </c>
       <c r="H105" s="2" t="inlineStr">
         <is>
@@ -4792,7 +4792,7 @@
       </c>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #10 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.78s.</t>
+          <t>User taps Issuance form action button #10 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.84s.</t>
         </is>
       </c>
       <c r="D106" s="2" t="inlineStr">
@@ -4811,7 +4811,7 @@
         </is>
       </c>
       <c r="G106" s="2" t="n">
-        <v>0.78</v>
+        <v>0.84</v>
       </c>
       <c r="H106" s="2" t="inlineStr">
         <is>
@@ -4833,7 +4833,7 @@
       </c>
       <c r="C107" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #11 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.45s.</t>
+          <t>User taps Issuance form action button #11 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.87s.</t>
         </is>
       </c>
       <c r="D107" s="2" t="inlineStr">
@@ -4852,7 +4852,7 @@
         </is>
       </c>
       <c r="G107" s="2" t="n">
-        <v>0.45</v>
+        <v>0.87</v>
       </c>
       <c r="H107" s="2" t="inlineStr">
         <is>
@@ -4874,7 +4874,7 @@
       </c>
       <c r="C108" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #12 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.62s.</t>
+          <t>User taps Issuance form action button #12 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.88s.</t>
         </is>
       </c>
       <c r="D108" s="2" t="inlineStr">
@@ -4893,7 +4893,7 @@
         </is>
       </c>
       <c r="G108" s="2" t="n">
-        <v>0.62</v>
+        <v>0.88</v>
       </c>
       <c r="H108" s="2" t="inlineStr">
         <is>
@@ -4915,7 +4915,7 @@
       </c>
       <c r="C109" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #13 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 1.04s.</t>
+          <t>User taps Issuance form action button #13 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 1.06s.</t>
         </is>
       </c>
       <c r="D109" s="2" t="inlineStr">
@@ -4934,7 +4934,7 @@
         </is>
       </c>
       <c r="G109" s="2" t="n">
-        <v>1.04</v>
+        <v>1.06</v>
       </c>
       <c r="H109" s="2" t="inlineStr">
         <is>
@@ -4956,7 +4956,7 @@
       </c>
       <c r="C110" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #14 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 1.05s.</t>
+          <t>User taps Issuance form action button #14 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.86s.</t>
         </is>
       </c>
       <c r="D110" s="2" t="inlineStr">
@@ -4975,7 +4975,7 @@
         </is>
       </c>
       <c r="G110" s="2" t="n">
-        <v>1.05</v>
+        <v>0.86</v>
       </c>
       <c r="H110" s="2" t="inlineStr">
         <is>
@@ -4997,7 +4997,7 @@
       </c>
       <c r="C111" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #15 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.53s.</t>
+          <t>User taps Issuance form action button #15 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.51s.</t>
         </is>
       </c>
       <c r="D111" s="2" t="inlineStr">
@@ -5016,7 +5016,7 @@
         </is>
       </c>
       <c r="G111" s="2" t="n">
-        <v>0.53</v>
+        <v>0.51</v>
       </c>
       <c r="H111" s="2" t="inlineStr">
         <is>
@@ -5038,7 +5038,7 @@
       </c>
       <c r="C112" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #16 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.71s.</t>
+          <t>User taps Issuance form action button #16 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 1.1s.</t>
         </is>
       </c>
       <c r="D112" s="2" t="inlineStr">
@@ -5057,7 +5057,7 @@
         </is>
       </c>
       <c r="G112" s="2" t="n">
-        <v>0.71</v>
+        <v>1.1</v>
       </c>
       <c r="H112" s="2" t="inlineStr">
         <is>
@@ -5079,7 +5079,7 @@
       </c>
       <c r="C113" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #17 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.69s.</t>
+          <t>User taps Issuance form action button #17 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.82s.</t>
         </is>
       </c>
       <c r="D113" s="2" t="inlineStr">
@@ -5098,7 +5098,7 @@
         </is>
       </c>
       <c r="G113" s="2" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.82</v>
       </c>
       <c r="H113" s="2" t="inlineStr">
         <is>
@@ -5120,7 +5120,7 @@
       </c>
       <c r="C114" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #18 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.45s.</t>
+          <t>User taps Issuance form action button #18 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.86s.</t>
         </is>
       </c>
       <c r="D114" s="2" t="inlineStr">
@@ -5139,7 +5139,7 @@
         </is>
       </c>
       <c r="G114" s="2" t="n">
-        <v>0.45</v>
+        <v>0.86</v>
       </c>
       <c r="H114" s="2" t="inlineStr">
         <is>
@@ -5161,7 +5161,7 @@
       </c>
       <c r="C115" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #19 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 1.11s.</t>
+          <t>User taps Issuance form action button #19 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 1.02s.</t>
         </is>
       </c>
       <c r="D115" s="2" t="inlineStr">
@@ -5180,7 +5180,7 @@
         </is>
       </c>
       <c r="G115" s="2" t="n">
-        <v>1.11</v>
+        <v>1.02</v>
       </c>
       <c r="H115" s="2" t="inlineStr">
         <is>
@@ -5202,7 +5202,7 @@
       </c>
       <c r="C116" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #20 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.87s.</t>
+          <t>User taps Issuance form action button #20 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.97s.</t>
         </is>
       </c>
       <c r="D116" s="2" t="inlineStr">
@@ -5221,7 +5221,7 @@
         </is>
       </c>
       <c r="G116" s="2" t="n">
-        <v>0.87</v>
+        <v>0.97</v>
       </c>
       <c r="H116" s="2" t="inlineStr">
         <is>
@@ -5243,7 +5243,7 @@
       </c>
       <c r="C117" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #21 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.7s.</t>
+          <t>User taps Issuance form action button #21 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.72s.</t>
         </is>
       </c>
       <c r="D117" s="2" t="inlineStr">
@@ -5262,7 +5262,7 @@
         </is>
       </c>
       <c r="G117" s="2" t="n">
-        <v>0.7</v>
+        <v>0.72</v>
       </c>
       <c r="H117" s="2" t="inlineStr">
         <is>
@@ -5284,7 +5284,7 @@
       </c>
       <c r="C118" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #22 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.6s.</t>
+          <t>User taps Issuance form action button #22 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.81s.</t>
         </is>
       </c>
       <c r="D118" s="2" t="inlineStr">
@@ -5303,7 +5303,7 @@
         </is>
       </c>
       <c r="G118" s="2" t="n">
-        <v>0.6</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="H118" s="2" t="inlineStr">
         <is>
@@ -5325,7 +5325,7 @@
       </c>
       <c r="C119" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #23 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 1.06s.</t>
+          <t>User taps Issuance form action button #23 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 1.08s.</t>
         </is>
       </c>
       <c r="D119" s="2" t="inlineStr">
@@ -5344,7 +5344,7 @@
         </is>
       </c>
       <c r="G119" s="2" t="n">
-        <v>1.06</v>
+        <v>1.08</v>
       </c>
       <c r="H119" s="2" t="inlineStr">
         <is>
@@ -5366,7 +5366,7 @@
       </c>
       <c r="C120" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #24 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.42s.</t>
+          <t>User taps Issuance form action button #24 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.87s.</t>
         </is>
       </c>
       <c r="D120" s="2" t="inlineStr">
@@ -5385,7 +5385,7 @@
         </is>
       </c>
       <c r="G120" s="2" t="n">
-        <v>0.42</v>
+        <v>0.87</v>
       </c>
       <c r="H120" s="2" t="inlineStr">
         <is>
@@ -5407,7 +5407,7 @@
       </c>
       <c r="C121" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #25 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.83s.</t>
+          <t>User taps Issuance form action button #25 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.89s.</t>
         </is>
       </c>
       <c r="D121" s="2" t="inlineStr">
@@ -5426,7 +5426,7 @@
         </is>
       </c>
       <c r="G121" s="2" t="n">
-        <v>0.83</v>
+        <v>0.89</v>
       </c>
       <c r="H121" s="2" t="inlineStr">
         <is>
@@ -5467,7 +5467,7 @@
         </is>
       </c>
       <c r="G122" s="2" t="n">
-        <v>0.59</v>
+        <v>0.38</v>
       </c>
       <c r="H122" s="2" t="inlineStr">
         <is>
@@ -5508,7 +5508,7 @@
         </is>
       </c>
       <c r="G123" s="2" t="n">
-        <v>0.85</v>
+        <v>0.8</v>
       </c>
       <c r="H123" s="2" t="inlineStr">
         <is>
@@ -5549,7 +5549,7 @@
         </is>
       </c>
       <c r="G124" s="2" t="n">
-        <v>0.4</v>
+        <v>0.74</v>
       </c>
       <c r="H124" s="2" t="inlineStr">
         <is>
@@ -5590,7 +5590,7 @@
         </is>
       </c>
       <c r="G125" s="2" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.62</v>
       </c>
       <c r="H125" s="2" t="inlineStr">
         <is>
@@ -5631,7 +5631,7 @@
         </is>
       </c>
       <c r="G126" s="2" t="n">
-        <v>0.64</v>
+        <v>0.67</v>
       </c>
       <c r="H126" s="2" t="inlineStr">
         <is>
@@ -5672,7 +5672,7 @@
         </is>
       </c>
       <c r="G127" s="2" t="n">
-        <v>0.4</v>
+        <v>0.42</v>
       </c>
       <c r="H127" s="2" t="inlineStr">
         <is>
@@ -5713,7 +5713,7 @@
         </is>
       </c>
       <c r="G128" s="2" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.58</v>
       </c>
       <c r="H128" s="2" t="inlineStr">
         <is>
@@ -5754,7 +5754,7 @@
         </is>
       </c>
       <c r="G129" s="2" t="n">
-        <v>0.43</v>
+        <v>0.36</v>
       </c>
       <c r="H129" s="2" t="inlineStr">
         <is>
@@ -5795,7 +5795,7 @@
         </is>
       </c>
       <c r="G130" s="2" t="n">
-        <v>0.34</v>
+        <v>0.79</v>
       </c>
       <c r="H130" s="2" t="inlineStr">
         <is>
@@ -5836,7 +5836,7 @@
         </is>
       </c>
       <c r="G131" s="2" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.51</v>
       </c>
       <c r="H131" s="2" t="inlineStr">
         <is>
@@ -5858,7 +5858,7 @@
       </c>
       <c r="C132" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #1 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.67s.</t>
+          <t>User taps Registry interactive card/button #1 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.39s.</t>
         </is>
       </c>
       <c r="D132" s="2" t="inlineStr">
@@ -5877,7 +5877,7 @@
         </is>
       </c>
       <c r="G132" s="2" t="n">
-        <v>0.67</v>
+        <v>0.39</v>
       </c>
       <c r="H132" s="2" t="inlineStr">
         <is>
@@ -5899,7 +5899,7 @@
       </c>
       <c r="C133" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #2 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.53s.</t>
+          <t>User taps Registry interactive card/button #2 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.38s.</t>
         </is>
       </c>
       <c r="D133" s="2" t="inlineStr">
@@ -5918,7 +5918,7 @@
         </is>
       </c>
       <c r="G133" s="2" t="n">
-        <v>0.53</v>
+        <v>0.38</v>
       </c>
       <c r="H133" s="2" t="inlineStr">
         <is>
@@ -5940,7 +5940,7 @@
       </c>
       <c r="C134" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #3 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.4s.</t>
+          <t>User taps Registry interactive card/button #3 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.85s.</t>
         </is>
       </c>
       <c r="D134" s="2" t="inlineStr">
@@ -5959,7 +5959,7 @@
         </is>
       </c>
       <c r="G134" s="2" t="n">
-        <v>0.4</v>
+        <v>0.85</v>
       </c>
       <c r="H134" s="2" t="inlineStr">
         <is>
@@ -5981,7 +5981,7 @@
       </c>
       <c r="C135" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #4 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.69s.</t>
+          <t>User taps Registry interactive card/button #4 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.56s.</t>
         </is>
       </c>
       <c r="D135" s="2" t="inlineStr">
@@ -6000,7 +6000,7 @@
         </is>
       </c>
       <c r="G135" s="2" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="H135" s="2" t="inlineStr">
         <is>
@@ -6022,7 +6022,7 @@
       </c>
       <c r="C136" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #5 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.42s.</t>
+          <t>User taps Registry interactive card/button #5 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.62s.</t>
         </is>
       </c>
       <c r="D136" s="2" t="inlineStr">
@@ -6041,7 +6041,7 @@
         </is>
       </c>
       <c r="G136" s="2" t="n">
-        <v>0.42</v>
+        <v>0.62</v>
       </c>
       <c r="H136" s="2" t="inlineStr">
         <is>
@@ -6063,7 +6063,7 @@
       </c>
       <c r="C137" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #6 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.66s.</t>
+          <t>User taps Registry interactive card/button #6 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.44s.</t>
         </is>
       </c>
       <c r="D137" s="2" t="inlineStr">
@@ -6082,7 +6082,7 @@
         </is>
       </c>
       <c r="G137" s="2" t="n">
-        <v>0.66</v>
+        <v>0.44</v>
       </c>
       <c r="H137" s="2" t="inlineStr">
         <is>
@@ -6104,7 +6104,7 @@
       </c>
       <c r="C138" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #7 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.58s.</t>
+          <t>User taps Registry interactive card/button #7 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.62s.</t>
         </is>
       </c>
       <c r="D138" s="2" t="inlineStr">
@@ -6123,7 +6123,7 @@
         </is>
       </c>
       <c r="G138" s="2" t="n">
-        <v>0.58</v>
+        <v>0.62</v>
       </c>
       <c r="H138" s="2" t="inlineStr">
         <is>
@@ -6145,7 +6145,7 @@
       </c>
       <c r="C139" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #8 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.36s.</t>
+          <t>User taps Registry interactive card/button #8 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.41s.</t>
         </is>
       </c>
       <c r="D139" s="2" t="inlineStr">
@@ -6164,7 +6164,7 @@
         </is>
       </c>
       <c r="G139" s="2" t="n">
-        <v>0.36</v>
+        <v>0.41</v>
       </c>
       <c r="H139" s="2" t="inlineStr">
         <is>
@@ -6186,7 +6186,7 @@
       </c>
       <c r="C140" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #9 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.6s.</t>
+          <t>User taps Registry interactive card/button #9 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.46s.</t>
         </is>
       </c>
       <c r="D140" s="2" t="inlineStr">
@@ -6205,7 +6205,7 @@
         </is>
       </c>
       <c r="G140" s="2" t="n">
-        <v>0.6</v>
+        <v>0.46</v>
       </c>
       <c r="H140" s="2" t="inlineStr">
         <is>
@@ -6227,7 +6227,7 @@
       </c>
       <c r="C141" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #10 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.6s.</t>
+          <t>User taps Registry interactive card/button #10 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.74s.</t>
         </is>
       </c>
       <c r="D141" s="2" t="inlineStr">
@@ -6246,7 +6246,7 @@
         </is>
       </c>
       <c r="G141" s="2" t="n">
-        <v>0.6</v>
+        <v>0.74</v>
       </c>
       <c r="H141" s="2" t="inlineStr">
         <is>
@@ -6268,7 +6268,7 @@
       </c>
       <c r="C142" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #11 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.53s.</t>
+          <t>User taps Registry interactive card/button #11 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.32s.</t>
         </is>
       </c>
       <c r="D142" s="2" t="inlineStr">
@@ -6287,7 +6287,7 @@
         </is>
       </c>
       <c r="G142" s="2" t="n">
-        <v>0.53</v>
+        <v>0.32</v>
       </c>
       <c r="H142" s="2" t="inlineStr">
         <is>
@@ -6350,7 +6350,7 @@
       </c>
       <c r="C144" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #13 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.51s.</t>
+          <t>User taps Registry interactive card/button #13 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.55s.</t>
         </is>
       </c>
       <c r="D144" s="2" t="inlineStr">
@@ -6369,7 +6369,7 @@
         </is>
       </c>
       <c r="G144" s="2" t="n">
-        <v>0.51</v>
+        <v>0.55</v>
       </c>
       <c r="H144" s="2" t="inlineStr">
         <is>
@@ -6391,7 +6391,7 @@
       </c>
       <c r="C145" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #14 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.46s.</t>
+          <t>User taps Registry interactive card/button #14 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.39s.</t>
         </is>
       </c>
       <c r="D145" s="2" t="inlineStr">
@@ -6410,7 +6410,7 @@
         </is>
       </c>
       <c r="G145" s="2" t="n">
-        <v>0.46</v>
+        <v>0.39</v>
       </c>
       <c r="H145" s="2" t="inlineStr">
         <is>
@@ -6432,7 +6432,7 @@
       </c>
       <c r="C146" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #15 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.65s.</t>
+          <t>User taps Registry interactive card/button #15 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.59s.</t>
         </is>
       </c>
       <c r="D146" s="2" t="inlineStr">
@@ -6451,7 +6451,7 @@
         </is>
       </c>
       <c r="G146" s="2" t="n">
-        <v>0.65</v>
+        <v>0.59</v>
       </c>
       <c r="H146" s="2" t="inlineStr">
         <is>
@@ -6473,7 +6473,7 @@
       </c>
       <c r="C147" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #16 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.53s.</t>
+          <t>User taps Registry interactive card/button #16 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.65s.</t>
         </is>
       </c>
       <c r="D147" s="2" t="inlineStr">
@@ -6492,7 +6492,7 @@
         </is>
       </c>
       <c r="G147" s="2" t="n">
-        <v>0.53</v>
+        <v>0.65</v>
       </c>
       <c r="H147" s="2" t="inlineStr">
         <is>
@@ -6514,7 +6514,7 @@
       </c>
       <c r="C148" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #17 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.32s.</t>
+          <t>User taps Registry interactive card/button #17 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.6s.</t>
         </is>
       </c>
       <c r="D148" s="2" t="inlineStr">
@@ -6533,7 +6533,7 @@
         </is>
       </c>
       <c r="G148" s="2" t="n">
-        <v>0.32</v>
+        <v>0.6</v>
       </c>
       <c r="H148" s="2" t="inlineStr">
         <is>
@@ -6555,7 +6555,7 @@
       </c>
       <c r="C149" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #18 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.84s.</t>
+          <t>User taps Registry interactive card/button #18 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.57s.</t>
         </is>
       </c>
       <c r="D149" s="2" t="inlineStr">
@@ -6574,7 +6574,7 @@
         </is>
       </c>
       <c r="G149" s="2" t="n">
-        <v>0.84</v>
+        <v>0.57</v>
       </c>
       <c r="H149" s="2" t="inlineStr">
         <is>
@@ -6596,7 +6596,7 @@
       </c>
       <c r="C150" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #19 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.68s.</t>
+          <t>User taps Registry interactive card/button #19 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.73s.</t>
         </is>
       </c>
       <c r="D150" s="2" t="inlineStr">
@@ -6615,7 +6615,7 @@
         </is>
       </c>
       <c r="G150" s="2" t="n">
-        <v>0.68</v>
+        <v>0.73</v>
       </c>
       <c r="H150" s="2" t="inlineStr">
         <is>
@@ -6637,7 +6637,7 @@
       </c>
       <c r="C151" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #20 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.79s.</t>
+          <t>User taps Registry interactive card/button #20 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.41s.</t>
         </is>
       </c>
       <c r="D151" s="2" t="inlineStr">
@@ -6656,7 +6656,7 @@
         </is>
       </c>
       <c r="G151" s="2" t="n">
-        <v>0.79</v>
+        <v>0.41</v>
       </c>
       <c r="H151" s="2" t="inlineStr">
         <is>
@@ -6678,7 +6678,7 @@
       </c>
       <c r="C152" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #21 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.46s.</t>
+          <t>User taps Registry interactive card/button #21 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.56s.</t>
         </is>
       </c>
       <c r="D152" s="2" t="inlineStr">
@@ -6697,7 +6697,7 @@
         </is>
       </c>
       <c r="G152" s="2" t="n">
-        <v>0.46</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="H152" s="2" t="inlineStr">
         <is>
@@ -6719,7 +6719,7 @@
       </c>
       <c r="C153" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #22 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.82s.</t>
+          <t>User taps Registry interactive card/button #22 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.64s.</t>
         </is>
       </c>
       <c r="D153" s="2" t="inlineStr">
@@ -6738,7 +6738,7 @@
         </is>
       </c>
       <c r="G153" s="2" t="n">
-        <v>0.82</v>
+        <v>0.64</v>
       </c>
       <c r="H153" s="2" t="inlineStr">
         <is>
@@ -6760,7 +6760,7 @@
       </c>
       <c r="C154" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #23 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.83s.</t>
+          <t>User taps Registry interactive card/button #23 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.78s.</t>
         </is>
       </c>
       <c r="D154" s="2" t="inlineStr">
@@ -6779,7 +6779,7 @@
         </is>
       </c>
       <c r="G154" s="2" t="n">
-        <v>0.83</v>
+        <v>0.78</v>
       </c>
       <c r="H154" s="2" t="inlineStr">
         <is>
@@ -6801,7 +6801,7 @@
       </c>
       <c r="C155" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #24 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.69s.</t>
+          <t>User taps Registry interactive card/button #24 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.35s.</t>
         </is>
       </c>
       <c r="D155" s="2" t="inlineStr">
@@ -6820,7 +6820,7 @@
         </is>
       </c>
       <c r="G155" s="2" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.35</v>
       </c>
       <c r="H155" s="2" t="inlineStr">
         <is>
@@ -6842,7 +6842,7 @@
       </c>
       <c r="C156" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #25 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.39s.</t>
+          <t>User taps Registry interactive card/button #25 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.62s.</t>
         </is>
       </c>
       <c r="D156" s="2" t="inlineStr">
@@ -6861,7 +6861,7 @@
         </is>
       </c>
       <c r="G156" s="2" t="n">
-        <v>0.39</v>
+        <v>0.62</v>
       </c>
       <c r="H156" s="2" t="inlineStr">
         <is>
@@ -6883,7 +6883,7 @@
       </c>
       <c r="C157" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #26 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.32s.</t>
+          <t>User taps Registry interactive card/button #26 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.54s.</t>
         </is>
       </c>
       <c r="D157" s="2" t="inlineStr">
@@ -6902,7 +6902,7 @@
         </is>
       </c>
       <c r="G157" s="2" t="n">
-        <v>0.32</v>
+        <v>0.54</v>
       </c>
       <c r="H157" s="2" t="inlineStr">
         <is>
@@ -6924,7 +6924,7 @@
       </c>
       <c r="C158" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #27 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.83s.</t>
+          <t>User taps Registry interactive card/button #27 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.61s.</t>
         </is>
       </c>
       <c r="D158" s="2" t="inlineStr">
@@ -6943,7 +6943,7 @@
         </is>
       </c>
       <c r="G158" s="2" t="n">
-        <v>0.83</v>
+        <v>0.61</v>
       </c>
       <c r="H158" s="2" t="inlineStr">
         <is>
@@ -6965,7 +6965,7 @@
       </c>
       <c r="C159" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #28 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.32s.</t>
+          <t>User taps Registry interactive card/button #28 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.79s.</t>
         </is>
       </c>
       <c r="D159" s="2" t="inlineStr">
@@ -6984,7 +6984,7 @@
         </is>
       </c>
       <c r="G159" s="2" t="n">
-        <v>0.32</v>
+        <v>0.79</v>
       </c>
       <c r="H159" s="2" t="inlineStr">
         <is>
@@ -7006,7 +7006,7 @@
       </c>
       <c r="C160" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #29 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.51s.</t>
+          <t>User taps Registry interactive card/button #29 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.44s.</t>
         </is>
       </c>
       <c r="D160" s="2" t="inlineStr">
@@ -7025,7 +7025,7 @@
         </is>
       </c>
       <c r="G160" s="2" t="n">
-        <v>0.51</v>
+        <v>0.44</v>
       </c>
       <c r="H160" s="2" t="inlineStr">
         <is>
@@ -7047,7 +7047,7 @@
       </c>
       <c r="C161" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #30 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.32s.</t>
+          <t>User taps Registry interactive card/button #30 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.78s.</t>
         </is>
       </c>
       <c r="D161" s="2" t="inlineStr">
@@ -7066,7 +7066,7 @@
         </is>
       </c>
       <c r="G161" s="2" t="n">
-        <v>0.32</v>
+        <v>0.78</v>
       </c>
       <c r="H161" s="2" t="inlineStr">
         <is>
@@ -7148,7 +7148,7 @@
         </is>
       </c>
       <c r="G163" s="2" t="n">
-        <v>0.53</v>
+        <v>0.49</v>
       </c>
       <c r="H163" s="2" t="inlineStr">
         <is>
@@ -7189,7 +7189,7 @@
         </is>
       </c>
       <c r="G164" s="2" t="n">
-        <v>0.43</v>
+        <v>0.4</v>
       </c>
       <c r="H164" s="2" t="inlineStr">
         <is>
@@ -7230,7 +7230,7 @@
         </is>
       </c>
       <c r="G165" s="2" t="n">
-        <v>0.48</v>
+        <v>0.51</v>
       </c>
       <c r="H165" s="2" t="inlineStr">
         <is>
@@ -7271,7 +7271,7 @@
         </is>
       </c>
       <c r="G166" s="2" t="n">
-        <v>0.32</v>
+        <v>0.42</v>
       </c>
       <c r="H166" s="2" t="inlineStr">
         <is>
@@ -7293,7 +7293,7 @@
       </c>
       <c r="C167" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #1 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.64s.</t>
+          <t>User taps Network diagnostic button #1 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.43s.</t>
         </is>
       </c>
       <c r="D167" s="2" t="inlineStr">
@@ -7312,7 +7312,7 @@
         </is>
       </c>
       <c r="G167" s="2" t="n">
-        <v>0.64</v>
+        <v>0.43</v>
       </c>
       <c r="H167" s="2" t="inlineStr">
         <is>
@@ -7334,7 +7334,7 @@
       </c>
       <c r="C168" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #2 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.78s.</t>
+          <t>User taps Network diagnostic button #2 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.74s.</t>
         </is>
       </c>
       <c r="D168" s="2" t="inlineStr">
@@ -7353,7 +7353,7 @@
         </is>
       </c>
       <c r="G168" s="2" t="n">
-        <v>0.78</v>
+        <v>0.74</v>
       </c>
       <c r="H168" s="2" t="inlineStr">
         <is>
@@ -7375,7 +7375,7 @@
       </c>
       <c r="C169" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #3 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.66s.</t>
+          <t>User taps Network diagnostic button #3 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.44s.</t>
         </is>
       </c>
       <c r="D169" s="2" t="inlineStr">
@@ -7394,7 +7394,7 @@
         </is>
       </c>
       <c r="G169" s="2" t="n">
-        <v>0.66</v>
+        <v>0.44</v>
       </c>
       <c r="H169" s="2" t="inlineStr">
         <is>
@@ -7416,7 +7416,7 @@
       </c>
       <c r="C170" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #4 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.38s.</t>
+          <t>User taps Network diagnostic button #4 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.67s.</t>
         </is>
       </c>
       <c r="D170" s="2" t="inlineStr">
@@ -7435,7 +7435,7 @@
         </is>
       </c>
       <c r="G170" s="2" t="n">
-        <v>0.38</v>
+        <v>0.67</v>
       </c>
       <c r="H170" s="2" t="inlineStr">
         <is>
@@ -7457,7 +7457,7 @@
       </c>
       <c r="C171" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #5 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.62s.</t>
+          <t>User taps Network diagnostic button #5 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.68s.</t>
         </is>
       </c>
       <c r="D171" s="2" t="inlineStr">
@@ -7476,7 +7476,7 @@
         </is>
       </c>
       <c r="G171" s="2" t="n">
-        <v>0.62</v>
+        <v>0.68</v>
       </c>
       <c r="H171" s="2" t="inlineStr">
         <is>
@@ -7498,7 +7498,7 @@
       </c>
       <c r="C172" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #6 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.41s.</t>
+          <t>User taps Network diagnostic button #6 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.39s.</t>
         </is>
       </c>
       <c r="D172" s="2" t="inlineStr">
@@ -7517,7 +7517,7 @@
         </is>
       </c>
       <c r="G172" s="2" t="n">
-        <v>0.41</v>
+        <v>0.39</v>
       </c>
       <c r="H172" s="2" t="inlineStr">
         <is>
@@ -7539,7 +7539,7 @@
       </c>
       <c r="C173" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #7 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.73s.</t>
+          <t>User taps Network diagnostic button #7 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.28s.</t>
         </is>
       </c>
       <c r="D173" s="2" t="inlineStr">
@@ -7558,7 +7558,7 @@
         </is>
       </c>
       <c r="G173" s="2" t="n">
-        <v>0.73</v>
+        <v>0.28</v>
       </c>
       <c r="H173" s="2" t="inlineStr">
         <is>
@@ -7580,7 +7580,7 @@
       </c>
       <c r="C174" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #8 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.47s.</t>
+          <t>User taps Network diagnostic button #8 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.41s.</t>
         </is>
       </c>
       <c r="D174" s="2" t="inlineStr">
@@ -7599,7 +7599,7 @@
         </is>
       </c>
       <c r="G174" s="2" t="n">
-        <v>0.47</v>
+        <v>0.41</v>
       </c>
       <c r="H174" s="2" t="inlineStr">
         <is>
@@ -7621,7 +7621,7 @@
       </c>
       <c r="C175" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #9 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.67s.</t>
+          <t>User taps Network diagnostic button #9 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.31s.</t>
         </is>
       </c>
       <c r="D175" s="2" t="inlineStr">
@@ -7640,7 +7640,7 @@
         </is>
       </c>
       <c r="G175" s="2" t="n">
-        <v>0.67</v>
+        <v>0.31</v>
       </c>
       <c r="H175" s="2" t="inlineStr">
         <is>
@@ -7662,7 +7662,7 @@
       </c>
       <c r="C176" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #10 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.57s.</t>
+          <t>User taps Network diagnostic button #10 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.61s.</t>
         </is>
       </c>
       <c r="D176" s="2" t="inlineStr">
@@ -7681,7 +7681,7 @@
         </is>
       </c>
       <c r="G176" s="2" t="n">
-        <v>0.57</v>
+        <v>0.61</v>
       </c>
       <c r="H176" s="2" t="inlineStr">
         <is>
@@ -7703,7 +7703,7 @@
       </c>
       <c r="C177" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #11 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.53s.</t>
+          <t>User taps Network diagnostic button #11 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.34s.</t>
         </is>
       </c>
       <c r="D177" s="2" t="inlineStr">
@@ -7722,7 +7722,7 @@
         </is>
       </c>
       <c r="G177" s="2" t="n">
-        <v>0.53</v>
+        <v>0.34</v>
       </c>
       <c r="H177" s="2" t="inlineStr">
         <is>
@@ -7744,7 +7744,7 @@
       </c>
       <c r="C178" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #12 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.56s.</t>
+          <t>User taps Network diagnostic button #12 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.78s.</t>
         </is>
       </c>
       <c r="D178" s="2" t="inlineStr">
@@ -7763,7 +7763,7 @@
         </is>
       </c>
       <c r="G178" s="2" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.78</v>
       </c>
       <c r="H178" s="2" t="inlineStr">
         <is>
@@ -7785,7 +7785,7 @@
       </c>
       <c r="C179" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #13 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.38s.</t>
+          <t>User taps Network diagnostic button #13 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.6s.</t>
         </is>
       </c>
       <c r="D179" s="2" t="inlineStr">
@@ -7804,7 +7804,7 @@
         </is>
       </c>
       <c r="G179" s="2" t="n">
-        <v>0.38</v>
+        <v>0.6</v>
       </c>
       <c r="H179" s="2" t="inlineStr">
         <is>
@@ -7826,7 +7826,7 @@
       </c>
       <c r="C180" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #14 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.52s.</t>
+          <t>User taps Network diagnostic button #14 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.57s.</t>
         </is>
       </c>
       <c r="D180" s="2" t="inlineStr">
@@ -7845,7 +7845,7 @@
         </is>
       </c>
       <c r="G180" s="2" t="n">
-        <v>0.52</v>
+        <v>0.57</v>
       </c>
       <c r="H180" s="2" t="inlineStr">
         <is>
@@ -7867,7 +7867,7 @@
       </c>
       <c r="C181" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #15 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.6s.</t>
+          <t>User taps Network diagnostic button #15 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.46s.</t>
         </is>
       </c>
       <c r="D181" s="2" t="inlineStr">
@@ -7886,7 +7886,7 @@
         </is>
       </c>
       <c r="G181" s="2" t="n">
-        <v>0.6</v>
+        <v>0.46</v>
       </c>
       <c r="H181" s="2" t="inlineStr">
         <is>
@@ -7908,7 +7908,7 @@
       </c>
       <c r="C182" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #16 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.59s.</t>
+          <t>User taps Network diagnostic button #16 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.7s.</t>
         </is>
       </c>
       <c r="D182" s="2" t="inlineStr">
@@ -7927,7 +7927,7 @@
         </is>
       </c>
       <c r="G182" s="2" t="n">
-        <v>0.59</v>
+        <v>0.7</v>
       </c>
       <c r="H182" s="2" t="inlineStr">
         <is>
@@ -7949,7 +7949,7 @@
       </c>
       <c r="C183" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #17 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.71s.</t>
+          <t>User taps Network diagnostic button #17 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.32s.</t>
         </is>
       </c>
       <c r="D183" s="2" t="inlineStr">
@@ -7968,7 +7968,7 @@
         </is>
       </c>
       <c r="G183" s="2" t="n">
-        <v>0.71</v>
+        <v>0.32</v>
       </c>
       <c r="H183" s="2" t="inlineStr">
         <is>
@@ -7990,7 +7990,7 @@
       </c>
       <c r="C184" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #18 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.78s.</t>
+          <t>User taps Network diagnostic button #18 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.45s.</t>
         </is>
       </c>
       <c r="D184" s="2" t="inlineStr">
@@ -8009,7 +8009,7 @@
         </is>
       </c>
       <c r="G184" s="2" t="n">
-        <v>0.78</v>
+        <v>0.45</v>
       </c>
       <c r="H184" s="2" t="inlineStr">
         <is>
@@ -8031,7 +8031,7 @@
       </c>
       <c r="C185" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #19 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.75s.</t>
+          <t>User taps Network diagnostic button #19 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.47s.</t>
         </is>
       </c>
       <c r="D185" s="2" t="inlineStr">
@@ -8050,7 +8050,7 @@
         </is>
       </c>
       <c r="G185" s="2" t="n">
-        <v>0.75</v>
+        <v>0.47</v>
       </c>
       <c r="H185" s="2" t="inlineStr">
         <is>
@@ -8072,7 +8072,7 @@
       </c>
       <c r="C186" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #20 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.28s.</t>
+          <t>User taps Network diagnostic button #20 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.73s.</t>
         </is>
       </c>
       <c r="D186" s="2" t="inlineStr">
@@ -8091,7 +8091,7 @@
         </is>
       </c>
       <c r="G186" s="2" t="n">
-        <v>0.28</v>
+        <v>0.73</v>
       </c>
       <c r="H186" s="2" t="inlineStr">
         <is>
@@ -8113,7 +8113,7 @@
       </c>
       <c r="C187" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #21 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.42s.</t>
+          <t>User taps Network diagnostic button #21 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.53s.</t>
         </is>
       </c>
       <c r="D187" s="2" t="inlineStr">
@@ -8132,7 +8132,7 @@
         </is>
       </c>
       <c r="G187" s="2" t="n">
-        <v>0.42</v>
+        <v>0.53</v>
       </c>
       <c r="H187" s="2" t="inlineStr">
         <is>
@@ -8154,7 +8154,7 @@
       </c>
       <c r="C188" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #22 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.34s.</t>
+          <t>User taps Network diagnostic button #22 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.65s.</t>
         </is>
       </c>
       <c r="D188" s="2" t="inlineStr">
@@ -8173,7 +8173,7 @@
         </is>
       </c>
       <c r="G188" s="2" t="n">
-        <v>0.34</v>
+        <v>0.65</v>
       </c>
       <c r="H188" s="2" t="inlineStr">
         <is>
@@ -8195,7 +8195,7 @@
       </c>
       <c r="C189" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #23 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.55s.</t>
+          <t>User taps Network diagnostic button #23 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.59s.</t>
         </is>
       </c>
       <c r="D189" s="2" t="inlineStr">
@@ -8214,7 +8214,7 @@
         </is>
       </c>
       <c r="G189" s="2" t="n">
-        <v>0.55</v>
+        <v>0.59</v>
       </c>
       <c r="H189" s="2" t="inlineStr">
         <is>
@@ -8236,7 +8236,7 @@
       </c>
       <c r="C190" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #24 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.45s.</t>
+          <t>User taps Network diagnostic button #24 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.54s.</t>
         </is>
       </c>
       <c r="D190" s="2" t="inlineStr">
@@ -8255,7 +8255,7 @@
         </is>
       </c>
       <c r="G190" s="2" t="n">
-        <v>0.45</v>
+        <v>0.54</v>
       </c>
       <c r="H190" s="2" t="inlineStr">
         <is>
@@ -8277,7 +8277,7 @@
       </c>
       <c r="C191" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #25 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.73s.</t>
+          <t>User taps Network diagnostic button #25 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.69s.</t>
         </is>
       </c>
       <c r="D191" s="2" t="inlineStr">
@@ -8296,7 +8296,7 @@
         </is>
       </c>
       <c r="G191" s="2" t="n">
-        <v>0.73</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="H191" s="2" t="inlineStr">
         <is>
@@ -8318,7 +8318,7 @@
       </c>
       <c r="C192" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #26 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.44s.</t>
+          <t>User taps Network diagnostic button #26 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.69s.</t>
         </is>
       </c>
       <c r="D192" s="2" t="inlineStr">
@@ -8337,7 +8337,7 @@
         </is>
       </c>
       <c r="G192" s="2" t="n">
-        <v>0.44</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="H192" s="2" t="inlineStr">
         <is>
@@ -8359,7 +8359,7 @@
       </c>
       <c r="C193" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #27 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.57s.</t>
+          <t>User taps Network diagnostic button #27 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.67s.</t>
         </is>
       </c>
       <c r="D193" s="2" t="inlineStr">
@@ -8378,7 +8378,7 @@
         </is>
       </c>
       <c r="G193" s="2" t="n">
-        <v>0.57</v>
+        <v>0.67</v>
       </c>
       <c r="H193" s="2" t="inlineStr">
         <is>
@@ -8400,7 +8400,7 @@
       </c>
       <c r="C194" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #28 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.47s.</t>
+          <t>User taps Network diagnostic button #28 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.6s.</t>
         </is>
       </c>
       <c r="D194" s="2" t="inlineStr">
@@ -8419,7 +8419,7 @@
         </is>
       </c>
       <c r="G194" s="2" t="n">
-        <v>0.47</v>
+        <v>0.6</v>
       </c>
       <c r="H194" s="2" t="inlineStr">
         <is>
@@ -8441,7 +8441,7 @@
       </c>
       <c r="C195" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #29 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.52s.</t>
+          <t>User taps Network diagnostic button #29 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.43s.</t>
         </is>
       </c>
       <c r="D195" s="2" t="inlineStr">
@@ -8460,7 +8460,7 @@
         </is>
       </c>
       <c r="G195" s="2" t="n">
-        <v>0.52</v>
+        <v>0.43</v>
       </c>
       <c r="H195" s="2" t="inlineStr">
         <is>
@@ -8482,7 +8482,7 @@
       </c>
       <c r="C196" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #30 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.63s.</t>
+          <t>User taps Network diagnostic button #30 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.68s.</t>
         </is>
       </c>
       <c r="D196" s="2" t="inlineStr">
@@ -8501,7 +8501,7 @@
         </is>
       </c>
       <c r="G196" s="2" t="n">
-        <v>0.63</v>
+        <v>0.68</v>
       </c>
       <c r="H196" s="2" t="inlineStr">
         <is>
@@ -8542,7 +8542,7 @@
         </is>
       </c>
       <c r="G197" s="2" t="n">
-        <v>0.88</v>
+        <v>1.16</v>
       </c>
       <c r="H197" s="2" t="inlineStr">
         <is>
@@ -8583,7 +8583,7 @@
         </is>
       </c>
       <c r="G198" s="2" t="n">
-        <v>0.59</v>
+        <v>0.47</v>
       </c>
       <c r="H198" s="2" t="inlineStr">
         <is>
@@ -8624,7 +8624,7 @@
         </is>
       </c>
       <c r="G199" s="2" t="n">
-        <v>0.5</v>
+        <v>1.12</v>
       </c>
       <c r="H199" s="2" t="inlineStr">
         <is>
@@ -8665,7 +8665,7 @@
         </is>
       </c>
       <c r="G200" s="2" t="n">
-        <v>0.8</v>
+        <v>1.17</v>
       </c>
       <c r="H200" s="2" t="inlineStr">
         <is>
@@ -8706,7 +8706,7 @@
         </is>
       </c>
       <c r="G201" s="2" t="n">
-        <v>0.86</v>
+        <v>0.95</v>
       </c>
       <c r="H201" s="2" t="inlineStr">
         <is>
@@ -8747,7 +8747,7 @@
         </is>
       </c>
       <c r="G202" s="2" t="n">
-        <v>0.76</v>
+        <v>0.67</v>
       </c>
       <c r="H202" s="2" t="inlineStr">
         <is>
@@ -8788,7 +8788,7 @@
         </is>
       </c>
       <c r="G203" s="2" t="n">
-        <v>1.13</v>
+        <v>0.89</v>
       </c>
       <c r="H203" s="2" t="inlineStr">
         <is>
@@ -8810,7 +8810,7 @@
       </c>
       <c r="C204" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #1 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.85s.</t>
+          <t>User executes touch gesture #1 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.95s.</t>
         </is>
       </c>
       <c r="D204" s="2" t="inlineStr">
@@ -8829,7 +8829,7 @@
         </is>
       </c>
       <c r="G204" s="2" t="n">
-        <v>0.85</v>
+        <v>0.95</v>
       </c>
       <c r="H204" s="2" t="inlineStr">
         <is>
@@ -8851,7 +8851,7 @@
       </c>
       <c r="C205" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #2 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.48s.</t>
+          <t>User executes touch gesture #2 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.43s.</t>
         </is>
       </c>
       <c r="D205" s="2" t="inlineStr">
@@ -8870,7 +8870,7 @@
         </is>
       </c>
       <c r="G205" s="2" t="n">
-        <v>0.48</v>
+        <v>0.43</v>
       </c>
       <c r="H205" s="2" t="inlineStr">
         <is>
@@ -8892,7 +8892,7 @@
       </c>
       <c r="C206" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #3 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.05s.</t>
+          <t>User executes touch gesture #3 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.92s.</t>
         </is>
       </c>
       <c r="D206" s="2" t="inlineStr">
@@ -8911,7 +8911,7 @@
         </is>
       </c>
       <c r="G206" s="2" t="n">
-        <v>1.05</v>
+        <v>0.92</v>
       </c>
       <c r="H206" s="2" t="inlineStr">
         <is>
@@ -8933,7 +8933,7 @@
       </c>
       <c r="C207" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #4 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.45s.</t>
+          <t>User executes touch gesture #4 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.7s.</t>
         </is>
       </c>
       <c r="D207" s="2" t="inlineStr">
@@ -8952,7 +8952,7 @@
         </is>
       </c>
       <c r="G207" s="2" t="n">
-        <v>0.45</v>
+        <v>0.7</v>
       </c>
       <c r="H207" s="2" t="inlineStr">
         <is>
@@ -8974,7 +8974,7 @@
       </c>
       <c r="C208" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #5 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.68s.</t>
+          <t>User executes touch gesture #5 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.02s.</t>
         </is>
       </c>
       <c r="D208" s="2" t="inlineStr">
@@ -8993,7 +8993,7 @@
         </is>
       </c>
       <c r="G208" s="2" t="n">
-        <v>0.68</v>
+        <v>1.02</v>
       </c>
       <c r="H208" s="2" t="inlineStr">
         <is>
@@ -9015,7 +9015,7 @@
       </c>
       <c r="C209" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #6 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.51s.</t>
+          <t>User executes touch gesture #6 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.45s.</t>
         </is>
       </c>
       <c r="D209" s="2" t="inlineStr">
@@ -9034,7 +9034,7 @@
         </is>
       </c>
       <c r="G209" s="2" t="n">
-        <v>0.51</v>
+        <v>0.45</v>
       </c>
       <c r="H209" s="2" t="inlineStr">
         <is>
@@ -9056,7 +9056,7 @@
       </c>
       <c r="C210" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #7 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.69s.</t>
+          <t>User executes touch gesture #7 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.63s.</t>
         </is>
       </c>
       <c r="D210" s="2" t="inlineStr">
@@ -9075,7 +9075,7 @@
         </is>
       </c>
       <c r="G210" s="2" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.63</v>
       </c>
       <c r="H210" s="2" t="inlineStr">
         <is>
@@ -9097,7 +9097,7 @@
       </c>
       <c r="C211" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #8 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.42s.</t>
+          <t>User executes touch gesture #8 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.19s.</t>
         </is>
       </c>
       <c r="D211" s="2" t="inlineStr">
@@ -9116,7 +9116,7 @@
         </is>
       </c>
       <c r="G211" s="2" t="n">
-        <v>0.42</v>
+        <v>1.19</v>
       </c>
       <c r="H211" s="2" t="inlineStr">
         <is>
@@ -9138,7 +9138,7 @@
       </c>
       <c r="C212" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #9 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.63s.</t>
+          <t>User executes touch gesture #9 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.73s.</t>
         </is>
       </c>
       <c r="D212" s="2" t="inlineStr">
@@ -9157,7 +9157,7 @@
         </is>
       </c>
       <c r="G212" s="2" t="n">
-        <v>0.63</v>
+        <v>0.73</v>
       </c>
       <c r="H212" s="2" t="inlineStr">
         <is>
@@ -9179,7 +9179,7 @@
       </c>
       <c r="C213" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #10 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.46s.</t>
+          <t>User executes touch gesture #10 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.25s.</t>
         </is>
       </c>
       <c r="D213" s="2" t="inlineStr">
@@ -9198,7 +9198,7 @@
         </is>
       </c>
       <c r="G213" s="2" t="n">
-        <v>0.46</v>
+        <v>1.25</v>
       </c>
       <c r="H213" s="2" t="inlineStr">
         <is>
@@ -9220,7 +9220,7 @@
       </c>
       <c r="C214" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #11 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.42s.</t>
+          <t>User executes touch gesture #11 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.01s.</t>
         </is>
       </c>
       <c r="D214" s="2" t="inlineStr">
@@ -9239,7 +9239,7 @@
         </is>
       </c>
       <c r="G214" s="2" t="n">
-        <v>0.42</v>
+        <v>1.01</v>
       </c>
       <c r="H214" s="2" t="inlineStr">
         <is>
@@ -9261,7 +9261,7 @@
       </c>
       <c r="C215" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #12 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.09s.</t>
+          <t>User executes touch gesture #12 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.63s.</t>
         </is>
       </c>
       <c r="D215" s="2" t="inlineStr">
@@ -9280,7 +9280,7 @@
         </is>
       </c>
       <c r="G215" s="2" t="n">
-        <v>1.09</v>
+        <v>0.63</v>
       </c>
       <c r="H215" s="2" t="inlineStr">
         <is>
@@ -9302,7 +9302,7 @@
       </c>
       <c r="C216" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #13 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.24s.</t>
+          <t>User executes touch gesture #13 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.77s.</t>
         </is>
       </c>
       <c r="D216" s="2" t="inlineStr">
@@ -9321,7 +9321,7 @@
         </is>
       </c>
       <c r="G216" s="2" t="n">
-        <v>1.24</v>
+        <v>0.77</v>
       </c>
       <c r="H216" s="2" t="inlineStr">
         <is>
@@ -9343,7 +9343,7 @@
       </c>
       <c r="C217" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #14 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.93s.</t>
+          <t>User executes touch gesture #14 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.97s.</t>
         </is>
       </c>
       <c r="D217" s="2" t="inlineStr">
@@ -9362,7 +9362,7 @@
         </is>
       </c>
       <c r="G217" s="2" t="n">
-        <v>0.93</v>
+        <v>0.97</v>
       </c>
       <c r="H217" s="2" t="inlineStr">
         <is>
@@ -9384,7 +9384,7 @@
       </c>
       <c r="C218" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #15 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.63s.</t>
+          <t>User executes touch gesture #15 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.25s.</t>
         </is>
       </c>
       <c r="D218" s="2" t="inlineStr">
@@ -9403,7 +9403,7 @@
         </is>
       </c>
       <c r="G218" s="2" t="n">
-        <v>0.63</v>
+        <v>1.25</v>
       </c>
       <c r="H218" s="2" t="inlineStr">
         <is>
@@ -9425,7 +9425,7 @@
       </c>
       <c r="C219" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #16 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.07s.</t>
+          <t>User executes touch gesture #16 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.38s.</t>
         </is>
       </c>
       <c r="D219" s="2" t="inlineStr">
@@ -9444,7 +9444,7 @@
         </is>
       </c>
       <c r="G219" s="2" t="n">
-        <v>1.07</v>
+        <v>0.38</v>
       </c>
       <c r="H219" s="2" t="inlineStr">
         <is>
@@ -9466,7 +9466,7 @@
       </c>
       <c r="C220" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #17 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.98s.</t>
+          <t>User executes touch gesture #17 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.74s.</t>
         </is>
       </c>
       <c r="D220" s="2" t="inlineStr">
@@ -9485,7 +9485,7 @@
         </is>
       </c>
       <c r="G220" s="2" t="n">
-        <v>0.98</v>
+        <v>0.74</v>
       </c>
       <c r="H220" s="2" t="inlineStr">
         <is>
@@ -9507,7 +9507,7 @@
       </c>
       <c r="C221" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #18 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.67s.</t>
+          <t>User executes touch gesture #18 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.59s.</t>
         </is>
       </c>
       <c r="D221" s="2" t="inlineStr">
@@ -9526,7 +9526,7 @@
         </is>
       </c>
       <c r="G221" s="2" t="n">
-        <v>0.67</v>
+        <v>0.59</v>
       </c>
       <c r="H221" s="2" t="inlineStr">
         <is>
@@ -9548,7 +9548,7 @@
       </c>
       <c r="C222" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #19 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.98s.</t>
+          <t>User executes touch gesture #19 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.17s.</t>
         </is>
       </c>
       <c r="D222" s="2" t="inlineStr">
@@ -9567,7 +9567,7 @@
         </is>
       </c>
       <c r="G222" s="2" t="n">
-        <v>0.98</v>
+        <v>1.17</v>
       </c>
       <c r="H222" s="2" t="inlineStr">
         <is>
@@ -9589,7 +9589,7 @@
       </c>
       <c r="C223" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #20 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.21s.</t>
+          <t>User executes touch gesture #20 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.06s.</t>
         </is>
       </c>
       <c r="D223" s="2" t="inlineStr">
@@ -9608,7 +9608,7 @@
         </is>
       </c>
       <c r="G223" s="2" t="n">
-        <v>1.21</v>
+        <v>1.06</v>
       </c>
       <c r="H223" s="2" t="inlineStr">
         <is>
@@ -9630,7 +9630,7 @@
       </c>
       <c r="C224" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #21 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.84s.</t>
+          <t>User executes touch gesture #21 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.15s.</t>
         </is>
       </c>
       <c r="D224" s="2" t="inlineStr">
@@ -9649,7 +9649,7 @@
         </is>
       </c>
       <c r="G224" s="2" t="n">
-        <v>0.84</v>
+        <v>1.15</v>
       </c>
       <c r="H224" s="2" t="inlineStr">
         <is>
@@ -9671,7 +9671,7 @@
       </c>
       <c r="C225" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #22 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.93s.</t>
+          <t>User executes touch gesture #22 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.71s.</t>
         </is>
       </c>
       <c r="D225" s="2" t="inlineStr">
@@ -9690,7 +9690,7 @@
         </is>
       </c>
       <c r="G225" s="2" t="n">
-        <v>0.93</v>
+        <v>0.71</v>
       </c>
       <c r="H225" s="2" t="inlineStr">
         <is>
@@ -9712,7 +9712,7 @@
       </c>
       <c r="C226" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #23 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.08s.</t>
+          <t>User executes touch gesture #23 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.72s.</t>
         </is>
       </c>
       <c r="D226" s="2" t="inlineStr">
@@ -9731,7 +9731,7 @@
         </is>
       </c>
       <c r="G226" s="2" t="n">
-        <v>1.08</v>
+        <v>0.72</v>
       </c>
       <c r="H226" s="2" t="inlineStr">
         <is>
@@ -9753,7 +9753,7 @@
       </c>
       <c r="C227" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #24 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.68s.</t>
+          <t>User executes touch gesture #24 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.97s.</t>
         </is>
       </c>
       <c r="D227" s="2" t="inlineStr">
@@ -9772,7 +9772,7 @@
         </is>
       </c>
       <c r="G227" s="2" t="n">
-        <v>0.68</v>
+        <v>0.97</v>
       </c>
       <c r="H227" s="2" t="inlineStr">
         <is>
@@ -9794,7 +9794,7 @@
       </c>
       <c r="C228" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #25 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.06s.</t>
+          <t>User executes touch gesture #25 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.71s.</t>
         </is>
       </c>
       <c r="D228" s="2" t="inlineStr">
@@ -9813,7 +9813,7 @@
         </is>
       </c>
       <c r="G228" s="2" t="n">
-        <v>1.06</v>
+        <v>0.71</v>
       </c>
       <c r="H228" s="2" t="inlineStr">
         <is>
@@ -9835,7 +9835,7 @@
       </c>
       <c r="C229" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #26 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.77s.</t>
+          <t>User executes touch gesture #26 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.94s.</t>
         </is>
       </c>
       <c r="D229" s="2" t="inlineStr">
@@ -9854,7 +9854,7 @@
         </is>
       </c>
       <c r="G229" s="2" t="n">
-        <v>0.77</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="H229" s="2" t="inlineStr">
         <is>
@@ -9876,7 +9876,7 @@
       </c>
       <c r="C230" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #27 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.12s.</t>
+          <t>User executes touch gesture #27 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.72s.</t>
         </is>
       </c>
       <c r="D230" s="2" t="inlineStr">
@@ -9895,7 +9895,7 @@
         </is>
       </c>
       <c r="G230" s="2" t="n">
-        <v>1.12</v>
+        <v>0.72</v>
       </c>
       <c r="H230" s="2" t="inlineStr">
         <is>
@@ -9917,7 +9917,7 @@
       </c>
       <c r="C231" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #28 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.52s.</t>
+          <t>User executes touch gesture #28 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.94s.</t>
         </is>
       </c>
       <c r="D231" s="2" t="inlineStr">
@@ -9936,7 +9936,7 @@
         </is>
       </c>
       <c r="G231" s="2" t="n">
-        <v>0.52</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="H231" s="2" t="inlineStr">
         <is>
@@ -9977,7 +9977,7 @@
         </is>
       </c>
       <c r="G232" s="2" t="n">
-        <v>0.58</v>
+        <v>0.73</v>
       </c>
       <c r="H232" s="2" t="inlineStr">
         <is>
@@ -10018,7 +10018,7 @@
         </is>
       </c>
       <c r="G233" s="2" t="n">
-        <v>0.51</v>
+        <v>0.38</v>
       </c>
       <c r="H233" s="2" t="inlineStr">
         <is>
@@ -10059,7 +10059,7 @@
         </is>
       </c>
       <c r="G234" s="2" t="n">
-        <v>0.52</v>
+        <v>0.37</v>
       </c>
       <c r="H234" s="2" t="inlineStr">
         <is>
@@ -10100,7 +10100,7 @@
         </is>
       </c>
       <c r="G235" s="2" t="n">
-        <v>0.49</v>
+        <v>0.72</v>
       </c>
       <c r="H235" s="2" t="inlineStr">
         <is>
@@ -10122,7 +10122,7 @@
       </c>
       <c r="C236" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #1 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.64s.</t>
+          <t>User executes offline storage operation #1 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.73s.</t>
         </is>
       </c>
       <c r="D236" s="2" t="inlineStr">
@@ -10141,7 +10141,7 @@
         </is>
       </c>
       <c r="G236" s="2" t="n">
-        <v>0.64</v>
+        <v>0.73</v>
       </c>
       <c r="H236" s="2" t="inlineStr">
         <is>
@@ -10163,7 +10163,7 @@
       </c>
       <c r="C237" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #2 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.54s.</t>
+          <t>User executes offline storage operation #2 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.41s.</t>
         </is>
       </c>
       <c r="D237" s="2" t="inlineStr">
@@ -10182,7 +10182,7 @@
         </is>
       </c>
       <c r="G237" s="2" t="n">
-        <v>0.54</v>
+        <v>0.41</v>
       </c>
       <c r="H237" s="2" t="inlineStr">
         <is>
@@ -10204,7 +10204,7 @@
       </c>
       <c r="C238" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #3 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.3s.</t>
+          <t>User executes offline storage operation #3 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.31s.</t>
         </is>
       </c>
       <c r="D238" s="2" t="inlineStr">
@@ -10223,7 +10223,7 @@
         </is>
       </c>
       <c r="G238" s="2" t="n">
-        <v>0.3</v>
+        <v>0.31</v>
       </c>
       <c r="H238" s="2" t="inlineStr">
         <is>
@@ -10245,7 +10245,7 @@
       </c>
       <c r="C239" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #4 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.73s.</t>
+          <t>User executes offline storage operation #4 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.39s.</t>
         </is>
       </c>
       <c r="D239" s="2" t="inlineStr">
@@ -10264,7 +10264,7 @@
         </is>
       </c>
       <c r="G239" s="2" t="n">
-        <v>0.73</v>
+        <v>0.39</v>
       </c>
       <c r="H239" s="2" t="inlineStr">
         <is>
@@ -10286,7 +10286,7 @@
       </c>
       <c r="C240" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #5 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.41s.</t>
+          <t>User executes offline storage operation #5 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.61s.</t>
         </is>
       </c>
       <c r="D240" s="2" t="inlineStr">
@@ -10305,7 +10305,7 @@
         </is>
       </c>
       <c r="G240" s="2" t="n">
-        <v>0.41</v>
+        <v>0.61</v>
       </c>
       <c r="H240" s="2" t="inlineStr">
         <is>
@@ -10327,7 +10327,7 @@
       </c>
       <c r="C241" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #6 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.59s.</t>
+          <t>User executes offline storage operation #6 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.27s.</t>
         </is>
       </c>
       <c r="D241" s="2" t="inlineStr">
@@ -10346,7 +10346,7 @@
         </is>
       </c>
       <c r="G241" s="2" t="n">
-        <v>0.59</v>
+        <v>0.27</v>
       </c>
       <c r="H241" s="2" t="inlineStr">
         <is>
@@ -10368,7 +10368,7 @@
       </c>
       <c r="C242" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #7 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.44s.</t>
+          <t>User executes offline storage operation #7 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.58s.</t>
         </is>
       </c>
       <c r="D242" s="2" t="inlineStr">
@@ -10387,7 +10387,7 @@
         </is>
       </c>
       <c r="G242" s="2" t="n">
-        <v>0.44</v>
+        <v>0.58</v>
       </c>
       <c r="H242" s="2" t="inlineStr">
         <is>
@@ -10409,7 +10409,7 @@
       </c>
       <c r="C243" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #8 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.67s.</t>
+          <t>User executes offline storage operation #8 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.42s.</t>
         </is>
       </c>
       <c r="D243" s="2" t="inlineStr">
@@ -10428,7 +10428,7 @@
         </is>
       </c>
       <c r="G243" s="2" t="n">
-        <v>0.67</v>
+        <v>0.42</v>
       </c>
       <c r="H243" s="2" t="inlineStr">
         <is>
@@ -10450,7 +10450,7 @@
       </c>
       <c r="C244" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #9 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.27s.</t>
+          <t>User executes offline storage operation #9 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.58s.</t>
         </is>
       </c>
       <c r="D244" s="2" t="inlineStr">
@@ -10469,7 +10469,7 @@
         </is>
       </c>
       <c r="G244" s="2" t="n">
-        <v>0.27</v>
+        <v>0.58</v>
       </c>
       <c r="H244" s="2" t="inlineStr">
         <is>
@@ -10491,7 +10491,7 @@
       </c>
       <c r="C245" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #10 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.46s.</t>
+          <t>User executes offline storage operation #10 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.32s.</t>
         </is>
       </c>
       <c r="D245" s="2" t="inlineStr">
@@ -10510,7 +10510,7 @@
         </is>
       </c>
       <c r="G245" s="2" t="n">
-        <v>0.46</v>
+        <v>0.32</v>
       </c>
       <c r="H245" s="2" t="inlineStr">
         <is>
@@ -10532,7 +10532,7 @@
       </c>
       <c r="C246" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #11 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.58s.</t>
+          <t>User executes offline storage operation #11 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.41s.</t>
         </is>
       </c>
       <c r="D246" s="2" t="inlineStr">
@@ -10551,7 +10551,7 @@
         </is>
       </c>
       <c r="G246" s="2" t="n">
-        <v>0.58</v>
+        <v>0.41</v>
       </c>
       <c r="H246" s="2" t="inlineStr">
         <is>
@@ -10573,7 +10573,7 @@
       </c>
       <c r="C247" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #12 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.41s.</t>
+          <t>User executes offline storage operation #12 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.26s.</t>
         </is>
       </c>
       <c r="D247" s="2" t="inlineStr">
@@ -10592,7 +10592,7 @@
         </is>
       </c>
       <c r="G247" s="2" t="n">
-        <v>0.41</v>
+        <v>0.26</v>
       </c>
       <c r="H247" s="2" t="inlineStr">
         <is>
@@ -10614,7 +10614,7 @@
       </c>
       <c r="C248" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #13 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.45s.</t>
+          <t>User executes offline storage operation #13 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.53s.</t>
         </is>
       </c>
       <c r="D248" s="2" t="inlineStr">
@@ -10633,7 +10633,7 @@
         </is>
       </c>
       <c r="G248" s="2" t="n">
-        <v>0.45</v>
+        <v>0.53</v>
       </c>
       <c r="H248" s="2" t="inlineStr">
         <is>
@@ -10655,7 +10655,7 @@
       </c>
       <c r="C249" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #14 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.39s.</t>
+          <t>User executes offline storage operation #14 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.65s.</t>
         </is>
       </c>
       <c r="D249" s="2" t="inlineStr">
@@ -10674,7 +10674,7 @@
         </is>
       </c>
       <c r="G249" s="2" t="n">
-        <v>0.39</v>
+        <v>0.65</v>
       </c>
       <c r="H249" s="2" t="inlineStr">
         <is>
@@ -10696,7 +10696,7 @@
       </c>
       <c r="C250" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #15 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.55s.</t>
+          <t>User executes offline storage operation #15 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.65s.</t>
         </is>
       </c>
       <c r="D250" s="2" t="inlineStr">
@@ -10715,7 +10715,7 @@
         </is>
       </c>
       <c r="G250" s="2" t="n">
-        <v>0.55</v>
+        <v>0.65</v>
       </c>
       <c r="H250" s="2" t="inlineStr">
         <is>
@@ -10737,7 +10737,7 @@
       </c>
       <c r="C251" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #16 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.65s.</t>
+          <t>User executes offline storage operation #16 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.61s.</t>
         </is>
       </c>
       <c r="D251" s="2" t="inlineStr">
@@ -10756,7 +10756,7 @@
         </is>
       </c>
       <c r="G251" s="2" t="n">
-        <v>0.65</v>
+        <v>0.61</v>
       </c>
       <c r="H251" s="2" t="inlineStr">
         <is>
@@ -10778,7 +10778,7 @@
       </c>
       <c r="C252" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #17 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.5s.</t>
+          <t>User executes offline storage operation #17 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.47s.</t>
         </is>
       </c>
       <c r="D252" s="2" t="inlineStr">
@@ -10797,7 +10797,7 @@
         </is>
       </c>
       <c r="G252" s="2" t="n">
-        <v>0.5</v>
+        <v>0.47</v>
       </c>
       <c r="H252" s="2" t="inlineStr">
         <is>
@@ -10819,7 +10819,7 @@
       </c>
       <c r="C253" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #18 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.27s.</t>
+          <t>User executes offline storage operation #18 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.26s.</t>
         </is>
       </c>
       <c r="D253" s="2" t="inlineStr">
@@ -10838,7 +10838,7 @@
         </is>
       </c>
       <c r="G253" s="2" t="n">
-        <v>0.27</v>
+        <v>0.26</v>
       </c>
       <c r="H253" s="2" t="inlineStr">
         <is>
@@ -10860,7 +10860,7 @@
       </c>
       <c r="C254" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #19 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.29s.</t>
+          <t>User executes offline storage operation #19 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.43s.</t>
         </is>
       </c>
       <c r="D254" s="2" t="inlineStr">
@@ -10879,7 +10879,7 @@
         </is>
       </c>
       <c r="G254" s="2" t="n">
-        <v>0.29</v>
+        <v>0.43</v>
       </c>
       <c r="H254" s="2" t="inlineStr">
         <is>
@@ -10901,7 +10901,7 @@
       </c>
       <c r="C255" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #20 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.41s.</t>
+          <t>User executes offline storage operation #20 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.67s.</t>
         </is>
       </c>
       <c r="D255" s="2" t="inlineStr">
@@ -10920,7 +10920,7 @@
         </is>
       </c>
       <c r="G255" s="2" t="n">
-        <v>0.41</v>
+        <v>0.67</v>
       </c>
       <c r="H255" s="2" t="inlineStr">
         <is>
@@ -10942,7 +10942,7 @@
       </c>
       <c r="C256" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #21 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.27s.</t>
+          <t>User executes offline storage operation #21 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.66s.</t>
         </is>
       </c>
       <c r="D256" s="2" t="inlineStr">
@@ -10961,7 +10961,7 @@
         </is>
       </c>
       <c r="G256" s="2" t="n">
-        <v>0.27</v>
+        <v>0.66</v>
       </c>
       <c r="H256" s="2" t="inlineStr">
         <is>
@@ -10983,7 +10983,7 @@
       </c>
       <c r="C257" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #22 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.54s.</t>
+          <t>User executes offline storage operation #22 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.28s.</t>
         </is>
       </c>
       <c r="D257" s="2" t="inlineStr">
@@ -11002,7 +11002,7 @@
         </is>
       </c>
       <c r="G257" s="2" t="n">
-        <v>0.54</v>
+        <v>0.28</v>
       </c>
       <c r="H257" s="2" t="inlineStr">
         <is>
@@ -11024,7 +11024,7 @@
       </c>
       <c r="C258" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #23 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.3s.</t>
+          <t>User executes offline storage operation #23 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.47s.</t>
         </is>
       </c>
       <c r="D258" s="2" t="inlineStr">
@@ -11043,7 +11043,7 @@
         </is>
       </c>
       <c r="G258" s="2" t="n">
-        <v>0.3</v>
+        <v>0.47</v>
       </c>
       <c r="H258" s="2" t="inlineStr">
         <is>
@@ -11065,7 +11065,7 @@
       </c>
       <c r="C259" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #24 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.55s.</t>
+          <t>User executes offline storage operation #24 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.45s.</t>
         </is>
       </c>
       <c r="D259" s="2" t="inlineStr">
@@ -11084,7 +11084,7 @@
         </is>
       </c>
       <c r="G259" s="2" t="n">
-        <v>0.55</v>
+        <v>0.45</v>
       </c>
       <c r="H259" s="2" t="inlineStr">
         <is>
@@ -11106,7 +11106,7 @@
       </c>
       <c r="C260" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #25 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.72s.</t>
+          <t>User executes offline storage operation #25 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.58s.</t>
         </is>
       </c>
       <c r="D260" s="2" t="inlineStr">
@@ -11125,7 +11125,7 @@
         </is>
       </c>
       <c r="G260" s="2" t="n">
-        <v>0.72</v>
+        <v>0.58</v>
       </c>
       <c r="H260" s="2" t="inlineStr">
         <is>
@@ -11147,7 +11147,7 @@
       </c>
       <c r="C261" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #26 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.49s.</t>
+          <t>User executes offline storage operation #26 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.27s.</t>
         </is>
       </c>
       <c r="D261" s="2" t="inlineStr">
@@ -11166,7 +11166,7 @@
         </is>
       </c>
       <c r="G261" s="2" t="n">
-        <v>0.49</v>
+        <v>0.27</v>
       </c>
       <c r="H261" s="2" t="inlineStr">
         <is>
@@ -11188,7 +11188,7 @@
       </c>
       <c r="C262" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #27 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.44s.</t>
+          <t>User executes offline storage operation #27 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.59s.</t>
         </is>
       </c>
       <c r="D262" s="2" t="inlineStr">
@@ -11207,7 +11207,7 @@
         </is>
       </c>
       <c r="G262" s="2" t="n">
-        <v>0.44</v>
+        <v>0.59</v>
       </c>
       <c r="H262" s="2" t="inlineStr">
         <is>
@@ -11229,7 +11229,7 @@
       </c>
       <c r="C263" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #28 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.67s.</t>
+          <t>User executes offline storage operation #28 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.36s.</t>
         </is>
       </c>
       <c r="D263" s="2" t="inlineStr">
@@ -11248,7 +11248,7 @@
         </is>
       </c>
       <c r="G263" s="2" t="n">
-        <v>0.67</v>
+        <v>0.36</v>
       </c>
       <c r="H263" s="2" t="inlineStr">
         <is>
@@ -11270,7 +11270,7 @@
       </c>
       <c r="C264" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #29 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.61s.</t>
+          <t>User executes offline storage operation #29 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.48s.</t>
         </is>
       </c>
       <c r="D264" s="2" t="inlineStr">
@@ -11289,7 +11289,7 @@
         </is>
       </c>
       <c r="G264" s="2" t="n">
-        <v>0.61</v>
+        <v>0.48</v>
       </c>
       <c r="H264" s="2" t="inlineStr">
         <is>
@@ -11311,7 +11311,7 @@
       </c>
       <c r="C265" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #30 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.47s.</t>
+          <t>User executes offline storage operation #30 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.36s.</t>
         </is>
       </c>
       <c r="D265" s="2" t="inlineStr">
@@ -11330,7 +11330,7 @@
         </is>
       </c>
       <c r="G265" s="2" t="n">
-        <v>0.47</v>
+        <v>0.36</v>
       </c>
       <c r="H265" s="2" t="inlineStr">
         <is>
@@ -11352,7 +11352,7 @@
       </c>
       <c r="C266" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #31 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.5s.</t>
+          <t>User executes offline storage operation #31 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.52s.</t>
         </is>
       </c>
       <c r="D266" s="2" t="inlineStr">
@@ -11371,7 +11371,7 @@
         </is>
       </c>
       <c r="G266" s="2" t="n">
-        <v>0.5</v>
+        <v>0.52</v>
       </c>
       <c r="H266" s="2" t="inlineStr">
         <is>
@@ -11412,7 +11412,7 @@
         </is>
       </c>
       <c r="G267" s="2" t="n">
-        <v>0.27</v>
+        <v>0.26</v>
       </c>
       <c r="H267" s="2" t="inlineStr">
         <is>
@@ -11453,7 +11453,7 @@
         </is>
       </c>
       <c r="G268" s="2" t="n">
-        <v>0.48</v>
+        <v>0.67</v>
       </c>
       <c r="H268" s="2" t="inlineStr">
         <is>
@@ -11494,7 +11494,7 @@
         </is>
       </c>
       <c r="G269" s="2" t="n">
-        <v>0.53</v>
+        <v>0.28</v>
       </c>
       <c r="H269" s="2" t="inlineStr">
         <is>
@@ -11535,7 +11535,7 @@
         </is>
       </c>
       <c r="G270" s="2" t="n">
-        <v>0.59</v>
+        <v>0.33</v>
       </c>
       <c r="H270" s="2" t="inlineStr">
         <is>
@@ -11557,7 +11557,7 @@
       </c>
       <c r="C271" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #1 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.65s.</t>
+          <t>User tests layout/memory scenario #1 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.57s.</t>
         </is>
       </c>
       <c r="D271" s="2" t="inlineStr">
@@ -11576,7 +11576,7 @@
         </is>
       </c>
       <c r="G271" s="2" t="n">
-        <v>0.65</v>
+        <v>0.57</v>
       </c>
       <c r="H271" s="2" t="inlineStr">
         <is>
@@ -11598,7 +11598,7 @@
       </c>
       <c r="C272" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #2 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.52s.</t>
+          <t>User tests layout/memory scenario #2 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.64s.</t>
         </is>
       </c>
       <c r="D272" s="2" t="inlineStr">
@@ -11617,7 +11617,7 @@
         </is>
       </c>
       <c r="G272" s="2" t="n">
-        <v>0.52</v>
+        <v>0.64</v>
       </c>
       <c r="H272" s="2" t="inlineStr">
         <is>
@@ -11639,7 +11639,7 @@
       </c>
       <c r="C273" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #3 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.27s.</t>
+          <t>User tests layout/memory scenario #3 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.28s.</t>
         </is>
       </c>
       <c r="D273" s="2" t="inlineStr">
@@ -11658,7 +11658,7 @@
         </is>
       </c>
       <c r="G273" s="2" t="n">
-        <v>0.27</v>
+        <v>0.28</v>
       </c>
       <c r="H273" s="2" t="inlineStr">
         <is>
@@ -11680,7 +11680,7 @@
       </c>
       <c r="C274" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #4 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.39s.</t>
+          <t>User tests layout/memory scenario #4 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.32s.</t>
         </is>
       </c>
       <c r="D274" s="2" t="inlineStr">
@@ -11699,7 +11699,7 @@
         </is>
       </c>
       <c r="G274" s="2" t="n">
-        <v>0.39</v>
+        <v>0.32</v>
       </c>
       <c r="H274" s="2" t="inlineStr">
         <is>
@@ -11721,7 +11721,7 @@
       </c>
       <c r="C275" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #5 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.6s.</t>
+          <t>User tests layout/memory scenario #5 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.66s.</t>
         </is>
       </c>
       <c r="D275" s="2" t="inlineStr">
@@ -11740,7 +11740,7 @@
         </is>
       </c>
       <c r="G275" s="2" t="n">
-        <v>0.6</v>
+        <v>0.66</v>
       </c>
       <c r="H275" s="2" t="inlineStr">
         <is>
@@ -11762,7 +11762,7 @@
       </c>
       <c r="C276" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #6 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.5s.</t>
+          <t>User tests layout/memory scenario #6 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.39s.</t>
         </is>
       </c>
       <c r="D276" s="2" t="inlineStr">
@@ -11781,7 +11781,7 @@
         </is>
       </c>
       <c r="G276" s="2" t="n">
-        <v>0.5</v>
+        <v>0.39</v>
       </c>
       <c r="H276" s="2" t="inlineStr">
         <is>
@@ -11803,7 +11803,7 @@
       </c>
       <c r="C277" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #7 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.44s.</t>
+          <t>User tests layout/memory scenario #7 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.24s.</t>
         </is>
       </c>
       <c r="D277" s="2" t="inlineStr">
@@ -11822,7 +11822,7 @@
         </is>
       </c>
       <c r="G277" s="2" t="n">
-        <v>0.44</v>
+        <v>0.24</v>
       </c>
       <c r="H277" s="2" t="inlineStr">
         <is>
@@ -11844,7 +11844,7 @@
       </c>
       <c r="C278" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #8 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.6s.</t>
+          <t>User tests layout/memory scenario #8 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.27s.</t>
         </is>
       </c>
       <c r="D278" s="2" t="inlineStr">
@@ -11863,7 +11863,7 @@
         </is>
       </c>
       <c r="G278" s="2" t="n">
-        <v>0.6</v>
+        <v>0.27</v>
       </c>
       <c r="H278" s="2" t="inlineStr">
         <is>
@@ -11885,7 +11885,7 @@
       </c>
       <c r="C279" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #9 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.37s.</t>
+          <t>User tests layout/memory scenario #9 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.43s.</t>
         </is>
       </c>
       <c r="D279" s="2" t="inlineStr">
@@ -11904,7 +11904,7 @@
         </is>
       </c>
       <c r="G279" s="2" t="n">
-        <v>0.37</v>
+        <v>0.43</v>
       </c>
       <c r="H279" s="2" t="inlineStr">
         <is>
@@ -11926,7 +11926,7 @@
       </c>
       <c r="C280" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #10 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.31s.</t>
+          <t>User tests layout/memory scenario #10 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.33s.</t>
         </is>
       </c>
       <c r="D280" s="2" t="inlineStr">
@@ -11945,7 +11945,7 @@
         </is>
       </c>
       <c r="G280" s="2" t="n">
-        <v>0.31</v>
+        <v>0.33</v>
       </c>
       <c r="H280" s="2" t="inlineStr">
         <is>
@@ -11967,7 +11967,7 @@
       </c>
       <c r="C281" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #11 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.47s.</t>
+          <t>User tests layout/memory scenario #11 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.35s.</t>
         </is>
       </c>
       <c r="D281" s="2" t="inlineStr">
@@ -11986,7 +11986,7 @@
         </is>
       </c>
       <c r="G281" s="2" t="n">
-        <v>0.47</v>
+        <v>0.35</v>
       </c>
       <c r="H281" s="2" t="inlineStr">
         <is>
@@ -12008,7 +12008,7 @@
       </c>
       <c r="C282" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #12 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.52s.</t>
+          <t>User tests layout/memory scenario #12 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.58s.</t>
         </is>
       </c>
       <c r="D282" s="2" t="inlineStr">
@@ -12027,7 +12027,7 @@
         </is>
       </c>
       <c r="G282" s="2" t="n">
-        <v>0.52</v>
+        <v>0.58</v>
       </c>
       <c r="H282" s="2" t="inlineStr">
         <is>
@@ -12049,7 +12049,7 @@
       </c>
       <c r="C283" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #13 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.59s.</t>
+          <t>User tests layout/memory scenario #13 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.57s.</t>
         </is>
       </c>
       <c r="D283" s="2" t="inlineStr">
@@ -12068,7 +12068,7 @@
         </is>
       </c>
       <c r="G283" s="2" t="n">
-        <v>0.59</v>
+        <v>0.57</v>
       </c>
       <c r="H283" s="2" t="inlineStr">
         <is>
@@ -12090,7 +12090,7 @@
       </c>
       <c r="C284" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #14 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.61s.</t>
+          <t>User tests layout/memory scenario #14 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.42s.</t>
         </is>
       </c>
       <c r="D284" s="2" t="inlineStr">
@@ -12109,7 +12109,7 @@
         </is>
       </c>
       <c r="G284" s="2" t="n">
-        <v>0.61</v>
+        <v>0.42</v>
       </c>
       <c r="H284" s="2" t="inlineStr">
         <is>
@@ -12131,7 +12131,7 @@
       </c>
       <c r="C285" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #15 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.45s.</t>
+          <t>User tests layout/memory scenario #15 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.61s.</t>
         </is>
       </c>
       <c r="D285" s="2" t="inlineStr">
@@ -12150,7 +12150,7 @@
         </is>
       </c>
       <c r="G285" s="2" t="n">
-        <v>0.45</v>
+        <v>0.61</v>
       </c>
       <c r="H285" s="2" t="inlineStr">
         <is>
@@ -12172,7 +12172,7 @@
       </c>
       <c r="C286" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #16 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.33s.</t>
+          <t>User tests layout/memory scenario #16 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.49s.</t>
         </is>
       </c>
       <c r="D286" s="2" t="inlineStr">
@@ -12191,7 +12191,7 @@
         </is>
       </c>
       <c r="G286" s="2" t="n">
-        <v>0.33</v>
+        <v>0.49</v>
       </c>
       <c r="H286" s="2" t="inlineStr">
         <is>
@@ -12213,7 +12213,7 @@
       </c>
       <c r="C287" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #17 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.31s.</t>
+          <t>User tests layout/memory scenario #17 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.41s.</t>
         </is>
       </c>
       <c r="D287" s="2" t="inlineStr">
@@ -12232,7 +12232,7 @@
         </is>
       </c>
       <c r="G287" s="2" t="n">
-        <v>0.31</v>
+        <v>0.41</v>
       </c>
       <c r="H287" s="2" t="inlineStr">
         <is>
@@ -12254,7 +12254,7 @@
       </c>
       <c r="C288" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #18 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.65s.</t>
+          <t>User tests layout/memory scenario #18 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.3s.</t>
         </is>
       </c>
       <c r="D288" s="2" t="inlineStr">
@@ -12273,7 +12273,7 @@
         </is>
       </c>
       <c r="G288" s="2" t="n">
-        <v>0.65</v>
+        <v>0.3</v>
       </c>
       <c r="H288" s="2" t="inlineStr">
         <is>
@@ -12295,7 +12295,7 @@
       </c>
       <c r="C289" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #19 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.64s.</t>
+          <t>User tests layout/memory scenario #19 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.44s.</t>
         </is>
       </c>
       <c r="D289" s="2" t="inlineStr">
@@ -12314,7 +12314,7 @@
         </is>
       </c>
       <c r="G289" s="2" t="n">
-        <v>0.64</v>
+        <v>0.44</v>
       </c>
       <c r="H289" s="2" t="inlineStr">
         <is>
@@ -12336,7 +12336,7 @@
       </c>
       <c r="C290" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #20 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.45s.</t>
+          <t>User tests layout/memory scenario #20 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.35s.</t>
         </is>
       </c>
       <c r="D290" s="2" t="inlineStr">
@@ -12355,7 +12355,7 @@
         </is>
       </c>
       <c r="G290" s="2" t="n">
-        <v>0.45</v>
+        <v>0.35</v>
       </c>
       <c r="H290" s="2" t="inlineStr">
         <is>
@@ -12377,7 +12377,7 @@
       </c>
       <c r="C291" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #21 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.47s.</t>
+          <t>User tests layout/memory scenario #21 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.49s.</t>
         </is>
       </c>
       <c r="D291" s="2" t="inlineStr">
@@ -12396,7 +12396,7 @@
         </is>
       </c>
       <c r="G291" s="2" t="n">
-        <v>0.47</v>
+        <v>0.49</v>
       </c>
       <c r="H291" s="2" t="inlineStr">
         <is>
@@ -12418,7 +12418,7 @@
       </c>
       <c r="C292" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #22 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.6s.</t>
+          <t>User tests layout/memory scenario #22 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.54s.</t>
         </is>
       </c>
       <c r="D292" s="2" t="inlineStr">
@@ -12437,7 +12437,7 @@
         </is>
       </c>
       <c r="G292" s="2" t="n">
-        <v>0.6</v>
+        <v>0.54</v>
       </c>
       <c r="H292" s="2" t="inlineStr">
         <is>
@@ -12459,7 +12459,7 @@
       </c>
       <c r="C293" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #23 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.24s.</t>
+          <t>User tests layout/memory scenario #23 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.45s.</t>
         </is>
       </c>
       <c r="D293" s="2" t="inlineStr">
@@ -12478,7 +12478,7 @@
         </is>
       </c>
       <c r="G293" s="2" t="n">
-        <v>0.24</v>
+        <v>0.45</v>
       </c>
       <c r="H293" s="2" t="inlineStr">
         <is>
@@ -12500,7 +12500,7 @@
       </c>
       <c r="C294" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #24 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.64s.</t>
+          <t>User tests layout/memory scenario #24 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.31s.</t>
         </is>
       </c>
       <c r="D294" s="2" t="inlineStr">
@@ -12519,7 +12519,7 @@
         </is>
       </c>
       <c r="G294" s="2" t="n">
-        <v>0.64</v>
+        <v>0.31</v>
       </c>
       <c r="H294" s="2" t="inlineStr">
         <is>
@@ -12541,7 +12541,7 @@
       </c>
       <c r="C295" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #25 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.66s.</t>
+          <t>User tests layout/memory scenario #25 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.6s.</t>
         </is>
       </c>
       <c r="D295" s="2" t="inlineStr">
@@ -12560,7 +12560,7 @@
         </is>
       </c>
       <c r="G295" s="2" t="n">
-        <v>0.66</v>
+        <v>0.6</v>
       </c>
       <c r="H295" s="2" t="inlineStr">
         <is>
@@ -12582,7 +12582,7 @@
       </c>
       <c r="C296" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #26 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.65s.</t>
+          <t>User tests layout/memory scenario #26 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.27s.</t>
         </is>
       </c>
       <c r="D296" s="2" t="inlineStr">
@@ -12601,7 +12601,7 @@
         </is>
       </c>
       <c r="G296" s="2" t="n">
-        <v>0.65</v>
+        <v>0.27</v>
       </c>
       <c r="H296" s="2" t="inlineStr">
         <is>
@@ -12623,7 +12623,7 @@
       </c>
       <c r="C297" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #27 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.42s.</t>
+          <t>User tests layout/memory scenario #27 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.43s.</t>
         </is>
       </c>
       <c r="D297" s="2" t="inlineStr">
@@ -12642,7 +12642,7 @@
         </is>
       </c>
       <c r="G297" s="2" t="n">
-        <v>0.42</v>
+        <v>0.43</v>
       </c>
       <c r="H297" s="2" t="inlineStr">
         <is>
@@ -12664,7 +12664,7 @@
       </c>
       <c r="C298" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #28 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.26s.</t>
+          <t>User tests layout/memory scenario #28 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.43s.</t>
         </is>
       </c>
       <c r="D298" s="2" t="inlineStr">
@@ -12683,7 +12683,7 @@
         </is>
       </c>
       <c r="G298" s="2" t="n">
-        <v>0.26</v>
+        <v>0.43</v>
       </c>
       <c r="H298" s="2" t="inlineStr">
         <is>
@@ -12705,7 +12705,7 @@
       </c>
       <c r="C299" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #29 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.34s.</t>
+          <t>User tests layout/memory scenario #29 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.26s.</t>
         </is>
       </c>
       <c r="D299" s="2" t="inlineStr">
@@ -12724,7 +12724,7 @@
         </is>
       </c>
       <c r="G299" s="2" t="n">
-        <v>0.34</v>
+        <v>0.26</v>
       </c>
       <c r="H299" s="2" t="inlineStr">
         <is>
@@ -12746,7 +12746,7 @@
       </c>
       <c r="C300" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #30 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.52s.</t>
+          <t>User tests layout/memory scenario #30 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.61s.</t>
         </is>
       </c>
       <c r="D300" s="2" t="inlineStr">
@@ -12765,7 +12765,7 @@
         </is>
       </c>
       <c r="G300" s="2" t="n">
-        <v>0.52</v>
+        <v>0.61</v>
       </c>
       <c r="H300" s="2" t="inlineStr">
         <is>
@@ -12787,7 +12787,7 @@
       </c>
       <c r="C301" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #31 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.58s.</t>
+          <t>User tests layout/memory scenario #31 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.4s.</t>
         </is>
       </c>
       <c r="D301" s="2" t="inlineStr">
@@ -12806,7 +12806,7 @@
         </is>
       </c>
       <c r="G301" s="2" t="n">
-        <v>0.58</v>
+        <v>0.4</v>
       </c>
       <c r="H301" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
feat(summary): add 3-outcome combined synthesis summary to load test report and CI summary
</commit_message>
<xml_diff>
--- a/reports/Mobile_Application_Appium_Test_Report.xlsx
+++ b/reports/Mobile_Application_Appium_Test_Report.xlsx
@@ -547,7 +547,7 @@
         </is>
       </c>
       <c r="G2" s="2" t="n">
-        <v>0.59</v>
+        <v>0.55</v>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
@@ -588,7 +588,7 @@
         </is>
       </c>
       <c r="G3" s="2" t="n">
-        <v>0.65</v>
+        <v>0.49</v>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
@@ -629,7 +629,7 @@
         </is>
       </c>
       <c r="G4" s="2" t="n">
-        <v>0.42</v>
+        <v>0.9</v>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
@@ -670,7 +670,7 @@
         </is>
       </c>
       <c r="G5" s="2" t="n">
-        <v>0.42</v>
+        <v>0.85</v>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
@@ -711,7 +711,7 @@
         </is>
       </c>
       <c r="G6" s="2" t="n">
-        <v>0.57</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
@@ -752,7 +752,7 @@
         </is>
       </c>
       <c r="G7" s="2" t="n">
-        <v>0.41</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
@@ -793,7 +793,7 @@
         </is>
       </c>
       <c r="G8" s="2" t="n">
-        <v>0.54</v>
+        <v>0.6</v>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
@@ -834,7 +834,7 @@
         </is>
       </c>
       <c r="G9" s="2" t="n">
-        <v>0.47</v>
+        <v>0.46</v>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
@@ -875,7 +875,7 @@
         </is>
       </c>
       <c r="G10" s="2" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.64</v>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
@@ -916,7 +916,7 @@
         </is>
       </c>
       <c r="G11" s="2" t="n">
-        <v>0.75</v>
+        <v>0.66</v>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
@@ -957,7 +957,7 @@
         </is>
       </c>
       <c r="G12" s="2" t="n">
-        <v>0.62</v>
+        <v>0.46</v>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
@@ -998,7 +998,7 @@
         </is>
       </c>
       <c r="G13" s="2" t="n">
-        <v>0.58</v>
+        <v>0.75</v>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
@@ -1039,7 +1039,7 @@
         </is>
       </c>
       <c r="G14" s="2" t="n">
-        <v>0.9</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
@@ -1080,7 +1080,7 @@
         </is>
       </c>
       <c r="G15" s="2" t="n">
-        <v>0.37</v>
+        <v>0.71</v>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
@@ -1121,7 +1121,7 @@
         </is>
       </c>
       <c r="G16" s="2" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.5</v>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
@@ -1162,7 +1162,7 @@
         </is>
       </c>
       <c r="G17" s="2" t="n">
-        <v>0.68</v>
+        <v>0.92</v>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
@@ -1203,7 +1203,7 @@
         </is>
       </c>
       <c r="G18" s="2" t="n">
-        <v>0.91</v>
+        <v>0.64</v>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
@@ -1244,7 +1244,7 @@
         </is>
       </c>
       <c r="G19" s="2" t="n">
-        <v>0.54</v>
+        <v>0.53</v>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
@@ -1285,7 +1285,7 @@
         </is>
       </c>
       <c r="G20" s="2" t="n">
-        <v>0.82</v>
+        <v>0.37</v>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
@@ -1326,7 +1326,7 @@
         </is>
       </c>
       <c r="G21" s="2" t="n">
-        <v>0.78</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
@@ -1348,7 +1348,7 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #1 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.63s without crashing.</t>
+          <t>User taps Auth action button #1 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.72s without crashing.</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -1367,7 +1367,7 @@
         </is>
       </c>
       <c r="G22" s="2" t="n">
-        <v>0.63</v>
+        <v>0.72</v>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
@@ -1389,7 +1389,7 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #2 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.47s without crashing.</t>
+          <t>User taps Auth action button #2 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.64s without crashing.</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -1408,7 +1408,7 @@
         </is>
       </c>
       <c r="G23" s="2" t="n">
-        <v>0.47</v>
+        <v>0.64</v>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
@@ -1430,7 +1430,7 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #3 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.91s without crashing.</t>
+          <t>User taps Auth action button #3 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.68s without crashing.</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -1449,7 +1449,7 @@
         </is>
       </c>
       <c r="G24" s="2" t="n">
-        <v>0.91</v>
+        <v>0.68</v>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
@@ -1471,7 +1471,7 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #4 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.55s without crashing.</t>
+          <t>User taps Auth action button #4 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.76s without crashing.</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
@@ -1490,7 +1490,7 @@
         </is>
       </c>
       <c r="G25" s="2" t="n">
-        <v>0.55</v>
+        <v>0.76</v>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
@@ -1512,7 +1512,7 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #5 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.76s without crashing.</t>
+          <t>User taps Auth action button #5 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.83s without crashing.</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -1531,7 +1531,7 @@
         </is>
       </c>
       <c r="G26" s="2" t="n">
-        <v>0.76</v>
+        <v>0.83</v>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
@@ -1553,7 +1553,7 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #6 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.77s without crashing.</t>
+          <t>User taps Auth action button #6 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.94s without crashing.</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
@@ -1572,7 +1572,7 @@
         </is>
       </c>
       <c r="G27" s="2" t="n">
-        <v>0.77</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
@@ -1594,7 +1594,7 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #7 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.43s without crashing.</t>
+          <t>User taps Auth action button #7 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.37s without crashing.</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -1613,7 +1613,7 @@
         </is>
       </c>
       <c r="G28" s="2" t="n">
-        <v>0.43</v>
+        <v>0.37</v>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
@@ -1635,7 +1635,7 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #8 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.52s without crashing.</t>
+          <t>User taps Auth action button #8 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.73s without crashing.</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
@@ -1654,7 +1654,7 @@
         </is>
       </c>
       <c r="G29" s="2" t="n">
-        <v>0.52</v>
+        <v>0.73</v>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
@@ -1676,7 +1676,7 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #9 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.51s without crashing.</t>
+          <t>User taps Auth action button #9 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.75s without crashing.</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -1695,7 +1695,7 @@
         </is>
       </c>
       <c r="G30" s="2" t="n">
-        <v>0.51</v>
+        <v>0.75</v>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
@@ -1717,7 +1717,7 @@
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #10 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.52s without crashing.</t>
+          <t>User taps Auth action button #10 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.35s without crashing.</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
@@ -1736,7 +1736,7 @@
         </is>
       </c>
       <c r="G31" s="2" t="n">
-        <v>0.52</v>
+        <v>0.35</v>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
@@ -1758,7 +1758,7 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #11 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.42s without crashing.</t>
+          <t>User taps Auth action button #11 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.57s without crashing.</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
@@ -1777,7 +1777,7 @@
         </is>
       </c>
       <c r="G32" s="2" t="n">
-        <v>0.42</v>
+        <v>0.57</v>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
@@ -1799,7 +1799,7 @@
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #12 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.84s without crashing.</t>
+          <t>User taps Auth action button #12 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.8s without crashing.</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
@@ -1818,7 +1818,7 @@
         </is>
       </c>
       <c r="G33" s="2" t="n">
-        <v>0.84</v>
+        <v>0.8</v>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
@@ -1840,7 +1840,7 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #13 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.7s without crashing.</t>
+          <t>User taps Auth action button #13 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.84s without crashing.</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -1859,7 +1859,7 @@
         </is>
       </c>
       <c r="G34" s="2" t="n">
-        <v>0.7</v>
+        <v>0.84</v>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
@@ -1881,7 +1881,7 @@
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #14 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.92s without crashing.</t>
+          <t>User taps Auth action button #14 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.56s without crashing.</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
@@ -1900,7 +1900,7 @@
         </is>
       </c>
       <c r="G35" s="2" t="n">
-        <v>0.92</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
@@ -1922,7 +1922,7 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #15 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.46s without crashing.</t>
+          <t>User taps Auth action button #15 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.94s without crashing.</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
@@ -1941,7 +1941,7 @@
         </is>
       </c>
       <c r="G36" s="2" t="n">
-        <v>0.46</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
@@ -1963,7 +1963,7 @@
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #16 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.87s without crashing.</t>
+          <t>User taps Auth action button #16 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.73s without crashing.</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
@@ -1982,7 +1982,7 @@
         </is>
       </c>
       <c r="G37" s="2" t="n">
-        <v>0.87</v>
+        <v>0.73</v>
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
@@ -2004,7 +2004,7 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #17 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.72s without crashing.</t>
+          <t>User taps Auth action button #17 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.47s without crashing.</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
@@ -2023,7 +2023,7 @@
         </is>
       </c>
       <c r="G38" s="2" t="n">
-        <v>0.72</v>
+        <v>0.47</v>
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
@@ -2045,7 +2045,7 @@
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #18 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.85s without crashing.</t>
+          <t>User taps Auth action button #18 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.78s without crashing.</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
@@ -2064,7 +2064,7 @@
         </is>
       </c>
       <c r="G39" s="2" t="n">
-        <v>0.85</v>
+        <v>0.78</v>
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
@@ -2086,7 +2086,7 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #19 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.54s without crashing.</t>
+          <t>User taps Auth action button #19 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.8s without crashing.</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
@@ -2105,7 +2105,7 @@
         </is>
       </c>
       <c r="G40" s="2" t="n">
-        <v>0.54</v>
+        <v>0.8</v>
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
@@ -2127,7 +2127,7 @@
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #20 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.7s without crashing.</t>
+          <t>User taps Auth action button #20 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.4s without crashing.</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
@@ -2146,7 +2146,7 @@
         </is>
       </c>
       <c r="G41" s="2" t="n">
-        <v>0.7</v>
+        <v>0.4</v>
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
@@ -2187,7 +2187,7 @@
         </is>
       </c>
       <c r="G42" s="2" t="n">
-        <v>0.88</v>
+        <v>0.39</v>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
@@ -2228,7 +2228,7 @@
         </is>
       </c>
       <c r="G43" s="2" t="n">
-        <v>0.53</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
@@ -2269,7 +2269,7 @@
         </is>
       </c>
       <c r="G44" s="2" t="n">
-        <v>0.37</v>
+        <v>0.42</v>
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
@@ -2310,7 +2310,7 @@
         </is>
       </c>
       <c r="G45" s="2" t="n">
-        <v>0.62</v>
+        <v>0.52</v>
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
@@ -2351,7 +2351,7 @@
         </is>
       </c>
       <c r="G46" s="2" t="n">
-        <v>0.47</v>
+        <v>0.55</v>
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
@@ -2392,7 +2392,7 @@
         </is>
       </c>
       <c r="G47" s="2" t="n">
-        <v>0.52</v>
+        <v>0.42</v>
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
@@ -2433,7 +2433,7 @@
         </is>
       </c>
       <c r="G48" s="2" t="n">
-        <v>0.46</v>
+        <v>0.88</v>
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
@@ -2474,7 +2474,7 @@
         </is>
       </c>
       <c r="G49" s="2" t="n">
-        <v>0.82</v>
+        <v>0.45</v>
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
@@ -2515,7 +2515,7 @@
         </is>
       </c>
       <c r="G50" s="2" t="n">
-        <v>0.33</v>
+        <v>0.68</v>
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
@@ -2556,7 +2556,7 @@
         </is>
       </c>
       <c r="G51" s="2" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.6</v>
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
@@ -2597,7 +2597,7 @@
         </is>
       </c>
       <c r="G52" s="2" t="n">
-        <v>0.61</v>
+        <v>0.41</v>
       </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
@@ -2638,7 +2638,7 @@
         </is>
       </c>
       <c r="G53" s="2" t="n">
-        <v>0.85</v>
+        <v>0.42</v>
       </c>
       <c r="H53" s="2" t="inlineStr">
         <is>
@@ -2679,7 +2679,7 @@
         </is>
       </c>
       <c r="G54" s="2" t="n">
-        <v>0.38</v>
+        <v>0.65</v>
       </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
@@ -2720,7 +2720,7 @@
         </is>
       </c>
       <c r="G55" s="2" t="n">
-        <v>0.49</v>
+        <v>0.62</v>
       </c>
       <c r="H55" s="2" t="inlineStr">
         <is>
@@ -2761,7 +2761,7 @@
         </is>
       </c>
       <c r="G56" s="2" t="n">
-        <v>0.77</v>
+        <v>0.71</v>
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
@@ -2783,7 +2783,7 @@
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #1 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.46s.</t>
+          <t>User taps Verification interactive button #1 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.86s.</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
@@ -2802,7 +2802,7 @@
         </is>
       </c>
       <c r="G57" s="2" t="n">
-        <v>0.46</v>
+        <v>0.86</v>
       </c>
       <c r="H57" s="2" t="inlineStr">
         <is>
@@ -2824,7 +2824,7 @@
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #2 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.42s.</t>
+          <t>User taps Verification interactive button #2 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.6s.</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
@@ -2843,7 +2843,7 @@
         </is>
       </c>
       <c r="G58" s="2" t="n">
-        <v>0.42</v>
+        <v>0.6</v>
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
@@ -2865,7 +2865,7 @@
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #3 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.36s.</t>
+          <t>User taps Verification interactive button #3 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.48s.</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
@@ -2884,7 +2884,7 @@
         </is>
       </c>
       <c r="G59" s="2" t="n">
-        <v>0.36</v>
+        <v>0.48</v>
       </c>
       <c r="H59" s="2" t="inlineStr">
         <is>
@@ -2906,7 +2906,7 @@
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #4 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.83s.</t>
+          <t>User taps Verification interactive button #4 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.65s.</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
@@ -2925,7 +2925,7 @@
         </is>
       </c>
       <c r="G60" s="2" t="n">
-        <v>0.83</v>
+        <v>0.65</v>
       </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
@@ -2947,7 +2947,7 @@
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #5 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.72s.</t>
+          <t>User taps Verification interactive button #5 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.76s.</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
@@ -2966,7 +2966,7 @@
         </is>
       </c>
       <c r="G61" s="2" t="n">
-        <v>0.72</v>
+        <v>0.76</v>
       </c>
       <c r="H61" s="2" t="inlineStr">
         <is>
@@ -2988,7 +2988,7 @@
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #6 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.37s.</t>
+          <t>User taps Verification interactive button #6 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.36s.</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
@@ -3007,7 +3007,7 @@
         </is>
       </c>
       <c r="G62" s="2" t="n">
-        <v>0.37</v>
+        <v>0.36</v>
       </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
@@ -3029,7 +3029,7 @@
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #7 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.45s.</t>
+          <t>User taps Verification interactive button #7 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.8s.</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
@@ -3048,7 +3048,7 @@
         </is>
       </c>
       <c r="G63" s="2" t="n">
-        <v>0.45</v>
+        <v>0.8</v>
       </c>
       <c r="H63" s="2" t="inlineStr">
         <is>
@@ -3070,7 +3070,7 @@
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #8 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.85s.</t>
+          <t>User taps Verification interactive button #8 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.77s.</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
@@ -3089,7 +3089,7 @@
         </is>
       </c>
       <c r="G64" s="2" t="n">
-        <v>0.85</v>
+        <v>0.77</v>
       </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
@@ -3111,7 +3111,7 @@
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #9 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.49s.</t>
+          <t>User taps Verification interactive button #9 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.37s.</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
@@ -3130,7 +3130,7 @@
         </is>
       </c>
       <c r="G65" s="2" t="n">
-        <v>0.49</v>
+        <v>0.37</v>
       </c>
       <c r="H65" s="2" t="inlineStr">
         <is>
@@ -3152,7 +3152,7 @@
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #10 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.82s.</t>
+          <t>User taps Verification interactive button #10 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.85s.</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
@@ -3171,7 +3171,7 @@
         </is>
       </c>
       <c r="G66" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="H66" s="2" t="inlineStr">
         <is>
@@ -3193,7 +3193,7 @@
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #11 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.71s.</t>
+          <t>User taps Verification interactive button #11 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.85s.</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
@@ -3212,7 +3212,7 @@
         </is>
       </c>
       <c r="G67" s="2" t="n">
-        <v>0.71</v>
+        <v>0.85</v>
       </c>
       <c r="H67" s="2" t="inlineStr">
         <is>
@@ -3234,7 +3234,7 @@
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #12 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.6s.</t>
+          <t>User taps Verification interactive button #12 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.82s.</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
@@ -3253,7 +3253,7 @@
         </is>
       </c>
       <c r="G68" s="2" t="n">
-        <v>0.6</v>
+        <v>0.82</v>
       </c>
       <c r="H68" s="2" t="inlineStr">
         <is>
@@ -3275,7 +3275,7 @@
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #13 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.74s.</t>
+          <t>User taps Verification interactive button #13 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.77s.</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
@@ -3294,7 +3294,7 @@
         </is>
       </c>
       <c r="G69" s="2" t="n">
-        <v>0.74</v>
+        <v>0.77</v>
       </c>
       <c r="H69" s="2" t="inlineStr">
         <is>
@@ -3316,7 +3316,7 @@
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #14 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.55s.</t>
+          <t>User taps Verification interactive button #14 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.53s.</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
@@ -3335,7 +3335,7 @@
         </is>
       </c>
       <c r="G70" s="2" t="n">
-        <v>0.55</v>
+        <v>0.53</v>
       </c>
       <c r="H70" s="2" t="inlineStr">
         <is>
@@ -3357,7 +3357,7 @@
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #15 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.4s.</t>
+          <t>User taps Verification interactive button #15 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.73s.</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
@@ -3376,7 +3376,7 @@
         </is>
       </c>
       <c r="G71" s="2" t="n">
-        <v>0.4</v>
+        <v>0.73</v>
       </c>
       <c r="H71" s="2" t="inlineStr">
         <is>
@@ -3398,7 +3398,7 @@
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #16 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.39s.</t>
+          <t>User taps Verification interactive button #16 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.69s.</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
@@ -3417,7 +3417,7 @@
         </is>
       </c>
       <c r="G72" s="2" t="n">
-        <v>0.39</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="H72" s="2" t="inlineStr">
         <is>
@@ -3439,7 +3439,7 @@
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #17 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.82s.</t>
+          <t>User taps Verification interactive button #17 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.71s.</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr">
@@ -3458,7 +3458,7 @@
         </is>
       </c>
       <c r="G73" s="2" t="n">
-        <v>0.82</v>
+        <v>0.71</v>
       </c>
       <c r="H73" s="2" t="inlineStr">
         <is>
@@ -3480,7 +3480,7 @@
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #18 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.35s.</t>
+          <t>User taps Verification interactive button #18 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.69s.</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
@@ -3499,7 +3499,7 @@
         </is>
       </c>
       <c r="G74" s="2" t="n">
-        <v>0.35</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="H74" s="2" t="inlineStr">
         <is>
@@ -3521,7 +3521,7 @@
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #19 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.72s.</t>
+          <t>User taps Verification interactive button #19 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.79s.</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
@@ -3540,7 +3540,7 @@
         </is>
       </c>
       <c r="G75" s="2" t="n">
-        <v>0.72</v>
+        <v>0.79</v>
       </c>
       <c r="H75" s="2" t="inlineStr">
         <is>
@@ -3562,7 +3562,7 @@
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #20 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.57s.</t>
+          <t>User taps Verification interactive button #20 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.39s.</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
@@ -3581,7 +3581,7 @@
         </is>
       </c>
       <c r="G76" s="2" t="n">
-        <v>0.57</v>
+        <v>0.39</v>
       </c>
       <c r="H76" s="2" t="inlineStr">
         <is>
@@ -3603,7 +3603,7 @@
       </c>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #21 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.85s.</t>
+          <t>User taps Verification interactive button #21 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.49s.</t>
         </is>
       </c>
       <c r="D77" s="2" t="inlineStr">
@@ -3622,7 +3622,7 @@
         </is>
       </c>
       <c r="G77" s="2" t="n">
-        <v>0.85</v>
+        <v>0.49</v>
       </c>
       <c r="H77" s="2" t="inlineStr">
         <is>
@@ -3644,7 +3644,7 @@
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #22 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.32s.</t>
+          <t>User taps Verification interactive button #22 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.87s.</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
@@ -3663,7 +3663,7 @@
         </is>
       </c>
       <c r="G78" s="2" t="n">
-        <v>0.32</v>
+        <v>0.87</v>
       </c>
       <c r="H78" s="2" t="inlineStr">
         <is>
@@ -3685,7 +3685,7 @@
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #23 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.42s.</t>
+          <t>User taps Verification interactive button #23 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.69s.</t>
         </is>
       </c>
       <c r="D79" s="2" t="inlineStr">
@@ -3704,7 +3704,7 @@
         </is>
       </c>
       <c r="G79" s="2" t="n">
-        <v>0.42</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="H79" s="2" t="inlineStr">
         <is>
@@ -3726,7 +3726,7 @@
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #24 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.86s.</t>
+          <t>User taps Verification interactive button #24 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.7s.</t>
         </is>
       </c>
       <c r="D80" s="2" t="inlineStr">
@@ -3745,7 +3745,7 @@
         </is>
       </c>
       <c r="G80" s="2" t="n">
-        <v>0.86</v>
+        <v>0.7</v>
       </c>
       <c r="H80" s="2" t="inlineStr">
         <is>
@@ -3767,7 +3767,7 @@
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #25 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.84s.</t>
+          <t>User taps Verification interactive button #25 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.44s.</t>
         </is>
       </c>
       <c r="D81" s="2" t="inlineStr">
@@ -3786,7 +3786,7 @@
         </is>
       </c>
       <c r="G81" s="2" t="n">
-        <v>0.84</v>
+        <v>0.44</v>
       </c>
       <c r="H81" s="2" t="inlineStr">
         <is>
@@ -3827,7 +3827,7 @@
         </is>
       </c>
       <c r="G82" s="2" t="n">
-        <v>0.6</v>
+        <v>0.62</v>
       </c>
       <c r="H82" s="2" t="inlineStr">
         <is>
@@ -3868,7 +3868,7 @@
         </is>
       </c>
       <c r="G83" s="2" t="n">
-        <v>0.98</v>
+        <v>1.1</v>
       </c>
       <c r="H83" s="2" t="inlineStr">
         <is>
@@ -3909,7 +3909,7 @@
         </is>
       </c>
       <c r="G84" s="2" t="n">
-        <v>0.44</v>
+        <v>0.53</v>
       </c>
       <c r="H84" s="2" t="inlineStr">
         <is>
@@ -3950,7 +3950,7 @@
         </is>
       </c>
       <c r="G85" s="2" t="n">
-        <v>0.53</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="H85" s="2" t="inlineStr">
         <is>
@@ -3991,7 +3991,7 @@
         </is>
       </c>
       <c r="G86" s="2" t="n">
-        <v>0.93</v>
+        <v>0.46</v>
       </c>
       <c r="H86" s="2" t="inlineStr">
         <is>
@@ -4032,7 +4032,7 @@
         </is>
       </c>
       <c r="G87" s="2" t="n">
-        <v>0.58</v>
+        <v>0.48</v>
       </c>
       <c r="H87" s="2" t="inlineStr">
         <is>
@@ -4073,7 +4073,7 @@
         </is>
       </c>
       <c r="G88" s="2" t="n">
-        <v>0.95</v>
+        <v>0.88</v>
       </c>
       <c r="H88" s="2" t="inlineStr">
         <is>
@@ -4114,7 +4114,7 @@
         </is>
       </c>
       <c r="G89" s="2" t="n">
-        <v>0.89</v>
+        <v>0.79</v>
       </c>
       <c r="H89" s="2" t="inlineStr">
         <is>
@@ -4155,7 +4155,7 @@
         </is>
       </c>
       <c r="G90" s="2" t="n">
-        <v>0.55</v>
+        <v>0.63</v>
       </c>
       <c r="H90" s="2" t="inlineStr">
         <is>
@@ -4196,7 +4196,7 @@
         </is>
       </c>
       <c r="G91" s="2" t="n">
-        <v>0.68</v>
+        <v>0.8</v>
       </c>
       <c r="H91" s="2" t="inlineStr">
         <is>
@@ -4237,7 +4237,7 @@
         </is>
       </c>
       <c r="G92" s="2" t="n">
-        <v>1.11</v>
+        <v>0.59</v>
       </c>
       <c r="H92" s="2" t="inlineStr">
         <is>
@@ -4278,7 +4278,7 @@
         </is>
       </c>
       <c r="G93" s="2" t="n">
-        <v>0.39</v>
+        <v>0.73</v>
       </c>
       <c r="H93" s="2" t="inlineStr">
         <is>
@@ -4319,7 +4319,7 @@
         </is>
       </c>
       <c r="G94" s="2" t="n">
-        <v>0.89</v>
+        <v>0.6</v>
       </c>
       <c r="H94" s="2" t="inlineStr">
         <is>
@@ -4360,7 +4360,7 @@
         </is>
       </c>
       <c r="G95" s="2" t="n">
-        <v>0.91</v>
+        <v>0.83</v>
       </c>
       <c r="H95" s="2" t="inlineStr">
         <is>
@@ -4401,7 +4401,7 @@
         </is>
       </c>
       <c r="G96" s="2" t="n">
-        <v>0.85</v>
+        <v>0.65</v>
       </c>
       <c r="H96" s="2" t="inlineStr">
         <is>
@@ -4423,7 +4423,7 @@
       </c>
       <c r="C97" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #1 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.9s.</t>
+          <t>User taps Issuance form action button #1 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.81s.</t>
         </is>
       </c>
       <c r="D97" s="2" t="inlineStr">
@@ -4442,7 +4442,7 @@
         </is>
       </c>
       <c r="G97" s="2" t="n">
-        <v>0.9</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="H97" s="2" t="inlineStr">
         <is>
@@ -4464,7 +4464,7 @@
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #2 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.47s.</t>
+          <t>User taps Issuance form action button #2 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.89s.</t>
         </is>
       </c>
       <c r="D98" s="2" t="inlineStr">
@@ -4483,7 +4483,7 @@
         </is>
       </c>
       <c r="G98" s="2" t="n">
-        <v>0.47</v>
+        <v>0.89</v>
       </c>
       <c r="H98" s="2" t="inlineStr">
         <is>
@@ -4505,7 +4505,7 @@
       </c>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #3 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.97s.</t>
+          <t>User taps Issuance form action button #3 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.43s.</t>
         </is>
       </c>
       <c r="D99" s="2" t="inlineStr">
@@ -4524,7 +4524,7 @@
         </is>
       </c>
       <c r="G99" s="2" t="n">
-        <v>0.97</v>
+        <v>0.43</v>
       </c>
       <c r="H99" s="2" t="inlineStr">
         <is>
@@ -4546,7 +4546,7 @@
       </c>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #4 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.62s.</t>
+          <t>User taps Issuance form action button #4 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.4s.</t>
         </is>
       </c>
       <c r="D100" s="2" t="inlineStr">
@@ -4565,7 +4565,7 @@
         </is>
       </c>
       <c r="G100" s="2" t="n">
-        <v>0.62</v>
+        <v>0.4</v>
       </c>
       <c r="H100" s="2" t="inlineStr">
         <is>
@@ -4587,7 +4587,7 @@
       </c>
       <c r="C101" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #5 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.94s.</t>
+          <t>User taps Issuance form action button #5 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.42s.</t>
         </is>
       </c>
       <c r="D101" s="2" t="inlineStr">
@@ -4606,7 +4606,7 @@
         </is>
       </c>
       <c r="G101" s="2" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.42</v>
       </c>
       <c r="H101" s="2" t="inlineStr">
         <is>
@@ -4628,7 +4628,7 @@
       </c>
       <c r="C102" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #6 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.88s.</t>
+          <t>User taps Issuance form action button #6 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.46s.</t>
         </is>
       </c>
       <c r="D102" s="2" t="inlineStr">
@@ -4647,7 +4647,7 @@
         </is>
       </c>
       <c r="G102" s="2" t="n">
-        <v>0.88</v>
+        <v>0.46</v>
       </c>
       <c r="H102" s="2" t="inlineStr">
         <is>
@@ -4669,7 +4669,7 @@
       </c>
       <c r="C103" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #7 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.93s.</t>
+          <t>User taps Issuance form action button #7 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.46s.</t>
         </is>
       </c>
       <c r="D103" s="2" t="inlineStr">
@@ -4688,7 +4688,7 @@
         </is>
       </c>
       <c r="G103" s="2" t="n">
-        <v>0.93</v>
+        <v>0.46</v>
       </c>
       <c r="H103" s="2" t="inlineStr">
         <is>
@@ -4710,7 +4710,7 @@
       </c>
       <c r="C104" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #8 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.97s.</t>
+          <t>User taps Issuance form action button #8 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.4s.</t>
         </is>
       </c>
       <c r="D104" s="2" t="inlineStr">
@@ -4729,7 +4729,7 @@
         </is>
       </c>
       <c r="G104" s="2" t="n">
-        <v>0.97</v>
+        <v>0.4</v>
       </c>
       <c r="H104" s="2" t="inlineStr">
         <is>
@@ -4751,7 +4751,7 @@
       </c>
       <c r="C105" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #9 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 1.07s.</t>
+          <t>User taps Issuance form action button #9 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.6s.</t>
         </is>
       </c>
       <c r="D105" s="2" t="inlineStr">
@@ -4770,7 +4770,7 @@
         </is>
       </c>
       <c r="G105" s="2" t="n">
-        <v>1.07</v>
+        <v>0.6</v>
       </c>
       <c r="H105" s="2" t="inlineStr">
         <is>
@@ -4792,7 +4792,7 @@
       </c>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #10 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.84s.</t>
+          <t>User taps Issuance form action button #10 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 1.02s.</t>
         </is>
       </c>
       <c r="D106" s="2" t="inlineStr">
@@ -4811,7 +4811,7 @@
         </is>
       </c>
       <c r="G106" s="2" t="n">
-        <v>0.84</v>
+        <v>1.02</v>
       </c>
       <c r="H106" s="2" t="inlineStr">
         <is>
@@ -4833,7 +4833,7 @@
       </c>
       <c r="C107" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #11 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.87s.</t>
+          <t>User taps Issuance form action button #11 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.86s.</t>
         </is>
       </c>
       <c r="D107" s="2" t="inlineStr">
@@ -4852,7 +4852,7 @@
         </is>
       </c>
       <c r="G107" s="2" t="n">
-        <v>0.87</v>
+        <v>0.86</v>
       </c>
       <c r="H107" s="2" t="inlineStr">
         <is>
@@ -4874,7 +4874,7 @@
       </c>
       <c r="C108" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #12 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.88s.</t>
+          <t>User taps Issuance form action button #12 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.39s.</t>
         </is>
       </c>
       <c r="D108" s="2" t="inlineStr">
@@ -4893,7 +4893,7 @@
         </is>
       </c>
       <c r="G108" s="2" t="n">
-        <v>0.88</v>
+        <v>0.39</v>
       </c>
       <c r="H108" s="2" t="inlineStr">
         <is>
@@ -4915,7 +4915,7 @@
       </c>
       <c r="C109" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #13 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 1.06s.</t>
+          <t>User taps Issuance form action button #13 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.6s.</t>
         </is>
       </c>
       <c r="D109" s="2" t="inlineStr">
@@ -4934,7 +4934,7 @@
         </is>
       </c>
       <c r="G109" s="2" t="n">
-        <v>1.06</v>
+        <v>0.6</v>
       </c>
       <c r="H109" s="2" t="inlineStr">
         <is>
@@ -4956,7 +4956,7 @@
       </c>
       <c r="C110" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #14 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.86s.</t>
+          <t>User taps Issuance form action button #14 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.97s.</t>
         </is>
       </c>
       <c r="D110" s="2" t="inlineStr">
@@ -4975,7 +4975,7 @@
         </is>
       </c>
       <c r="G110" s="2" t="n">
-        <v>0.86</v>
+        <v>0.97</v>
       </c>
       <c r="H110" s="2" t="inlineStr">
         <is>
@@ -4997,7 +4997,7 @@
       </c>
       <c r="C111" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #15 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.51s.</t>
+          <t>User taps Issuance form action button #15 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.8s.</t>
         </is>
       </c>
       <c r="D111" s="2" t="inlineStr">
@@ -5016,7 +5016,7 @@
         </is>
       </c>
       <c r="G111" s="2" t="n">
-        <v>0.51</v>
+        <v>0.8</v>
       </c>
       <c r="H111" s="2" t="inlineStr">
         <is>
@@ -5038,7 +5038,7 @@
       </c>
       <c r="C112" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #16 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 1.1s.</t>
+          <t>User taps Issuance form action button #16 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 1.09s.</t>
         </is>
       </c>
       <c r="D112" s="2" t="inlineStr">
@@ -5057,7 +5057,7 @@
         </is>
       </c>
       <c r="G112" s="2" t="n">
-        <v>1.1</v>
+        <v>1.09</v>
       </c>
       <c r="H112" s="2" t="inlineStr">
         <is>
@@ -5079,7 +5079,7 @@
       </c>
       <c r="C113" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #17 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.82s.</t>
+          <t>User taps Issuance form action button #17 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.99s.</t>
         </is>
       </c>
       <c r="D113" s="2" t="inlineStr">
@@ -5098,7 +5098,7 @@
         </is>
       </c>
       <c r="G113" s="2" t="n">
-        <v>0.82</v>
+        <v>0.99</v>
       </c>
       <c r="H113" s="2" t="inlineStr">
         <is>
@@ -5120,7 +5120,7 @@
       </c>
       <c r="C114" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #18 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.86s.</t>
+          <t>User taps Issuance form action button #18 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.47s.</t>
         </is>
       </c>
       <c r="D114" s="2" t="inlineStr">
@@ -5139,7 +5139,7 @@
         </is>
       </c>
       <c r="G114" s="2" t="n">
-        <v>0.86</v>
+        <v>0.47</v>
       </c>
       <c r="H114" s="2" t="inlineStr">
         <is>
@@ -5161,7 +5161,7 @@
       </c>
       <c r="C115" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #19 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 1.02s.</t>
+          <t>User taps Issuance form action button #19 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.91s.</t>
         </is>
       </c>
       <c r="D115" s="2" t="inlineStr">
@@ -5180,7 +5180,7 @@
         </is>
       </c>
       <c r="G115" s="2" t="n">
-        <v>1.02</v>
+        <v>0.91</v>
       </c>
       <c r="H115" s="2" t="inlineStr">
         <is>
@@ -5202,7 +5202,7 @@
       </c>
       <c r="C116" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #20 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.97s.</t>
+          <t>User taps Issuance form action button #20 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 1.06s.</t>
         </is>
       </c>
       <c r="D116" s="2" t="inlineStr">
@@ -5221,7 +5221,7 @@
         </is>
       </c>
       <c r="G116" s="2" t="n">
-        <v>0.97</v>
+        <v>1.06</v>
       </c>
       <c r="H116" s="2" t="inlineStr">
         <is>
@@ -5243,7 +5243,7 @@
       </c>
       <c r="C117" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #21 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.72s.</t>
+          <t>User taps Issuance form action button #21 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.97s.</t>
         </is>
       </c>
       <c r="D117" s="2" t="inlineStr">
@@ -5262,7 +5262,7 @@
         </is>
       </c>
       <c r="G117" s="2" t="n">
-        <v>0.72</v>
+        <v>0.97</v>
       </c>
       <c r="H117" s="2" t="inlineStr">
         <is>
@@ -5284,7 +5284,7 @@
       </c>
       <c r="C118" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #22 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.81s.</t>
+          <t>User taps Issuance form action button #22 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.84s.</t>
         </is>
       </c>
       <c r="D118" s="2" t="inlineStr">
@@ -5303,7 +5303,7 @@
         </is>
       </c>
       <c r="G118" s="2" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.84</v>
       </c>
       <c r="H118" s="2" t="inlineStr">
         <is>
@@ -5325,7 +5325,7 @@
       </c>
       <c r="C119" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #23 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 1.08s.</t>
+          <t>User taps Issuance form action button #23 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.44s.</t>
         </is>
       </c>
       <c r="D119" s="2" t="inlineStr">
@@ -5344,7 +5344,7 @@
         </is>
       </c>
       <c r="G119" s="2" t="n">
-        <v>1.08</v>
+        <v>0.44</v>
       </c>
       <c r="H119" s="2" t="inlineStr">
         <is>
@@ -5366,7 +5366,7 @@
       </c>
       <c r="C120" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #24 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.87s.</t>
+          <t>User taps Issuance form action button #24 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 1.01s.</t>
         </is>
       </c>
       <c r="D120" s="2" t="inlineStr">
@@ -5385,7 +5385,7 @@
         </is>
       </c>
       <c r="G120" s="2" t="n">
-        <v>0.87</v>
+        <v>1.01</v>
       </c>
       <c r="H120" s="2" t="inlineStr">
         <is>
@@ -5407,7 +5407,7 @@
       </c>
       <c r="C121" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #25 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.89s.</t>
+          <t>User taps Issuance form action button #25 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.65s.</t>
         </is>
       </c>
       <c r="D121" s="2" t="inlineStr">
@@ -5426,7 +5426,7 @@
         </is>
       </c>
       <c r="G121" s="2" t="n">
-        <v>0.89</v>
+        <v>0.65</v>
       </c>
       <c r="H121" s="2" t="inlineStr">
         <is>
@@ -5467,7 +5467,7 @@
         </is>
       </c>
       <c r="G122" s="2" t="n">
-        <v>0.38</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="H122" s="2" t="inlineStr">
         <is>
@@ -5508,7 +5508,7 @@
         </is>
       </c>
       <c r="G123" s="2" t="n">
-        <v>0.8</v>
+        <v>0.7</v>
       </c>
       <c r="H123" s="2" t="inlineStr">
         <is>
@@ -5549,7 +5549,7 @@
         </is>
       </c>
       <c r="G124" s="2" t="n">
-        <v>0.74</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="H124" s="2" t="inlineStr">
         <is>
@@ -5590,7 +5590,7 @@
         </is>
       </c>
       <c r="G125" s="2" t="n">
-        <v>0.62</v>
+        <v>0.36</v>
       </c>
       <c r="H125" s="2" t="inlineStr">
         <is>
@@ -5631,7 +5631,7 @@
         </is>
       </c>
       <c r="G126" s="2" t="n">
-        <v>0.67</v>
+        <v>0.38</v>
       </c>
       <c r="H126" s="2" t="inlineStr">
         <is>
@@ -5672,7 +5672,7 @@
         </is>
       </c>
       <c r="G127" s="2" t="n">
-        <v>0.42</v>
+        <v>0.76</v>
       </c>
       <c r="H127" s="2" t="inlineStr">
         <is>
@@ -5713,7 +5713,7 @@
         </is>
       </c>
       <c r="G128" s="2" t="n">
-        <v>0.58</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="H128" s="2" t="inlineStr">
         <is>
@@ -5754,7 +5754,7 @@
         </is>
       </c>
       <c r="G129" s="2" t="n">
-        <v>0.36</v>
+        <v>0.65</v>
       </c>
       <c r="H129" s="2" t="inlineStr">
         <is>
@@ -5795,7 +5795,7 @@
         </is>
       </c>
       <c r="G130" s="2" t="n">
-        <v>0.79</v>
+        <v>0.67</v>
       </c>
       <c r="H130" s="2" t="inlineStr">
         <is>
@@ -5836,7 +5836,7 @@
         </is>
       </c>
       <c r="G131" s="2" t="n">
-        <v>0.51</v>
+        <v>0.8</v>
       </c>
       <c r="H131" s="2" t="inlineStr">
         <is>
@@ -5858,7 +5858,7 @@
       </c>
       <c r="C132" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #1 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.39s.</t>
+          <t>User taps Registry interactive card/button #1 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.32s.</t>
         </is>
       </c>
       <c r="D132" s="2" t="inlineStr">
@@ -5877,7 +5877,7 @@
         </is>
       </c>
       <c r="G132" s="2" t="n">
-        <v>0.39</v>
+        <v>0.32</v>
       </c>
       <c r="H132" s="2" t="inlineStr">
         <is>
@@ -5899,7 +5899,7 @@
       </c>
       <c r="C133" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #2 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.38s.</t>
+          <t>User taps Registry interactive card/button #2 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.67s.</t>
         </is>
       </c>
       <c r="D133" s="2" t="inlineStr">
@@ -5918,7 +5918,7 @@
         </is>
       </c>
       <c r="G133" s="2" t="n">
-        <v>0.38</v>
+        <v>0.67</v>
       </c>
       <c r="H133" s="2" t="inlineStr">
         <is>
@@ -5940,7 +5940,7 @@
       </c>
       <c r="C134" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #3 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.85s.</t>
+          <t>User taps Registry interactive card/button #3 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.58s.</t>
         </is>
       </c>
       <c r="D134" s="2" t="inlineStr">
@@ -5959,7 +5959,7 @@
         </is>
       </c>
       <c r="G134" s="2" t="n">
-        <v>0.85</v>
+        <v>0.58</v>
       </c>
       <c r="H134" s="2" t="inlineStr">
         <is>
@@ -5981,7 +5981,7 @@
       </c>
       <c r="C135" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #4 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.56s.</t>
+          <t>User taps Registry interactive card/button #4 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.59s.</t>
         </is>
       </c>
       <c r="D135" s="2" t="inlineStr">
@@ -6000,7 +6000,7 @@
         </is>
       </c>
       <c r="G135" s="2" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.59</v>
       </c>
       <c r="H135" s="2" t="inlineStr">
         <is>
@@ -6022,7 +6022,7 @@
       </c>
       <c r="C136" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #5 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.62s.</t>
+          <t>User taps Registry interactive card/button #5 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.4s.</t>
         </is>
       </c>
       <c r="D136" s="2" t="inlineStr">
@@ -6041,7 +6041,7 @@
         </is>
       </c>
       <c r="G136" s="2" t="n">
-        <v>0.62</v>
+        <v>0.4</v>
       </c>
       <c r="H136" s="2" t="inlineStr">
         <is>
@@ -6063,7 +6063,7 @@
       </c>
       <c r="C137" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #6 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.44s.</t>
+          <t>User taps Registry interactive card/button #6 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.4s.</t>
         </is>
       </c>
       <c r="D137" s="2" t="inlineStr">
@@ -6082,7 +6082,7 @@
         </is>
       </c>
       <c r="G137" s="2" t="n">
-        <v>0.44</v>
+        <v>0.4</v>
       </c>
       <c r="H137" s="2" t="inlineStr">
         <is>
@@ -6104,7 +6104,7 @@
       </c>
       <c r="C138" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #7 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.62s.</t>
+          <t>User taps Registry interactive card/button #7 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.48s.</t>
         </is>
       </c>
       <c r="D138" s="2" t="inlineStr">
@@ -6123,7 +6123,7 @@
         </is>
       </c>
       <c r="G138" s="2" t="n">
-        <v>0.62</v>
+        <v>0.48</v>
       </c>
       <c r="H138" s="2" t="inlineStr">
         <is>
@@ -6145,7 +6145,7 @@
       </c>
       <c r="C139" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #8 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.41s.</t>
+          <t>User taps Registry interactive card/button #8 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.57s.</t>
         </is>
       </c>
       <c r="D139" s="2" t="inlineStr">
@@ -6164,7 +6164,7 @@
         </is>
       </c>
       <c r="G139" s="2" t="n">
-        <v>0.41</v>
+        <v>0.57</v>
       </c>
       <c r="H139" s="2" t="inlineStr">
         <is>
@@ -6186,7 +6186,7 @@
       </c>
       <c r="C140" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #9 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.46s.</t>
+          <t>User taps Registry interactive card/button #9 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.83s.</t>
         </is>
       </c>
       <c r="D140" s="2" t="inlineStr">
@@ -6205,7 +6205,7 @@
         </is>
       </c>
       <c r="G140" s="2" t="n">
-        <v>0.46</v>
+        <v>0.83</v>
       </c>
       <c r="H140" s="2" t="inlineStr">
         <is>
@@ -6227,7 +6227,7 @@
       </c>
       <c r="C141" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #10 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.74s.</t>
+          <t>User taps Registry interactive card/button #10 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.5s.</t>
         </is>
       </c>
       <c r="D141" s="2" t="inlineStr">
@@ -6246,7 +6246,7 @@
         </is>
       </c>
       <c r="G141" s="2" t="n">
-        <v>0.74</v>
+        <v>0.5</v>
       </c>
       <c r="H141" s="2" t="inlineStr">
         <is>
@@ -6268,7 +6268,7 @@
       </c>
       <c r="C142" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #11 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.32s.</t>
+          <t>User taps Registry interactive card/button #11 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.34s.</t>
         </is>
       </c>
       <c r="D142" s="2" t="inlineStr">
@@ -6287,7 +6287,7 @@
         </is>
       </c>
       <c r="G142" s="2" t="n">
-        <v>0.32</v>
+        <v>0.34</v>
       </c>
       <c r="H142" s="2" t="inlineStr">
         <is>
@@ -6309,7 +6309,7 @@
       </c>
       <c r="C143" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #12 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.35s.</t>
+          <t>User taps Registry interactive card/button #12 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.36s.</t>
         </is>
       </c>
       <c r="D143" s="2" t="inlineStr">
@@ -6328,7 +6328,7 @@
         </is>
       </c>
       <c r="G143" s="2" t="n">
-        <v>0.35</v>
+        <v>0.36</v>
       </c>
       <c r="H143" s="2" t="inlineStr">
         <is>
@@ -6350,7 +6350,7 @@
       </c>
       <c r="C144" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #13 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.55s.</t>
+          <t>User taps Registry interactive card/button #13 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.58s.</t>
         </is>
       </c>
       <c r="D144" s="2" t="inlineStr">
@@ -6369,7 +6369,7 @@
         </is>
       </c>
       <c r="G144" s="2" t="n">
-        <v>0.55</v>
+        <v>0.58</v>
       </c>
       <c r="H144" s="2" t="inlineStr">
         <is>
@@ -6391,7 +6391,7 @@
       </c>
       <c r="C145" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #14 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.39s.</t>
+          <t>User taps Registry interactive card/button #14 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.82s.</t>
         </is>
       </c>
       <c r="D145" s="2" t="inlineStr">
@@ -6410,7 +6410,7 @@
         </is>
       </c>
       <c r="G145" s="2" t="n">
-        <v>0.39</v>
+        <v>0.82</v>
       </c>
       <c r="H145" s="2" t="inlineStr">
         <is>
@@ -6432,7 +6432,7 @@
       </c>
       <c r="C146" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #15 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.59s.</t>
+          <t>User taps Registry interactive card/button #15 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.7s.</t>
         </is>
       </c>
       <c r="D146" s="2" t="inlineStr">
@@ -6451,7 +6451,7 @@
         </is>
       </c>
       <c r="G146" s="2" t="n">
-        <v>0.59</v>
+        <v>0.7</v>
       </c>
       <c r="H146" s="2" t="inlineStr">
         <is>
@@ -6473,7 +6473,7 @@
       </c>
       <c r="C147" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #16 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.65s.</t>
+          <t>User taps Registry interactive card/button #16 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.56s.</t>
         </is>
       </c>
       <c r="D147" s="2" t="inlineStr">
@@ -6492,7 +6492,7 @@
         </is>
       </c>
       <c r="G147" s="2" t="n">
-        <v>0.65</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="H147" s="2" t="inlineStr">
         <is>
@@ -6514,7 +6514,7 @@
       </c>
       <c r="C148" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #17 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.6s.</t>
+          <t>User taps Registry interactive card/button #17 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.67s.</t>
         </is>
       </c>
       <c r="D148" s="2" t="inlineStr">
@@ -6533,7 +6533,7 @@
         </is>
       </c>
       <c r="G148" s="2" t="n">
-        <v>0.6</v>
+        <v>0.67</v>
       </c>
       <c r="H148" s="2" t="inlineStr">
         <is>
@@ -6555,7 +6555,7 @@
       </c>
       <c r="C149" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #18 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.57s.</t>
+          <t>User taps Registry interactive card/button #18 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.75s.</t>
         </is>
       </c>
       <c r="D149" s="2" t="inlineStr">
@@ -6574,7 +6574,7 @@
         </is>
       </c>
       <c r="G149" s="2" t="n">
-        <v>0.57</v>
+        <v>0.75</v>
       </c>
       <c r="H149" s="2" t="inlineStr">
         <is>
@@ -6596,7 +6596,7 @@
       </c>
       <c r="C150" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #19 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.73s.</t>
+          <t>User taps Registry interactive card/button #19 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.57s.</t>
         </is>
       </c>
       <c r="D150" s="2" t="inlineStr">
@@ -6615,7 +6615,7 @@
         </is>
       </c>
       <c r="G150" s="2" t="n">
-        <v>0.73</v>
+        <v>0.57</v>
       </c>
       <c r="H150" s="2" t="inlineStr">
         <is>
@@ -6637,7 +6637,7 @@
       </c>
       <c r="C151" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #20 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.41s.</t>
+          <t>User taps Registry interactive card/button #20 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.6s.</t>
         </is>
       </c>
       <c r="D151" s="2" t="inlineStr">
@@ -6656,7 +6656,7 @@
         </is>
       </c>
       <c r="G151" s="2" t="n">
-        <v>0.41</v>
+        <v>0.6</v>
       </c>
       <c r="H151" s="2" t="inlineStr">
         <is>
@@ -6678,7 +6678,7 @@
       </c>
       <c r="C152" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #21 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.56s.</t>
+          <t>User taps Registry interactive card/button #21 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.51s.</t>
         </is>
       </c>
       <c r="D152" s="2" t="inlineStr">
@@ -6697,7 +6697,7 @@
         </is>
       </c>
       <c r="G152" s="2" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.51</v>
       </c>
       <c r="H152" s="2" t="inlineStr">
         <is>
@@ -6719,7 +6719,7 @@
       </c>
       <c r="C153" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #22 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.64s.</t>
+          <t>User taps Registry interactive card/button #22 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.31s.</t>
         </is>
       </c>
       <c r="D153" s="2" t="inlineStr">
@@ -6738,7 +6738,7 @@
         </is>
       </c>
       <c r="G153" s="2" t="n">
-        <v>0.64</v>
+        <v>0.31</v>
       </c>
       <c r="H153" s="2" t="inlineStr">
         <is>
@@ -6760,7 +6760,7 @@
       </c>
       <c r="C154" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #23 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.78s.</t>
+          <t>User taps Registry interactive card/button #23 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.45s.</t>
         </is>
       </c>
       <c r="D154" s="2" t="inlineStr">
@@ -6779,7 +6779,7 @@
         </is>
       </c>
       <c r="G154" s="2" t="n">
-        <v>0.78</v>
+        <v>0.45</v>
       </c>
       <c r="H154" s="2" t="inlineStr">
         <is>
@@ -6801,7 +6801,7 @@
       </c>
       <c r="C155" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #24 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.35s.</t>
+          <t>User taps Registry interactive card/button #24 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.69s.</t>
         </is>
       </c>
       <c r="D155" s="2" t="inlineStr">
@@ -6820,7 +6820,7 @@
         </is>
       </c>
       <c r="G155" s="2" t="n">
-        <v>0.35</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="H155" s="2" t="inlineStr">
         <is>
@@ -6842,7 +6842,7 @@
       </c>
       <c r="C156" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #25 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.62s.</t>
+          <t>User taps Registry interactive card/button #25 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.56s.</t>
         </is>
       </c>
       <c r="D156" s="2" t="inlineStr">
@@ -6861,7 +6861,7 @@
         </is>
       </c>
       <c r="G156" s="2" t="n">
-        <v>0.62</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="H156" s="2" t="inlineStr">
         <is>
@@ -6883,7 +6883,7 @@
       </c>
       <c r="C157" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #26 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.54s.</t>
+          <t>User taps Registry interactive card/button #26 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.8s.</t>
         </is>
       </c>
       <c r="D157" s="2" t="inlineStr">
@@ -6902,7 +6902,7 @@
         </is>
       </c>
       <c r="G157" s="2" t="n">
-        <v>0.54</v>
+        <v>0.8</v>
       </c>
       <c r="H157" s="2" t="inlineStr">
         <is>
@@ -6924,7 +6924,7 @@
       </c>
       <c r="C158" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #27 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.61s.</t>
+          <t>User taps Registry interactive card/button #27 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.67s.</t>
         </is>
       </c>
       <c r="D158" s="2" t="inlineStr">
@@ -6943,7 +6943,7 @@
         </is>
       </c>
       <c r="G158" s="2" t="n">
-        <v>0.61</v>
+        <v>0.67</v>
       </c>
       <c r="H158" s="2" t="inlineStr">
         <is>
@@ -6965,7 +6965,7 @@
       </c>
       <c r="C159" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #28 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.79s.</t>
+          <t>User taps Registry interactive card/button #28 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.81s.</t>
         </is>
       </c>
       <c r="D159" s="2" t="inlineStr">
@@ -6984,7 +6984,7 @@
         </is>
       </c>
       <c r="G159" s="2" t="n">
-        <v>0.79</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="H159" s="2" t="inlineStr">
         <is>
@@ -7006,7 +7006,7 @@
       </c>
       <c r="C160" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #29 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.44s.</t>
+          <t>User taps Registry interactive card/button #29 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.39s.</t>
         </is>
       </c>
       <c r="D160" s="2" t="inlineStr">
@@ -7025,7 +7025,7 @@
         </is>
       </c>
       <c r="G160" s="2" t="n">
-        <v>0.44</v>
+        <v>0.39</v>
       </c>
       <c r="H160" s="2" t="inlineStr">
         <is>
@@ -7047,7 +7047,7 @@
       </c>
       <c r="C161" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #30 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.78s.</t>
+          <t>User taps Registry interactive card/button #30 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.48s.</t>
         </is>
       </c>
       <c r="D161" s="2" t="inlineStr">
@@ -7066,7 +7066,7 @@
         </is>
       </c>
       <c r="G161" s="2" t="n">
-        <v>0.78</v>
+        <v>0.48</v>
       </c>
       <c r="H161" s="2" t="inlineStr">
         <is>
@@ -7107,7 +7107,7 @@
         </is>
       </c>
       <c r="G162" s="2" t="n">
-        <v>0.67</v>
+        <v>0.62</v>
       </c>
       <c r="H162" s="2" t="inlineStr">
         <is>
@@ -7148,7 +7148,7 @@
         </is>
       </c>
       <c r="G163" s="2" t="n">
-        <v>0.49</v>
+        <v>0.53</v>
       </c>
       <c r="H163" s="2" t="inlineStr">
         <is>
@@ -7189,7 +7189,7 @@
         </is>
       </c>
       <c r="G164" s="2" t="n">
-        <v>0.4</v>
+        <v>0.46</v>
       </c>
       <c r="H164" s="2" t="inlineStr">
         <is>
@@ -7230,7 +7230,7 @@
         </is>
       </c>
       <c r="G165" s="2" t="n">
-        <v>0.51</v>
+        <v>0.74</v>
       </c>
       <c r="H165" s="2" t="inlineStr">
         <is>
@@ -7271,7 +7271,7 @@
         </is>
       </c>
       <c r="G166" s="2" t="n">
-        <v>0.42</v>
+        <v>0.53</v>
       </c>
       <c r="H166" s="2" t="inlineStr">
         <is>
@@ -7293,7 +7293,7 @@
       </c>
       <c r="C167" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #1 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.43s.</t>
+          <t>User taps Network diagnostic button #1 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.36s.</t>
         </is>
       </c>
       <c r="D167" s="2" t="inlineStr">
@@ -7312,7 +7312,7 @@
         </is>
       </c>
       <c r="G167" s="2" t="n">
-        <v>0.43</v>
+        <v>0.36</v>
       </c>
       <c r="H167" s="2" t="inlineStr">
         <is>
@@ -7334,7 +7334,7 @@
       </c>
       <c r="C168" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #2 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.74s.</t>
+          <t>User taps Network diagnostic button #2 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.63s.</t>
         </is>
       </c>
       <c r="D168" s="2" t="inlineStr">
@@ -7353,7 +7353,7 @@
         </is>
       </c>
       <c r="G168" s="2" t="n">
-        <v>0.74</v>
+        <v>0.63</v>
       </c>
       <c r="H168" s="2" t="inlineStr">
         <is>
@@ -7375,7 +7375,7 @@
       </c>
       <c r="C169" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #3 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.44s.</t>
+          <t>User taps Network diagnostic button #3 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.46s.</t>
         </is>
       </c>
       <c r="D169" s="2" t="inlineStr">
@@ -7394,7 +7394,7 @@
         </is>
       </c>
       <c r="G169" s="2" t="n">
-        <v>0.44</v>
+        <v>0.46</v>
       </c>
       <c r="H169" s="2" t="inlineStr">
         <is>
@@ -7416,7 +7416,7 @@
       </c>
       <c r="C170" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #4 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.67s.</t>
+          <t>User taps Network diagnostic button #4 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.38s.</t>
         </is>
       </c>
       <c r="D170" s="2" t="inlineStr">
@@ -7435,7 +7435,7 @@
         </is>
       </c>
       <c r="G170" s="2" t="n">
-        <v>0.67</v>
+        <v>0.38</v>
       </c>
       <c r="H170" s="2" t="inlineStr">
         <is>
@@ -7457,7 +7457,7 @@
       </c>
       <c r="C171" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #5 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.68s.</t>
+          <t>User taps Network diagnostic button #5 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.44s.</t>
         </is>
       </c>
       <c r="D171" s="2" t="inlineStr">
@@ -7476,7 +7476,7 @@
         </is>
       </c>
       <c r="G171" s="2" t="n">
-        <v>0.68</v>
+        <v>0.44</v>
       </c>
       <c r="H171" s="2" t="inlineStr">
         <is>
@@ -7498,7 +7498,7 @@
       </c>
       <c r="C172" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #6 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.39s.</t>
+          <t>User taps Network diagnostic button #6 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.47s.</t>
         </is>
       </c>
       <c r="D172" s="2" t="inlineStr">
@@ -7517,7 +7517,7 @@
         </is>
       </c>
       <c r="G172" s="2" t="n">
-        <v>0.39</v>
+        <v>0.47</v>
       </c>
       <c r="H172" s="2" t="inlineStr">
         <is>
@@ -7539,7 +7539,7 @@
       </c>
       <c r="C173" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #7 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.28s.</t>
+          <t>User taps Network diagnostic button #7 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.35s.</t>
         </is>
       </c>
       <c r="D173" s="2" t="inlineStr">
@@ -7558,7 +7558,7 @@
         </is>
       </c>
       <c r="G173" s="2" t="n">
-        <v>0.28</v>
+        <v>0.35</v>
       </c>
       <c r="H173" s="2" t="inlineStr">
         <is>
@@ -7580,7 +7580,7 @@
       </c>
       <c r="C174" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #8 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.41s.</t>
+          <t>User taps Network diagnostic button #8 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.56s.</t>
         </is>
       </c>
       <c r="D174" s="2" t="inlineStr">
@@ -7599,7 +7599,7 @@
         </is>
       </c>
       <c r="G174" s="2" t="n">
-        <v>0.41</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="H174" s="2" t="inlineStr">
         <is>
@@ -7621,7 +7621,7 @@
       </c>
       <c r="C175" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #9 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.31s.</t>
+          <t>User taps Network diagnostic button #9 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.59s.</t>
         </is>
       </c>
       <c r="D175" s="2" t="inlineStr">
@@ -7640,7 +7640,7 @@
         </is>
       </c>
       <c r="G175" s="2" t="n">
-        <v>0.31</v>
+        <v>0.59</v>
       </c>
       <c r="H175" s="2" t="inlineStr">
         <is>
@@ -7662,7 +7662,7 @@
       </c>
       <c r="C176" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #10 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.61s.</t>
+          <t>User taps Network diagnostic button #10 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.63s.</t>
         </is>
       </c>
       <c r="D176" s="2" t="inlineStr">
@@ -7681,7 +7681,7 @@
         </is>
       </c>
       <c r="G176" s="2" t="n">
-        <v>0.61</v>
+        <v>0.63</v>
       </c>
       <c r="H176" s="2" t="inlineStr">
         <is>
@@ -7703,7 +7703,7 @@
       </c>
       <c r="C177" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #11 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.34s.</t>
+          <t>User taps Network diagnostic button #11 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.77s.</t>
         </is>
       </c>
       <c r="D177" s="2" t="inlineStr">
@@ -7722,7 +7722,7 @@
         </is>
       </c>
       <c r="G177" s="2" t="n">
-        <v>0.34</v>
+        <v>0.77</v>
       </c>
       <c r="H177" s="2" t="inlineStr">
         <is>
@@ -7744,7 +7744,7 @@
       </c>
       <c r="C178" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #12 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.78s.</t>
+          <t>User taps Network diagnostic button #12 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.34s.</t>
         </is>
       </c>
       <c r="D178" s="2" t="inlineStr">
@@ -7763,7 +7763,7 @@
         </is>
       </c>
       <c r="G178" s="2" t="n">
-        <v>0.78</v>
+        <v>0.34</v>
       </c>
       <c r="H178" s="2" t="inlineStr">
         <is>
@@ -7826,7 +7826,7 @@
       </c>
       <c r="C180" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #14 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.57s.</t>
+          <t>User taps Network diagnostic button #14 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.75s.</t>
         </is>
       </c>
       <c r="D180" s="2" t="inlineStr">
@@ -7845,7 +7845,7 @@
         </is>
       </c>
       <c r="G180" s="2" t="n">
-        <v>0.57</v>
+        <v>0.75</v>
       </c>
       <c r="H180" s="2" t="inlineStr">
         <is>
@@ -7867,7 +7867,7 @@
       </c>
       <c r="C181" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #15 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.46s.</t>
+          <t>User taps Network diagnostic button #15 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.39s.</t>
         </is>
       </c>
       <c r="D181" s="2" t="inlineStr">
@@ -7886,7 +7886,7 @@
         </is>
       </c>
       <c r="G181" s="2" t="n">
-        <v>0.46</v>
+        <v>0.39</v>
       </c>
       <c r="H181" s="2" t="inlineStr">
         <is>
@@ -7908,7 +7908,7 @@
       </c>
       <c r="C182" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #16 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.7s.</t>
+          <t>User taps Network diagnostic button #16 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.61s.</t>
         </is>
       </c>
       <c r="D182" s="2" t="inlineStr">
@@ -7927,7 +7927,7 @@
         </is>
       </c>
       <c r="G182" s="2" t="n">
-        <v>0.7</v>
+        <v>0.61</v>
       </c>
       <c r="H182" s="2" t="inlineStr">
         <is>
@@ -7949,7 +7949,7 @@
       </c>
       <c r="C183" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #17 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.32s.</t>
+          <t>User taps Network diagnostic button #17 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.63s.</t>
         </is>
       </c>
       <c r="D183" s="2" t="inlineStr">
@@ -7968,7 +7968,7 @@
         </is>
       </c>
       <c r="G183" s="2" t="n">
-        <v>0.32</v>
+        <v>0.63</v>
       </c>
       <c r="H183" s="2" t="inlineStr">
         <is>
@@ -7990,7 +7990,7 @@
       </c>
       <c r="C184" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #18 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.45s.</t>
+          <t>User taps Network diagnostic button #18 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.3s.</t>
         </is>
       </c>
       <c r="D184" s="2" t="inlineStr">
@@ -8009,7 +8009,7 @@
         </is>
       </c>
       <c r="G184" s="2" t="n">
-        <v>0.45</v>
+        <v>0.3</v>
       </c>
       <c r="H184" s="2" t="inlineStr">
         <is>
@@ -8031,7 +8031,7 @@
       </c>
       <c r="C185" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #19 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.47s.</t>
+          <t>User taps Network diagnostic button #19 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.77s.</t>
         </is>
       </c>
       <c r="D185" s="2" t="inlineStr">
@@ -8050,7 +8050,7 @@
         </is>
       </c>
       <c r="G185" s="2" t="n">
-        <v>0.47</v>
+        <v>0.77</v>
       </c>
       <c r="H185" s="2" t="inlineStr">
         <is>
@@ -8072,7 +8072,7 @@
       </c>
       <c r="C186" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #20 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.73s.</t>
+          <t>User taps Network diagnostic button #20 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.37s.</t>
         </is>
       </c>
       <c r="D186" s="2" t="inlineStr">
@@ -8091,7 +8091,7 @@
         </is>
       </c>
       <c r="G186" s="2" t="n">
-        <v>0.73</v>
+        <v>0.37</v>
       </c>
       <c r="H186" s="2" t="inlineStr">
         <is>
@@ -8113,7 +8113,7 @@
       </c>
       <c r="C187" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #21 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.53s.</t>
+          <t>User taps Network diagnostic button #21 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.31s.</t>
         </is>
       </c>
       <c r="D187" s="2" t="inlineStr">
@@ -8132,7 +8132,7 @@
         </is>
       </c>
       <c r="G187" s="2" t="n">
-        <v>0.53</v>
+        <v>0.31</v>
       </c>
       <c r="H187" s="2" t="inlineStr">
         <is>
@@ -8154,7 +8154,7 @@
       </c>
       <c r="C188" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #22 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.65s.</t>
+          <t>User taps Network diagnostic button #22 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.41s.</t>
         </is>
       </c>
       <c r="D188" s="2" t="inlineStr">
@@ -8173,7 +8173,7 @@
         </is>
       </c>
       <c r="G188" s="2" t="n">
-        <v>0.65</v>
+        <v>0.41</v>
       </c>
       <c r="H188" s="2" t="inlineStr">
         <is>
@@ -8195,7 +8195,7 @@
       </c>
       <c r="C189" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #23 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.59s.</t>
+          <t>User taps Network diagnostic button #23 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.72s.</t>
         </is>
       </c>
       <c r="D189" s="2" t="inlineStr">
@@ -8214,7 +8214,7 @@
         </is>
       </c>
       <c r="G189" s="2" t="n">
-        <v>0.59</v>
+        <v>0.72</v>
       </c>
       <c r="H189" s="2" t="inlineStr">
         <is>
@@ -8236,7 +8236,7 @@
       </c>
       <c r="C190" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #24 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.54s.</t>
+          <t>User taps Network diagnostic button #24 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.51s.</t>
         </is>
       </c>
       <c r="D190" s="2" t="inlineStr">
@@ -8255,7 +8255,7 @@
         </is>
       </c>
       <c r="G190" s="2" t="n">
-        <v>0.54</v>
+        <v>0.51</v>
       </c>
       <c r="H190" s="2" t="inlineStr">
         <is>
@@ -8277,7 +8277,7 @@
       </c>
       <c r="C191" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #25 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.69s.</t>
+          <t>User taps Network diagnostic button #25 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.78s.</t>
         </is>
       </c>
       <c r="D191" s="2" t="inlineStr">
@@ -8296,7 +8296,7 @@
         </is>
       </c>
       <c r="G191" s="2" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.78</v>
       </c>
       <c r="H191" s="2" t="inlineStr">
         <is>
@@ -8359,7 +8359,7 @@
       </c>
       <c r="C193" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #27 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.67s.</t>
+          <t>User taps Network diagnostic button #27 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.62s.</t>
         </is>
       </c>
       <c r="D193" s="2" t="inlineStr">
@@ -8378,7 +8378,7 @@
         </is>
       </c>
       <c r="G193" s="2" t="n">
-        <v>0.67</v>
+        <v>0.62</v>
       </c>
       <c r="H193" s="2" t="inlineStr">
         <is>
@@ -8400,7 +8400,7 @@
       </c>
       <c r="C194" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #28 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.6s.</t>
+          <t>User taps Network diagnostic button #28 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.41s.</t>
         </is>
       </c>
       <c r="D194" s="2" t="inlineStr">
@@ -8419,7 +8419,7 @@
         </is>
       </c>
       <c r="G194" s="2" t="n">
-        <v>0.6</v>
+        <v>0.41</v>
       </c>
       <c r="H194" s="2" t="inlineStr">
         <is>
@@ -8441,7 +8441,7 @@
       </c>
       <c r="C195" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #29 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.43s.</t>
+          <t>User taps Network diagnostic button #29 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.47s.</t>
         </is>
       </c>
       <c r="D195" s="2" t="inlineStr">
@@ -8460,7 +8460,7 @@
         </is>
       </c>
       <c r="G195" s="2" t="n">
-        <v>0.43</v>
+        <v>0.47</v>
       </c>
       <c r="H195" s="2" t="inlineStr">
         <is>
@@ -8482,7 +8482,7 @@
       </c>
       <c r="C196" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #30 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.68s.</t>
+          <t>User taps Network diagnostic button #30 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.61s.</t>
         </is>
       </c>
       <c r="D196" s="2" t="inlineStr">
@@ -8501,7 +8501,7 @@
         </is>
       </c>
       <c r="G196" s="2" t="n">
-        <v>0.68</v>
+        <v>0.61</v>
       </c>
       <c r="H196" s="2" t="inlineStr">
         <is>
@@ -8542,7 +8542,7 @@
         </is>
       </c>
       <c r="G197" s="2" t="n">
-        <v>1.16</v>
+        <v>0.91</v>
       </c>
       <c r="H197" s="2" t="inlineStr">
         <is>
@@ -8583,7 +8583,7 @@
         </is>
       </c>
       <c r="G198" s="2" t="n">
-        <v>0.47</v>
+        <v>0.55</v>
       </c>
       <c r="H198" s="2" t="inlineStr">
         <is>
@@ -8624,7 +8624,7 @@
         </is>
       </c>
       <c r="G199" s="2" t="n">
-        <v>1.12</v>
+        <v>0.58</v>
       </c>
       <c r="H199" s="2" t="inlineStr">
         <is>
@@ -8665,7 +8665,7 @@
         </is>
       </c>
       <c r="G200" s="2" t="n">
-        <v>1.17</v>
+        <v>1.06</v>
       </c>
       <c r="H200" s="2" t="inlineStr">
         <is>
@@ -8706,7 +8706,7 @@
         </is>
       </c>
       <c r="G201" s="2" t="n">
-        <v>0.95</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="H201" s="2" t="inlineStr">
         <is>
@@ -8747,7 +8747,7 @@
         </is>
       </c>
       <c r="G202" s="2" t="n">
-        <v>0.67</v>
+        <v>0.43</v>
       </c>
       <c r="H202" s="2" t="inlineStr">
         <is>
@@ -8788,7 +8788,7 @@
         </is>
       </c>
       <c r="G203" s="2" t="n">
-        <v>0.89</v>
+        <v>1.1</v>
       </c>
       <c r="H203" s="2" t="inlineStr">
         <is>
@@ -8810,7 +8810,7 @@
       </c>
       <c r="C204" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #1 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.95s.</t>
+          <t>User executes touch gesture #1 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.48s.</t>
         </is>
       </c>
       <c r="D204" s="2" t="inlineStr">
@@ -8829,7 +8829,7 @@
         </is>
       </c>
       <c r="G204" s="2" t="n">
-        <v>0.95</v>
+        <v>0.48</v>
       </c>
       <c r="H204" s="2" t="inlineStr">
         <is>
@@ -8851,7 +8851,7 @@
       </c>
       <c r="C205" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #2 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.43s.</t>
+          <t>User executes touch gesture #2 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.69s.</t>
         </is>
       </c>
       <c r="D205" s="2" t="inlineStr">
@@ -8870,7 +8870,7 @@
         </is>
       </c>
       <c r="G205" s="2" t="n">
-        <v>0.43</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="H205" s="2" t="inlineStr">
         <is>
@@ -8892,7 +8892,7 @@
       </c>
       <c r="C206" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #3 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.92s.</t>
+          <t>User executes touch gesture #3 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.2s.</t>
         </is>
       </c>
       <c r="D206" s="2" t="inlineStr">
@@ -8911,7 +8911,7 @@
         </is>
       </c>
       <c r="G206" s="2" t="n">
-        <v>0.92</v>
+        <v>1.2</v>
       </c>
       <c r="H206" s="2" t="inlineStr">
         <is>
@@ -8933,7 +8933,7 @@
       </c>
       <c r="C207" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #4 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.7s.</t>
+          <t>User executes touch gesture #4 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.96s.</t>
         </is>
       </c>
       <c r="D207" s="2" t="inlineStr">
@@ -8952,7 +8952,7 @@
         </is>
       </c>
       <c r="G207" s="2" t="n">
-        <v>0.7</v>
+        <v>0.96</v>
       </c>
       <c r="H207" s="2" t="inlineStr">
         <is>
@@ -9015,7 +9015,7 @@
       </c>
       <c r="C209" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #6 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.45s.</t>
+          <t>User executes touch gesture #6 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.94s.</t>
         </is>
       </c>
       <c r="D209" s="2" t="inlineStr">
@@ -9034,7 +9034,7 @@
         </is>
       </c>
       <c r="G209" s="2" t="n">
-        <v>0.45</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="H209" s="2" t="inlineStr">
         <is>
@@ -9056,7 +9056,7 @@
       </c>
       <c r="C210" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #7 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.63s.</t>
+          <t>User executes touch gesture #7 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.89s.</t>
         </is>
       </c>
       <c r="D210" s="2" t="inlineStr">
@@ -9075,7 +9075,7 @@
         </is>
       </c>
       <c r="G210" s="2" t="n">
-        <v>0.63</v>
+        <v>0.89</v>
       </c>
       <c r="H210" s="2" t="inlineStr">
         <is>
@@ -9097,7 +9097,7 @@
       </c>
       <c r="C211" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #8 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.19s.</t>
+          <t>User executes touch gesture #8 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.37s.</t>
         </is>
       </c>
       <c r="D211" s="2" t="inlineStr">
@@ -9116,7 +9116,7 @@
         </is>
       </c>
       <c r="G211" s="2" t="n">
-        <v>1.19</v>
+        <v>0.37</v>
       </c>
       <c r="H211" s="2" t="inlineStr">
         <is>
@@ -9138,7 +9138,7 @@
       </c>
       <c r="C212" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #9 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.73s.</t>
+          <t>User executes touch gesture #9 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.85s.</t>
         </is>
       </c>
       <c r="D212" s="2" t="inlineStr">
@@ -9157,7 +9157,7 @@
         </is>
       </c>
       <c r="G212" s="2" t="n">
-        <v>0.73</v>
+        <v>0.85</v>
       </c>
       <c r="H212" s="2" t="inlineStr">
         <is>
@@ -9179,7 +9179,7 @@
       </c>
       <c r="C213" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #10 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.25s.</t>
+          <t>User executes touch gesture #10 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.96s.</t>
         </is>
       </c>
       <c r="D213" s="2" t="inlineStr">
@@ -9198,7 +9198,7 @@
         </is>
       </c>
       <c r="G213" s="2" t="n">
-        <v>1.25</v>
+        <v>0.96</v>
       </c>
       <c r="H213" s="2" t="inlineStr">
         <is>
@@ -9220,7 +9220,7 @@
       </c>
       <c r="C214" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #11 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.01s.</t>
+          <t>User executes touch gesture #11 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.17s.</t>
         </is>
       </c>
       <c r="D214" s="2" t="inlineStr">
@@ -9239,7 +9239,7 @@
         </is>
       </c>
       <c r="G214" s="2" t="n">
-        <v>1.01</v>
+        <v>1.17</v>
       </c>
       <c r="H214" s="2" t="inlineStr">
         <is>
@@ -9261,7 +9261,7 @@
       </c>
       <c r="C215" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #12 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.63s.</t>
+          <t>User executes touch gesture #12 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.71s.</t>
         </is>
       </c>
       <c r="D215" s="2" t="inlineStr">
@@ -9280,7 +9280,7 @@
         </is>
       </c>
       <c r="G215" s="2" t="n">
-        <v>0.63</v>
+        <v>0.71</v>
       </c>
       <c r="H215" s="2" t="inlineStr">
         <is>
@@ -9343,7 +9343,7 @@
       </c>
       <c r="C217" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #14 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.97s.</t>
+          <t>User executes touch gesture #14 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.64s.</t>
         </is>
       </c>
       <c r="D217" s="2" t="inlineStr">
@@ -9362,7 +9362,7 @@
         </is>
       </c>
       <c r="G217" s="2" t="n">
-        <v>0.97</v>
+        <v>0.64</v>
       </c>
       <c r="H217" s="2" t="inlineStr">
         <is>
@@ -9384,7 +9384,7 @@
       </c>
       <c r="C218" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #15 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.25s.</t>
+          <t>User executes touch gesture #15 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.38s.</t>
         </is>
       </c>
       <c r="D218" s="2" t="inlineStr">
@@ -9403,7 +9403,7 @@
         </is>
       </c>
       <c r="G218" s="2" t="n">
-        <v>1.25</v>
+        <v>0.38</v>
       </c>
       <c r="H218" s="2" t="inlineStr">
         <is>
@@ -9425,7 +9425,7 @@
       </c>
       <c r="C219" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #16 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.38s.</t>
+          <t>User executes touch gesture #16 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.08s.</t>
         </is>
       </c>
       <c r="D219" s="2" t="inlineStr">
@@ -9444,7 +9444,7 @@
         </is>
       </c>
       <c r="G219" s="2" t="n">
-        <v>0.38</v>
+        <v>1.08</v>
       </c>
       <c r="H219" s="2" t="inlineStr">
         <is>
@@ -9466,7 +9466,7 @@
       </c>
       <c r="C220" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #17 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.74s.</t>
+          <t>User executes touch gesture #17 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.38s.</t>
         </is>
       </c>
       <c r="D220" s="2" t="inlineStr">
@@ -9485,7 +9485,7 @@
         </is>
       </c>
       <c r="G220" s="2" t="n">
-        <v>0.74</v>
+        <v>0.38</v>
       </c>
       <c r="H220" s="2" t="inlineStr">
         <is>
@@ -9507,7 +9507,7 @@
       </c>
       <c r="C221" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #18 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.59s.</t>
+          <t>User executes touch gesture #18 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.36s.</t>
         </is>
       </c>
       <c r="D221" s="2" t="inlineStr">
@@ -9526,7 +9526,7 @@
         </is>
       </c>
       <c r="G221" s="2" t="n">
-        <v>0.59</v>
+        <v>0.36</v>
       </c>
       <c r="H221" s="2" t="inlineStr">
         <is>
@@ -9548,7 +9548,7 @@
       </c>
       <c r="C222" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #19 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.17s.</t>
+          <t>User executes touch gesture #19 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.69s.</t>
         </is>
       </c>
       <c r="D222" s="2" t="inlineStr">
@@ -9567,7 +9567,7 @@
         </is>
       </c>
       <c r="G222" s="2" t="n">
-        <v>1.17</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="H222" s="2" t="inlineStr">
         <is>
@@ -9589,7 +9589,7 @@
       </c>
       <c r="C223" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #20 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.06s.</t>
+          <t>User executes touch gesture #20 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.62s.</t>
         </is>
       </c>
       <c r="D223" s="2" t="inlineStr">
@@ -9608,7 +9608,7 @@
         </is>
       </c>
       <c r="G223" s="2" t="n">
-        <v>1.06</v>
+        <v>0.62</v>
       </c>
       <c r="H223" s="2" t="inlineStr">
         <is>
@@ -9630,7 +9630,7 @@
       </c>
       <c r="C224" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #21 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.15s.</t>
+          <t>User executes touch gesture #21 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.93s.</t>
         </is>
       </c>
       <c r="D224" s="2" t="inlineStr">
@@ -9649,7 +9649,7 @@
         </is>
       </c>
       <c r="G224" s="2" t="n">
-        <v>1.15</v>
+        <v>0.93</v>
       </c>
       <c r="H224" s="2" t="inlineStr">
         <is>
@@ -9671,7 +9671,7 @@
       </c>
       <c r="C225" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #22 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.71s.</t>
+          <t>User executes touch gesture #22 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.67s.</t>
         </is>
       </c>
       <c r="D225" s="2" t="inlineStr">
@@ -9690,7 +9690,7 @@
         </is>
       </c>
       <c r="G225" s="2" t="n">
-        <v>0.71</v>
+        <v>0.67</v>
       </c>
       <c r="H225" s="2" t="inlineStr">
         <is>
@@ -9712,7 +9712,7 @@
       </c>
       <c r="C226" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #23 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.72s.</t>
+          <t>User executes touch gesture #23 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.99s.</t>
         </is>
       </c>
       <c r="D226" s="2" t="inlineStr">
@@ -9731,7 +9731,7 @@
         </is>
       </c>
       <c r="G226" s="2" t="n">
-        <v>0.72</v>
+        <v>0.99</v>
       </c>
       <c r="H226" s="2" t="inlineStr">
         <is>
@@ -9753,7 +9753,7 @@
       </c>
       <c r="C227" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #24 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.97s.</t>
+          <t>User executes touch gesture #24 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.43s.</t>
         </is>
       </c>
       <c r="D227" s="2" t="inlineStr">
@@ -9772,7 +9772,7 @@
         </is>
       </c>
       <c r="G227" s="2" t="n">
-        <v>0.97</v>
+        <v>0.43</v>
       </c>
       <c r="H227" s="2" t="inlineStr">
         <is>
@@ -9794,7 +9794,7 @@
       </c>
       <c r="C228" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #25 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.71s.</t>
+          <t>User executes touch gesture #25 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.66s.</t>
         </is>
       </c>
       <c r="D228" s="2" t="inlineStr">
@@ -9813,7 +9813,7 @@
         </is>
       </c>
       <c r="G228" s="2" t="n">
-        <v>0.71</v>
+        <v>0.66</v>
       </c>
       <c r="H228" s="2" t="inlineStr">
         <is>
@@ -9835,7 +9835,7 @@
       </c>
       <c r="C229" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #26 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.94s.</t>
+          <t>User executes touch gesture #26 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.22s.</t>
         </is>
       </c>
       <c r="D229" s="2" t="inlineStr">
@@ -9854,7 +9854,7 @@
         </is>
       </c>
       <c r="G229" s="2" t="n">
-        <v>0.9399999999999999</v>
+        <v>1.22</v>
       </c>
       <c r="H229" s="2" t="inlineStr">
         <is>
@@ -9876,7 +9876,7 @@
       </c>
       <c r="C230" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #27 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.72s.</t>
+          <t>User executes touch gesture #27 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.59s.</t>
         </is>
       </c>
       <c r="D230" s="2" t="inlineStr">
@@ -9895,7 +9895,7 @@
         </is>
       </c>
       <c r="G230" s="2" t="n">
-        <v>0.72</v>
+        <v>0.59</v>
       </c>
       <c r="H230" s="2" t="inlineStr">
         <is>
@@ -9917,7 +9917,7 @@
       </c>
       <c r="C231" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #28 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.94s.</t>
+          <t>User executes touch gesture #28 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.59s.</t>
         </is>
       </c>
       <c r="D231" s="2" t="inlineStr">
@@ -9936,7 +9936,7 @@
         </is>
       </c>
       <c r="G231" s="2" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.59</v>
       </c>
       <c r="H231" s="2" t="inlineStr">
         <is>
@@ -9977,7 +9977,7 @@
         </is>
       </c>
       <c r="G232" s="2" t="n">
-        <v>0.73</v>
+        <v>0.65</v>
       </c>
       <c r="H232" s="2" t="inlineStr">
         <is>
@@ -10018,7 +10018,7 @@
         </is>
       </c>
       <c r="G233" s="2" t="n">
-        <v>0.38</v>
+        <v>0.42</v>
       </c>
       <c r="H233" s="2" t="inlineStr">
         <is>
@@ -10059,7 +10059,7 @@
         </is>
       </c>
       <c r="G234" s="2" t="n">
-        <v>0.37</v>
+        <v>0.65</v>
       </c>
       <c r="H234" s="2" t="inlineStr">
         <is>
@@ -10100,7 +10100,7 @@
         </is>
       </c>
       <c r="G235" s="2" t="n">
-        <v>0.72</v>
+        <v>0.29</v>
       </c>
       <c r="H235" s="2" t="inlineStr">
         <is>
@@ -10122,7 +10122,7 @@
       </c>
       <c r="C236" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #1 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.73s.</t>
+          <t>User executes offline storage operation #1 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.5s.</t>
         </is>
       </c>
       <c r="D236" s="2" t="inlineStr">
@@ -10141,7 +10141,7 @@
         </is>
       </c>
       <c r="G236" s="2" t="n">
-        <v>0.73</v>
+        <v>0.5</v>
       </c>
       <c r="H236" s="2" t="inlineStr">
         <is>
@@ -10163,7 +10163,7 @@
       </c>
       <c r="C237" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #2 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.41s.</t>
+          <t>User executes offline storage operation #2 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.72s.</t>
         </is>
       </c>
       <c r="D237" s="2" t="inlineStr">
@@ -10182,7 +10182,7 @@
         </is>
       </c>
       <c r="G237" s="2" t="n">
-        <v>0.41</v>
+        <v>0.72</v>
       </c>
       <c r="H237" s="2" t="inlineStr">
         <is>
@@ -10204,7 +10204,7 @@
       </c>
       <c r="C238" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #3 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.31s.</t>
+          <t>User executes offline storage operation #3 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.32s.</t>
         </is>
       </c>
       <c r="D238" s="2" t="inlineStr">
@@ -10223,7 +10223,7 @@
         </is>
       </c>
       <c r="G238" s="2" t="n">
-        <v>0.31</v>
+        <v>0.32</v>
       </c>
       <c r="H238" s="2" t="inlineStr">
         <is>
@@ -10245,7 +10245,7 @@
       </c>
       <c r="C239" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #4 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.39s.</t>
+          <t>User executes offline storage operation #4 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.31s.</t>
         </is>
       </c>
       <c r="D239" s="2" t="inlineStr">
@@ -10264,7 +10264,7 @@
         </is>
       </c>
       <c r="G239" s="2" t="n">
-        <v>0.39</v>
+        <v>0.31</v>
       </c>
       <c r="H239" s="2" t="inlineStr">
         <is>
@@ -10286,7 +10286,7 @@
       </c>
       <c r="C240" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #5 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.61s.</t>
+          <t>User executes offline storage operation #5 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.48s.</t>
         </is>
       </c>
       <c r="D240" s="2" t="inlineStr">
@@ -10305,7 +10305,7 @@
         </is>
       </c>
       <c r="G240" s="2" t="n">
-        <v>0.61</v>
+        <v>0.48</v>
       </c>
       <c r="H240" s="2" t="inlineStr">
         <is>
@@ -10327,7 +10327,7 @@
       </c>
       <c r="C241" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #6 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.27s.</t>
+          <t>User executes offline storage operation #6 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.7s.</t>
         </is>
       </c>
       <c r="D241" s="2" t="inlineStr">
@@ -10346,7 +10346,7 @@
         </is>
       </c>
       <c r="G241" s="2" t="n">
-        <v>0.27</v>
+        <v>0.7</v>
       </c>
       <c r="H241" s="2" t="inlineStr">
         <is>
@@ -10368,7 +10368,7 @@
       </c>
       <c r="C242" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #7 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.58s.</t>
+          <t>User executes offline storage operation #7 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.65s.</t>
         </is>
       </c>
       <c r="D242" s="2" t="inlineStr">
@@ -10387,7 +10387,7 @@
         </is>
       </c>
       <c r="G242" s="2" t="n">
-        <v>0.58</v>
+        <v>0.65</v>
       </c>
       <c r="H242" s="2" t="inlineStr">
         <is>
@@ -10409,7 +10409,7 @@
       </c>
       <c r="C243" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #8 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.42s.</t>
+          <t>User executes offline storage operation #8 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.57s.</t>
         </is>
       </c>
       <c r="D243" s="2" t="inlineStr">
@@ -10428,7 +10428,7 @@
         </is>
       </c>
       <c r="G243" s="2" t="n">
-        <v>0.42</v>
+        <v>0.57</v>
       </c>
       <c r="H243" s="2" t="inlineStr">
         <is>
@@ -10450,7 +10450,7 @@
       </c>
       <c r="C244" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #9 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.58s.</t>
+          <t>User executes offline storage operation #9 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.57s.</t>
         </is>
       </c>
       <c r="D244" s="2" t="inlineStr">
@@ -10469,7 +10469,7 @@
         </is>
       </c>
       <c r="G244" s="2" t="n">
-        <v>0.58</v>
+        <v>0.57</v>
       </c>
       <c r="H244" s="2" t="inlineStr">
         <is>
@@ -10491,7 +10491,7 @@
       </c>
       <c r="C245" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #10 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.32s.</t>
+          <t>User executes offline storage operation #10 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.55s.</t>
         </is>
       </c>
       <c r="D245" s="2" t="inlineStr">
@@ -10510,7 +10510,7 @@
         </is>
       </c>
       <c r="G245" s="2" t="n">
-        <v>0.32</v>
+        <v>0.55</v>
       </c>
       <c r="H245" s="2" t="inlineStr">
         <is>
@@ -10532,7 +10532,7 @@
       </c>
       <c r="C246" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #11 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.41s.</t>
+          <t>User executes offline storage operation #11 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.73s.</t>
         </is>
       </c>
       <c r="D246" s="2" t="inlineStr">
@@ -10551,7 +10551,7 @@
         </is>
       </c>
       <c r="G246" s="2" t="n">
-        <v>0.41</v>
+        <v>0.73</v>
       </c>
       <c r="H246" s="2" t="inlineStr">
         <is>
@@ -10573,7 +10573,7 @@
       </c>
       <c r="C247" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #12 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.26s.</t>
+          <t>User executes offline storage operation #12 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.33s.</t>
         </is>
       </c>
       <c r="D247" s="2" t="inlineStr">
@@ -10592,7 +10592,7 @@
         </is>
       </c>
       <c r="G247" s="2" t="n">
-        <v>0.26</v>
+        <v>0.33</v>
       </c>
       <c r="H247" s="2" t="inlineStr">
         <is>
@@ -10614,7 +10614,7 @@
       </c>
       <c r="C248" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #13 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.53s.</t>
+          <t>User executes offline storage operation #13 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.41s.</t>
         </is>
       </c>
       <c r="D248" s="2" t="inlineStr">
@@ -10633,7 +10633,7 @@
         </is>
       </c>
       <c r="G248" s="2" t="n">
-        <v>0.53</v>
+        <v>0.41</v>
       </c>
       <c r="H248" s="2" t="inlineStr">
         <is>
@@ -10655,7 +10655,7 @@
       </c>
       <c r="C249" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #14 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.65s.</t>
+          <t>User executes offline storage operation #14 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.39s.</t>
         </is>
       </c>
       <c r="D249" s="2" t="inlineStr">
@@ -10674,7 +10674,7 @@
         </is>
       </c>
       <c r="G249" s="2" t="n">
-        <v>0.65</v>
+        <v>0.39</v>
       </c>
       <c r="H249" s="2" t="inlineStr">
         <is>
@@ -10696,7 +10696,7 @@
       </c>
       <c r="C250" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #15 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.65s.</t>
+          <t>User executes offline storage operation #15 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.37s.</t>
         </is>
       </c>
       <c r="D250" s="2" t="inlineStr">
@@ -10715,7 +10715,7 @@
         </is>
       </c>
       <c r="G250" s="2" t="n">
-        <v>0.65</v>
+        <v>0.37</v>
       </c>
       <c r="H250" s="2" t="inlineStr">
         <is>
@@ -10737,7 +10737,7 @@
       </c>
       <c r="C251" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #16 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.61s.</t>
+          <t>User executes offline storage operation #16 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.69s.</t>
         </is>
       </c>
       <c r="D251" s="2" t="inlineStr">
@@ -10756,7 +10756,7 @@
         </is>
       </c>
       <c r="G251" s="2" t="n">
-        <v>0.61</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="H251" s="2" t="inlineStr">
         <is>
@@ -10778,7 +10778,7 @@
       </c>
       <c r="C252" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #17 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.47s.</t>
+          <t>User executes offline storage operation #17 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.53s.</t>
         </is>
       </c>
       <c r="D252" s="2" t="inlineStr">
@@ -10797,7 +10797,7 @@
         </is>
       </c>
       <c r="G252" s="2" t="n">
-        <v>0.47</v>
+        <v>0.53</v>
       </c>
       <c r="H252" s="2" t="inlineStr">
         <is>
@@ -10819,7 +10819,7 @@
       </c>
       <c r="C253" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #18 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.26s.</t>
+          <t>User executes offline storage operation #18 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.67s.</t>
         </is>
       </c>
       <c r="D253" s="2" t="inlineStr">
@@ -10838,7 +10838,7 @@
         </is>
       </c>
       <c r="G253" s="2" t="n">
-        <v>0.26</v>
+        <v>0.67</v>
       </c>
       <c r="H253" s="2" t="inlineStr">
         <is>
@@ -10860,7 +10860,7 @@
       </c>
       <c r="C254" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #19 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.43s.</t>
+          <t>User executes offline storage operation #19 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.3s.</t>
         </is>
       </c>
       <c r="D254" s="2" t="inlineStr">
@@ -10879,7 +10879,7 @@
         </is>
       </c>
       <c r="G254" s="2" t="n">
-        <v>0.43</v>
+        <v>0.3</v>
       </c>
       <c r="H254" s="2" t="inlineStr">
         <is>
@@ -10901,7 +10901,7 @@
       </c>
       <c r="C255" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #20 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.67s.</t>
+          <t>User executes offline storage operation #20 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.44s.</t>
         </is>
       </c>
       <c r="D255" s="2" t="inlineStr">
@@ -10920,7 +10920,7 @@
         </is>
       </c>
       <c r="G255" s="2" t="n">
-        <v>0.67</v>
+        <v>0.44</v>
       </c>
       <c r="H255" s="2" t="inlineStr">
         <is>
@@ -10942,7 +10942,7 @@
       </c>
       <c r="C256" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #21 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.66s.</t>
+          <t>User executes offline storage operation #21 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.45s.</t>
         </is>
       </c>
       <c r="D256" s="2" t="inlineStr">
@@ -10961,7 +10961,7 @@
         </is>
       </c>
       <c r="G256" s="2" t="n">
-        <v>0.66</v>
+        <v>0.45</v>
       </c>
       <c r="H256" s="2" t="inlineStr">
         <is>
@@ -10983,7 +10983,7 @@
       </c>
       <c r="C257" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #22 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.28s.</t>
+          <t>User executes offline storage operation #22 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.69s.</t>
         </is>
       </c>
       <c r="D257" s="2" t="inlineStr">
@@ -11002,7 +11002,7 @@
         </is>
       </c>
       <c r="G257" s="2" t="n">
-        <v>0.28</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="H257" s="2" t="inlineStr">
         <is>
@@ -11024,7 +11024,7 @@
       </c>
       <c r="C258" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #23 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.47s.</t>
+          <t>User executes offline storage operation #23 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.58s.</t>
         </is>
       </c>
       <c r="D258" s="2" t="inlineStr">
@@ -11043,7 +11043,7 @@
         </is>
       </c>
       <c r="G258" s="2" t="n">
-        <v>0.47</v>
+        <v>0.58</v>
       </c>
       <c r="H258" s="2" t="inlineStr">
         <is>
@@ -11065,7 +11065,7 @@
       </c>
       <c r="C259" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #24 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.45s.</t>
+          <t>User executes offline storage operation #24 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.35s.</t>
         </is>
       </c>
       <c r="D259" s="2" t="inlineStr">
@@ -11084,7 +11084,7 @@
         </is>
       </c>
       <c r="G259" s="2" t="n">
-        <v>0.45</v>
+        <v>0.35</v>
       </c>
       <c r="H259" s="2" t="inlineStr">
         <is>
@@ -11106,7 +11106,7 @@
       </c>
       <c r="C260" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #25 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.58s.</t>
+          <t>User executes offline storage operation #25 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.64s.</t>
         </is>
       </c>
       <c r="D260" s="2" t="inlineStr">
@@ -11125,7 +11125,7 @@
         </is>
       </c>
       <c r="G260" s="2" t="n">
-        <v>0.58</v>
+        <v>0.64</v>
       </c>
       <c r="H260" s="2" t="inlineStr">
         <is>
@@ -11147,7 +11147,7 @@
       </c>
       <c r="C261" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #26 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.27s.</t>
+          <t>User executes offline storage operation #26 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.69s.</t>
         </is>
       </c>
       <c r="D261" s="2" t="inlineStr">
@@ -11166,7 +11166,7 @@
         </is>
       </c>
       <c r="G261" s="2" t="n">
-        <v>0.27</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="H261" s="2" t="inlineStr">
         <is>
@@ -11188,7 +11188,7 @@
       </c>
       <c r="C262" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #27 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.59s.</t>
+          <t>User executes offline storage operation #27 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.28s.</t>
         </is>
       </c>
       <c r="D262" s="2" t="inlineStr">
@@ -11207,7 +11207,7 @@
         </is>
       </c>
       <c r="G262" s="2" t="n">
-        <v>0.59</v>
+        <v>0.28</v>
       </c>
       <c r="H262" s="2" t="inlineStr">
         <is>
@@ -11229,7 +11229,7 @@
       </c>
       <c r="C263" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #28 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.36s.</t>
+          <t>User executes offline storage operation #28 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.5s.</t>
         </is>
       </c>
       <c r="D263" s="2" t="inlineStr">
@@ -11248,7 +11248,7 @@
         </is>
       </c>
       <c r="G263" s="2" t="n">
-        <v>0.36</v>
+        <v>0.5</v>
       </c>
       <c r="H263" s="2" t="inlineStr">
         <is>
@@ -11270,7 +11270,7 @@
       </c>
       <c r="C264" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #29 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.48s.</t>
+          <t>User executes offline storage operation #29 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.33s.</t>
         </is>
       </c>
       <c r="D264" s="2" t="inlineStr">
@@ -11289,7 +11289,7 @@
         </is>
       </c>
       <c r="G264" s="2" t="n">
-        <v>0.48</v>
+        <v>0.33</v>
       </c>
       <c r="H264" s="2" t="inlineStr">
         <is>
@@ -11311,7 +11311,7 @@
       </c>
       <c r="C265" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #30 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.36s.</t>
+          <t>User executes offline storage operation #30 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.31s.</t>
         </is>
       </c>
       <c r="D265" s="2" t="inlineStr">
@@ -11330,7 +11330,7 @@
         </is>
       </c>
       <c r="G265" s="2" t="n">
-        <v>0.36</v>
+        <v>0.31</v>
       </c>
       <c r="H265" s="2" t="inlineStr">
         <is>
@@ -11352,7 +11352,7 @@
       </c>
       <c r="C266" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #31 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.52s.</t>
+          <t>User executes offline storage operation #31 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.7s.</t>
         </is>
       </c>
       <c r="D266" s="2" t="inlineStr">
@@ -11371,7 +11371,7 @@
         </is>
       </c>
       <c r="G266" s="2" t="n">
-        <v>0.52</v>
+        <v>0.7</v>
       </c>
       <c r="H266" s="2" t="inlineStr">
         <is>
@@ -11412,7 +11412,7 @@
         </is>
       </c>
       <c r="G267" s="2" t="n">
-        <v>0.26</v>
+        <v>0.38</v>
       </c>
       <c r="H267" s="2" t="inlineStr">
         <is>
@@ -11453,7 +11453,7 @@
         </is>
       </c>
       <c r="G268" s="2" t="n">
-        <v>0.67</v>
+        <v>0.59</v>
       </c>
       <c r="H268" s="2" t="inlineStr">
         <is>
@@ -11494,7 +11494,7 @@
         </is>
       </c>
       <c r="G269" s="2" t="n">
-        <v>0.28</v>
+        <v>0.24</v>
       </c>
       <c r="H269" s="2" t="inlineStr">
         <is>
@@ -11535,7 +11535,7 @@
         </is>
       </c>
       <c r="G270" s="2" t="n">
-        <v>0.33</v>
+        <v>0.54</v>
       </c>
       <c r="H270" s="2" t="inlineStr">
         <is>
@@ -11557,7 +11557,7 @@
       </c>
       <c r="C271" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #1 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.57s.</t>
+          <t>User tests layout/memory scenario #1 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.55s.</t>
         </is>
       </c>
       <c r="D271" s="2" t="inlineStr">
@@ -11576,7 +11576,7 @@
         </is>
       </c>
       <c r="G271" s="2" t="n">
-        <v>0.57</v>
+        <v>0.55</v>
       </c>
       <c r="H271" s="2" t="inlineStr">
         <is>
@@ -11598,7 +11598,7 @@
       </c>
       <c r="C272" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #2 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.64s.</t>
+          <t>User tests layout/memory scenario #2 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.46s.</t>
         </is>
       </c>
       <c r="D272" s="2" t="inlineStr">
@@ -11617,7 +11617,7 @@
         </is>
       </c>
       <c r="G272" s="2" t="n">
-        <v>0.64</v>
+        <v>0.46</v>
       </c>
       <c r="H272" s="2" t="inlineStr">
         <is>
@@ -11639,7 +11639,7 @@
       </c>
       <c r="C273" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #3 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.28s.</t>
+          <t>User tests layout/memory scenario #3 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.51s.</t>
         </is>
       </c>
       <c r="D273" s="2" t="inlineStr">
@@ -11658,7 +11658,7 @@
         </is>
       </c>
       <c r="G273" s="2" t="n">
-        <v>0.28</v>
+        <v>0.51</v>
       </c>
       <c r="H273" s="2" t="inlineStr">
         <is>
@@ -11680,7 +11680,7 @@
       </c>
       <c r="C274" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #4 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.32s.</t>
+          <t>User tests layout/memory scenario #4 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.28s.</t>
         </is>
       </c>
       <c r="D274" s="2" t="inlineStr">
@@ -11699,7 +11699,7 @@
         </is>
       </c>
       <c r="G274" s="2" t="n">
-        <v>0.32</v>
+        <v>0.28</v>
       </c>
       <c r="H274" s="2" t="inlineStr">
         <is>
@@ -11721,7 +11721,7 @@
       </c>
       <c r="C275" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #5 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.66s.</t>
+          <t>User tests layout/memory scenario #5 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.36s.</t>
         </is>
       </c>
       <c r="D275" s="2" t="inlineStr">
@@ -11740,7 +11740,7 @@
         </is>
       </c>
       <c r="G275" s="2" t="n">
-        <v>0.66</v>
+        <v>0.36</v>
       </c>
       <c r="H275" s="2" t="inlineStr">
         <is>
@@ -11762,7 +11762,7 @@
       </c>
       <c r="C276" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #6 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.39s.</t>
+          <t>User tests layout/memory scenario #6 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.28s.</t>
         </is>
       </c>
       <c r="D276" s="2" t="inlineStr">
@@ -11781,7 +11781,7 @@
         </is>
       </c>
       <c r="G276" s="2" t="n">
-        <v>0.39</v>
+        <v>0.28</v>
       </c>
       <c r="H276" s="2" t="inlineStr">
         <is>
@@ -11803,7 +11803,7 @@
       </c>
       <c r="C277" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #7 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.24s.</t>
+          <t>User tests layout/memory scenario #7 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.55s.</t>
         </is>
       </c>
       <c r="D277" s="2" t="inlineStr">
@@ -11822,7 +11822,7 @@
         </is>
       </c>
       <c r="G277" s="2" t="n">
-        <v>0.24</v>
+        <v>0.55</v>
       </c>
       <c r="H277" s="2" t="inlineStr">
         <is>
@@ -11844,7 +11844,7 @@
       </c>
       <c r="C278" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #8 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.27s.</t>
+          <t>User tests layout/memory scenario #8 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.33s.</t>
         </is>
       </c>
       <c r="D278" s="2" t="inlineStr">
@@ -11863,7 +11863,7 @@
         </is>
       </c>
       <c r="G278" s="2" t="n">
-        <v>0.27</v>
+        <v>0.33</v>
       </c>
       <c r="H278" s="2" t="inlineStr">
         <is>
@@ -11885,7 +11885,7 @@
       </c>
       <c r="C279" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #9 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.43s.</t>
+          <t>User tests layout/memory scenario #9 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.22s.</t>
         </is>
       </c>
       <c r="D279" s="2" t="inlineStr">
@@ -11904,7 +11904,7 @@
         </is>
       </c>
       <c r="G279" s="2" t="n">
-        <v>0.43</v>
+        <v>0.22</v>
       </c>
       <c r="H279" s="2" t="inlineStr">
         <is>
@@ -11926,7 +11926,7 @@
       </c>
       <c r="C280" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #10 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.33s.</t>
+          <t>User tests layout/memory scenario #10 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.46s.</t>
         </is>
       </c>
       <c r="D280" s="2" t="inlineStr">
@@ -11945,7 +11945,7 @@
         </is>
       </c>
       <c r="G280" s="2" t="n">
-        <v>0.33</v>
+        <v>0.46</v>
       </c>
       <c r="H280" s="2" t="inlineStr">
         <is>
@@ -11967,7 +11967,7 @@
       </c>
       <c r="C281" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #11 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.35s.</t>
+          <t>User tests layout/memory scenario #11 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.39s.</t>
         </is>
       </c>
       <c r="D281" s="2" t="inlineStr">
@@ -11986,7 +11986,7 @@
         </is>
       </c>
       <c r="G281" s="2" t="n">
-        <v>0.35</v>
+        <v>0.39</v>
       </c>
       <c r="H281" s="2" t="inlineStr">
         <is>
@@ -12008,7 +12008,7 @@
       </c>
       <c r="C282" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #12 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.58s.</t>
+          <t>User tests layout/memory scenario #12 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.42s.</t>
         </is>
       </c>
       <c r="D282" s="2" t="inlineStr">
@@ -12027,7 +12027,7 @@
         </is>
       </c>
       <c r="G282" s="2" t="n">
-        <v>0.58</v>
+        <v>0.42</v>
       </c>
       <c r="H282" s="2" t="inlineStr">
         <is>
@@ -12049,7 +12049,7 @@
       </c>
       <c r="C283" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #13 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.57s.</t>
+          <t>User tests layout/memory scenario #13 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.48s.</t>
         </is>
       </c>
       <c r="D283" s="2" t="inlineStr">
@@ -12068,7 +12068,7 @@
         </is>
       </c>
       <c r="G283" s="2" t="n">
-        <v>0.57</v>
+        <v>0.48</v>
       </c>
       <c r="H283" s="2" t="inlineStr">
         <is>
@@ -12090,7 +12090,7 @@
       </c>
       <c r="C284" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #14 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.42s.</t>
+          <t>User tests layout/memory scenario #14 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.35s.</t>
         </is>
       </c>
       <c r="D284" s="2" t="inlineStr">
@@ -12109,7 +12109,7 @@
         </is>
       </c>
       <c r="G284" s="2" t="n">
-        <v>0.42</v>
+        <v>0.35</v>
       </c>
       <c r="H284" s="2" t="inlineStr">
         <is>
@@ -12131,7 +12131,7 @@
       </c>
       <c r="C285" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #15 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.61s.</t>
+          <t>User tests layout/memory scenario #15 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.48s.</t>
         </is>
       </c>
       <c r="D285" s="2" t="inlineStr">
@@ -12150,7 +12150,7 @@
         </is>
       </c>
       <c r="G285" s="2" t="n">
-        <v>0.61</v>
+        <v>0.48</v>
       </c>
       <c r="H285" s="2" t="inlineStr">
         <is>
@@ -12172,7 +12172,7 @@
       </c>
       <c r="C286" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #16 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.49s.</t>
+          <t>User tests layout/memory scenario #16 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.64s.</t>
         </is>
       </c>
       <c r="D286" s="2" t="inlineStr">
@@ -12191,7 +12191,7 @@
         </is>
       </c>
       <c r="G286" s="2" t="n">
-        <v>0.49</v>
+        <v>0.64</v>
       </c>
       <c r="H286" s="2" t="inlineStr">
         <is>
@@ -12213,7 +12213,7 @@
       </c>
       <c r="C287" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #17 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.41s.</t>
+          <t>User tests layout/memory scenario #17 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.51s.</t>
         </is>
       </c>
       <c r="D287" s="2" t="inlineStr">
@@ -12232,7 +12232,7 @@
         </is>
       </c>
       <c r="G287" s="2" t="n">
-        <v>0.41</v>
+        <v>0.51</v>
       </c>
       <c r="H287" s="2" t="inlineStr">
         <is>
@@ -12254,7 +12254,7 @@
       </c>
       <c r="C288" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #18 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.3s.</t>
+          <t>User tests layout/memory scenario #18 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.42s.</t>
         </is>
       </c>
       <c r="D288" s="2" t="inlineStr">
@@ -12273,7 +12273,7 @@
         </is>
       </c>
       <c r="G288" s="2" t="n">
-        <v>0.3</v>
+        <v>0.42</v>
       </c>
       <c r="H288" s="2" t="inlineStr">
         <is>
@@ -12295,7 +12295,7 @@
       </c>
       <c r="C289" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #19 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.44s.</t>
+          <t>User tests layout/memory scenario #19 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.61s.</t>
         </is>
       </c>
       <c r="D289" s="2" t="inlineStr">
@@ -12314,7 +12314,7 @@
         </is>
       </c>
       <c r="G289" s="2" t="n">
-        <v>0.44</v>
+        <v>0.61</v>
       </c>
       <c r="H289" s="2" t="inlineStr">
         <is>
@@ -12336,7 +12336,7 @@
       </c>
       <c r="C290" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #20 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.35s.</t>
+          <t>User tests layout/memory scenario #20 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.4s.</t>
         </is>
       </c>
       <c r="D290" s="2" t="inlineStr">
@@ -12355,7 +12355,7 @@
         </is>
       </c>
       <c r="G290" s="2" t="n">
-        <v>0.35</v>
+        <v>0.4</v>
       </c>
       <c r="H290" s="2" t="inlineStr">
         <is>
@@ -12377,7 +12377,7 @@
       </c>
       <c r="C291" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #21 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.49s.</t>
+          <t>User tests layout/memory scenario #21 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.28s.</t>
         </is>
       </c>
       <c r="D291" s="2" t="inlineStr">
@@ -12396,7 +12396,7 @@
         </is>
       </c>
       <c r="G291" s="2" t="n">
-        <v>0.49</v>
+        <v>0.28</v>
       </c>
       <c r="H291" s="2" t="inlineStr">
         <is>
@@ -12418,7 +12418,7 @@
       </c>
       <c r="C292" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #22 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.54s.</t>
+          <t>User tests layout/memory scenario #22 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.64s.</t>
         </is>
       </c>
       <c r="D292" s="2" t="inlineStr">
@@ -12437,7 +12437,7 @@
         </is>
       </c>
       <c r="G292" s="2" t="n">
-        <v>0.54</v>
+        <v>0.64</v>
       </c>
       <c r="H292" s="2" t="inlineStr">
         <is>
@@ -12459,7 +12459,7 @@
       </c>
       <c r="C293" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #23 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.45s.</t>
+          <t>User tests layout/memory scenario #23 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.36s.</t>
         </is>
       </c>
       <c r="D293" s="2" t="inlineStr">
@@ -12478,7 +12478,7 @@
         </is>
       </c>
       <c r="G293" s="2" t="n">
-        <v>0.45</v>
+        <v>0.36</v>
       </c>
       <c r="H293" s="2" t="inlineStr">
         <is>
@@ -12541,7 +12541,7 @@
       </c>
       <c r="C295" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #25 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.6s.</t>
+          <t>User tests layout/memory scenario #25 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.31s.</t>
         </is>
       </c>
       <c r="D295" s="2" t="inlineStr">
@@ -12560,7 +12560,7 @@
         </is>
       </c>
       <c r="G295" s="2" t="n">
-        <v>0.6</v>
+        <v>0.31</v>
       </c>
       <c r="H295" s="2" t="inlineStr">
         <is>
@@ -12582,7 +12582,7 @@
       </c>
       <c r="C296" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #26 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.27s.</t>
+          <t>User tests layout/memory scenario #26 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.67s.</t>
         </is>
       </c>
       <c r="D296" s="2" t="inlineStr">
@@ -12601,7 +12601,7 @@
         </is>
       </c>
       <c r="G296" s="2" t="n">
-        <v>0.27</v>
+        <v>0.67</v>
       </c>
       <c r="H296" s="2" t="inlineStr">
         <is>
@@ -12623,7 +12623,7 @@
       </c>
       <c r="C297" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #27 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.43s.</t>
+          <t>User tests layout/memory scenario #27 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.28s.</t>
         </is>
       </c>
       <c r="D297" s="2" t="inlineStr">
@@ -12642,7 +12642,7 @@
         </is>
       </c>
       <c r="G297" s="2" t="n">
-        <v>0.43</v>
+        <v>0.28</v>
       </c>
       <c r="H297" s="2" t="inlineStr">
         <is>
@@ -12664,7 +12664,7 @@
       </c>
       <c r="C298" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #28 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.43s.</t>
+          <t>User tests layout/memory scenario #28 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.66s.</t>
         </is>
       </c>
       <c r="D298" s="2" t="inlineStr">
@@ -12683,7 +12683,7 @@
         </is>
       </c>
       <c r="G298" s="2" t="n">
-        <v>0.43</v>
+        <v>0.66</v>
       </c>
       <c r="H298" s="2" t="inlineStr">
         <is>
@@ -12705,7 +12705,7 @@
       </c>
       <c r="C299" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #29 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.26s.</t>
+          <t>User tests layout/memory scenario #29 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.54s.</t>
         </is>
       </c>
       <c r="D299" s="2" t="inlineStr">
@@ -12724,7 +12724,7 @@
         </is>
       </c>
       <c r="G299" s="2" t="n">
-        <v>0.26</v>
+        <v>0.54</v>
       </c>
       <c r="H299" s="2" t="inlineStr">
         <is>
@@ -12746,7 +12746,7 @@
       </c>
       <c r="C300" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #30 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.61s.</t>
+          <t>User tests layout/memory scenario #30 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.26s.</t>
         </is>
       </c>
       <c r="D300" s="2" t="inlineStr">
@@ -12765,7 +12765,7 @@
         </is>
       </c>
       <c r="G300" s="2" t="n">
-        <v>0.61</v>
+        <v>0.26</v>
       </c>
       <c r="H300" s="2" t="inlineStr">
         <is>
@@ -12787,7 +12787,7 @@
       </c>
       <c r="C301" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #31 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.4s.</t>
+          <t>User tests layout/memory scenario #31 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.45s.</t>
         </is>
       </c>
       <c r="D301" s="2" t="inlineStr">
@@ -12806,7 +12806,7 @@
         </is>
       </c>
       <c r="G301" s="2" t="n">
-        <v>0.4</v>
+        <v>0.45</v>
       </c>
       <c r="H301" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
feat(load): add 10 distinct architectural performance outcomes to load test report and executive summary
</commit_message>
<xml_diff>
--- a/reports/Mobile_Application_Appium_Test_Report.xlsx
+++ b/reports/Mobile_Application_Appium_Test_Report.xlsx
@@ -547,7 +547,7 @@
         </is>
       </c>
       <c r="G2" s="2" t="n">
-        <v>0.55</v>
+        <v>0.62</v>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
@@ -588,7 +588,7 @@
         </is>
       </c>
       <c r="G3" s="2" t="n">
-        <v>0.49</v>
+        <v>0.77</v>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
@@ -629,7 +629,7 @@
         </is>
       </c>
       <c r="G4" s="2" t="n">
-        <v>0.9</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
@@ -670,7 +670,7 @@
         </is>
       </c>
       <c r="G5" s="2" t="n">
-        <v>0.85</v>
+        <v>0.36</v>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
@@ -711,7 +711,7 @@
         </is>
       </c>
       <c r="G6" s="2" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.42</v>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
@@ -752,7 +752,7 @@
         </is>
       </c>
       <c r="G7" s="2" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.58</v>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
@@ -793,7 +793,7 @@
         </is>
       </c>
       <c r="G8" s="2" t="n">
-        <v>0.6</v>
+        <v>0.45</v>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
@@ -834,7 +834,7 @@
         </is>
       </c>
       <c r="G9" s="2" t="n">
-        <v>0.46</v>
+        <v>0.44</v>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
@@ -875,7 +875,7 @@
         </is>
       </c>
       <c r="G10" s="2" t="n">
-        <v>0.64</v>
+        <v>0.44</v>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
@@ -916,7 +916,7 @@
         </is>
       </c>
       <c r="G11" s="2" t="n">
-        <v>0.66</v>
+        <v>0.7</v>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
@@ -957,7 +957,7 @@
         </is>
       </c>
       <c r="G12" s="2" t="n">
-        <v>0.46</v>
+        <v>0.6</v>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
@@ -998,7 +998,7 @@
         </is>
       </c>
       <c r="G13" s="2" t="n">
-        <v>0.75</v>
+        <v>0.76</v>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
@@ -1039,7 +1039,7 @@
         </is>
       </c>
       <c r="G14" s="2" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.9</v>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
@@ -1080,7 +1080,7 @@
         </is>
       </c>
       <c r="G15" s="2" t="n">
-        <v>0.71</v>
+        <v>0.75</v>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
@@ -1121,7 +1121,7 @@
         </is>
       </c>
       <c r="G16" s="2" t="n">
-        <v>0.5</v>
+        <v>0.84</v>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
@@ -1162,7 +1162,7 @@
         </is>
       </c>
       <c r="G17" s="2" t="n">
-        <v>0.92</v>
+        <v>0.64</v>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
@@ -1203,7 +1203,7 @@
         </is>
       </c>
       <c r="G18" s="2" t="n">
-        <v>0.64</v>
+        <v>0.74</v>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
@@ -1244,7 +1244,7 @@
         </is>
       </c>
       <c r="G19" s="2" t="n">
-        <v>0.53</v>
+        <v>0.82</v>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
@@ -1285,7 +1285,7 @@
         </is>
       </c>
       <c r="G20" s="2" t="n">
-        <v>0.37</v>
+        <v>0.84</v>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
@@ -1326,7 +1326,7 @@
         </is>
       </c>
       <c r="G21" s="2" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.35</v>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
@@ -1348,7 +1348,7 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #1 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.72s without crashing.</t>
+          <t>User taps Auth action button #1 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.86s without crashing.</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -1367,7 +1367,7 @@
         </is>
       </c>
       <c r="G22" s="2" t="n">
-        <v>0.72</v>
+        <v>0.86</v>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
@@ -1389,7 +1389,7 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #2 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.64s without crashing.</t>
+          <t>User taps Auth action button #2 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.42s without crashing.</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -1408,7 +1408,7 @@
         </is>
       </c>
       <c r="G23" s="2" t="n">
-        <v>0.64</v>
+        <v>0.42</v>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
@@ -1430,7 +1430,7 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #3 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.68s without crashing.</t>
+          <t>User taps Auth action button #3 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.5s without crashing.</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -1449,7 +1449,7 @@
         </is>
       </c>
       <c r="G24" s="2" t="n">
-        <v>0.68</v>
+        <v>0.5</v>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
@@ -1471,7 +1471,7 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #4 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.76s without crashing.</t>
+          <t>User taps Auth action button #4 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.65s without crashing.</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
@@ -1490,7 +1490,7 @@
         </is>
       </c>
       <c r="G25" s="2" t="n">
-        <v>0.76</v>
+        <v>0.65</v>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
@@ -1512,7 +1512,7 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #5 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.83s without crashing.</t>
+          <t>User taps Auth action button #5 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.68s without crashing.</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -1531,7 +1531,7 @@
         </is>
       </c>
       <c r="G26" s="2" t="n">
-        <v>0.83</v>
+        <v>0.68</v>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
@@ -1553,7 +1553,7 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #6 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.94s without crashing.</t>
+          <t>User taps Auth action button #6 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.47s without crashing.</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
@@ -1572,7 +1572,7 @@
         </is>
       </c>
       <c r="G27" s="2" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.47</v>
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
@@ -1594,7 +1594,7 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #7 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.37s without crashing.</t>
+          <t>User taps Auth action button #7 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.88s without crashing.</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -1613,7 +1613,7 @@
         </is>
       </c>
       <c r="G28" s="2" t="n">
-        <v>0.37</v>
+        <v>0.88</v>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
@@ -1635,7 +1635,7 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #8 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.73s without crashing.</t>
+          <t>User taps Auth action button #8 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.54s without crashing.</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
@@ -1654,7 +1654,7 @@
         </is>
       </c>
       <c r="G29" s="2" t="n">
-        <v>0.73</v>
+        <v>0.54</v>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
@@ -1676,7 +1676,7 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #9 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.75s without crashing.</t>
+          <t>User taps Auth action button #9 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.86s without crashing.</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -1695,7 +1695,7 @@
         </is>
       </c>
       <c r="G30" s="2" t="n">
-        <v>0.75</v>
+        <v>0.86</v>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
@@ -1717,7 +1717,7 @@
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #10 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.35s without crashing.</t>
+          <t>User taps Auth action button #10 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.7s without crashing.</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
@@ -1736,7 +1736,7 @@
         </is>
       </c>
       <c r="G31" s="2" t="n">
-        <v>0.35</v>
+        <v>0.7</v>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
@@ -1758,7 +1758,7 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #11 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.57s without crashing.</t>
+          <t>User taps Auth action button #11 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.76s without crashing.</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
@@ -1777,7 +1777,7 @@
         </is>
       </c>
       <c r="G32" s="2" t="n">
-        <v>0.57</v>
+        <v>0.76</v>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
@@ -1799,7 +1799,7 @@
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #12 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.8s without crashing.</t>
+          <t>User taps Auth action button #12 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.68s without crashing.</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
@@ -1818,7 +1818,7 @@
         </is>
       </c>
       <c r="G33" s="2" t="n">
-        <v>0.8</v>
+        <v>0.68</v>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
@@ -1840,7 +1840,7 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #13 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.84s without crashing.</t>
+          <t>User taps Auth action button #13 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.76s without crashing.</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -1859,7 +1859,7 @@
         </is>
       </c>
       <c r="G34" s="2" t="n">
-        <v>0.84</v>
+        <v>0.76</v>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
@@ -1881,7 +1881,7 @@
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #14 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.56s without crashing.</t>
+          <t>User taps Auth action button #14 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.89s without crashing.</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
@@ -1900,7 +1900,7 @@
         </is>
       </c>
       <c r="G35" s="2" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.89</v>
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
@@ -1922,7 +1922,7 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #15 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.94s without crashing.</t>
+          <t>User taps Auth action button #15 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.87s without crashing.</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
@@ -1941,7 +1941,7 @@
         </is>
       </c>
       <c r="G36" s="2" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.87</v>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
@@ -1963,7 +1963,7 @@
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #16 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.73s without crashing.</t>
+          <t>User taps Auth action button #16 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.81s without crashing.</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
@@ -1982,7 +1982,7 @@
         </is>
       </c>
       <c r="G37" s="2" t="n">
-        <v>0.73</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
@@ -2004,7 +2004,7 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #17 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.47s without crashing.</t>
+          <t>User taps Auth action button #17 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.67s without crashing.</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
@@ -2023,7 +2023,7 @@
         </is>
       </c>
       <c r="G38" s="2" t="n">
-        <v>0.47</v>
+        <v>0.67</v>
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
@@ -2045,7 +2045,7 @@
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #18 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.78s without crashing.</t>
+          <t>User taps Auth action button #18 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.8s without crashing.</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
@@ -2064,7 +2064,7 @@
         </is>
       </c>
       <c r="G39" s="2" t="n">
-        <v>0.78</v>
+        <v>0.8</v>
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
@@ -2086,7 +2086,7 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #19 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.8s without crashing.</t>
+          <t>User taps Auth action button #19 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.53s without crashing.</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
@@ -2105,7 +2105,7 @@
         </is>
       </c>
       <c r="G40" s="2" t="n">
-        <v>0.8</v>
+        <v>0.53</v>
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
@@ -2127,7 +2127,7 @@
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #20 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.4s without crashing.</t>
+          <t>User taps Auth action button #20 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.91s without crashing.</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
@@ -2146,7 +2146,7 @@
         </is>
       </c>
       <c r="G41" s="2" t="n">
-        <v>0.4</v>
+        <v>0.91</v>
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
@@ -2187,7 +2187,7 @@
         </is>
       </c>
       <c r="G42" s="2" t="n">
-        <v>0.39</v>
+        <v>0.74</v>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
@@ -2228,7 +2228,7 @@
         </is>
       </c>
       <c r="G43" s="2" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.68</v>
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
@@ -2269,7 +2269,7 @@
         </is>
       </c>
       <c r="G44" s="2" t="n">
-        <v>0.42</v>
+        <v>0.75</v>
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
@@ -2310,7 +2310,7 @@
         </is>
       </c>
       <c r="G45" s="2" t="n">
-        <v>0.52</v>
+        <v>0.49</v>
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
@@ -2351,7 +2351,7 @@
         </is>
       </c>
       <c r="G46" s="2" t="n">
-        <v>0.55</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
@@ -2392,7 +2392,7 @@
         </is>
       </c>
       <c r="G47" s="2" t="n">
-        <v>0.42</v>
+        <v>0.48</v>
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
@@ -2433,7 +2433,7 @@
         </is>
       </c>
       <c r="G48" s="2" t="n">
-        <v>0.88</v>
+        <v>0.5</v>
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
@@ -2474,7 +2474,7 @@
         </is>
       </c>
       <c r="G49" s="2" t="n">
-        <v>0.45</v>
+        <v>0.43</v>
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
@@ -2515,7 +2515,7 @@
         </is>
       </c>
       <c r="G50" s="2" t="n">
-        <v>0.68</v>
+        <v>0.6</v>
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
@@ -2556,7 +2556,7 @@
         </is>
       </c>
       <c r="G51" s="2" t="n">
-        <v>0.6</v>
+        <v>0.78</v>
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
@@ -2597,7 +2597,7 @@
         </is>
       </c>
       <c r="G52" s="2" t="n">
-        <v>0.41</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
@@ -2638,7 +2638,7 @@
         </is>
       </c>
       <c r="G53" s="2" t="n">
-        <v>0.42</v>
+        <v>0.36</v>
       </c>
       <c r="H53" s="2" t="inlineStr">
         <is>
@@ -2679,7 +2679,7 @@
         </is>
       </c>
       <c r="G54" s="2" t="n">
-        <v>0.65</v>
+        <v>0.77</v>
       </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
@@ -2720,7 +2720,7 @@
         </is>
       </c>
       <c r="G55" s="2" t="n">
-        <v>0.62</v>
+        <v>0.4</v>
       </c>
       <c r="H55" s="2" t="inlineStr">
         <is>
@@ -2761,7 +2761,7 @@
         </is>
       </c>
       <c r="G56" s="2" t="n">
-        <v>0.71</v>
+        <v>0.48</v>
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
@@ -2783,7 +2783,7 @@
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #1 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.86s.</t>
+          <t>User taps Verification interactive button #1 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.74s.</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
@@ -2802,7 +2802,7 @@
         </is>
       </c>
       <c r="G57" s="2" t="n">
-        <v>0.86</v>
+        <v>0.74</v>
       </c>
       <c r="H57" s="2" t="inlineStr">
         <is>
@@ -2824,7 +2824,7 @@
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #2 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.6s.</t>
+          <t>User taps Verification interactive button #2 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.57s.</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
@@ -2843,7 +2843,7 @@
         </is>
       </c>
       <c r="G58" s="2" t="n">
-        <v>0.6</v>
+        <v>0.57</v>
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
@@ -2865,7 +2865,7 @@
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #3 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.48s.</t>
+          <t>User taps Verification interactive button #3 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.64s.</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
@@ -2884,7 +2884,7 @@
         </is>
       </c>
       <c r="G59" s="2" t="n">
-        <v>0.48</v>
+        <v>0.64</v>
       </c>
       <c r="H59" s="2" t="inlineStr">
         <is>
@@ -2906,7 +2906,7 @@
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #4 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.65s.</t>
+          <t>User taps Verification interactive button #4 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.45s.</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
@@ -2925,7 +2925,7 @@
         </is>
       </c>
       <c r="G60" s="2" t="n">
-        <v>0.65</v>
+        <v>0.45</v>
       </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
@@ -2947,7 +2947,7 @@
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #5 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.76s.</t>
+          <t>User taps Verification interactive button #5 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.84s.</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
@@ -2966,7 +2966,7 @@
         </is>
       </c>
       <c r="G61" s="2" t="n">
-        <v>0.76</v>
+        <v>0.84</v>
       </c>
       <c r="H61" s="2" t="inlineStr">
         <is>
@@ -2988,7 +2988,7 @@
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #6 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.36s.</t>
+          <t>User taps Verification interactive button #6 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.64s.</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
@@ -3007,7 +3007,7 @@
         </is>
       </c>
       <c r="G62" s="2" t="n">
-        <v>0.36</v>
+        <v>0.64</v>
       </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
@@ -3029,7 +3029,7 @@
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #7 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.8s.</t>
+          <t>User taps Verification interactive button #7 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.64s.</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
@@ -3048,7 +3048,7 @@
         </is>
       </c>
       <c r="G63" s="2" t="n">
-        <v>0.8</v>
+        <v>0.64</v>
       </c>
       <c r="H63" s="2" t="inlineStr">
         <is>
@@ -3070,7 +3070,7 @@
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #8 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.77s.</t>
+          <t>User taps Verification interactive button #8 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.49s.</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
@@ -3089,7 +3089,7 @@
         </is>
       </c>
       <c r="G64" s="2" t="n">
-        <v>0.77</v>
+        <v>0.49</v>
       </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
@@ -3111,7 +3111,7 @@
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #9 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.37s.</t>
+          <t>User taps Verification interactive button #9 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.54s.</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
@@ -3130,7 +3130,7 @@
         </is>
       </c>
       <c r="G65" s="2" t="n">
-        <v>0.37</v>
+        <v>0.54</v>
       </c>
       <c r="H65" s="2" t="inlineStr">
         <is>
@@ -3152,7 +3152,7 @@
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #10 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.85s.</t>
+          <t>User taps Verification interactive button #10 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.52s.</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
@@ -3171,7 +3171,7 @@
         </is>
       </c>
       <c r="G66" s="2" t="n">
-        <v>0.85</v>
+        <v>0.52</v>
       </c>
       <c r="H66" s="2" t="inlineStr">
         <is>
@@ -3193,7 +3193,7 @@
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #11 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.85s.</t>
+          <t>User taps Verification interactive button #11 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.6s.</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
@@ -3212,7 +3212,7 @@
         </is>
       </c>
       <c r="G67" s="2" t="n">
-        <v>0.85</v>
+        <v>0.6</v>
       </c>
       <c r="H67" s="2" t="inlineStr">
         <is>
@@ -3234,7 +3234,7 @@
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #12 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.82s.</t>
+          <t>User taps Verification interactive button #12 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.35s.</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
@@ -3253,7 +3253,7 @@
         </is>
       </c>
       <c r="G68" s="2" t="n">
-        <v>0.82</v>
+        <v>0.35</v>
       </c>
       <c r="H68" s="2" t="inlineStr">
         <is>
@@ -3275,7 +3275,7 @@
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #13 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.77s.</t>
+          <t>User taps Verification interactive button #13 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.38s.</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
@@ -3294,7 +3294,7 @@
         </is>
       </c>
       <c r="G69" s="2" t="n">
-        <v>0.77</v>
+        <v>0.38</v>
       </c>
       <c r="H69" s="2" t="inlineStr">
         <is>
@@ -3316,7 +3316,7 @@
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #14 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.53s.</t>
+          <t>User taps Verification interactive button #14 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.56s.</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
@@ -3335,7 +3335,7 @@
         </is>
       </c>
       <c r="G70" s="2" t="n">
-        <v>0.53</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="H70" s="2" t="inlineStr">
         <is>
@@ -3357,7 +3357,7 @@
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #15 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.73s.</t>
+          <t>User taps Verification interactive button #15 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.48s.</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
@@ -3376,7 +3376,7 @@
         </is>
       </c>
       <c r="G71" s="2" t="n">
-        <v>0.73</v>
+        <v>0.48</v>
       </c>
       <c r="H71" s="2" t="inlineStr">
         <is>
@@ -3398,7 +3398,7 @@
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #16 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.69s.</t>
+          <t>User taps Verification interactive button #16 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.78s.</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
@@ -3417,7 +3417,7 @@
         </is>
       </c>
       <c r="G72" s="2" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.78</v>
       </c>
       <c r="H72" s="2" t="inlineStr">
         <is>
@@ -3439,7 +3439,7 @@
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #17 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.71s.</t>
+          <t>User taps Verification interactive button #17 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.44s.</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr">
@@ -3458,7 +3458,7 @@
         </is>
       </c>
       <c r="G73" s="2" t="n">
-        <v>0.71</v>
+        <v>0.44</v>
       </c>
       <c r="H73" s="2" t="inlineStr">
         <is>
@@ -3480,7 +3480,7 @@
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #18 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.69s.</t>
+          <t>User taps Verification interactive button #18 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.35s.</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
@@ -3499,7 +3499,7 @@
         </is>
       </c>
       <c r="G74" s="2" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.35</v>
       </c>
       <c r="H74" s="2" t="inlineStr">
         <is>
@@ -3521,7 +3521,7 @@
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #19 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.79s.</t>
+          <t>User taps Verification interactive button #19 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.52s.</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
@@ -3540,7 +3540,7 @@
         </is>
       </c>
       <c r="G75" s="2" t="n">
-        <v>0.79</v>
+        <v>0.52</v>
       </c>
       <c r="H75" s="2" t="inlineStr">
         <is>
@@ -3562,7 +3562,7 @@
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #20 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.39s.</t>
+          <t>User taps Verification interactive button #20 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.68s.</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
@@ -3581,7 +3581,7 @@
         </is>
       </c>
       <c r="G76" s="2" t="n">
-        <v>0.39</v>
+        <v>0.68</v>
       </c>
       <c r="H76" s="2" t="inlineStr">
         <is>
@@ -3603,7 +3603,7 @@
       </c>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #21 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.49s.</t>
+          <t>User taps Verification interactive button #21 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.6s.</t>
         </is>
       </c>
       <c r="D77" s="2" t="inlineStr">
@@ -3622,7 +3622,7 @@
         </is>
       </c>
       <c r="G77" s="2" t="n">
-        <v>0.49</v>
+        <v>0.6</v>
       </c>
       <c r="H77" s="2" t="inlineStr">
         <is>
@@ -3644,7 +3644,7 @@
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #22 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.87s.</t>
+          <t>User taps Verification interactive button #22 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.85s.</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
@@ -3663,7 +3663,7 @@
         </is>
       </c>
       <c r="G78" s="2" t="n">
-        <v>0.87</v>
+        <v>0.85</v>
       </c>
       <c r="H78" s="2" t="inlineStr">
         <is>
@@ -3685,7 +3685,7 @@
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #23 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.69s.</t>
+          <t>User taps Verification interactive button #23 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.85s.</t>
         </is>
       </c>
       <c r="D79" s="2" t="inlineStr">
@@ -3704,7 +3704,7 @@
         </is>
       </c>
       <c r="G79" s="2" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.85</v>
       </c>
       <c r="H79" s="2" t="inlineStr">
         <is>
@@ -3726,7 +3726,7 @@
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #24 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.7s.</t>
+          <t>User taps Verification interactive button #24 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.37s.</t>
         </is>
       </c>
       <c r="D80" s="2" t="inlineStr">
@@ -3745,7 +3745,7 @@
         </is>
       </c>
       <c r="G80" s="2" t="n">
-        <v>0.7</v>
+        <v>0.37</v>
       </c>
       <c r="H80" s="2" t="inlineStr">
         <is>
@@ -3767,7 +3767,7 @@
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #25 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.44s.</t>
+          <t>User taps Verification interactive button #25 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.35s.</t>
         </is>
       </c>
       <c r="D81" s="2" t="inlineStr">
@@ -3786,7 +3786,7 @@
         </is>
       </c>
       <c r="G81" s="2" t="n">
-        <v>0.44</v>
+        <v>0.35</v>
       </c>
       <c r="H81" s="2" t="inlineStr">
         <is>
@@ -3827,7 +3827,7 @@
         </is>
       </c>
       <c r="G82" s="2" t="n">
-        <v>0.62</v>
+        <v>0.66</v>
       </c>
       <c r="H82" s="2" t="inlineStr">
         <is>
@@ -3868,7 +3868,7 @@
         </is>
       </c>
       <c r="G83" s="2" t="n">
-        <v>1.1</v>
+        <v>1.06</v>
       </c>
       <c r="H83" s="2" t="inlineStr">
         <is>
@@ -3909,7 +3909,7 @@
         </is>
       </c>
       <c r="G84" s="2" t="n">
-        <v>0.53</v>
+        <v>0.88</v>
       </c>
       <c r="H84" s="2" t="inlineStr">
         <is>
@@ -3950,7 +3950,7 @@
         </is>
       </c>
       <c r="G85" s="2" t="n">
-        <v>0.9399999999999999</v>
+        <v>1.11</v>
       </c>
       <c r="H85" s="2" t="inlineStr">
         <is>
@@ -3991,7 +3991,7 @@
         </is>
       </c>
       <c r="G86" s="2" t="n">
-        <v>0.46</v>
+        <v>0.73</v>
       </c>
       <c r="H86" s="2" t="inlineStr">
         <is>
@@ -4032,7 +4032,7 @@
         </is>
       </c>
       <c r="G87" s="2" t="n">
-        <v>0.48</v>
+        <v>0.53</v>
       </c>
       <c r="H87" s="2" t="inlineStr">
         <is>
@@ -4073,7 +4073,7 @@
         </is>
       </c>
       <c r="G88" s="2" t="n">
-        <v>0.88</v>
+        <v>1.01</v>
       </c>
       <c r="H88" s="2" t="inlineStr">
         <is>
@@ -4114,7 +4114,7 @@
         </is>
       </c>
       <c r="G89" s="2" t="n">
-        <v>0.79</v>
+        <v>0.65</v>
       </c>
       <c r="H89" s="2" t="inlineStr">
         <is>
@@ -4155,7 +4155,7 @@
         </is>
       </c>
       <c r="G90" s="2" t="n">
-        <v>0.63</v>
+        <v>0.62</v>
       </c>
       <c r="H90" s="2" t="inlineStr">
         <is>
@@ -4196,7 +4196,7 @@
         </is>
       </c>
       <c r="G91" s="2" t="n">
-        <v>0.8</v>
+        <v>0.54</v>
       </c>
       <c r="H91" s="2" t="inlineStr">
         <is>
@@ -4237,7 +4237,7 @@
         </is>
       </c>
       <c r="G92" s="2" t="n">
-        <v>0.59</v>
+        <v>0.39</v>
       </c>
       <c r="H92" s="2" t="inlineStr">
         <is>
@@ -4278,7 +4278,7 @@
         </is>
       </c>
       <c r="G93" s="2" t="n">
-        <v>0.73</v>
+        <v>0.54</v>
       </c>
       <c r="H93" s="2" t="inlineStr">
         <is>
@@ -4319,7 +4319,7 @@
         </is>
       </c>
       <c r="G94" s="2" t="n">
-        <v>0.6</v>
+        <v>0.93</v>
       </c>
       <c r="H94" s="2" t="inlineStr">
         <is>
@@ -4360,7 +4360,7 @@
         </is>
       </c>
       <c r="G95" s="2" t="n">
-        <v>0.83</v>
+        <v>0.57</v>
       </c>
       <c r="H95" s="2" t="inlineStr">
         <is>
@@ -4401,7 +4401,7 @@
         </is>
       </c>
       <c r="G96" s="2" t="n">
-        <v>0.65</v>
+        <v>0.79</v>
       </c>
       <c r="H96" s="2" t="inlineStr">
         <is>
@@ -4423,7 +4423,7 @@
       </c>
       <c r="C97" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #1 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.81s.</t>
+          <t>User taps Issuance form action button #1 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.5s.</t>
         </is>
       </c>
       <c r="D97" s="2" t="inlineStr">
@@ -4442,7 +4442,7 @@
         </is>
       </c>
       <c r="G97" s="2" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.5</v>
       </c>
       <c r="H97" s="2" t="inlineStr">
         <is>
@@ -4464,7 +4464,7 @@
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #2 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.89s.</t>
+          <t>User taps Issuance form action button #2 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.96s.</t>
         </is>
       </c>
       <c r="D98" s="2" t="inlineStr">
@@ -4483,7 +4483,7 @@
         </is>
       </c>
       <c r="G98" s="2" t="n">
-        <v>0.89</v>
+        <v>0.96</v>
       </c>
       <c r="H98" s="2" t="inlineStr">
         <is>
@@ -4505,7 +4505,7 @@
       </c>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #3 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.43s.</t>
+          <t>User taps Issuance form action button #3 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.77s.</t>
         </is>
       </c>
       <c r="D99" s="2" t="inlineStr">
@@ -4524,7 +4524,7 @@
         </is>
       </c>
       <c r="G99" s="2" t="n">
-        <v>0.43</v>
+        <v>0.77</v>
       </c>
       <c r="H99" s="2" t="inlineStr">
         <is>
@@ -4546,7 +4546,7 @@
       </c>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #4 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.4s.</t>
+          <t>User taps Issuance form action button #4 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.63s.</t>
         </is>
       </c>
       <c r="D100" s="2" t="inlineStr">
@@ -4565,7 +4565,7 @@
         </is>
       </c>
       <c r="G100" s="2" t="n">
-        <v>0.4</v>
+        <v>0.63</v>
       </c>
       <c r="H100" s="2" t="inlineStr">
         <is>
@@ -4587,7 +4587,7 @@
       </c>
       <c r="C101" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #5 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.42s.</t>
+          <t>User taps Issuance form action button #5 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.51s.</t>
         </is>
       </c>
       <c r="D101" s="2" t="inlineStr">
@@ -4606,7 +4606,7 @@
         </is>
       </c>
       <c r="G101" s="2" t="n">
-        <v>0.42</v>
+        <v>0.51</v>
       </c>
       <c r="H101" s="2" t="inlineStr">
         <is>
@@ -4628,7 +4628,7 @@
       </c>
       <c r="C102" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #6 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.46s.</t>
+          <t>User taps Issuance form action button #6 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.42s.</t>
         </is>
       </c>
       <c r="D102" s="2" t="inlineStr">
@@ -4647,7 +4647,7 @@
         </is>
       </c>
       <c r="G102" s="2" t="n">
-        <v>0.46</v>
+        <v>0.42</v>
       </c>
       <c r="H102" s="2" t="inlineStr">
         <is>
@@ -4669,7 +4669,7 @@
       </c>
       <c r="C103" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #7 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.46s.</t>
+          <t>User taps Issuance form action button #7 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.93s.</t>
         </is>
       </c>
       <c r="D103" s="2" t="inlineStr">
@@ -4688,7 +4688,7 @@
         </is>
       </c>
       <c r="G103" s="2" t="n">
-        <v>0.46</v>
+        <v>0.93</v>
       </c>
       <c r="H103" s="2" t="inlineStr">
         <is>
@@ -4710,7 +4710,7 @@
       </c>
       <c r="C104" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #8 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.4s.</t>
+          <t>User taps Issuance form action button #8 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.71s.</t>
         </is>
       </c>
       <c r="D104" s="2" t="inlineStr">
@@ -4729,7 +4729,7 @@
         </is>
       </c>
       <c r="G104" s="2" t="n">
-        <v>0.4</v>
+        <v>0.71</v>
       </c>
       <c r="H104" s="2" t="inlineStr">
         <is>
@@ -4751,7 +4751,7 @@
       </c>
       <c r="C105" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #9 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.6s.</t>
+          <t>User taps Issuance form action button #9 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.87s.</t>
         </is>
       </c>
       <c r="D105" s="2" t="inlineStr">
@@ -4770,7 +4770,7 @@
         </is>
       </c>
       <c r="G105" s="2" t="n">
-        <v>0.6</v>
+        <v>0.87</v>
       </c>
       <c r="H105" s="2" t="inlineStr">
         <is>
@@ -4792,7 +4792,7 @@
       </c>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #10 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 1.02s.</t>
+          <t>User taps Issuance form action button #10 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 1.05s.</t>
         </is>
       </c>
       <c r="D106" s="2" t="inlineStr">
@@ -4811,7 +4811,7 @@
         </is>
       </c>
       <c r="G106" s="2" t="n">
-        <v>1.02</v>
+        <v>1.05</v>
       </c>
       <c r="H106" s="2" t="inlineStr">
         <is>
@@ -4833,7 +4833,7 @@
       </c>
       <c r="C107" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #11 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.86s.</t>
+          <t>User taps Issuance form action button #11 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.64s.</t>
         </is>
       </c>
       <c r="D107" s="2" t="inlineStr">
@@ -4852,7 +4852,7 @@
         </is>
       </c>
       <c r="G107" s="2" t="n">
-        <v>0.86</v>
+        <v>0.64</v>
       </c>
       <c r="H107" s="2" t="inlineStr">
         <is>
@@ -4874,7 +4874,7 @@
       </c>
       <c r="C108" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #12 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.39s.</t>
+          <t>User taps Issuance form action button #12 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.8s.</t>
         </is>
       </c>
       <c r="D108" s="2" t="inlineStr">
@@ -4893,7 +4893,7 @@
         </is>
       </c>
       <c r="G108" s="2" t="n">
-        <v>0.39</v>
+        <v>0.8</v>
       </c>
       <c r="H108" s="2" t="inlineStr">
         <is>
@@ -4915,7 +4915,7 @@
       </c>
       <c r="C109" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #13 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.6s.</t>
+          <t>User taps Issuance form action button #13 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.52s.</t>
         </is>
       </c>
       <c r="D109" s="2" t="inlineStr">
@@ -4934,7 +4934,7 @@
         </is>
       </c>
       <c r="G109" s="2" t="n">
-        <v>0.6</v>
+        <v>0.52</v>
       </c>
       <c r="H109" s="2" t="inlineStr">
         <is>
@@ -4956,7 +4956,7 @@
       </c>
       <c r="C110" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #14 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.97s.</t>
+          <t>User taps Issuance form action button #14 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 1.12s.</t>
         </is>
       </c>
       <c r="D110" s="2" t="inlineStr">
@@ -4975,7 +4975,7 @@
         </is>
       </c>
       <c r="G110" s="2" t="n">
-        <v>0.97</v>
+        <v>1.12</v>
       </c>
       <c r="H110" s="2" t="inlineStr">
         <is>
@@ -4997,7 +4997,7 @@
       </c>
       <c r="C111" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #15 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.8s.</t>
+          <t>User taps Issuance form action button #15 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.78s.</t>
         </is>
       </c>
       <c r="D111" s="2" t="inlineStr">
@@ -5016,7 +5016,7 @@
         </is>
       </c>
       <c r="G111" s="2" t="n">
-        <v>0.8</v>
+        <v>0.78</v>
       </c>
       <c r="H111" s="2" t="inlineStr">
         <is>
@@ -5038,7 +5038,7 @@
       </c>
       <c r="C112" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #16 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 1.09s.</t>
+          <t>User taps Issuance form action button #16 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.54s.</t>
         </is>
       </c>
       <c r="D112" s="2" t="inlineStr">
@@ -5057,7 +5057,7 @@
         </is>
       </c>
       <c r="G112" s="2" t="n">
-        <v>1.09</v>
+        <v>0.54</v>
       </c>
       <c r="H112" s="2" t="inlineStr">
         <is>
@@ -5079,7 +5079,7 @@
       </c>
       <c r="C113" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #17 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.99s.</t>
+          <t>User taps Issuance form action button #17 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.55s.</t>
         </is>
       </c>
       <c r="D113" s="2" t="inlineStr">
@@ -5098,7 +5098,7 @@
         </is>
       </c>
       <c r="G113" s="2" t="n">
-        <v>0.99</v>
+        <v>0.55</v>
       </c>
       <c r="H113" s="2" t="inlineStr">
         <is>
@@ -5120,7 +5120,7 @@
       </c>
       <c r="C114" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #18 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.47s.</t>
+          <t>User taps Issuance form action button #18 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.4s.</t>
         </is>
       </c>
       <c r="D114" s="2" t="inlineStr">
@@ -5139,7 +5139,7 @@
         </is>
       </c>
       <c r="G114" s="2" t="n">
-        <v>0.47</v>
+        <v>0.4</v>
       </c>
       <c r="H114" s="2" t="inlineStr">
         <is>
@@ -5161,7 +5161,7 @@
       </c>
       <c r="C115" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #19 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.91s.</t>
+          <t>User taps Issuance form action button #19 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.38s.</t>
         </is>
       </c>
       <c r="D115" s="2" t="inlineStr">
@@ -5180,7 +5180,7 @@
         </is>
       </c>
       <c r="G115" s="2" t="n">
-        <v>0.91</v>
+        <v>0.38</v>
       </c>
       <c r="H115" s="2" t="inlineStr">
         <is>
@@ -5202,7 +5202,7 @@
       </c>
       <c r="C116" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #20 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 1.06s.</t>
+          <t>User taps Issuance form action button #20 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.67s.</t>
         </is>
       </c>
       <c r="D116" s="2" t="inlineStr">
@@ -5221,7 +5221,7 @@
         </is>
       </c>
       <c r="G116" s="2" t="n">
-        <v>1.06</v>
+        <v>0.67</v>
       </c>
       <c r="H116" s="2" t="inlineStr">
         <is>
@@ -5243,7 +5243,7 @@
       </c>
       <c r="C117" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #21 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.97s.</t>
+          <t>User taps Issuance form action button #21 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.66s.</t>
         </is>
       </c>
       <c r="D117" s="2" t="inlineStr">
@@ -5262,7 +5262,7 @@
         </is>
       </c>
       <c r="G117" s="2" t="n">
-        <v>0.97</v>
+        <v>0.66</v>
       </c>
       <c r="H117" s="2" t="inlineStr">
         <is>
@@ -5284,7 +5284,7 @@
       </c>
       <c r="C118" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #22 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.84s.</t>
+          <t>User taps Issuance form action button #22 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 1.11s.</t>
         </is>
       </c>
       <c r="D118" s="2" t="inlineStr">
@@ -5303,7 +5303,7 @@
         </is>
       </c>
       <c r="G118" s="2" t="n">
-        <v>0.84</v>
+        <v>1.11</v>
       </c>
       <c r="H118" s="2" t="inlineStr">
         <is>
@@ -5325,7 +5325,7 @@
       </c>
       <c r="C119" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #23 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.44s.</t>
+          <t>User taps Issuance form action button #23 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 1.01s.</t>
         </is>
       </c>
       <c r="D119" s="2" t="inlineStr">
@@ -5344,7 +5344,7 @@
         </is>
       </c>
       <c r="G119" s="2" t="n">
-        <v>0.44</v>
+        <v>1.01</v>
       </c>
       <c r="H119" s="2" t="inlineStr">
         <is>
@@ -5366,7 +5366,7 @@
       </c>
       <c r="C120" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #24 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 1.01s.</t>
+          <t>User taps Issuance form action button #24 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.54s.</t>
         </is>
       </c>
       <c r="D120" s="2" t="inlineStr">
@@ -5385,7 +5385,7 @@
         </is>
       </c>
       <c r="G120" s="2" t="n">
-        <v>1.01</v>
+        <v>0.54</v>
       </c>
       <c r="H120" s="2" t="inlineStr">
         <is>
@@ -5407,7 +5407,7 @@
       </c>
       <c r="C121" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #25 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.65s.</t>
+          <t>User taps Issuance form action button #25 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 1.06s.</t>
         </is>
       </c>
       <c r="D121" s="2" t="inlineStr">
@@ -5426,7 +5426,7 @@
         </is>
       </c>
       <c r="G121" s="2" t="n">
-        <v>0.65</v>
+        <v>1.06</v>
       </c>
       <c r="H121" s="2" t="inlineStr">
         <is>
@@ -5467,7 +5467,7 @@
         </is>
       </c>
       <c r="G122" s="2" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.4</v>
       </c>
       <c r="H122" s="2" t="inlineStr">
         <is>
@@ -5508,7 +5508,7 @@
         </is>
       </c>
       <c r="G123" s="2" t="n">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="H123" s="2" t="inlineStr">
         <is>
@@ -5549,7 +5549,7 @@
         </is>
       </c>
       <c r="G124" s="2" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.74</v>
       </c>
       <c r="H124" s="2" t="inlineStr">
         <is>
@@ -5590,7 +5590,7 @@
         </is>
       </c>
       <c r="G125" s="2" t="n">
-        <v>0.36</v>
+        <v>0.73</v>
       </c>
       <c r="H125" s="2" t="inlineStr">
         <is>
@@ -5631,7 +5631,7 @@
         </is>
       </c>
       <c r="G126" s="2" t="n">
-        <v>0.38</v>
+        <v>0.37</v>
       </c>
       <c r="H126" s="2" t="inlineStr">
         <is>
@@ -5672,7 +5672,7 @@
         </is>
       </c>
       <c r="G127" s="2" t="n">
-        <v>0.76</v>
+        <v>0.73</v>
       </c>
       <c r="H127" s="2" t="inlineStr">
         <is>
@@ -5713,7 +5713,7 @@
         </is>
       </c>
       <c r="G128" s="2" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.7</v>
       </c>
       <c r="H128" s="2" t="inlineStr">
         <is>
@@ -5754,7 +5754,7 @@
         </is>
       </c>
       <c r="G129" s="2" t="n">
-        <v>0.65</v>
+        <v>0.35</v>
       </c>
       <c r="H129" s="2" t="inlineStr">
         <is>
@@ -5795,7 +5795,7 @@
         </is>
       </c>
       <c r="G130" s="2" t="n">
-        <v>0.67</v>
+        <v>0.41</v>
       </c>
       <c r="H130" s="2" t="inlineStr">
         <is>
@@ -5836,7 +5836,7 @@
         </is>
       </c>
       <c r="G131" s="2" t="n">
-        <v>0.8</v>
+        <v>0.42</v>
       </c>
       <c r="H131" s="2" t="inlineStr">
         <is>
@@ -5858,7 +5858,7 @@
       </c>
       <c r="C132" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #1 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.32s.</t>
+          <t>User taps Registry interactive card/button #1 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.35s.</t>
         </is>
       </c>
       <c r="D132" s="2" t="inlineStr">
@@ -5877,7 +5877,7 @@
         </is>
       </c>
       <c r="G132" s="2" t="n">
-        <v>0.32</v>
+        <v>0.35</v>
       </c>
       <c r="H132" s="2" t="inlineStr">
         <is>
@@ -5899,7 +5899,7 @@
       </c>
       <c r="C133" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #2 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.67s.</t>
+          <t>User taps Registry interactive card/button #2 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.55s.</t>
         </is>
       </c>
       <c r="D133" s="2" t="inlineStr">
@@ -5918,7 +5918,7 @@
         </is>
       </c>
       <c r="G133" s="2" t="n">
-        <v>0.67</v>
+        <v>0.55</v>
       </c>
       <c r="H133" s="2" t="inlineStr">
         <is>
@@ -5940,7 +5940,7 @@
       </c>
       <c r="C134" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #3 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.58s.</t>
+          <t>User taps Registry interactive card/button #3 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.65s.</t>
         </is>
       </c>
       <c r="D134" s="2" t="inlineStr">
@@ -5959,7 +5959,7 @@
         </is>
       </c>
       <c r="G134" s="2" t="n">
-        <v>0.58</v>
+        <v>0.65</v>
       </c>
       <c r="H134" s="2" t="inlineStr">
         <is>
@@ -5981,7 +5981,7 @@
       </c>
       <c r="C135" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #4 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.59s.</t>
+          <t>User taps Registry interactive card/button #4 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.49s.</t>
         </is>
       </c>
       <c r="D135" s="2" t="inlineStr">
@@ -6000,7 +6000,7 @@
         </is>
       </c>
       <c r="G135" s="2" t="n">
-        <v>0.59</v>
+        <v>0.49</v>
       </c>
       <c r="H135" s="2" t="inlineStr">
         <is>
@@ -6022,7 +6022,7 @@
       </c>
       <c r="C136" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #5 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.4s.</t>
+          <t>User taps Registry interactive card/button #5 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.36s.</t>
         </is>
       </c>
       <c r="D136" s="2" t="inlineStr">
@@ -6041,7 +6041,7 @@
         </is>
       </c>
       <c r="G136" s="2" t="n">
-        <v>0.4</v>
+        <v>0.36</v>
       </c>
       <c r="H136" s="2" t="inlineStr">
         <is>
@@ -6063,7 +6063,7 @@
       </c>
       <c r="C137" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #6 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.4s.</t>
+          <t>User taps Registry interactive card/button #6 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.72s.</t>
         </is>
       </c>
       <c r="D137" s="2" t="inlineStr">
@@ -6082,7 +6082,7 @@
         </is>
       </c>
       <c r="G137" s="2" t="n">
-        <v>0.4</v>
+        <v>0.72</v>
       </c>
       <c r="H137" s="2" t="inlineStr">
         <is>
@@ -6104,7 +6104,7 @@
       </c>
       <c r="C138" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #7 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.48s.</t>
+          <t>User taps Registry interactive card/button #7 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.61s.</t>
         </is>
       </c>
       <c r="D138" s="2" t="inlineStr">
@@ -6123,7 +6123,7 @@
         </is>
       </c>
       <c r="G138" s="2" t="n">
-        <v>0.48</v>
+        <v>0.61</v>
       </c>
       <c r="H138" s="2" t="inlineStr">
         <is>
@@ -6145,7 +6145,7 @@
       </c>
       <c r="C139" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #8 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.57s.</t>
+          <t>User taps Registry interactive card/button #8 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.6s.</t>
         </is>
       </c>
       <c r="D139" s="2" t="inlineStr">
@@ -6164,7 +6164,7 @@
         </is>
       </c>
       <c r="G139" s="2" t="n">
-        <v>0.57</v>
+        <v>0.6</v>
       </c>
       <c r="H139" s="2" t="inlineStr">
         <is>
@@ -6186,7 +6186,7 @@
       </c>
       <c r="C140" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #9 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.83s.</t>
+          <t>User taps Registry interactive card/button #9 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.76s.</t>
         </is>
       </c>
       <c r="D140" s="2" t="inlineStr">
@@ -6205,7 +6205,7 @@
         </is>
       </c>
       <c r="G140" s="2" t="n">
-        <v>0.83</v>
+        <v>0.76</v>
       </c>
       <c r="H140" s="2" t="inlineStr">
         <is>
@@ -6227,7 +6227,7 @@
       </c>
       <c r="C141" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #10 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.5s.</t>
+          <t>User taps Registry interactive card/button #10 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.7s.</t>
         </is>
       </c>
       <c r="D141" s="2" t="inlineStr">
@@ -6246,7 +6246,7 @@
         </is>
       </c>
       <c r="G141" s="2" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="H141" s="2" t="inlineStr">
         <is>
@@ -6268,7 +6268,7 @@
       </c>
       <c r="C142" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #11 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.34s.</t>
+          <t>User taps Registry interactive card/button #11 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.42s.</t>
         </is>
       </c>
       <c r="D142" s="2" t="inlineStr">
@@ -6287,7 +6287,7 @@
         </is>
       </c>
       <c r="G142" s="2" t="n">
-        <v>0.34</v>
+        <v>0.42</v>
       </c>
       <c r="H142" s="2" t="inlineStr">
         <is>
@@ -6309,7 +6309,7 @@
       </c>
       <c r="C143" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #12 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.36s.</t>
+          <t>User taps Registry interactive card/button #12 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.31s.</t>
         </is>
       </c>
       <c r="D143" s="2" t="inlineStr">
@@ -6328,7 +6328,7 @@
         </is>
       </c>
       <c r="G143" s="2" t="n">
-        <v>0.36</v>
+        <v>0.31</v>
       </c>
       <c r="H143" s="2" t="inlineStr">
         <is>
@@ -6350,7 +6350,7 @@
       </c>
       <c r="C144" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #13 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.58s.</t>
+          <t>User taps Registry interactive card/button #13 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.83s.</t>
         </is>
       </c>
       <c r="D144" s="2" t="inlineStr">
@@ -6369,7 +6369,7 @@
         </is>
       </c>
       <c r="G144" s="2" t="n">
-        <v>0.58</v>
+        <v>0.83</v>
       </c>
       <c r="H144" s="2" t="inlineStr">
         <is>
@@ -6391,7 +6391,7 @@
       </c>
       <c r="C145" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #14 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.82s.</t>
+          <t>User taps Registry interactive card/button #14 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.81s.</t>
         </is>
       </c>
       <c r="D145" s="2" t="inlineStr">
@@ -6410,7 +6410,7 @@
         </is>
       </c>
       <c r="G145" s="2" t="n">
-        <v>0.82</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="H145" s="2" t="inlineStr">
         <is>
@@ -6432,7 +6432,7 @@
       </c>
       <c r="C146" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #15 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.7s.</t>
+          <t>User taps Registry interactive card/button #15 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.45s.</t>
         </is>
       </c>
       <c r="D146" s="2" t="inlineStr">
@@ -6451,7 +6451,7 @@
         </is>
       </c>
       <c r="G146" s="2" t="n">
-        <v>0.7</v>
+        <v>0.45</v>
       </c>
       <c r="H146" s="2" t="inlineStr">
         <is>
@@ -6473,7 +6473,7 @@
       </c>
       <c r="C147" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #16 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.56s.</t>
+          <t>User taps Registry interactive card/button #16 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.58s.</t>
         </is>
       </c>
       <c r="D147" s="2" t="inlineStr">
@@ -6492,7 +6492,7 @@
         </is>
       </c>
       <c r="G147" s="2" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.58</v>
       </c>
       <c r="H147" s="2" t="inlineStr">
         <is>
@@ -6514,7 +6514,7 @@
       </c>
       <c r="C148" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #17 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.67s.</t>
+          <t>User taps Registry interactive card/button #17 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.39s.</t>
         </is>
       </c>
       <c r="D148" s="2" t="inlineStr">
@@ -6533,7 +6533,7 @@
         </is>
       </c>
       <c r="G148" s="2" t="n">
-        <v>0.67</v>
+        <v>0.39</v>
       </c>
       <c r="H148" s="2" t="inlineStr">
         <is>
@@ -6555,7 +6555,7 @@
       </c>
       <c r="C149" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #18 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.75s.</t>
+          <t>User taps Registry interactive card/button #18 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.53s.</t>
         </is>
       </c>
       <c r="D149" s="2" t="inlineStr">
@@ -6574,7 +6574,7 @@
         </is>
       </c>
       <c r="G149" s="2" t="n">
-        <v>0.75</v>
+        <v>0.53</v>
       </c>
       <c r="H149" s="2" t="inlineStr">
         <is>
@@ -6637,7 +6637,7 @@
       </c>
       <c r="C151" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #20 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.6s.</t>
+          <t>User taps Registry interactive card/button #20 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.66s.</t>
         </is>
       </c>
       <c r="D151" s="2" t="inlineStr">
@@ -6656,7 +6656,7 @@
         </is>
       </c>
       <c r="G151" s="2" t="n">
-        <v>0.6</v>
+        <v>0.66</v>
       </c>
       <c r="H151" s="2" t="inlineStr">
         <is>
@@ -6678,7 +6678,7 @@
       </c>
       <c r="C152" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #21 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.51s.</t>
+          <t>User taps Registry interactive card/button #21 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.35s.</t>
         </is>
       </c>
       <c r="D152" s="2" t="inlineStr">
@@ -6697,7 +6697,7 @@
         </is>
       </c>
       <c r="G152" s="2" t="n">
-        <v>0.51</v>
+        <v>0.35</v>
       </c>
       <c r="H152" s="2" t="inlineStr">
         <is>
@@ -6719,7 +6719,7 @@
       </c>
       <c r="C153" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #22 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.31s.</t>
+          <t>User taps Registry interactive card/button #22 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.53s.</t>
         </is>
       </c>
       <c r="D153" s="2" t="inlineStr">
@@ -6738,7 +6738,7 @@
         </is>
       </c>
       <c r="G153" s="2" t="n">
-        <v>0.31</v>
+        <v>0.53</v>
       </c>
       <c r="H153" s="2" t="inlineStr">
         <is>
@@ -6760,7 +6760,7 @@
       </c>
       <c r="C154" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #23 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.45s.</t>
+          <t>User taps Registry interactive card/button #23 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.67s.</t>
         </is>
       </c>
       <c r="D154" s="2" t="inlineStr">
@@ -6779,7 +6779,7 @@
         </is>
       </c>
       <c r="G154" s="2" t="n">
-        <v>0.45</v>
+        <v>0.67</v>
       </c>
       <c r="H154" s="2" t="inlineStr">
         <is>
@@ -6801,7 +6801,7 @@
       </c>
       <c r="C155" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #24 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.69s.</t>
+          <t>User taps Registry interactive card/button #24 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.73s.</t>
         </is>
       </c>
       <c r="D155" s="2" t="inlineStr">
@@ -6820,7 +6820,7 @@
         </is>
       </c>
       <c r="G155" s="2" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.73</v>
       </c>
       <c r="H155" s="2" t="inlineStr">
         <is>
@@ -6842,7 +6842,7 @@
       </c>
       <c r="C156" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #25 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.56s.</t>
+          <t>User taps Registry interactive card/button #25 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.49s.</t>
         </is>
       </c>
       <c r="D156" s="2" t="inlineStr">
@@ -6861,7 +6861,7 @@
         </is>
       </c>
       <c r="G156" s="2" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.49</v>
       </c>
       <c r="H156" s="2" t="inlineStr">
         <is>
@@ -6883,7 +6883,7 @@
       </c>
       <c r="C157" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #26 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.8s.</t>
+          <t>User taps Registry interactive card/button #26 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.81s.</t>
         </is>
       </c>
       <c r="D157" s="2" t="inlineStr">
@@ -6902,7 +6902,7 @@
         </is>
       </c>
       <c r="G157" s="2" t="n">
-        <v>0.8</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="H157" s="2" t="inlineStr">
         <is>
@@ -6924,7 +6924,7 @@
       </c>
       <c r="C158" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #27 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.67s.</t>
+          <t>User taps Registry interactive card/button #27 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.3s.</t>
         </is>
       </c>
       <c r="D158" s="2" t="inlineStr">
@@ -6943,7 +6943,7 @@
         </is>
       </c>
       <c r="G158" s="2" t="n">
-        <v>0.67</v>
+        <v>0.3</v>
       </c>
       <c r="H158" s="2" t="inlineStr">
         <is>
@@ -6965,7 +6965,7 @@
       </c>
       <c r="C159" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #28 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.81s.</t>
+          <t>User taps Registry interactive card/button #28 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.7s.</t>
         </is>
       </c>
       <c r="D159" s="2" t="inlineStr">
@@ -6984,7 +6984,7 @@
         </is>
       </c>
       <c r="G159" s="2" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.7</v>
       </c>
       <c r="H159" s="2" t="inlineStr">
         <is>
@@ -7006,7 +7006,7 @@
       </c>
       <c r="C160" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #29 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.39s.</t>
+          <t>User taps Registry interactive card/button #29 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.69s.</t>
         </is>
       </c>
       <c r="D160" s="2" t="inlineStr">
@@ -7025,7 +7025,7 @@
         </is>
       </c>
       <c r="G160" s="2" t="n">
-        <v>0.39</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="H160" s="2" t="inlineStr">
         <is>
@@ -7047,7 +7047,7 @@
       </c>
       <c r="C161" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #30 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.48s.</t>
+          <t>User taps Registry interactive card/button #30 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.46s.</t>
         </is>
       </c>
       <c r="D161" s="2" t="inlineStr">
@@ -7066,7 +7066,7 @@
         </is>
       </c>
       <c r="G161" s="2" t="n">
-        <v>0.48</v>
+        <v>0.46</v>
       </c>
       <c r="H161" s="2" t="inlineStr">
         <is>
@@ -7107,7 +7107,7 @@
         </is>
       </c>
       <c r="G162" s="2" t="n">
-        <v>0.62</v>
+        <v>0.31</v>
       </c>
       <c r="H162" s="2" t="inlineStr">
         <is>
@@ -7148,7 +7148,7 @@
         </is>
       </c>
       <c r="G163" s="2" t="n">
-        <v>0.53</v>
+        <v>0.44</v>
       </c>
       <c r="H163" s="2" t="inlineStr">
         <is>
@@ -7189,7 +7189,7 @@
         </is>
       </c>
       <c r="G164" s="2" t="n">
-        <v>0.46</v>
+        <v>0.62</v>
       </c>
       <c r="H164" s="2" t="inlineStr">
         <is>
@@ -7230,7 +7230,7 @@
         </is>
       </c>
       <c r="G165" s="2" t="n">
-        <v>0.74</v>
+        <v>0.63</v>
       </c>
       <c r="H165" s="2" t="inlineStr">
         <is>
@@ -7271,7 +7271,7 @@
         </is>
       </c>
       <c r="G166" s="2" t="n">
-        <v>0.53</v>
+        <v>0.49</v>
       </c>
       <c r="H166" s="2" t="inlineStr">
         <is>
@@ -7293,7 +7293,7 @@
       </c>
       <c r="C167" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #1 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.36s.</t>
+          <t>User taps Network diagnostic button #1 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.39s.</t>
         </is>
       </c>
       <c r="D167" s="2" t="inlineStr">
@@ -7312,7 +7312,7 @@
         </is>
       </c>
       <c r="G167" s="2" t="n">
-        <v>0.36</v>
+        <v>0.39</v>
       </c>
       <c r="H167" s="2" t="inlineStr">
         <is>
@@ -7334,7 +7334,7 @@
       </c>
       <c r="C168" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #2 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.63s.</t>
+          <t>User taps Network diagnostic button #2 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.31s.</t>
         </is>
       </c>
       <c r="D168" s="2" t="inlineStr">
@@ -7353,7 +7353,7 @@
         </is>
       </c>
       <c r="G168" s="2" t="n">
-        <v>0.63</v>
+        <v>0.31</v>
       </c>
       <c r="H168" s="2" t="inlineStr">
         <is>
@@ -7375,7 +7375,7 @@
       </c>
       <c r="C169" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #3 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.46s.</t>
+          <t>User taps Network diagnostic button #3 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.54s.</t>
         </is>
       </c>
       <c r="D169" s="2" t="inlineStr">
@@ -7394,7 +7394,7 @@
         </is>
       </c>
       <c r="G169" s="2" t="n">
-        <v>0.46</v>
+        <v>0.54</v>
       </c>
       <c r="H169" s="2" t="inlineStr">
         <is>
@@ -7416,7 +7416,7 @@
       </c>
       <c r="C170" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #4 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.38s.</t>
+          <t>User taps Network diagnostic button #4 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.52s.</t>
         </is>
       </c>
       <c r="D170" s="2" t="inlineStr">
@@ -7435,7 +7435,7 @@
         </is>
       </c>
       <c r="G170" s="2" t="n">
-        <v>0.38</v>
+        <v>0.52</v>
       </c>
       <c r="H170" s="2" t="inlineStr">
         <is>
@@ -7457,7 +7457,7 @@
       </c>
       <c r="C171" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #5 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.44s.</t>
+          <t>User taps Network diagnostic button #5 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.3s.</t>
         </is>
       </c>
       <c r="D171" s="2" t="inlineStr">
@@ -7476,7 +7476,7 @@
         </is>
       </c>
       <c r="G171" s="2" t="n">
-        <v>0.44</v>
+        <v>0.3</v>
       </c>
       <c r="H171" s="2" t="inlineStr">
         <is>
@@ -7498,7 +7498,7 @@
       </c>
       <c r="C172" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #6 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.47s.</t>
+          <t>User taps Network diagnostic button #6 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.7s.</t>
         </is>
       </c>
       <c r="D172" s="2" t="inlineStr">
@@ -7517,7 +7517,7 @@
         </is>
       </c>
       <c r="G172" s="2" t="n">
-        <v>0.47</v>
+        <v>0.7</v>
       </c>
       <c r="H172" s="2" t="inlineStr">
         <is>
@@ -7539,7 +7539,7 @@
       </c>
       <c r="C173" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #7 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.35s.</t>
+          <t>User taps Network diagnostic button #7 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.76s.</t>
         </is>
       </c>
       <c r="D173" s="2" t="inlineStr">
@@ -7558,7 +7558,7 @@
         </is>
       </c>
       <c r="G173" s="2" t="n">
-        <v>0.35</v>
+        <v>0.76</v>
       </c>
       <c r="H173" s="2" t="inlineStr">
         <is>
@@ -7580,7 +7580,7 @@
       </c>
       <c r="C174" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #8 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.56s.</t>
+          <t>User taps Network diagnostic button #8 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.38s.</t>
         </is>
       </c>
       <c r="D174" s="2" t="inlineStr">
@@ -7599,7 +7599,7 @@
         </is>
       </c>
       <c r="G174" s="2" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.38</v>
       </c>
       <c r="H174" s="2" t="inlineStr">
         <is>
@@ -7621,7 +7621,7 @@
       </c>
       <c r="C175" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #9 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.59s.</t>
+          <t>User taps Network diagnostic button #9 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.56s.</t>
         </is>
       </c>
       <c r="D175" s="2" t="inlineStr">
@@ -7640,7 +7640,7 @@
         </is>
       </c>
       <c r="G175" s="2" t="n">
-        <v>0.59</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="H175" s="2" t="inlineStr">
         <is>
@@ -7662,7 +7662,7 @@
       </c>
       <c r="C176" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #10 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.63s.</t>
+          <t>User taps Network diagnostic button #10 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.72s.</t>
         </is>
       </c>
       <c r="D176" s="2" t="inlineStr">
@@ -7681,7 +7681,7 @@
         </is>
       </c>
       <c r="G176" s="2" t="n">
-        <v>0.63</v>
+        <v>0.72</v>
       </c>
       <c r="H176" s="2" t="inlineStr">
         <is>
@@ -7703,7 +7703,7 @@
       </c>
       <c r="C177" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #11 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.77s.</t>
+          <t>User taps Network diagnostic button #11 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.5s.</t>
         </is>
       </c>
       <c r="D177" s="2" t="inlineStr">
@@ -7722,7 +7722,7 @@
         </is>
       </c>
       <c r="G177" s="2" t="n">
-        <v>0.77</v>
+        <v>0.5</v>
       </c>
       <c r="H177" s="2" t="inlineStr">
         <is>
@@ -7744,7 +7744,7 @@
       </c>
       <c r="C178" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #12 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.34s.</t>
+          <t>User taps Network diagnostic button #12 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.39s.</t>
         </is>
       </c>
       <c r="D178" s="2" t="inlineStr">
@@ -7763,7 +7763,7 @@
         </is>
       </c>
       <c r="G178" s="2" t="n">
-        <v>0.34</v>
+        <v>0.39</v>
       </c>
       <c r="H178" s="2" t="inlineStr">
         <is>
@@ -7785,7 +7785,7 @@
       </c>
       <c r="C179" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #13 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.6s.</t>
+          <t>User taps Network diagnostic button #13 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.73s.</t>
         </is>
       </c>
       <c r="D179" s="2" t="inlineStr">
@@ -7804,7 +7804,7 @@
         </is>
       </c>
       <c r="G179" s="2" t="n">
-        <v>0.6</v>
+        <v>0.73</v>
       </c>
       <c r="H179" s="2" t="inlineStr">
         <is>
@@ -7826,7 +7826,7 @@
       </c>
       <c r="C180" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #14 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.75s.</t>
+          <t>User taps Network diagnostic button #14 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.33s.</t>
         </is>
       </c>
       <c r="D180" s="2" t="inlineStr">
@@ -7845,7 +7845,7 @@
         </is>
       </c>
       <c r="G180" s="2" t="n">
-        <v>0.75</v>
+        <v>0.33</v>
       </c>
       <c r="H180" s="2" t="inlineStr">
         <is>
@@ -7867,7 +7867,7 @@
       </c>
       <c r="C181" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #15 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.39s.</t>
+          <t>User taps Network diagnostic button #15 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.42s.</t>
         </is>
       </c>
       <c r="D181" s="2" t="inlineStr">
@@ -7886,7 +7886,7 @@
         </is>
       </c>
       <c r="G181" s="2" t="n">
-        <v>0.39</v>
+        <v>0.42</v>
       </c>
       <c r="H181" s="2" t="inlineStr">
         <is>
@@ -7908,7 +7908,7 @@
       </c>
       <c r="C182" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #16 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.61s.</t>
+          <t>User taps Network diagnostic button #16 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.51s.</t>
         </is>
       </c>
       <c r="D182" s="2" t="inlineStr">
@@ -7927,7 +7927,7 @@
         </is>
       </c>
       <c r="G182" s="2" t="n">
-        <v>0.61</v>
+        <v>0.51</v>
       </c>
       <c r="H182" s="2" t="inlineStr">
         <is>
@@ -7949,7 +7949,7 @@
       </c>
       <c r="C183" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #17 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.63s.</t>
+          <t>User taps Network diagnostic button #17 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.52s.</t>
         </is>
       </c>
       <c r="D183" s="2" t="inlineStr">
@@ -7968,7 +7968,7 @@
         </is>
       </c>
       <c r="G183" s="2" t="n">
-        <v>0.63</v>
+        <v>0.52</v>
       </c>
       <c r="H183" s="2" t="inlineStr">
         <is>
@@ -7990,7 +7990,7 @@
       </c>
       <c r="C184" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #18 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.3s.</t>
+          <t>User taps Network diagnostic button #18 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.54s.</t>
         </is>
       </c>
       <c r="D184" s="2" t="inlineStr">
@@ -8009,7 +8009,7 @@
         </is>
       </c>
       <c r="G184" s="2" t="n">
-        <v>0.3</v>
+        <v>0.54</v>
       </c>
       <c r="H184" s="2" t="inlineStr">
         <is>
@@ -8031,7 +8031,7 @@
       </c>
       <c r="C185" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #19 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.77s.</t>
+          <t>User taps Network diagnostic button #19 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.67s.</t>
         </is>
       </c>
       <c r="D185" s="2" t="inlineStr">
@@ -8050,7 +8050,7 @@
         </is>
       </c>
       <c r="G185" s="2" t="n">
-        <v>0.77</v>
+        <v>0.67</v>
       </c>
       <c r="H185" s="2" t="inlineStr">
         <is>
@@ -8072,7 +8072,7 @@
       </c>
       <c r="C186" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #20 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.37s.</t>
+          <t>User taps Network diagnostic button #20 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.73s.</t>
         </is>
       </c>
       <c r="D186" s="2" t="inlineStr">
@@ -8091,7 +8091,7 @@
         </is>
       </c>
       <c r="G186" s="2" t="n">
-        <v>0.37</v>
+        <v>0.73</v>
       </c>
       <c r="H186" s="2" t="inlineStr">
         <is>
@@ -8113,7 +8113,7 @@
       </c>
       <c r="C187" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #21 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.31s.</t>
+          <t>User taps Network diagnostic button #21 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.33s.</t>
         </is>
       </c>
       <c r="D187" s="2" t="inlineStr">
@@ -8132,7 +8132,7 @@
         </is>
       </c>
       <c r="G187" s="2" t="n">
-        <v>0.31</v>
+        <v>0.33</v>
       </c>
       <c r="H187" s="2" t="inlineStr">
         <is>
@@ -8154,7 +8154,7 @@
       </c>
       <c r="C188" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #22 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.41s.</t>
+          <t>User taps Network diagnostic button #22 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.74s.</t>
         </is>
       </c>
       <c r="D188" s="2" t="inlineStr">
@@ -8173,7 +8173,7 @@
         </is>
       </c>
       <c r="G188" s="2" t="n">
-        <v>0.41</v>
+        <v>0.74</v>
       </c>
       <c r="H188" s="2" t="inlineStr">
         <is>
@@ -8195,7 +8195,7 @@
       </c>
       <c r="C189" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #23 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.72s.</t>
+          <t>User taps Network diagnostic button #23 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.71s.</t>
         </is>
       </c>
       <c r="D189" s="2" t="inlineStr">
@@ -8214,7 +8214,7 @@
         </is>
       </c>
       <c r="G189" s="2" t="n">
-        <v>0.72</v>
+        <v>0.71</v>
       </c>
       <c r="H189" s="2" t="inlineStr">
         <is>
@@ -8236,7 +8236,7 @@
       </c>
       <c r="C190" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #24 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.51s.</t>
+          <t>User taps Network diagnostic button #24 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.59s.</t>
         </is>
       </c>
       <c r="D190" s="2" t="inlineStr">
@@ -8255,7 +8255,7 @@
         </is>
       </c>
       <c r="G190" s="2" t="n">
-        <v>0.51</v>
+        <v>0.59</v>
       </c>
       <c r="H190" s="2" t="inlineStr">
         <is>
@@ -8277,7 +8277,7 @@
       </c>
       <c r="C191" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #25 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.78s.</t>
+          <t>User taps Network diagnostic button #25 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.36s.</t>
         </is>
       </c>
       <c r="D191" s="2" t="inlineStr">
@@ -8296,7 +8296,7 @@
         </is>
       </c>
       <c r="G191" s="2" t="n">
-        <v>0.78</v>
+        <v>0.36</v>
       </c>
       <c r="H191" s="2" t="inlineStr">
         <is>
@@ -8318,7 +8318,7 @@
       </c>
       <c r="C192" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #26 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.69s.</t>
+          <t>User taps Network diagnostic button #26 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.52s.</t>
         </is>
       </c>
       <c r="D192" s="2" t="inlineStr">
@@ -8337,7 +8337,7 @@
         </is>
       </c>
       <c r="G192" s="2" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.52</v>
       </c>
       <c r="H192" s="2" t="inlineStr">
         <is>
@@ -8359,7 +8359,7 @@
       </c>
       <c r="C193" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #27 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.62s.</t>
+          <t>User taps Network diagnostic button #27 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.28s.</t>
         </is>
       </c>
       <c r="D193" s="2" t="inlineStr">
@@ -8378,7 +8378,7 @@
         </is>
       </c>
       <c r="G193" s="2" t="n">
-        <v>0.62</v>
+        <v>0.28</v>
       </c>
       <c r="H193" s="2" t="inlineStr">
         <is>
@@ -8400,7 +8400,7 @@
       </c>
       <c r="C194" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #28 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.41s.</t>
+          <t>User taps Network diagnostic button #28 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.77s.</t>
         </is>
       </c>
       <c r="D194" s="2" t="inlineStr">
@@ -8419,7 +8419,7 @@
         </is>
       </c>
       <c r="G194" s="2" t="n">
-        <v>0.41</v>
+        <v>0.77</v>
       </c>
       <c r="H194" s="2" t="inlineStr">
         <is>
@@ -8441,7 +8441,7 @@
       </c>
       <c r="C195" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #29 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.47s.</t>
+          <t>User taps Network diagnostic button #29 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.66s.</t>
         </is>
       </c>
       <c r="D195" s="2" t="inlineStr">
@@ -8460,7 +8460,7 @@
         </is>
       </c>
       <c r="G195" s="2" t="n">
-        <v>0.47</v>
+        <v>0.66</v>
       </c>
       <c r="H195" s="2" t="inlineStr">
         <is>
@@ -8482,7 +8482,7 @@
       </c>
       <c r="C196" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #30 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.61s.</t>
+          <t>User taps Network diagnostic button #30 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.38s.</t>
         </is>
       </c>
       <c r="D196" s="2" t="inlineStr">
@@ -8501,7 +8501,7 @@
         </is>
       </c>
       <c r="G196" s="2" t="n">
-        <v>0.61</v>
+        <v>0.38</v>
       </c>
       <c r="H196" s="2" t="inlineStr">
         <is>
@@ -8542,7 +8542,7 @@
         </is>
       </c>
       <c r="G197" s="2" t="n">
-        <v>0.91</v>
+        <v>0.58</v>
       </c>
       <c r="H197" s="2" t="inlineStr">
         <is>
@@ -8583,7 +8583,7 @@
         </is>
       </c>
       <c r="G198" s="2" t="n">
-        <v>0.55</v>
+        <v>0.79</v>
       </c>
       <c r="H198" s="2" t="inlineStr">
         <is>
@@ -8624,7 +8624,7 @@
         </is>
       </c>
       <c r="G199" s="2" t="n">
-        <v>0.58</v>
+        <v>0.67</v>
       </c>
       <c r="H199" s="2" t="inlineStr">
         <is>
@@ -8665,7 +8665,7 @@
         </is>
       </c>
       <c r="G200" s="2" t="n">
-        <v>1.06</v>
+        <v>0.64</v>
       </c>
       <c r="H200" s="2" t="inlineStr">
         <is>
@@ -8706,7 +8706,7 @@
         </is>
       </c>
       <c r="G201" s="2" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.36</v>
       </c>
       <c r="H201" s="2" t="inlineStr">
         <is>
@@ -8747,7 +8747,7 @@
         </is>
       </c>
       <c r="G202" s="2" t="n">
-        <v>0.43</v>
+        <v>0.74</v>
       </c>
       <c r="H202" s="2" t="inlineStr">
         <is>
@@ -8788,7 +8788,7 @@
         </is>
       </c>
       <c r="G203" s="2" t="n">
-        <v>1.1</v>
+        <v>0.78</v>
       </c>
       <c r="H203" s="2" t="inlineStr">
         <is>
@@ -8810,7 +8810,7 @@
       </c>
       <c r="C204" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #1 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.48s.</t>
+          <t>User executes touch gesture #1 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.09s.</t>
         </is>
       </c>
       <c r="D204" s="2" t="inlineStr">
@@ -8829,7 +8829,7 @@
         </is>
       </c>
       <c r="G204" s="2" t="n">
-        <v>0.48</v>
+        <v>1.09</v>
       </c>
       <c r="H204" s="2" t="inlineStr">
         <is>
@@ -8851,7 +8851,7 @@
       </c>
       <c r="C205" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #2 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.69s.</t>
+          <t>User executes touch gesture #2 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.0s.</t>
         </is>
       </c>
       <c r="D205" s="2" t="inlineStr">
@@ -8870,7 +8870,7 @@
         </is>
       </c>
       <c r="G205" s="2" t="n">
-        <v>0.6899999999999999</v>
+        <v>1</v>
       </c>
       <c r="H205" s="2" t="inlineStr">
         <is>
@@ -8892,7 +8892,7 @@
       </c>
       <c r="C206" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #3 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.2s.</t>
+          <t>User executes touch gesture #3 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.61s.</t>
         </is>
       </c>
       <c r="D206" s="2" t="inlineStr">
@@ -8911,7 +8911,7 @@
         </is>
       </c>
       <c r="G206" s="2" t="n">
-        <v>1.2</v>
+        <v>0.61</v>
       </c>
       <c r="H206" s="2" t="inlineStr">
         <is>
@@ -8933,7 +8933,7 @@
       </c>
       <c r="C207" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #4 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.96s.</t>
+          <t>User executes touch gesture #4 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.47s.</t>
         </is>
       </c>
       <c r="D207" s="2" t="inlineStr">
@@ -8952,7 +8952,7 @@
         </is>
       </c>
       <c r="G207" s="2" t="n">
-        <v>0.96</v>
+        <v>0.47</v>
       </c>
       <c r="H207" s="2" t="inlineStr">
         <is>
@@ -8974,7 +8974,7 @@
       </c>
       <c r="C208" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #5 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.02s.</t>
+          <t>User executes touch gesture #5 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.7s.</t>
         </is>
       </c>
       <c r="D208" s="2" t="inlineStr">
@@ -8993,7 +8993,7 @@
         </is>
       </c>
       <c r="G208" s="2" t="n">
-        <v>1.02</v>
+        <v>0.7</v>
       </c>
       <c r="H208" s="2" t="inlineStr">
         <is>
@@ -9015,7 +9015,7 @@
       </c>
       <c r="C209" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #6 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.94s.</t>
+          <t>User executes touch gesture #6 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.38s.</t>
         </is>
       </c>
       <c r="D209" s="2" t="inlineStr">
@@ -9034,7 +9034,7 @@
         </is>
       </c>
       <c r="G209" s="2" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.38</v>
       </c>
       <c r="H209" s="2" t="inlineStr">
         <is>
@@ -9056,7 +9056,7 @@
       </c>
       <c r="C210" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #7 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.89s.</t>
+          <t>User executes touch gesture #7 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.68s.</t>
         </is>
       </c>
       <c r="D210" s="2" t="inlineStr">
@@ -9075,7 +9075,7 @@
         </is>
       </c>
       <c r="G210" s="2" t="n">
-        <v>0.89</v>
+        <v>0.68</v>
       </c>
       <c r="H210" s="2" t="inlineStr">
         <is>
@@ -9097,7 +9097,7 @@
       </c>
       <c r="C211" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #8 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.37s.</t>
+          <t>User executes touch gesture #8 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.91s.</t>
         </is>
       </c>
       <c r="D211" s="2" t="inlineStr">
@@ -9116,7 +9116,7 @@
         </is>
       </c>
       <c r="G211" s="2" t="n">
-        <v>0.37</v>
+        <v>0.91</v>
       </c>
       <c r="H211" s="2" t="inlineStr">
         <is>
@@ -9138,7 +9138,7 @@
       </c>
       <c r="C212" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #9 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.85s.</t>
+          <t>User executes touch gesture #9 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.1s.</t>
         </is>
       </c>
       <c r="D212" s="2" t="inlineStr">
@@ -9157,7 +9157,7 @@
         </is>
       </c>
       <c r="G212" s="2" t="n">
-        <v>0.85</v>
+        <v>1.1</v>
       </c>
       <c r="H212" s="2" t="inlineStr">
         <is>
@@ -9179,7 +9179,7 @@
       </c>
       <c r="C213" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #10 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.96s.</t>
+          <t>User executes touch gesture #10 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.02s.</t>
         </is>
       </c>
       <c r="D213" s="2" t="inlineStr">
@@ -9198,7 +9198,7 @@
         </is>
       </c>
       <c r="G213" s="2" t="n">
-        <v>0.96</v>
+        <v>1.02</v>
       </c>
       <c r="H213" s="2" t="inlineStr">
         <is>
@@ -9220,7 +9220,7 @@
       </c>
       <c r="C214" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #11 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.17s.</t>
+          <t>User executes touch gesture #11 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.51s.</t>
         </is>
       </c>
       <c r="D214" s="2" t="inlineStr">
@@ -9239,7 +9239,7 @@
         </is>
       </c>
       <c r="G214" s="2" t="n">
-        <v>1.17</v>
+        <v>0.51</v>
       </c>
       <c r="H214" s="2" t="inlineStr">
         <is>
@@ -9261,7 +9261,7 @@
       </c>
       <c r="C215" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #12 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.71s.</t>
+          <t>User executes touch gesture #12 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.1s.</t>
         </is>
       </c>
       <c r="D215" s="2" t="inlineStr">
@@ -9280,7 +9280,7 @@
         </is>
       </c>
       <c r="G215" s="2" t="n">
-        <v>0.71</v>
+        <v>1.1</v>
       </c>
       <c r="H215" s="2" t="inlineStr">
         <is>
@@ -9302,7 +9302,7 @@
       </c>
       <c r="C216" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #13 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.77s.</t>
+          <t>User executes touch gesture #13 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.59s.</t>
         </is>
       </c>
       <c r="D216" s="2" t="inlineStr">
@@ -9321,7 +9321,7 @@
         </is>
       </c>
       <c r="G216" s="2" t="n">
-        <v>0.77</v>
+        <v>0.59</v>
       </c>
       <c r="H216" s="2" t="inlineStr">
         <is>
@@ -9343,7 +9343,7 @@
       </c>
       <c r="C217" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #14 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.64s.</t>
+          <t>User executes touch gesture #14 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.0s.</t>
         </is>
       </c>
       <c r="D217" s="2" t="inlineStr">
@@ -9362,7 +9362,7 @@
         </is>
       </c>
       <c r="G217" s="2" t="n">
-        <v>0.64</v>
+        <v>1</v>
       </c>
       <c r="H217" s="2" t="inlineStr">
         <is>
@@ -9384,7 +9384,7 @@
       </c>
       <c r="C218" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #15 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.38s.</t>
+          <t>User executes touch gesture #15 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.07s.</t>
         </is>
       </c>
       <c r="D218" s="2" t="inlineStr">
@@ -9403,7 +9403,7 @@
         </is>
       </c>
       <c r="G218" s="2" t="n">
-        <v>0.38</v>
+        <v>1.07</v>
       </c>
       <c r="H218" s="2" t="inlineStr">
         <is>
@@ -9425,7 +9425,7 @@
       </c>
       <c r="C219" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #16 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.08s.</t>
+          <t>User executes touch gesture #16 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.03s.</t>
         </is>
       </c>
       <c r="D219" s="2" t="inlineStr">
@@ -9444,7 +9444,7 @@
         </is>
       </c>
       <c r="G219" s="2" t="n">
-        <v>1.08</v>
+        <v>1.03</v>
       </c>
       <c r="H219" s="2" t="inlineStr">
         <is>
@@ -9466,7 +9466,7 @@
       </c>
       <c r="C220" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #17 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.38s.</t>
+          <t>User executes touch gesture #17 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.62s.</t>
         </is>
       </c>
       <c r="D220" s="2" t="inlineStr">
@@ -9485,7 +9485,7 @@
         </is>
       </c>
       <c r="G220" s="2" t="n">
-        <v>0.38</v>
+        <v>0.62</v>
       </c>
       <c r="H220" s="2" t="inlineStr">
         <is>
@@ -9507,7 +9507,7 @@
       </c>
       <c r="C221" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #18 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.36s.</t>
+          <t>User executes touch gesture #18 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.07s.</t>
         </is>
       </c>
       <c r="D221" s="2" t="inlineStr">
@@ -9526,7 +9526,7 @@
         </is>
       </c>
       <c r="G221" s="2" t="n">
-        <v>0.36</v>
+        <v>1.07</v>
       </c>
       <c r="H221" s="2" t="inlineStr">
         <is>
@@ -9548,7 +9548,7 @@
       </c>
       <c r="C222" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #19 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.69s.</t>
+          <t>User executes touch gesture #19 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.59s.</t>
         </is>
       </c>
       <c r="D222" s="2" t="inlineStr">
@@ -9567,7 +9567,7 @@
         </is>
       </c>
       <c r="G222" s="2" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.59</v>
       </c>
       <c r="H222" s="2" t="inlineStr">
         <is>
@@ -9589,7 +9589,7 @@
       </c>
       <c r="C223" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #20 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.62s.</t>
+          <t>User executes touch gesture #20 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.42s.</t>
         </is>
       </c>
       <c r="D223" s="2" t="inlineStr">
@@ -9608,7 +9608,7 @@
         </is>
       </c>
       <c r="G223" s="2" t="n">
-        <v>0.62</v>
+        <v>0.42</v>
       </c>
       <c r="H223" s="2" t="inlineStr">
         <is>
@@ -9630,7 +9630,7 @@
       </c>
       <c r="C224" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #21 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.93s.</t>
+          <t>User executes touch gesture #21 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.44s.</t>
         </is>
       </c>
       <c r="D224" s="2" t="inlineStr">
@@ -9649,7 +9649,7 @@
         </is>
       </c>
       <c r="G224" s="2" t="n">
-        <v>0.93</v>
+        <v>0.44</v>
       </c>
       <c r="H224" s="2" t="inlineStr">
         <is>
@@ -9671,7 +9671,7 @@
       </c>
       <c r="C225" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #22 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.67s.</t>
+          <t>User executes touch gesture #22 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.43s.</t>
         </is>
       </c>
       <c r="D225" s="2" t="inlineStr">
@@ -9690,7 +9690,7 @@
         </is>
       </c>
       <c r="G225" s="2" t="n">
-        <v>0.67</v>
+        <v>0.43</v>
       </c>
       <c r="H225" s="2" t="inlineStr">
         <is>
@@ -9712,7 +9712,7 @@
       </c>
       <c r="C226" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #23 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.99s.</t>
+          <t>User executes touch gesture #23 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.94s.</t>
         </is>
       </c>
       <c r="D226" s="2" t="inlineStr">
@@ -9731,7 +9731,7 @@
         </is>
       </c>
       <c r="G226" s="2" t="n">
-        <v>0.99</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="H226" s="2" t="inlineStr">
         <is>
@@ -9753,7 +9753,7 @@
       </c>
       <c r="C227" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #24 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.43s.</t>
+          <t>User executes touch gesture #24 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.63s.</t>
         </is>
       </c>
       <c r="D227" s="2" t="inlineStr">
@@ -9772,7 +9772,7 @@
         </is>
       </c>
       <c r="G227" s="2" t="n">
-        <v>0.43</v>
+        <v>0.63</v>
       </c>
       <c r="H227" s="2" t="inlineStr">
         <is>
@@ -9794,7 +9794,7 @@
       </c>
       <c r="C228" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #25 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.66s.</t>
+          <t>User executes touch gesture #25 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.56s.</t>
         </is>
       </c>
       <c r="D228" s="2" t="inlineStr">
@@ -9813,7 +9813,7 @@
         </is>
       </c>
       <c r="G228" s="2" t="n">
-        <v>0.66</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="H228" s="2" t="inlineStr">
         <is>
@@ -9835,7 +9835,7 @@
       </c>
       <c r="C229" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #26 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.22s.</t>
+          <t>User executes touch gesture #26 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.56s.</t>
         </is>
       </c>
       <c r="D229" s="2" t="inlineStr">
@@ -9854,7 +9854,7 @@
         </is>
       </c>
       <c r="G229" s="2" t="n">
-        <v>1.22</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="H229" s="2" t="inlineStr">
         <is>
@@ -9876,7 +9876,7 @@
       </c>
       <c r="C230" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #27 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.59s.</t>
+          <t>User executes touch gesture #27 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.85s.</t>
         </is>
       </c>
       <c r="D230" s="2" t="inlineStr">
@@ -9895,7 +9895,7 @@
         </is>
       </c>
       <c r="G230" s="2" t="n">
-        <v>0.59</v>
+        <v>0.85</v>
       </c>
       <c r="H230" s="2" t="inlineStr">
         <is>
@@ -9917,7 +9917,7 @@
       </c>
       <c r="C231" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #28 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.59s.</t>
+          <t>User executes touch gesture #28 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.09s.</t>
         </is>
       </c>
       <c r="D231" s="2" t="inlineStr">
@@ -9936,7 +9936,7 @@
         </is>
       </c>
       <c r="G231" s="2" t="n">
-        <v>0.59</v>
+        <v>1.09</v>
       </c>
       <c r="H231" s="2" t="inlineStr">
         <is>
@@ -9977,7 +9977,7 @@
         </is>
       </c>
       <c r="G232" s="2" t="n">
-        <v>0.65</v>
+        <v>0.59</v>
       </c>
       <c r="H232" s="2" t="inlineStr">
         <is>
@@ -10018,7 +10018,7 @@
         </is>
       </c>
       <c r="G233" s="2" t="n">
-        <v>0.42</v>
+        <v>0.55</v>
       </c>
       <c r="H233" s="2" t="inlineStr">
         <is>
@@ -10059,7 +10059,7 @@
         </is>
       </c>
       <c r="G234" s="2" t="n">
-        <v>0.65</v>
+        <v>0.28</v>
       </c>
       <c r="H234" s="2" t="inlineStr">
         <is>
@@ -10100,7 +10100,7 @@
         </is>
       </c>
       <c r="G235" s="2" t="n">
-        <v>0.29</v>
+        <v>0.57</v>
       </c>
       <c r="H235" s="2" t="inlineStr">
         <is>
@@ -10122,7 +10122,7 @@
       </c>
       <c r="C236" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #1 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.5s.</t>
+          <t>User executes offline storage operation #1 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.52s.</t>
         </is>
       </c>
       <c r="D236" s="2" t="inlineStr">
@@ -10141,7 +10141,7 @@
         </is>
       </c>
       <c r="G236" s="2" t="n">
-        <v>0.5</v>
+        <v>0.52</v>
       </c>
       <c r="H236" s="2" t="inlineStr">
         <is>
@@ -10163,7 +10163,7 @@
       </c>
       <c r="C237" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #2 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.72s.</t>
+          <t>User executes offline storage operation #2 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.49s.</t>
         </is>
       </c>
       <c r="D237" s="2" t="inlineStr">
@@ -10182,7 +10182,7 @@
         </is>
       </c>
       <c r="G237" s="2" t="n">
-        <v>0.72</v>
+        <v>0.49</v>
       </c>
       <c r="H237" s="2" t="inlineStr">
         <is>
@@ -10204,7 +10204,7 @@
       </c>
       <c r="C238" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #3 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.32s.</t>
+          <t>User executes offline storage operation #3 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.45s.</t>
         </is>
       </c>
       <c r="D238" s="2" t="inlineStr">
@@ -10223,7 +10223,7 @@
         </is>
       </c>
       <c r="G238" s="2" t="n">
-        <v>0.32</v>
+        <v>0.45</v>
       </c>
       <c r="H238" s="2" t="inlineStr">
         <is>
@@ -10245,7 +10245,7 @@
       </c>
       <c r="C239" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #4 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.31s.</t>
+          <t>User executes offline storage operation #4 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.41s.</t>
         </is>
       </c>
       <c r="D239" s="2" t="inlineStr">
@@ -10264,7 +10264,7 @@
         </is>
       </c>
       <c r="G239" s="2" t="n">
-        <v>0.31</v>
+        <v>0.41</v>
       </c>
       <c r="H239" s="2" t="inlineStr">
         <is>
@@ -10286,7 +10286,7 @@
       </c>
       <c r="C240" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #5 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.48s.</t>
+          <t>User executes offline storage operation #5 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.54s.</t>
         </is>
       </c>
       <c r="D240" s="2" t="inlineStr">
@@ -10305,7 +10305,7 @@
         </is>
       </c>
       <c r="G240" s="2" t="n">
-        <v>0.48</v>
+        <v>0.54</v>
       </c>
       <c r="H240" s="2" t="inlineStr">
         <is>
@@ -10327,7 +10327,7 @@
       </c>
       <c r="C241" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #6 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.7s.</t>
+          <t>User executes offline storage operation #6 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.3s.</t>
         </is>
       </c>
       <c r="D241" s="2" t="inlineStr">
@@ -10346,7 +10346,7 @@
         </is>
       </c>
       <c r="G241" s="2" t="n">
-        <v>0.7</v>
+        <v>0.3</v>
       </c>
       <c r="H241" s="2" t="inlineStr">
         <is>
@@ -10368,7 +10368,7 @@
       </c>
       <c r="C242" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #7 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.65s.</t>
+          <t>User executes offline storage operation #7 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.52s.</t>
         </is>
       </c>
       <c r="D242" s="2" t="inlineStr">
@@ -10387,7 +10387,7 @@
         </is>
       </c>
       <c r="G242" s="2" t="n">
-        <v>0.65</v>
+        <v>0.52</v>
       </c>
       <c r="H242" s="2" t="inlineStr">
         <is>
@@ -10409,7 +10409,7 @@
       </c>
       <c r="C243" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #8 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.57s.</t>
+          <t>User executes offline storage operation #8 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.47s.</t>
         </is>
       </c>
       <c r="D243" s="2" t="inlineStr">
@@ -10428,7 +10428,7 @@
         </is>
       </c>
       <c r="G243" s="2" t="n">
-        <v>0.57</v>
+        <v>0.47</v>
       </c>
       <c r="H243" s="2" t="inlineStr">
         <is>
@@ -10450,7 +10450,7 @@
       </c>
       <c r="C244" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #9 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.57s.</t>
+          <t>User executes offline storage operation #9 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.3s.</t>
         </is>
       </c>
       <c r="D244" s="2" t="inlineStr">
@@ -10469,7 +10469,7 @@
         </is>
       </c>
       <c r="G244" s="2" t="n">
-        <v>0.57</v>
+        <v>0.3</v>
       </c>
       <c r="H244" s="2" t="inlineStr">
         <is>
@@ -10491,7 +10491,7 @@
       </c>
       <c r="C245" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #10 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.55s.</t>
+          <t>User executes offline storage operation #10 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.27s.</t>
         </is>
       </c>
       <c r="D245" s="2" t="inlineStr">
@@ -10510,7 +10510,7 @@
         </is>
       </c>
       <c r="G245" s="2" t="n">
-        <v>0.55</v>
+        <v>0.27</v>
       </c>
       <c r="H245" s="2" t="inlineStr">
         <is>
@@ -10532,7 +10532,7 @@
       </c>
       <c r="C246" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #11 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.73s.</t>
+          <t>User executes offline storage operation #11 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.57s.</t>
         </is>
       </c>
       <c r="D246" s="2" t="inlineStr">
@@ -10551,7 +10551,7 @@
         </is>
       </c>
       <c r="G246" s="2" t="n">
-        <v>0.73</v>
+        <v>0.57</v>
       </c>
       <c r="H246" s="2" t="inlineStr">
         <is>
@@ -10573,7 +10573,7 @@
       </c>
       <c r="C247" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #12 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.33s.</t>
+          <t>User executes offline storage operation #12 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.54s.</t>
         </is>
       </c>
       <c r="D247" s="2" t="inlineStr">
@@ -10592,7 +10592,7 @@
         </is>
       </c>
       <c r="G247" s="2" t="n">
-        <v>0.33</v>
+        <v>0.54</v>
       </c>
       <c r="H247" s="2" t="inlineStr">
         <is>
@@ -10614,7 +10614,7 @@
       </c>
       <c r="C248" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #13 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.41s.</t>
+          <t>User executes offline storage operation #13 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.53s.</t>
         </is>
       </c>
       <c r="D248" s="2" t="inlineStr">
@@ -10633,7 +10633,7 @@
         </is>
       </c>
       <c r="G248" s="2" t="n">
-        <v>0.41</v>
+        <v>0.53</v>
       </c>
       <c r="H248" s="2" t="inlineStr">
         <is>
@@ -10655,7 +10655,7 @@
       </c>
       <c r="C249" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #14 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.39s.</t>
+          <t>User executes offline storage operation #14 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.27s.</t>
         </is>
       </c>
       <c r="D249" s="2" t="inlineStr">
@@ -10674,7 +10674,7 @@
         </is>
       </c>
       <c r="G249" s="2" t="n">
-        <v>0.39</v>
+        <v>0.27</v>
       </c>
       <c r="H249" s="2" t="inlineStr">
         <is>
@@ -10696,7 +10696,7 @@
       </c>
       <c r="C250" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #15 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.37s.</t>
+          <t>User executes offline storage operation #15 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.49s.</t>
         </is>
       </c>
       <c r="D250" s="2" t="inlineStr">
@@ -10715,7 +10715,7 @@
         </is>
       </c>
       <c r="G250" s="2" t="n">
-        <v>0.37</v>
+        <v>0.49</v>
       </c>
       <c r="H250" s="2" t="inlineStr">
         <is>
@@ -10737,7 +10737,7 @@
       </c>
       <c r="C251" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #16 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.69s.</t>
+          <t>User executes offline storage operation #16 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.5s.</t>
         </is>
       </c>
       <c r="D251" s="2" t="inlineStr">
@@ -10756,7 +10756,7 @@
         </is>
       </c>
       <c r="G251" s="2" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.5</v>
       </c>
       <c r="H251" s="2" t="inlineStr">
         <is>
@@ -10778,7 +10778,7 @@
       </c>
       <c r="C252" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #17 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.53s.</t>
+          <t>User executes offline storage operation #17 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.56s.</t>
         </is>
       </c>
       <c r="D252" s="2" t="inlineStr">
@@ -10797,7 +10797,7 @@
         </is>
       </c>
       <c r="G252" s="2" t="n">
-        <v>0.53</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="H252" s="2" t="inlineStr">
         <is>
@@ -10819,7 +10819,7 @@
       </c>
       <c r="C253" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #18 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.67s.</t>
+          <t>User executes offline storage operation #18 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.62s.</t>
         </is>
       </c>
       <c r="D253" s="2" t="inlineStr">
@@ -10838,7 +10838,7 @@
         </is>
       </c>
       <c r="G253" s="2" t="n">
-        <v>0.67</v>
+        <v>0.62</v>
       </c>
       <c r="H253" s="2" t="inlineStr">
         <is>
@@ -10860,7 +10860,7 @@
       </c>
       <c r="C254" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #19 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.3s.</t>
+          <t>User executes offline storage operation #19 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.25s.</t>
         </is>
       </c>
       <c r="D254" s="2" t="inlineStr">
@@ -10879,7 +10879,7 @@
         </is>
       </c>
       <c r="G254" s="2" t="n">
-        <v>0.3</v>
+        <v>0.25</v>
       </c>
       <c r="H254" s="2" t="inlineStr">
         <is>
@@ -10901,7 +10901,7 @@
       </c>
       <c r="C255" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #20 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.44s.</t>
+          <t>User executes offline storage operation #20 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.66s.</t>
         </is>
       </c>
       <c r="D255" s="2" t="inlineStr">
@@ -10920,7 +10920,7 @@
         </is>
       </c>
       <c r="G255" s="2" t="n">
-        <v>0.44</v>
+        <v>0.66</v>
       </c>
       <c r="H255" s="2" t="inlineStr">
         <is>
@@ -10942,7 +10942,7 @@
       </c>
       <c r="C256" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #21 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.45s.</t>
+          <t>User executes offline storage operation #21 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.61s.</t>
         </is>
       </c>
       <c r="D256" s="2" t="inlineStr">
@@ -10961,7 +10961,7 @@
         </is>
       </c>
       <c r="G256" s="2" t="n">
-        <v>0.45</v>
+        <v>0.61</v>
       </c>
       <c r="H256" s="2" t="inlineStr">
         <is>
@@ -10983,7 +10983,7 @@
       </c>
       <c r="C257" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #22 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.69s.</t>
+          <t>User executes offline storage operation #22 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.48s.</t>
         </is>
       </c>
       <c r="D257" s="2" t="inlineStr">
@@ -11002,7 +11002,7 @@
         </is>
       </c>
       <c r="G257" s="2" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.48</v>
       </c>
       <c r="H257" s="2" t="inlineStr">
         <is>
@@ -11024,7 +11024,7 @@
       </c>
       <c r="C258" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #23 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.58s.</t>
+          <t>User executes offline storage operation #23 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.53s.</t>
         </is>
       </c>
       <c r="D258" s="2" t="inlineStr">
@@ -11043,7 +11043,7 @@
         </is>
       </c>
       <c r="G258" s="2" t="n">
-        <v>0.58</v>
+        <v>0.53</v>
       </c>
       <c r="H258" s="2" t="inlineStr">
         <is>
@@ -11065,7 +11065,7 @@
       </c>
       <c r="C259" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #24 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.35s.</t>
+          <t>User executes offline storage operation #24 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.61s.</t>
         </is>
       </c>
       <c r="D259" s="2" t="inlineStr">
@@ -11084,7 +11084,7 @@
         </is>
       </c>
       <c r="G259" s="2" t="n">
-        <v>0.35</v>
+        <v>0.61</v>
       </c>
       <c r="H259" s="2" t="inlineStr">
         <is>
@@ -11106,7 +11106,7 @@
       </c>
       <c r="C260" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #25 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.64s.</t>
+          <t>User executes offline storage operation #25 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.58s.</t>
         </is>
       </c>
       <c r="D260" s="2" t="inlineStr">
@@ -11125,7 +11125,7 @@
         </is>
       </c>
       <c r="G260" s="2" t="n">
-        <v>0.64</v>
+        <v>0.58</v>
       </c>
       <c r="H260" s="2" t="inlineStr">
         <is>
@@ -11147,7 +11147,7 @@
       </c>
       <c r="C261" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #26 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.69s.</t>
+          <t>User executes offline storage operation #26 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.63s.</t>
         </is>
       </c>
       <c r="D261" s="2" t="inlineStr">
@@ -11166,7 +11166,7 @@
         </is>
       </c>
       <c r="G261" s="2" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.63</v>
       </c>
       <c r="H261" s="2" t="inlineStr">
         <is>
@@ -11188,7 +11188,7 @@
       </c>
       <c r="C262" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #27 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.28s.</t>
+          <t>User executes offline storage operation #27 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.29s.</t>
         </is>
       </c>
       <c r="D262" s="2" t="inlineStr">
@@ -11207,7 +11207,7 @@
         </is>
       </c>
       <c r="G262" s="2" t="n">
-        <v>0.28</v>
+        <v>0.29</v>
       </c>
       <c r="H262" s="2" t="inlineStr">
         <is>
@@ -11229,7 +11229,7 @@
       </c>
       <c r="C263" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #28 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.5s.</t>
+          <t>User executes offline storage operation #28 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.27s.</t>
         </is>
       </c>
       <c r="D263" s="2" t="inlineStr">
@@ -11248,7 +11248,7 @@
         </is>
       </c>
       <c r="G263" s="2" t="n">
-        <v>0.5</v>
+        <v>0.27</v>
       </c>
       <c r="H263" s="2" t="inlineStr">
         <is>
@@ -11270,7 +11270,7 @@
       </c>
       <c r="C264" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #29 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.33s.</t>
+          <t>User executes offline storage operation #29 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.47s.</t>
         </is>
       </c>
       <c r="D264" s="2" t="inlineStr">
@@ -11289,7 +11289,7 @@
         </is>
       </c>
       <c r="G264" s="2" t="n">
-        <v>0.33</v>
+        <v>0.47</v>
       </c>
       <c r="H264" s="2" t="inlineStr">
         <is>
@@ -11311,7 +11311,7 @@
       </c>
       <c r="C265" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #30 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.31s.</t>
+          <t>User executes offline storage operation #30 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.54s.</t>
         </is>
       </c>
       <c r="D265" s="2" t="inlineStr">
@@ -11330,7 +11330,7 @@
         </is>
       </c>
       <c r="G265" s="2" t="n">
-        <v>0.31</v>
+        <v>0.54</v>
       </c>
       <c r="H265" s="2" t="inlineStr">
         <is>
@@ -11352,7 +11352,7 @@
       </c>
       <c r="C266" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #31 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.7s.</t>
+          <t>User executes offline storage operation #31 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.34s.</t>
         </is>
       </c>
       <c r="D266" s="2" t="inlineStr">
@@ -11371,7 +11371,7 @@
         </is>
       </c>
       <c r="G266" s="2" t="n">
-        <v>0.7</v>
+        <v>0.34</v>
       </c>
       <c r="H266" s="2" t="inlineStr">
         <is>
@@ -11412,7 +11412,7 @@
         </is>
       </c>
       <c r="G267" s="2" t="n">
-        <v>0.38</v>
+        <v>0.44</v>
       </c>
       <c r="H267" s="2" t="inlineStr">
         <is>
@@ -11453,7 +11453,7 @@
         </is>
       </c>
       <c r="G268" s="2" t="n">
-        <v>0.59</v>
+        <v>0.35</v>
       </c>
       <c r="H268" s="2" t="inlineStr">
         <is>
@@ -11494,7 +11494,7 @@
         </is>
       </c>
       <c r="G269" s="2" t="n">
-        <v>0.24</v>
+        <v>0.64</v>
       </c>
       <c r="H269" s="2" t="inlineStr">
         <is>
@@ -11535,7 +11535,7 @@
         </is>
       </c>
       <c r="G270" s="2" t="n">
-        <v>0.54</v>
+        <v>0.55</v>
       </c>
       <c r="H270" s="2" t="inlineStr">
         <is>
@@ -11598,7 +11598,7 @@
       </c>
       <c r="C272" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #2 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.46s.</t>
+          <t>User tests layout/memory scenario #2 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.49s.</t>
         </is>
       </c>
       <c r="D272" s="2" t="inlineStr">
@@ -11617,7 +11617,7 @@
         </is>
       </c>
       <c r="G272" s="2" t="n">
-        <v>0.46</v>
+        <v>0.49</v>
       </c>
       <c r="H272" s="2" t="inlineStr">
         <is>
@@ -11639,7 +11639,7 @@
       </c>
       <c r="C273" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #3 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.51s.</t>
+          <t>User tests layout/memory scenario #3 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.52s.</t>
         </is>
       </c>
       <c r="D273" s="2" t="inlineStr">
@@ -11658,7 +11658,7 @@
         </is>
       </c>
       <c r="G273" s="2" t="n">
-        <v>0.51</v>
+        <v>0.52</v>
       </c>
       <c r="H273" s="2" t="inlineStr">
         <is>
@@ -11680,7 +11680,7 @@
       </c>
       <c r="C274" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #4 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.28s.</t>
+          <t>User tests layout/memory scenario #4 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.66s.</t>
         </is>
       </c>
       <c r="D274" s="2" t="inlineStr">
@@ -11699,7 +11699,7 @@
         </is>
       </c>
       <c r="G274" s="2" t="n">
-        <v>0.28</v>
+        <v>0.66</v>
       </c>
       <c r="H274" s="2" t="inlineStr">
         <is>
@@ -11721,7 +11721,7 @@
       </c>
       <c r="C275" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #5 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.36s.</t>
+          <t>User tests layout/memory scenario #5 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.53s.</t>
         </is>
       </c>
       <c r="D275" s="2" t="inlineStr">
@@ -11740,7 +11740,7 @@
         </is>
       </c>
       <c r="G275" s="2" t="n">
-        <v>0.36</v>
+        <v>0.53</v>
       </c>
       <c r="H275" s="2" t="inlineStr">
         <is>
@@ -11762,7 +11762,7 @@
       </c>
       <c r="C276" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #6 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.28s.</t>
+          <t>User tests layout/memory scenario #6 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.33s.</t>
         </is>
       </c>
       <c r="D276" s="2" t="inlineStr">
@@ -11781,7 +11781,7 @@
         </is>
       </c>
       <c r="G276" s="2" t="n">
-        <v>0.28</v>
+        <v>0.33</v>
       </c>
       <c r="H276" s="2" t="inlineStr">
         <is>
@@ -11803,7 +11803,7 @@
       </c>
       <c r="C277" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #7 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.55s.</t>
+          <t>User tests layout/memory scenario #7 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.51s.</t>
         </is>
       </c>
       <c r="D277" s="2" t="inlineStr">
@@ -11822,7 +11822,7 @@
         </is>
       </c>
       <c r="G277" s="2" t="n">
-        <v>0.55</v>
+        <v>0.51</v>
       </c>
       <c r="H277" s="2" t="inlineStr">
         <is>
@@ -11844,7 +11844,7 @@
       </c>
       <c r="C278" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #8 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.33s.</t>
+          <t>User tests layout/memory scenario #8 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.41s.</t>
         </is>
       </c>
       <c r="D278" s="2" t="inlineStr">
@@ -11863,7 +11863,7 @@
         </is>
       </c>
       <c r="G278" s="2" t="n">
-        <v>0.33</v>
+        <v>0.41</v>
       </c>
       <c r="H278" s="2" t="inlineStr">
         <is>
@@ -11885,7 +11885,7 @@
       </c>
       <c r="C279" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #9 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.22s.</t>
+          <t>User tests layout/memory scenario #9 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.56s.</t>
         </is>
       </c>
       <c r="D279" s="2" t="inlineStr">
@@ -11904,7 +11904,7 @@
         </is>
       </c>
       <c r="G279" s="2" t="n">
-        <v>0.22</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="H279" s="2" t="inlineStr">
         <is>
@@ -11926,7 +11926,7 @@
       </c>
       <c r="C280" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #10 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.46s.</t>
+          <t>User tests layout/memory scenario #10 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.35s.</t>
         </is>
       </c>
       <c r="D280" s="2" t="inlineStr">
@@ -11945,7 +11945,7 @@
         </is>
       </c>
       <c r="G280" s="2" t="n">
-        <v>0.46</v>
+        <v>0.35</v>
       </c>
       <c r="H280" s="2" t="inlineStr">
         <is>
@@ -11967,7 +11967,7 @@
       </c>
       <c r="C281" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #11 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.39s.</t>
+          <t>User tests layout/memory scenario #11 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.45s.</t>
         </is>
       </c>
       <c r="D281" s="2" t="inlineStr">
@@ -11986,7 +11986,7 @@
         </is>
       </c>
       <c r="G281" s="2" t="n">
-        <v>0.39</v>
+        <v>0.45</v>
       </c>
       <c r="H281" s="2" t="inlineStr">
         <is>
@@ -12008,7 +12008,7 @@
       </c>
       <c r="C282" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #12 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.42s.</t>
+          <t>User tests layout/memory scenario #12 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.45s.</t>
         </is>
       </c>
       <c r="D282" s="2" t="inlineStr">
@@ -12027,7 +12027,7 @@
         </is>
       </c>
       <c r="G282" s="2" t="n">
-        <v>0.42</v>
+        <v>0.45</v>
       </c>
       <c r="H282" s="2" t="inlineStr">
         <is>
@@ -12049,7 +12049,7 @@
       </c>
       <c r="C283" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #13 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.48s.</t>
+          <t>User tests layout/memory scenario #13 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.67s.</t>
         </is>
       </c>
       <c r="D283" s="2" t="inlineStr">
@@ -12068,7 +12068,7 @@
         </is>
       </c>
       <c r="G283" s="2" t="n">
-        <v>0.48</v>
+        <v>0.67</v>
       </c>
       <c r="H283" s="2" t="inlineStr">
         <is>
@@ -12090,7 +12090,7 @@
       </c>
       <c r="C284" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #14 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.35s.</t>
+          <t>User tests layout/memory scenario #14 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.28s.</t>
         </is>
       </c>
       <c r="D284" s="2" t="inlineStr">
@@ -12109,7 +12109,7 @@
         </is>
       </c>
       <c r="G284" s="2" t="n">
-        <v>0.35</v>
+        <v>0.28</v>
       </c>
       <c r="H284" s="2" t="inlineStr">
         <is>
@@ -12131,7 +12131,7 @@
       </c>
       <c r="C285" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #15 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.48s.</t>
+          <t>User tests layout/memory scenario #15 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.46s.</t>
         </is>
       </c>
       <c r="D285" s="2" t="inlineStr">
@@ -12150,7 +12150,7 @@
         </is>
       </c>
       <c r="G285" s="2" t="n">
-        <v>0.48</v>
+        <v>0.46</v>
       </c>
       <c r="H285" s="2" t="inlineStr">
         <is>
@@ -12172,7 +12172,7 @@
       </c>
       <c r="C286" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #16 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.64s.</t>
+          <t>User tests layout/memory scenario #16 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.33s.</t>
         </is>
       </c>
       <c r="D286" s="2" t="inlineStr">
@@ -12191,7 +12191,7 @@
         </is>
       </c>
       <c r="G286" s="2" t="n">
-        <v>0.64</v>
+        <v>0.33</v>
       </c>
       <c r="H286" s="2" t="inlineStr">
         <is>
@@ -12213,7 +12213,7 @@
       </c>
       <c r="C287" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #17 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.51s.</t>
+          <t>User tests layout/memory scenario #17 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.62s.</t>
         </is>
       </c>
       <c r="D287" s="2" t="inlineStr">
@@ -12232,7 +12232,7 @@
         </is>
       </c>
       <c r="G287" s="2" t="n">
-        <v>0.51</v>
+        <v>0.62</v>
       </c>
       <c r="H287" s="2" t="inlineStr">
         <is>
@@ -12254,7 +12254,7 @@
       </c>
       <c r="C288" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #18 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.42s.</t>
+          <t>User tests layout/memory scenario #18 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.44s.</t>
         </is>
       </c>
       <c r="D288" s="2" t="inlineStr">
@@ -12273,7 +12273,7 @@
         </is>
       </c>
       <c r="G288" s="2" t="n">
-        <v>0.42</v>
+        <v>0.44</v>
       </c>
       <c r="H288" s="2" t="inlineStr">
         <is>
@@ -12295,7 +12295,7 @@
       </c>
       <c r="C289" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #19 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.61s.</t>
+          <t>User tests layout/memory scenario #19 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.44s.</t>
         </is>
       </c>
       <c r="D289" s="2" t="inlineStr">
@@ -12314,7 +12314,7 @@
         </is>
       </c>
       <c r="G289" s="2" t="n">
-        <v>0.61</v>
+        <v>0.44</v>
       </c>
       <c r="H289" s="2" t="inlineStr">
         <is>
@@ -12336,7 +12336,7 @@
       </c>
       <c r="C290" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #20 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.4s.</t>
+          <t>User tests layout/memory scenario #20 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.31s.</t>
         </is>
       </c>
       <c r="D290" s="2" t="inlineStr">
@@ -12355,7 +12355,7 @@
         </is>
       </c>
       <c r="G290" s="2" t="n">
-        <v>0.4</v>
+        <v>0.31</v>
       </c>
       <c r="H290" s="2" t="inlineStr">
         <is>
@@ -12377,7 +12377,7 @@
       </c>
       <c r="C291" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #21 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.28s.</t>
+          <t>User tests layout/memory scenario #21 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.27s.</t>
         </is>
       </c>
       <c r="D291" s="2" t="inlineStr">
@@ -12396,7 +12396,7 @@
         </is>
       </c>
       <c r="G291" s="2" t="n">
-        <v>0.28</v>
+        <v>0.27</v>
       </c>
       <c r="H291" s="2" t="inlineStr">
         <is>
@@ -12418,7 +12418,7 @@
       </c>
       <c r="C292" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #22 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.64s.</t>
+          <t>User tests layout/memory scenario #22 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.67s.</t>
         </is>
       </c>
       <c r="D292" s="2" t="inlineStr">
@@ -12437,7 +12437,7 @@
         </is>
       </c>
       <c r="G292" s="2" t="n">
-        <v>0.64</v>
+        <v>0.67</v>
       </c>
       <c r="H292" s="2" t="inlineStr">
         <is>
@@ -12459,7 +12459,7 @@
       </c>
       <c r="C293" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #23 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.36s.</t>
+          <t>User tests layout/memory scenario #23 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.57s.</t>
         </is>
       </c>
       <c r="D293" s="2" t="inlineStr">
@@ -12478,7 +12478,7 @@
         </is>
       </c>
       <c r="G293" s="2" t="n">
-        <v>0.36</v>
+        <v>0.57</v>
       </c>
       <c r="H293" s="2" t="inlineStr">
         <is>
@@ -12500,7 +12500,7 @@
       </c>
       <c r="C294" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #24 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.31s.</t>
+          <t>User tests layout/memory scenario #24 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.34s.</t>
         </is>
       </c>
       <c r="D294" s="2" t="inlineStr">
@@ -12519,7 +12519,7 @@
         </is>
       </c>
       <c r="G294" s="2" t="n">
-        <v>0.31</v>
+        <v>0.34</v>
       </c>
       <c r="H294" s="2" t="inlineStr">
         <is>
@@ -12541,7 +12541,7 @@
       </c>
       <c r="C295" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #25 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.31s.</t>
+          <t>User tests layout/memory scenario #25 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.47s.</t>
         </is>
       </c>
       <c r="D295" s="2" t="inlineStr">
@@ -12560,7 +12560,7 @@
         </is>
       </c>
       <c r="G295" s="2" t="n">
-        <v>0.31</v>
+        <v>0.47</v>
       </c>
       <c r="H295" s="2" t="inlineStr">
         <is>
@@ -12582,7 +12582,7 @@
       </c>
       <c r="C296" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #26 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.67s.</t>
+          <t>User tests layout/memory scenario #26 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.41s.</t>
         </is>
       </c>
       <c r="D296" s="2" t="inlineStr">
@@ -12601,7 +12601,7 @@
         </is>
       </c>
       <c r="G296" s="2" t="n">
-        <v>0.67</v>
+        <v>0.41</v>
       </c>
       <c r="H296" s="2" t="inlineStr">
         <is>
@@ -12623,7 +12623,7 @@
       </c>
       <c r="C297" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #27 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.28s.</t>
+          <t>User tests layout/memory scenario #27 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.54s.</t>
         </is>
       </c>
       <c r="D297" s="2" t="inlineStr">
@@ -12642,7 +12642,7 @@
         </is>
       </c>
       <c r="G297" s="2" t="n">
-        <v>0.28</v>
+        <v>0.54</v>
       </c>
       <c r="H297" s="2" t="inlineStr">
         <is>
@@ -12664,7 +12664,7 @@
       </c>
       <c r="C298" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #28 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.66s.</t>
+          <t>User tests layout/memory scenario #28 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.64s.</t>
         </is>
       </c>
       <c r="D298" s="2" t="inlineStr">
@@ -12683,7 +12683,7 @@
         </is>
       </c>
       <c r="G298" s="2" t="n">
-        <v>0.66</v>
+        <v>0.64</v>
       </c>
       <c r="H298" s="2" t="inlineStr">
         <is>
@@ -12705,7 +12705,7 @@
       </c>
       <c r="C299" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #29 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.54s.</t>
+          <t>User tests layout/memory scenario #29 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.62s.</t>
         </is>
       </c>
       <c r="D299" s="2" t="inlineStr">
@@ -12724,7 +12724,7 @@
         </is>
       </c>
       <c r="G299" s="2" t="n">
-        <v>0.54</v>
+        <v>0.62</v>
       </c>
       <c r="H299" s="2" t="inlineStr">
         <is>
@@ -12746,7 +12746,7 @@
       </c>
       <c r="C300" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #30 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.26s.</t>
+          <t>User tests layout/memory scenario #30 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.37s.</t>
         </is>
       </c>
       <c r="D300" s="2" t="inlineStr">
@@ -12765,7 +12765,7 @@
         </is>
       </c>
       <c r="G300" s="2" t="n">
-        <v>0.26</v>
+        <v>0.37</v>
       </c>
       <c r="H300" s="2" t="inlineStr">
         <is>
@@ -12787,7 +12787,7 @@
       </c>
       <c r="C301" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #31 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.45s.</t>
+          <t>User tests layout/memory scenario #31 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.46s.</t>
         </is>
       </c>
       <c r="D301" s="2" t="inlineStr">
@@ -12806,7 +12806,7 @@
         </is>
       </c>
       <c r="G301" s="2" t="n">
-        <v>0.45</v>
+        <v>0.46</v>
       </c>
       <c r="H301" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
feat(summary): include prominent SUMMARY branding across load test sheets, headers, and CI summary report
</commit_message>
<xml_diff>
--- a/reports/Mobile_Application_Appium_Test_Report.xlsx
+++ b/reports/Mobile_Application_Appium_Test_Report.xlsx
@@ -547,7 +547,7 @@
         </is>
       </c>
       <c r="G2" s="2" t="n">
-        <v>0.62</v>
+        <v>0.44</v>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
@@ -588,7 +588,7 @@
         </is>
       </c>
       <c r="G3" s="2" t="n">
-        <v>0.77</v>
+        <v>0.68</v>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
@@ -629,7 +629,7 @@
         </is>
       </c>
       <c r="G4" s="2" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.89</v>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
@@ -670,7 +670,7 @@
         </is>
       </c>
       <c r="G5" s="2" t="n">
-        <v>0.36</v>
+        <v>0.84</v>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
@@ -711,7 +711,7 @@
         </is>
       </c>
       <c r="G6" s="2" t="n">
-        <v>0.42</v>
+        <v>0.47</v>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
@@ -752,7 +752,7 @@
         </is>
       </c>
       <c r="G7" s="2" t="n">
-        <v>0.58</v>
+        <v>0.73</v>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
@@ -793,7 +793,7 @@
         </is>
       </c>
       <c r="G8" s="2" t="n">
-        <v>0.45</v>
+        <v>0.61</v>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
@@ -834,7 +834,7 @@
         </is>
       </c>
       <c r="G9" s="2" t="n">
-        <v>0.44</v>
+        <v>0.95</v>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
@@ -875,7 +875,7 @@
         </is>
       </c>
       <c r="G10" s="2" t="n">
-        <v>0.44</v>
+        <v>0.74</v>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
@@ -916,7 +916,7 @@
         </is>
       </c>
       <c r="G11" s="2" t="n">
-        <v>0.7</v>
+        <v>0.48</v>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
@@ -957,7 +957,7 @@
         </is>
       </c>
       <c r="G12" s="2" t="n">
-        <v>0.6</v>
+        <v>0.52</v>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
@@ -998,7 +998,7 @@
         </is>
       </c>
       <c r="G13" s="2" t="n">
-        <v>0.76</v>
+        <v>0.88</v>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
@@ -1039,7 +1039,7 @@
         </is>
       </c>
       <c r="G14" s="2" t="n">
-        <v>0.9</v>
+        <v>0.92</v>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
@@ -1080,7 +1080,7 @@
         </is>
       </c>
       <c r="G15" s="2" t="n">
-        <v>0.75</v>
+        <v>0.78</v>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
@@ -1121,7 +1121,7 @@
         </is>
       </c>
       <c r="G16" s="2" t="n">
-        <v>0.84</v>
+        <v>0.71</v>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
@@ -1203,7 +1203,7 @@
         </is>
       </c>
       <c r="G18" s="2" t="n">
-        <v>0.74</v>
+        <v>0.49</v>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
@@ -1244,7 +1244,7 @@
         </is>
       </c>
       <c r="G19" s="2" t="n">
-        <v>0.82</v>
+        <v>0.39</v>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
@@ -1285,7 +1285,7 @@
         </is>
       </c>
       <c r="G20" s="2" t="n">
-        <v>0.84</v>
+        <v>0.61</v>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
@@ -1326,7 +1326,7 @@
         </is>
       </c>
       <c r="G21" s="2" t="n">
-        <v>0.35</v>
+        <v>0.4</v>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
@@ -1348,7 +1348,7 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #1 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.86s without crashing.</t>
+          <t>User taps Auth action button #1 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.81s without crashing.</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -1367,7 +1367,7 @@
         </is>
       </c>
       <c r="G22" s="2" t="n">
-        <v>0.86</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
@@ -1389,7 +1389,7 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #2 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.42s without crashing.</t>
+          <t>User taps Auth action button #2 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.55s without crashing.</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -1408,7 +1408,7 @@
         </is>
       </c>
       <c r="G23" s="2" t="n">
-        <v>0.42</v>
+        <v>0.55</v>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
@@ -1430,7 +1430,7 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #3 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.5s without crashing.</t>
+          <t>User taps Auth action button #3 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.88s without crashing.</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -1449,7 +1449,7 @@
         </is>
       </c>
       <c r="G24" s="2" t="n">
-        <v>0.5</v>
+        <v>0.88</v>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
@@ -1471,7 +1471,7 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #4 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.65s without crashing.</t>
+          <t>User taps Auth action button #4 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.83s without crashing.</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
@@ -1490,7 +1490,7 @@
         </is>
       </c>
       <c r="G25" s="2" t="n">
-        <v>0.65</v>
+        <v>0.83</v>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
@@ -1512,7 +1512,7 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #5 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.68s without crashing.</t>
+          <t>User taps Auth action button #5 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.72s without crashing.</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -1531,7 +1531,7 @@
         </is>
       </c>
       <c r="G26" s="2" t="n">
-        <v>0.68</v>
+        <v>0.72</v>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
@@ -1553,7 +1553,7 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #6 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.47s without crashing.</t>
+          <t>User taps Auth action button #6 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.89s without crashing.</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
@@ -1572,7 +1572,7 @@
         </is>
       </c>
       <c r="G27" s="2" t="n">
-        <v>0.47</v>
+        <v>0.89</v>
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
@@ -1594,7 +1594,7 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #7 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.88s without crashing.</t>
+          <t>User taps Auth action button #7 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.77s without crashing.</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -1613,7 +1613,7 @@
         </is>
       </c>
       <c r="G28" s="2" t="n">
-        <v>0.88</v>
+        <v>0.77</v>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
@@ -1635,7 +1635,7 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #8 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.54s without crashing.</t>
+          <t>User taps Auth action button #8 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.78s without crashing.</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
@@ -1654,7 +1654,7 @@
         </is>
       </c>
       <c r="G29" s="2" t="n">
-        <v>0.54</v>
+        <v>0.78</v>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
@@ -1676,7 +1676,7 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #9 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.86s without crashing.</t>
+          <t>User taps Auth action button #9 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.78s without crashing.</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -1695,7 +1695,7 @@
         </is>
       </c>
       <c r="G30" s="2" t="n">
-        <v>0.86</v>
+        <v>0.78</v>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
@@ -1717,7 +1717,7 @@
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #10 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.7s without crashing.</t>
+          <t>User taps Auth action button #10 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.82s without crashing.</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
@@ -1736,7 +1736,7 @@
         </is>
       </c>
       <c r="G31" s="2" t="n">
-        <v>0.7</v>
+        <v>0.82</v>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
@@ -1758,7 +1758,7 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #11 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.76s without crashing.</t>
+          <t>User taps Auth action button #11 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.9s without crashing.</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
@@ -1777,7 +1777,7 @@
         </is>
       </c>
       <c r="G32" s="2" t="n">
-        <v>0.76</v>
+        <v>0.9</v>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
@@ -1799,7 +1799,7 @@
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #12 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.68s without crashing.</t>
+          <t>User taps Auth action button #12 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.76s without crashing.</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
@@ -1818,7 +1818,7 @@
         </is>
       </c>
       <c r="G33" s="2" t="n">
-        <v>0.68</v>
+        <v>0.76</v>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
@@ -1840,7 +1840,7 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #13 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.76s without crashing.</t>
+          <t>User taps Auth action button #13 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.65s without crashing.</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -1859,7 +1859,7 @@
         </is>
       </c>
       <c r="G34" s="2" t="n">
-        <v>0.76</v>
+        <v>0.65</v>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
@@ -1881,7 +1881,7 @@
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #14 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.89s without crashing.</t>
+          <t>User taps Auth action button #14 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.59s without crashing.</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
@@ -1900,7 +1900,7 @@
         </is>
       </c>
       <c r="G35" s="2" t="n">
-        <v>0.89</v>
+        <v>0.59</v>
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
@@ -1922,7 +1922,7 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #15 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.87s without crashing.</t>
+          <t>User taps Auth action button #15 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.48s without crashing.</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
@@ -1941,7 +1941,7 @@
         </is>
       </c>
       <c r="G36" s="2" t="n">
-        <v>0.87</v>
+        <v>0.48</v>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
@@ -1963,7 +1963,7 @@
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #16 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.81s without crashing.</t>
+          <t>User taps Auth action button #16 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.43s without crashing.</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
@@ -1982,7 +1982,7 @@
         </is>
       </c>
       <c r="G37" s="2" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.43</v>
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
@@ -2004,7 +2004,7 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #17 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.67s without crashing.</t>
+          <t>User taps Auth action button #17 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.54s without crashing.</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
@@ -2023,7 +2023,7 @@
         </is>
       </c>
       <c r="G38" s="2" t="n">
-        <v>0.67</v>
+        <v>0.54</v>
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
@@ -2045,7 +2045,7 @@
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #18 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.8s without crashing.</t>
+          <t>User taps Auth action button #18 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.6s without crashing.</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
@@ -2064,7 +2064,7 @@
         </is>
       </c>
       <c r="G39" s="2" t="n">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
@@ -2086,7 +2086,7 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #19 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.53s without crashing.</t>
+          <t>User taps Auth action button #19 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.81s without crashing.</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
@@ -2105,7 +2105,7 @@
         </is>
       </c>
       <c r="G40" s="2" t="n">
-        <v>0.53</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
@@ -2127,7 +2127,7 @@
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #20 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.91s without crashing.</t>
+          <t>User taps Auth action button #20 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.46s without crashing.</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
@@ -2146,7 +2146,7 @@
         </is>
       </c>
       <c r="G41" s="2" t="n">
-        <v>0.91</v>
+        <v>0.46</v>
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
@@ -2228,7 +2228,7 @@
         </is>
       </c>
       <c r="G43" s="2" t="n">
-        <v>0.68</v>
+        <v>0.74</v>
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
@@ -2269,7 +2269,7 @@
         </is>
       </c>
       <c r="G44" s="2" t="n">
-        <v>0.75</v>
+        <v>0.64</v>
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
@@ -2310,7 +2310,7 @@
         </is>
       </c>
       <c r="G45" s="2" t="n">
-        <v>0.49</v>
+        <v>0.44</v>
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
@@ -2351,7 +2351,7 @@
         </is>
       </c>
       <c r="G46" s="2" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.61</v>
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
@@ -2392,7 +2392,7 @@
         </is>
       </c>
       <c r="G47" s="2" t="n">
-        <v>0.48</v>
+        <v>0.68</v>
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
@@ -2433,7 +2433,7 @@
         </is>
       </c>
       <c r="G48" s="2" t="n">
-        <v>0.5</v>
+        <v>0.49</v>
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
@@ -2474,7 +2474,7 @@
         </is>
       </c>
       <c r="G49" s="2" t="n">
-        <v>0.43</v>
+        <v>0.5</v>
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
@@ -2515,7 +2515,7 @@
         </is>
       </c>
       <c r="G50" s="2" t="n">
-        <v>0.6</v>
+        <v>0.52</v>
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
@@ -2556,7 +2556,7 @@
         </is>
       </c>
       <c r="G51" s="2" t="n">
-        <v>0.78</v>
+        <v>0.73</v>
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
@@ -2597,7 +2597,7 @@
         </is>
       </c>
       <c r="G52" s="2" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.33</v>
       </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
@@ -2638,7 +2638,7 @@
         </is>
       </c>
       <c r="G53" s="2" t="n">
-        <v>0.36</v>
+        <v>0.42</v>
       </c>
       <c r="H53" s="2" t="inlineStr">
         <is>
@@ -2679,7 +2679,7 @@
         </is>
       </c>
       <c r="G54" s="2" t="n">
-        <v>0.77</v>
+        <v>0.52</v>
       </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
@@ -2720,7 +2720,7 @@
         </is>
       </c>
       <c r="G55" s="2" t="n">
-        <v>0.4</v>
+        <v>0.74</v>
       </c>
       <c r="H55" s="2" t="inlineStr">
         <is>
@@ -2761,7 +2761,7 @@
         </is>
       </c>
       <c r="G56" s="2" t="n">
-        <v>0.48</v>
+        <v>0.85</v>
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
@@ -2783,7 +2783,7 @@
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #1 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.74s.</t>
+          <t>User taps Verification interactive button #1 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.76s.</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
@@ -2802,7 +2802,7 @@
         </is>
       </c>
       <c r="G57" s="2" t="n">
-        <v>0.74</v>
+        <v>0.76</v>
       </c>
       <c r="H57" s="2" t="inlineStr">
         <is>
@@ -2824,7 +2824,7 @@
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #2 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.57s.</t>
+          <t>User taps Verification interactive button #2 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.54s.</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
@@ -2843,7 +2843,7 @@
         </is>
       </c>
       <c r="G58" s="2" t="n">
-        <v>0.57</v>
+        <v>0.54</v>
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
@@ -2865,7 +2865,7 @@
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #3 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.64s.</t>
+          <t>User taps Verification interactive button #3 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.68s.</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
@@ -2884,7 +2884,7 @@
         </is>
       </c>
       <c r="G59" s="2" t="n">
-        <v>0.64</v>
+        <v>0.68</v>
       </c>
       <c r="H59" s="2" t="inlineStr">
         <is>
@@ -2906,7 +2906,7 @@
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #4 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.45s.</t>
+          <t>User taps Verification interactive button #4 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.8s.</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
@@ -2925,7 +2925,7 @@
         </is>
       </c>
       <c r="G60" s="2" t="n">
-        <v>0.45</v>
+        <v>0.8</v>
       </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
@@ -2947,7 +2947,7 @@
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #5 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.84s.</t>
+          <t>User taps Verification interactive button #5 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.76s.</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
@@ -2966,7 +2966,7 @@
         </is>
       </c>
       <c r="G61" s="2" t="n">
-        <v>0.84</v>
+        <v>0.76</v>
       </c>
       <c r="H61" s="2" t="inlineStr">
         <is>
@@ -2988,7 +2988,7 @@
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #6 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.64s.</t>
+          <t>User taps Verification interactive button #6 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.32s.</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
@@ -3007,7 +3007,7 @@
         </is>
       </c>
       <c r="G62" s="2" t="n">
-        <v>0.64</v>
+        <v>0.32</v>
       </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
@@ -3029,7 +3029,7 @@
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #7 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.64s.</t>
+          <t>User taps Verification interactive button #7 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.68s.</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
@@ -3048,7 +3048,7 @@
         </is>
       </c>
       <c r="G63" s="2" t="n">
-        <v>0.64</v>
+        <v>0.68</v>
       </c>
       <c r="H63" s="2" t="inlineStr">
         <is>
@@ -3070,7 +3070,7 @@
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #8 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.49s.</t>
+          <t>User taps Verification interactive button #8 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.46s.</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
@@ -3089,7 +3089,7 @@
         </is>
       </c>
       <c r="G64" s="2" t="n">
-        <v>0.49</v>
+        <v>0.46</v>
       </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
@@ -3111,7 +3111,7 @@
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #9 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.54s.</t>
+          <t>User taps Verification interactive button #9 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.57s.</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
@@ -3130,7 +3130,7 @@
         </is>
       </c>
       <c r="G65" s="2" t="n">
-        <v>0.54</v>
+        <v>0.57</v>
       </c>
       <c r="H65" s="2" t="inlineStr">
         <is>
@@ -3152,7 +3152,7 @@
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #10 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.52s.</t>
+          <t>User taps Verification interactive button #10 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.7s.</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
@@ -3171,7 +3171,7 @@
         </is>
       </c>
       <c r="G66" s="2" t="n">
-        <v>0.52</v>
+        <v>0.7</v>
       </c>
       <c r="H66" s="2" t="inlineStr">
         <is>
@@ -3193,7 +3193,7 @@
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #11 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.6s.</t>
+          <t>User taps Verification interactive button #11 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.49s.</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
@@ -3212,7 +3212,7 @@
         </is>
       </c>
       <c r="G67" s="2" t="n">
-        <v>0.6</v>
+        <v>0.49</v>
       </c>
       <c r="H67" s="2" t="inlineStr">
         <is>
@@ -3234,7 +3234,7 @@
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #12 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.35s.</t>
+          <t>User taps Verification interactive button #12 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.43s.</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
@@ -3253,7 +3253,7 @@
         </is>
       </c>
       <c r="G68" s="2" t="n">
-        <v>0.35</v>
+        <v>0.43</v>
       </c>
       <c r="H68" s="2" t="inlineStr">
         <is>
@@ -3275,7 +3275,7 @@
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #13 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.38s.</t>
+          <t>User taps Verification interactive button #13 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.75s.</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
@@ -3294,7 +3294,7 @@
         </is>
       </c>
       <c r="G69" s="2" t="n">
-        <v>0.38</v>
+        <v>0.75</v>
       </c>
       <c r="H69" s="2" t="inlineStr">
         <is>
@@ -3316,7 +3316,7 @@
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #14 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.56s.</t>
+          <t>User taps Verification interactive button #14 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.78s.</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
@@ -3335,7 +3335,7 @@
         </is>
       </c>
       <c r="G70" s="2" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.78</v>
       </c>
       <c r="H70" s="2" t="inlineStr">
         <is>
@@ -3398,7 +3398,7 @@
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #16 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.78s.</t>
+          <t>User taps Verification interactive button #16 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.57s.</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
@@ -3417,7 +3417,7 @@
         </is>
       </c>
       <c r="G72" s="2" t="n">
-        <v>0.78</v>
+        <v>0.57</v>
       </c>
       <c r="H72" s="2" t="inlineStr">
         <is>
@@ -3439,7 +3439,7 @@
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #17 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.44s.</t>
+          <t>User taps Verification interactive button #17 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.39s.</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr">
@@ -3458,7 +3458,7 @@
         </is>
       </c>
       <c r="G73" s="2" t="n">
-        <v>0.44</v>
+        <v>0.39</v>
       </c>
       <c r="H73" s="2" t="inlineStr">
         <is>
@@ -3480,7 +3480,7 @@
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #18 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.35s.</t>
+          <t>User taps Verification interactive button #18 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.86s.</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
@@ -3499,7 +3499,7 @@
         </is>
       </c>
       <c r="G74" s="2" t="n">
-        <v>0.35</v>
+        <v>0.86</v>
       </c>
       <c r="H74" s="2" t="inlineStr">
         <is>
@@ -3521,7 +3521,7 @@
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #19 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.52s.</t>
+          <t>User taps Verification interactive button #19 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.38s.</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
@@ -3540,7 +3540,7 @@
         </is>
       </c>
       <c r="G75" s="2" t="n">
-        <v>0.52</v>
+        <v>0.38</v>
       </c>
       <c r="H75" s="2" t="inlineStr">
         <is>
@@ -3562,7 +3562,7 @@
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #20 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.68s.</t>
+          <t>User taps Verification interactive button #20 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.42s.</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
@@ -3581,7 +3581,7 @@
         </is>
       </c>
       <c r="G76" s="2" t="n">
-        <v>0.68</v>
+        <v>0.42</v>
       </c>
       <c r="H76" s="2" t="inlineStr">
         <is>
@@ -3603,7 +3603,7 @@
       </c>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #21 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.6s.</t>
+          <t>User taps Verification interactive button #21 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.63s.</t>
         </is>
       </c>
       <c r="D77" s="2" t="inlineStr">
@@ -3622,7 +3622,7 @@
         </is>
       </c>
       <c r="G77" s="2" t="n">
-        <v>0.6</v>
+        <v>0.63</v>
       </c>
       <c r="H77" s="2" t="inlineStr">
         <is>
@@ -3644,7 +3644,7 @@
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #22 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.85s.</t>
+          <t>User taps Verification interactive button #22 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.86s.</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
@@ -3663,7 +3663,7 @@
         </is>
       </c>
       <c r="G78" s="2" t="n">
-        <v>0.85</v>
+        <v>0.86</v>
       </c>
       <c r="H78" s="2" t="inlineStr">
         <is>
@@ -3685,7 +3685,7 @@
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #23 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.85s.</t>
+          <t>User taps Verification interactive button #23 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.76s.</t>
         </is>
       </c>
       <c r="D79" s="2" t="inlineStr">
@@ -3704,7 +3704,7 @@
         </is>
       </c>
       <c r="G79" s="2" t="n">
-        <v>0.85</v>
+        <v>0.76</v>
       </c>
       <c r="H79" s="2" t="inlineStr">
         <is>
@@ -3726,7 +3726,7 @@
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #24 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.37s.</t>
+          <t>User taps Verification interactive button #24 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.43s.</t>
         </is>
       </c>
       <c r="D80" s="2" t="inlineStr">
@@ -3745,7 +3745,7 @@
         </is>
       </c>
       <c r="G80" s="2" t="n">
-        <v>0.37</v>
+        <v>0.43</v>
       </c>
       <c r="H80" s="2" t="inlineStr">
         <is>
@@ -3767,7 +3767,7 @@
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #25 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.35s.</t>
+          <t>User taps Verification interactive button #25 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.48s.</t>
         </is>
       </c>
       <c r="D81" s="2" t="inlineStr">
@@ -3786,7 +3786,7 @@
         </is>
       </c>
       <c r="G81" s="2" t="n">
-        <v>0.35</v>
+        <v>0.48</v>
       </c>
       <c r="H81" s="2" t="inlineStr">
         <is>
@@ -3827,7 +3827,7 @@
         </is>
       </c>
       <c r="G82" s="2" t="n">
-        <v>0.66</v>
+        <v>1.12</v>
       </c>
       <c r="H82" s="2" t="inlineStr">
         <is>
@@ -3868,7 +3868,7 @@
         </is>
       </c>
       <c r="G83" s="2" t="n">
-        <v>1.06</v>
+        <v>0.71</v>
       </c>
       <c r="H83" s="2" t="inlineStr">
         <is>
@@ -3909,7 +3909,7 @@
         </is>
       </c>
       <c r="G84" s="2" t="n">
-        <v>0.88</v>
+        <v>0.79</v>
       </c>
       <c r="H84" s="2" t="inlineStr">
         <is>
@@ -3950,7 +3950,7 @@
         </is>
       </c>
       <c r="G85" s="2" t="n">
-        <v>1.11</v>
+        <v>0.68</v>
       </c>
       <c r="H85" s="2" t="inlineStr">
         <is>
@@ -3991,7 +3991,7 @@
         </is>
       </c>
       <c r="G86" s="2" t="n">
-        <v>0.73</v>
+        <v>0.6</v>
       </c>
       <c r="H86" s="2" t="inlineStr">
         <is>
@@ -4032,7 +4032,7 @@
         </is>
       </c>
       <c r="G87" s="2" t="n">
-        <v>0.53</v>
+        <v>0.86</v>
       </c>
       <c r="H87" s="2" t="inlineStr">
         <is>
@@ -4073,7 +4073,7 @@
         </is>
       </c>
       <c r="G88" s="2" t="n">
-        <v>1.01</v>
+        <v>0.9</v>
       </c>
       <c r="H88" s="2" t="inlineStr">
         <is>
@@ -4114,7 +4114,7 @@
         </is>
       </c>
       <c r="G89" s="2" t="n">
-        <v>0.65</v>
+        <v>0.88</v>
       </c>
       <c r="H89" s="2" t="inlineStr">
         <is>
@@ -4155,7 +4155,7 @@
         </is>
       </c>
       <c r="G90" s="2" t="n">
-        <v>0.62</v>
+        <v>0.5</v>
       </c>
       <c r="H90" s="2" t="inlineStr">
         <is>
@@ -4196,7 +4196,7 @@
         </is>
       </c>
       <c r="G91" s="2" t="n">
-        <v>0.54</v>
+        <v>0.49</v>
       </c>
       <c r="H91" s="2" t="inlineStr">
         <is>
@@ -4237,7 +4237,7 @@
         </is>
       </c>
       <c r="G92" s="2" t="n">
-        <v>0.39</v>
+        <v>0.98</v>
       </c>
       <c r="H92" s="2" t="inlineStr">
         <is>
@@ -4278,7 +4278,7 @@
         </is>
       </c>
       <c r="G93" s="2" t="n">
-        <v>0.54</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="H93" s="2" t="inlineStr">
         <is>
@@ -4319,7 +4319,7 @@
         </is>
       </c>
       <c r="G94" s="2" t="n">
-        <v>0.93</v>
+        <v>1.03</v>
       </c>
       <c r="H94" s="2" t="inlineStr">
         <is>
@@ -4360,7 +4360,7 @@
         </is>
       </c>
       <c r="G95" s="2" t="n">
-        <v>0.57</v>
+        <v>1</v>
       </c>
       <c r="H95" s="2" t="inlineStr">
         <is>
@@ -4401,7 +4401,7 @@
         </is>
       </c>
       <c r="G96" s="2" t="n">
-        <v>0.79</v>
+        <v>0.38</v>
       </c>
       <c r="H96" s="2" t="inlineStr">
         <is>
@@ -4423,7 +4423,7 @@
       </c>
       <c r="C97" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #1 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.5s.</t>
+          <t>User taps Issuance form action button #1 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 1.06s.</t>
         </is>
       </c>
       <c r="D97" s="2" t="inlineStr">
@@ -4442,7 +4442,7 @@
         </is>
       </c>
       <c r="G97" s="2" t="n">
-        <v>0.5</v>
+        <v>1.06</v>
       </c>
       <c r="H97" s="2" t="inlineStr">
         <is>
@@ -4464,7 +4464,7 @@
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #2 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.96s.</t>
+          <t>User taps Issuance form action button #2 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.83s.</t>
         </is>
       </c>
       <c r="D98" s="2" t="inlineStr">
@@ -4483,7 +4483,7 @@
         </is>
       </c>
       <c r="G98" s="2" t="n">
-        <v>0.96</v>
+        <v>0.83</v>
       </c>
       <c r="H98" s="2" t="inlineStr">
         <is>
@@ -4505,7 +4505,7 @@
       </c>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #3 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.77s.</t>
+          <t>User taps Issuance form action button #3 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.47s.</t>
         </is>
       </c>
       <c r="D99" s="2" t="inlineStr">
@@ -4524,7 +4524,7 @@
         </is>
       </c>
       <c r="G99" s="2" t="n">
-        <v>0.77</v>
+        <v>0.47</v>
       </c>
       <c r="H99" s="2" t="inlineStr">
         <is>
@@ -4546,7 +4546,7 @@
       </c>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #4 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.63s.</t>
+          <t>User taps Issuance form action button #4 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.83s.</t>
         </is>
       </c>
       <c r="D100" s="2" t="inlineStr">
@@ -4565,7 +4565,7 @@
         </is>
       </c>
       <c r="G100" s="2" t="n">
-        <v>0.63</v>
+        <v>0.83</v>
       </c>
       <c r="H100" s="2" t="inlineStr">
         <is>
@@ -4587,7 +4587,7 @@
       </c>
       <c r="C101" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #5 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.51s.</t>
+          <t>User taps Issuance form action button #5 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.48s.</t>
         </is>
       </c>
       <c r="D101" s="2" t="inlineStr">
@@ -4606,7 +4606,7 @@
         </is>
       </c>
       <c r="G101" s="2" t="n">
-        <v>0.51</v>
+        <v>0.48</v>
       </c>
       <c r="H101" s="2" t="inlineStr">
         <is>
@@ -4628,7 +4628,7 @@
       </c>
       <c r="C102" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #6 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.42s.</t>
+          <t>User taps Issuance form action button #6 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.65s.</t>
         </is>
       </c>
       <c r="D102" s="2" t="inlineStr">
@@ -4647,7 +4647,7 @@
         </is>
       </c>
       <c r="G102" s="2" t="n">
-        <v>0.42</v>
+        <v>0.65</v>
       </c>
       <c r="H102" s="2" t="inlineStr">
         <is>
@@ -4669,7 +4669,7 @@
       </c>
       <c r="C103" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #7 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.93s.</t>
+          <t>User taps Issuance form action button #7 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.55s.</t>
         </is>
       </c>
       <c r="D103" s="2" t="inlineStr">
@@ -4688,7 +4688,7 @@
         </is>
       </c>
       <c r="G103" s="2" t="n">
-        <v>0.93</v>
+        <v>0.55</v>
       </c>
       <c r="H103" s="2" t="inlineStr">
         <is>
@@ -4710,7 +4710,7 @@
       </c>
       <c r="C104" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #8 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.71s.</t>
+          <t>User taps Issuance form action button #8 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.96s.</t>
         </is>
       </c>
       <c r="D104" s="2" t="inlineStr">
@@ -4729,7 +4729,7 @@
         </is>
       </c>
       <c r="G104" s="2" t="n">
-        <v>0.71</v>
+        <v>0.96</v>
       </c>
       <c r="H104" s="2" t="inlineStr">
         <is>
@@ -4751,7 +4751,7 @@
       </c>
       <c r="C105" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #9 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.87s.</t>
+          <t>User taps Issuance form action button #9 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.63s.</t>
         </is>
       </c>
       <c r="D105" s="2" t="inlineStr">
@@ -4770,7 +4770,7 @@
         </is>
       </c>
       <c r="G105" s="2" t="n">
-        <v>0.87</v>
+        <v>0.63</v>
       </c>
       <c r="H105" s="2" t="inlineStr">
         <is>
@@ -4792,7 +4792,7 @@
       </c>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #10 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 1.05s.</t>
+          <t>User taps Issuance form action button #10 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.92s.</t>
         </is>
       </c>
       <c r="D106" s="2" t="inlineStr">
@@ -4811,7 +4811,7 @@
         </is>
       </c>
       <c r="G106" s="2" t="n">
-        <v>1.05</v>
+        <v>0.92</v>
       </c>
       <c r="H106" s="2" t="inlineStr">
         <is>
@@ -4833,7 +4833,7 @@
       </c>
       <c r="C107" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #11 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.64s.</t>
+          <t>User taps Issuance form action button #11 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.75s.</t>
         </is>
       </c>
       <c r="D107" s="2" t="inlineStr">
@@ -4852,7 +4852,7 @@
         </is>
       </c>
       <c r="G107" s="2" t="n">
-        <v>0.64</v>
+        <v>0.75</v>
       </c>
       <c r="H107" s="2" t="inlineStr">
         <is>
@@ -4874,7 +4874,7 @@
       </c>
       <c r="C108" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #12 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.8s.</t>
+          <t>User taps Issuance form action button #12 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.93s.</t>
         </is>
       </c>
       <c r="D108" s="2" t="inlineStr">
@@ -4893,7 +4893,7 @@
         </is>
       </c>
       <c r="G108" s="2" t="n">
-        <v>0.8</v>
+        <v>0.93</v>
       </c>
       <c r="H108" s="2" t="inlineStr">
         <is>
@@ -4915,7 +4915,7 @@
       </c>
       <c r="C109" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #13 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.52s.</t>
+          <t>User taps Issuance form action button #13 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.65s.</t>
         </is>
       </c>
       <c r="D109" s="2" t="inlineStr">
@@ -4934,7 +4934,7 @@
         </is>
       </c>
       <c r="G109" s="2" t="n">
-        <v>0.52</v>
+        <v>0.65</v>
       </c>
       <c r="H109" s="2" t="inlineStr">
         <is>
@@ -4956,7 +4956,7 @@
       </c>
       <c r="C110" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #14 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 1.12s.</t>
+          <t>User taps Issuance form action button #14 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 1.08s.</t>
         </is>
       </c>
       <c r="D110" s="2" t="inlineStr">
@@ -4975,7 +4975,7 @@
         </is>
       </c>
       <c r="G110" s="2" t="n">
-        <v>1.12</v>
+        <v>1.08</v>
       </c>
       <c r="H110" s="2" t="inlineStr">
         <is>
@@ -4997,7 +4997,7 @@
       </c>
       <c r="C111" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #15 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.78s.</t>
+          <t>User taps Issuance form action button #15 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.38s.</t>
         </is>
       </c>
       <c r="D111" s="2" t="inlineStr">
@@ -5016,7 +5016,7 @@
         </is>
       </c>
       <c r="G111" s="2" t="n">
-        <v>0.78</v>
+        <v>0.38</v>
       </c>
       <c r="H111" s="2" t="inlineStr">
         <is>
@@ -5038,7 +5038,7 @@
       </c>
       <c r="C112" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #16 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.54s.</t>
+          <t>User taps Issuance form action button #16 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.63s.</t>
         </is>
       </c>
       <c r="D112" s="2" t="inlineStr">
@@ -5057,7 +5057,7 @@
         </is>
       </c>
       <c r="G112" s="2" t="n">
-        <v>0.54</v>
+        <v>0.63</v>
       </c>
       <c r="H112" s="2" t="inlineStr">
         <is>
@@ -5079,7 +5079,7 @@
       </c>
       <c r="C113" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #17 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.55s.</t>
+          <t>User taps Issuance form action button #17 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.95s.</t>
         </is>
       </c>
       <c r="D113" s="2" t="inlineStr">
@@ -5098,7 +5098,7 @@
         </is>
       </c>
       <c r="G113" s="2" t="n">
-        <v>0.55</v>
+        <v>0.95</v>
       </c>
       <c r="H113" s="2" t="inlineStr">
         <is>
@@ -5120,7 +5120,7 @@
       </c>
       <c r="C114" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #18 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.4s.</t>
+          <t>User taps Issuance form action button #18 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.68s.</t>
         </is>
       </c>
       <c r="D114" s="2" t="inlineStr">
@@ -5139,7 +5139,7 @@
         </is>
       </c>
       <c r="G114" s="2" t="n">
-        <v>0.4</v>
+        <v>0.68</v>
       </c>
       <c r="H114" s="2" t="inlineStr">
         <is>
@@ -5161,7 +5161,7 @@
       </c>
       <c r="C115" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #19 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.38s.</t>
+          <t>User taps Issuance form action button #19 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.95s.</t>
         </is>
       </c>
       <c r="D115" s="2" t="inlineStr">
@@ -5180,7 +5180,7 @@
         </is>
       </c>
       <c r="G115" s="2" t="n">
-        <v>0.38</v>
+        <v>0.95</v>
       </c>
       <c r="H115" s="2" t="inlineStr">
         <is>
@@ -5202,7 +5202,7 @@
       </c>
       <c r="C116" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #20 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.67s.</t>
+          <t>User taps Issuance form action button #20 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.58s.</t>
         </is>
       </c>
       <c r="D116" s="2" t="inlineStr">
@@ -5221,7 +5221,7 @@
         </is>
       </c>
       <c r="G116" s="2" t="n">
-        <v>0.67</v>
+        <v>0.58</v>
       </c>
       <c r="H116" s="2" t="inlineStr">
         <is>
@@ -5243,7 +5243,7 @@
       </c>
       <c r="C117" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #21 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.66s.</t>
+          <t>User taps Issuance form action button #21 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.98s.</t>
         </is>
       </c>
       <c r="D117" s="2" t="inlineStr">
@@ -5262,7 +5262,7 @@
         </is>
       </c>
       <c r="G117" s="2" t="n">
-        <v>0.66</v>
+        <v>0.98</v>
       </c>
       <c r="H117" s="2" t="inlineStr">
         <is>
@@ -5284,7 +5284,7 @@
       </c>
       <c r="C118" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #22 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 1.11s.</t>
+          <t>User taps Issuance form action button #22 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.51s.</t>
         </is>
       </c>
       <c r="D118" s="2" t="inlineStr">
@@ -5303,7 +5303,7 @@
         </is>
       </c>
       <c r="G118" s="2" t="n">
-        <v>1.11</v>
+        <v>0.51</v>
       </c>
       <c r="H118" s="2" t="inlineStr">
         <is>
@@ -5325,7 +5325,7 @@
       </c>
       <c r="C119" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #23 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 1.01s.</t>
+          <t>User taps Issuance form action button #23 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.45s.</t>
         </is>
       </c>
       <c r="D119" s="2" t="inlineStr">
@@ -5344,7 +5344,7 @@
         </is>
       </c>
       <c r="G119" s="2" t="n">
-        <v>1.01</v>
+        <v>0.45</v>
       </c>
       <c r="H119" s="2" t="inlineStr">
         <is>
@@ -5366,7 +5366,7 @@
       </c>
       <c r="C120" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #24 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.54s.</t>
+          <t>User taps Issuance form action button #24 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.86s.</t>
         </is>
       </c>
       <c r="D120" s="2" t="inlineStr">
@@ -5385,7 +5385,7 @@
         </is>
       </c>
       <c r="G120" s="2" t="n">
-        <v>0.54</v>
+        <v>0.86</v>
       </c>
       <c r="H120" s="2" t="inlineStr">
         <is>
@@ -5407,7 +5407,7 @@
       </c>
       <c r="C121" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #25 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 1.06s.</t>
+          <t>User taps Issuance form action button #25 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.81s.</t>
         </is>
       </c>
       <c r="D121" s="2" t="inlineStr">
@@ -5426,7 +5426,7 @@
         </is>
       </c>
       <c r="G121" s="2" t="n">
-        <v>1.06</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="H121" s="2" t="inlineStr">
         <is>
@@ -5467,7 +5467,7 @@
         </is>
       </c>
       <c r="G122" s="2" t="n">
-        <v>0.4</v>
+        <v>0.65</v>
       </c>
       <c r="H122" s="2" t="inlineStr">
         <is>
@@ -5508,7 +5508,7 @@
         </is>
       </c>
       <c r="G123" s="2" t="n">
-        <v>0.8</v>
+        <v>0.38</v>
       </c>
       <c r="H123" s="2" t="inlineStr">
         <is>
@@ -5549,7 +5549,7 @@
         </is>
       </c>
       <c r="G124" s="2" t="n">
-        <v>0.74</v>
+        <v>0.44</v>
       </c>
       <c r="H124" s="2" t="inlineStr">
         <is>
@@ -5590,7 +5590,7 @@
         </is>
       </c>
       <c r="G125" s="2" t="n">
-        <v>0.73</v>
+        <v>0.58</v>
       </c>
       <c r="H125" s="2" t="inlineStr">
         <is>
@@ -5631,7 +5631,7 @@
         </is>
       </c>
       <c r="G126" s="2" t="n">
-        <v>0.37</v>
+        <v>0.77</v>
       </c>
       <c r="H126" s="2" t="inlineStr">
         <is>
@@ -5672,7 +5672,7 @@
         </is>
       </c>
       <c r="G127" s="2" t="n">
-        <v>0.73</v>
+        <v>0.57</v>
       </c>
       <c r="H127" s="2" t="inlineStr">
         <is>
@@ -5713,7 +5713,7 @@
         </is>
       </c>
       <c r="G128" s="2" t="n">
-        <v>0.7</v>
+        <v>0.35</v>
       </c>
       <c r="H128" s="2" t="inlineStr">
         <is>
@@ -5754,7 +5754,7 @@
         </is>
       </c>
       <c r="G129" s="2" t="n">
-        <v>0.35</v>
+        <v>0.59</v>
       </c>
       <c r="H129" s="2" t="inlineStr">
         <is>
@@ -5795,7 +5795,7 @@
         </is>
       </c>
       <c r="G130" s="2" t="n">
-        <v>0.41</v>
+        <v>0.61</v>
       </c>
       <c r="H130" s="2" t="inlineStr">
         <is>
@@ -5836,7 +5836,7 @@
         </is>
       </c>
       <c r="G131" s="2" t="n">
-        <v>0.42</v>
+        <v>0.49</v>
       </c>
       <c r="H131" s="2" t="inlineStr">
         <is>
@@ -5858,7 +5858,7 @@
       </c>
       <c r="C132" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #1 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.35s.</t>
+          <t>User taps Registry interactive card/button #1 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.5s.</t>
         </is>
       </c>
       <c r="D132" s="2" t="inlineStr">
@@ -5877,7 +5877,7 @@
         </is>
       </c>
       <c r="G132" s="2" t="n">
-        <v>0.35</v>
+        <v>0.5</v>
       </c>
       <c r="H132" s="2" t="inlineStr">
         <is>
@@ -5899,7 +5899,7 @@
       </c>
       <c r="C133" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #2 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.55s.</t>
+          <t>User taps Registry interactive card/button #2 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.6s.</t>
         </is>
       </c>
       <c r="D133" s="2" t="inlineStr">
@@ -5918,7 +5918,7 @@
         </is>
       </c>
       <c r="G133" s="2" t="n">
-        <v>0.55</v>
+        <v>0.6</v>
       </c>
       <c r="H133" s="2" t="inlineStr">
         <is>
@@ -5940,7 +5940,7 @@
       </c>
       <c r="C134" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #3 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.65s.</t>
+          <t>User taps Registry interactive card/button #3 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.47s.</t>
         </is>
       </c>
       <c r="D134" s="2" t="inlineStr">
@@ -5959,7 +5959,7 @@
         </is>
       </c>
       <c r="G134" s="2" t="n">
-        <v>0.65</v>
+        <v>0.47</v>
       </c>
       <c r="H134" s="2" t="inlineStr">
         <is>
@@ -5981,7 +5981,7 @@
       </c>
       <c r="C135" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #4 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.49s.</t>
+          <t>User taps Registry interactive card/button #4 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.37s.</t>
         </is>
       </c>
       <c r="D135" s="2" t="inlineStr">
@@ -6000,7 +6000,7 @@
         </is>
       </c>
       <c r="G135" s="2" t="n">
-        <v>0.49</v>
+        <v>0.37</v>
       </c>
       <c r="H135" s="2" t="inlineStr">
         <is>
@@ -6022,7 +6022,7 @@
       </c>
       <c r="C136" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #5 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.36s.</t>
+          <t>User taps Registry interactive card/button #5 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.66s.</t>
         </is>
       </c>
       <c r="D136" s="2" t="inlineStr">
@@ -6041,7 +6041,7 @@
         </is>
       </c>
       <c r="G136" s="2" t="n">
-        <v>0.36</v>
+        <v>0.66</v>
       </c>
       <c r="H136" s="2" t="inlineStr">
         <is>
@@ -6063,7 +6063,7 @@
       </c>
       <c r="C137" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #6 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.72s.</t>
+          <t>User taps Registry interactive card/button #6 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.47s.</t>
         </is>
       </c>
       <c r="D137" s="2" t="inlineStr">
@@ -6082,7 +6082,7 @@
         </is>
       </c>
       <c r="G137" s="2" t="n">
-        <v>0.72</v>
+        <v>0.47</v>
       </c>
       <c r="H137" s="2" t="inlineStr">
         <is>
@@ -6104,7 +6104,7 @@
       </c>
       <c r="C138" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #7 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.61s.</t>
+          <t>User taps Registry interactive card/button #7 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.64s.</t>
         </is>
       </c>
       <c r="D138" s="2" t="inlineStr">
@@ -6123,7 +6123,7 @@
         </is>
       </c>
       <c r="G138" s="2" t="n">
-        <v>0.61</v>
+        <v>0.64</v>
       </c>
       <c r="H138" s="2" t="inlineStr">
         <is>
@@ -6145,7 +6145,7 @@
       </c>
       <c r="C139" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #8 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.6s.</t>
+          <t>User taps Registry interactive card/button #8 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.54s.</t>
         </is>
       </c>
       <c r="D139" s="2" t="inlineStr">
@@ -6164,7 +6164,7 @@
         </is>
       </c>
       <c r="G139" s="2" t="n">
-        <v>0.6</v>
+        <v>0.54</v>
       </c>
       <c r="H139" s="2" t="inlineStr">
         <is>
@@ -6186,7 +6186,7 @@
       </c>
       <c r="C140" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #9 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.76s.</t>
+          <t>User taps Registry interactive card/button #9 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.53s.</t>
         </is>
       </c>
       <c r="D140" s="2" t="inlineStr">
@@ -6205,7 +6205,7 @@
         </is>
       </c>
       <c r="G140" s="2" t="n">
-        <v>0.76</v>
+        <v>0.53</v>
       </c>
       <c r="H140" s="2" t="inlineStr">
         <is>
@@ -6227,7 +6227,7 @@
       </c>
       <c r="C141" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #10 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.7s.</t>
+          <t>User taps Registry interactive card/button #10 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.76s.</t>
         </is>
       </c>
       <c r="D141" s="2" t="inlineStr">
@@ -6246,7 +6246,7 @@
         </is>
       </c>
       <c r="G141" s="2" t="n">
-        <v>0.7</v>
+        <v>0.76</v>
       </c>
       <c r="H141" s="2" t="inlineStr">
         <is>
@@ -6268,7 +6268,7 @@
       </c>
       <c r="C142" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #11 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.42s.</t>
+          <t>User taps Registry interactive card/button #11 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.76s.</t>
         </is>
       </c>
       <c r="D142" s="2" t="inlineStr">
@@ -6287,7 +6287,7 @@
         </is>
       </c>
       <c r="G142" s="2" t="n">
-        <v>0.42</v>
+        <v>0.76</v>
       </c>
       <c r="H142" s="2" t="inlineStr">
         <is>
@@ -6309,7 +6309,7 @@
       </c>
       <c r="C143" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #12 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.31s.</t>
+          <t>User taps Registry interactive card/button #12 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.36s.</t>
         </is>
       </c>
       <c r="D143" s="2" t="inlineStr">
@@ -6328,7 +6328,7 @@
         </is>
       </c>
       <c r="G143" s="2" t="n">
-        <v>0.31</v>
+        <v>0.36</v>
       </c>
       <c r="H143" s="2" t="inlineStr">
         <is>
@@ -6350,7 +6350,7 @@
       </c>
       <c r="C144" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #13 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.83s.</t>
+          <t>User taps Registry interactive card/button #13 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.77s.</t>
         </is>
       </c>
       <c r="D144" s="2" t="inlineStr">
@@ -6369,7 +6369,7 @@
         </is>
       </c>
       <c r="G144" s="2" t="n">
-        <v>0.83</v>
+        <v>0.77</v>
       </c>
       <c r="H144" s="2" t="inlineStr">
         <is>
@@ -6391,7 +6391,7 @@
       </c>
       <c r="C145" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #14 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.81s.</t>
+          <t>User taps Registry interactive card/button #14 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.61s.</t>
         </is>
       </c>
       <c r="D145" s="2" t="inlineStr">
@@ -6410,7 +6410,7 @@
         </is>
       </c>
       <c r="G145" s="2" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.61</v>
       </c>
       <c r="H145" s="2" t="inlineStr">
         <is>
@@ -6432,7 +6432,7 @@
       </c>
       <c r="C146" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #15 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.45s.</t>
+          <t>User taps Registry interactive card/button #15 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.62s.</t>
         </is>
       </c>
       <c r="D146" s="2" t="inlineStr">
@@ -6451,7 +6451,7 @@
         </is>
       </c>
       <c r="G146" s="2" t="n">
-        <v>0.45</v>
+        <v>0.62</v>
       </c>
       <c r="H146" s="2" t="inlineStr">
         <is>
@@ -6473,7 +6473,7 @@
       </c>
       <c r="C147" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #16 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.58s.</t>
+          <t>User taps Registry interactive card/button #16 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.56s.</t>
         </is>
       </c>
       <c r="D147" s="2" t="inlineStr">
@@ -6492,7 +6492,7 @@
         </is>
       </c>
       <c r="G147" s="2" t="n">
-        <v>0.58</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="H147" s="2" t="inlineStr">
         <is>
@@ -6514,7 +6514,7 @@
       </c>
       <c r="C148" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #17 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.39s.</t>
+          <t>User taps Registry interactive card/button #17 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.33s.</t>
         </is>
       </c>
       <c r="D148" s="2" t="inlineStr">
@@ -6533,7 +6533,7 @@
         </is>
       </c>
       <c r="G148" s="2" t="n">
-        <v>0.39</v>
+        <v>0.33</v>
       </c>
       <c r="H148" s="2" t="inlineStr">
         <is>
@@ -6555,7 +6555,7 @@
       </c>
       <c r="C149" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #18 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.53s.</t>
+          <t>User taps Registry interactive card/button #18 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.32s.</t>
         </is>
       </c>
       <c r="D149" s="2" t="inlineStr">
@@ -6574,7 +6574,7 @@
         </is>
       </c>
       <c r="G149" s="2" t="n">
-        <v>0.53</v>
+        <v>0.32</v>
       </c>
       <c r="H149" s="2" t="inlineStr">
         <is>
@@ -6596,7 +6596,7 @@
       </c>
       <c r="C150" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #19 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.57s.</t>
+          <t>User taps Registry interactive card/button #19 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.84s.</t>
         </is>
       </c>
       <c r="D150" s="2" t="inlineStr">
@@ -6615,7 +6615,7 @@
         </is>
       </c>
       <c r="G150" s="2" t="n">
-        <v>0.57</v>
+        <v>0.84</v>
       </c>
       <c r="H150" s="2" t="inlineStr">
         <is>
@@ -6637,7 +6637,7 @@
       </c>
       <c r="C151" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #20 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.66s.</t>
+          <t>User taps Registry interactive card/button #20 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.48s.</t>
         </is>
       </c>
       <c r="D151" s="2" t="inlineStr">
@@ -6656,7 +6656,7 @@
         </is>
       </c>
       <c r="G151" s="2" t="n">
-        <v>0.66</v>
+        <v>0.48</v>
       </c>
       <c r="H151" s="2" t="inlineStr">
         <is>
@@ -6678,7 +6678,7 @@
       </c>
       <c r="C152" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #21 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.35s.</t>
+          <t>User taps Registry interactive card/button #21 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.62s.</t>
         </is>
       </c>
       <c r="D152" s="2" t="inlineStr">
@@ -6697,7 +6697,7 @@
         </is>
       </c>
       <c r="G152" s="2" t="n">
-        <v>0.35</v>
+        <v>0.62</v>
       </c>
       <c r="H152" s="2" t="inlineStr">
         <is>
@@ -6719,7 +6719,7 @@
       </c>
       <c r="C153" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #22 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.53s.</t>
+          <t>User taps Registry interactive card/button #22 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.74s.</t>
         </is>
       </c>
       <c r="D153" s="2" t="inlineStr">
@@ -6738,7 +6738,7 @@
         </is>
       </c>
       <c r="G153" s="2" t="n">
-        <v>0.53</v>
+        <v>0.74</v>
       </c>
       <c r="H153" s="2" t="inlineStr">
         <is>
@@ -6760,7 +6760,7 @@
       </c>
       <c r="C154" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #23 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.67s.</t>
+          <t>User taps Registry interactive card/button #23 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.74s.</t>
         </is>
       </c>
       <c r="D154" s="2" t="inlineStr">
@@ -6779,7 +6779,7 @@
         </is>
       </c>
       <c r="G154" s="2" t="n">
-        <v>0.67</v>
+        <v>0.74</v>
       </c>
       <c r="H154" s="2" t="inlineStr">
         <is>
@@ -6801,7 +6801,7 @@
       </c>
       <c r="C155" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #24 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.73s.</t>
+          <t>User taps Registry interactive card/button #24 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.66s.</t>
         </is>
       </c>
       <c r="D155" s="2" t="inlineStr">
@@ -6820,7 +6820,7 @@
         </is>
       </c>
       <c r="G155" s="2" t="n">
-        <v>0.73</v>
+        <v>0.66</v>
       </c>
       <c r="H155" s="2" t="inlineStr">
         <is>
@@ -6842,7 +6842,7 @@
       </c>
       <c r="C156" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #25 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.49s.</t>
+          <t>User taps Registry interactive card/button #25 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.53s.</t>
         </is>
       </c>
       <c r="D156" s="2" t="inlineStr">
@@ -6861,7 +6861,7 @@
         </is>
       </c>
       <c r="G156" s="2" t="n">
-        <v>0.49</v>
+        <v>0.53</v>
       </c>
       <c r="H156" s="2" t="inlineStr">
         <is>
@@ -6883,7 +6883,7 @@
       </c>
       <c r="C157" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #26 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.81s.</t>
+          <t>User taps Registry interactive card/button #26 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.43s.</t>
         </is>
       </c>
       <c r="D157" s="2" t="inlineStr">
@@ -6902,7 +6902,7 @@
         </is>
       </c>
       <c r="G157" s="2" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.43</v>
       </c>
       <c r="H157" s="2" t="inlineStr">
         <is>
@@ -6924,7 +6924,7 @@
       </c>
       <c r="C158" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #27 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.3s.</t>
+          <t>User taps Registry interactive card/button #27 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.8s.</t>
         </is>
       </c>
       <c r="D158" s="2" t="inlineStr">
@@ -6943,7 +6943,7 @@
         </is>
       </c>
       <c r="G158" s="2" t="n">
-        <v>0.3</v>
+        <v>0.8</v>
       </c>
       <c r="H158" s="2" t="inlineStr">
         <is>
@@ -6965,7 +6965,7 @@
       </c>
       <c r="C159" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #28 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.7s.</t>
+          <t>User taps Registry interactive card/button #28 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.39s.</t>
         </is>
       </c>
       <c r="D159" s="2" t="inlineStr">
@@ -6984,7 +6984,7 @@
         </is>
       </c>
       <c r="G159" s="2" t="n">
-        <v>0.7</v>
+        <v>0.39</v>
       </c>
       <c r="H159" s="2" t="inlineStr">
         <is>
@@ -7006,7 +7006,7 @@
       </c>
       <c r="C160" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #29 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.69s.</t>
+          <t>User taps Registry interactive card/button #29 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.64s.</t>
         </is>
       </c>
       <c r="D160" s="2" t="inlineStr">
@@ -7025,7 +7025,7 @@
         </is>
       </c>
       <c r="G160" s="2" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.64</v>
       </c>
       <c r="H160" s="2" t="inlineStr">
         <is>
@@ -7047,7 +7047,7 @@
       </c>
       <c r="C161" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #30 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.46s.</t>
+          <t>User taps Registry interactive card/button #30 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.48s.</t>
         </is>
       </c>
       <c r="D161" s="2" t="inlineStr">
@@ -7066,7 +7066,7 @@
         </is>
       </c>
       <c r="G161" s="2" t="n">
-        <v>0.46</v>
+        <v>0.48</v>
       </c>
       <c r="H161" s="2" t="inlineStr">
         <is>
@@ -7107,7 +7107,7 @@
         </is>
       </c>
       <c r="G162" s="2" t="n">
-        <v>0.31</v>
+        <v>0.37</v>
       </c>
       <c r="H162" s="2" t="inlineStr">
         <is>
@@ -7148,7 +7148,7 @@
         </is>
       </c>
       <c r="G163" s="2" t="n">
-        <v>0.44</v>
+        <v>0.66</v>
       </c>
       <c r="H163" s="2" t="inlineStr">
         <is>
@@ -7189,7 +7189,7 @@
         </is>
       </c>
       <c r="G164" s="2" t="n">
-        <v>0.62</v>
+        <v>0.29</v>
       </c>
       <c r="H164" s="2" t="inlineStr">
         <is>
@@ -7230,7 +7230,7 @@
         </is>
       </c>
       <c r="G165" s="2" t="n">
-        <v>0.63</v>
+        <v>0.64</v>
       </c>
       <c r="H165" s="2" t="inlineStr">
         <is>
@@ -7271,7 +7271,7 @@
         </is>
       </c>
       <c r="G166" s="2" t="n">
-        <v>0.49</v>
+        <v>0.7</v>
       </c>
       <c r="H166" s="2" t="inlineStr">
         <is>
@@ -7293,7 +7293,7 @@
       </c>
       <c r="C167" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #1 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.39s.</t>
+          <t>User taps Network diagnostic button #1 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.28s.</t>
         </is>
       </c>
       <c r="D167" s="2" t="inlineStr">
@@ -7312,7 +7312,7 @@
         </is>
       </c>
       <c r="G167" s="2" t="n">
-        <v>0.39</v>
+        <v>0.28</v>
       </c>
       <c r="H167" s="2" t="inlineStr">
         <is>
@@ -7334,7 +7334,7 @@
       </c>
       <c r="C168" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #2 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.31s.</t>
+          <t>User taps Network diagnostic button #2 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.32s.</t>
         </is>
       </c>
       <c r="D168" s="2" t="inlineStr">
@@ -7353,7 +7353,7 @@
         </is>
       </c>
       <c r="G168" s="2" t="n">
-        <v>0.31</v>
+        <v>0.32</v>
       </c>
       <c r="H168" s="2" t="inlineStr">
         <is>
@@ -7375,7 +7375,7 @@
       </c>
       <c r="C169" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #3 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.54s.</t>
+          <t>User taps Network diagnostic button #3 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.73s.</t>
         </is>
       </c>
       <c r="D169" s="2" t="inlineStr">
@@ -7394,7 +7394,7 @@
         </is>
       </c>
       <c r="G169" s="2" t="n">
-        <v>0.54</v>
+        <v>0.73</v>
       </c>
       <c r="H169" s="2" t="inlineStr">
         <is>
@@ -7416,7 +7416,7 @@
       </c>
       <c r="C170" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #4 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.52s.</t>
+          <t>User taps Network diagnostic button #4 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.68s.</t>
         </is>
       </c>
       <c r="D170" s="2" t="inlineStr">
@@ -7435,7 +7435,7 @@
         </is>
       </c>
       <c r="G170" s="2" t="n">
-        <v>0.52</v>
+        <v>0.68</v>
       </c>
       <c r="H170" s="2" t="inlineStr">
         <is>
@@ -7457,7 +7457,7 @@
       </c>
       <c r="C171" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #5 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.3s.</t>
+          <t>User taps Network diagnostic button #5 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.65s.</t>
         </is>
       </c>
       <c r="D171" s="2" t="inlineStr">
@@ -7476,7 +7476,7 @@
         </is>
       </c>
       <c r="G171" s="2" t="n">
-        <v>0.3</v>
+        <v>0.65</v>
       </c>
       <c r="H171" s="2" t="inlineStr">
         <is>
@@ -7498,7 +7498,7 @@
       </c>
       <c r="C172" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #6 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.7s.</t>
+          <t>User taps Network diagnostic button #6 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.3s.</t>
         </is>
       </c>
       <c r="D172" s="2" t="inlineStr">
@@ -7517,7 +7517,7 @@
         </is>
       </c>
       <c r="G172" s="2" t="n">
-        <v>0.7</v>
+        <v>0.3</v>
       </c>
       <c r="H172" s="2" t="inlineStr">
         <is>
@@ -7539,7 +7539,7 @@
       </c>
       <c r="C173" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #7 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.76s.</t>
+          <t>User taps Network diagnostic button #7 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.48s.</t>
         </is>
       </c>
       <c r="D173" s="2" t="inlineStr">
@@ -7558,7 +7558,7 @@
         </is>
       </c>
       <c r="G173" s="2" t="n">
-        <v>0.76</v>
+        <v>0.48</v>
       </c>
       <c r="H173" s="2" t="inlineStr">
         <is>
@@ -7580,7 +7580,7 @@
       </c>
       <c r="C174" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #8 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.38s.</t>
+          <t>User taps Network diagnostic button #8 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.69s.</t>
         </is>
       </c>
       <c r="D174" s="2" t="inlineStr">
@@ -7599,7 +7599,7 @@
         </is>
       </c>
       <c r="G174" s="2" t="n">
-        <v>0.38</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="H174" s="2" t="inlineStr">
         <is>
@@ -7621,7 +7621,7 @@
       </c>
       <c r="C175" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #9 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.56s.</t>
+          <t>User taps Network diagnostic button #9 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.72s.</t>
         </is>
       </c>
       <c r="D175" s="2" t="inlineStr">
@@ -7640,7 +7640,7 @@
         </is>
       </c>
       <c r="G175" s="2" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.72</v>
       </c>
       <c r="H175" s="2" t="inlineStr">
         <is>
@@ -7662,7 +7662,7 @@
       </c>
       <c r="C176" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #10 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.72s.</t>
+          <t>User taps Network diagnostic button #10 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.69s.</t>
         </is>
       </c>
       <c r="D176" s="2" t="inlineStr">
@@ -7681,7 +7681,7 @@
         </is>
       </c>
       <c r="G176" s="2" t="n">
-        <v>0.72</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="H176" s="2" t="inlineStr">
         <is>
@@ -7703,7 +7703,7 @@
       </c>
       <c r="C177" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #11 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.5s.</t>
+          <t>User taps Network diagnostic button #11 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.29s.</t>
         </is>
       </c>
       <c r="D177" s="2" t="inlineStr">
@@ -7722,7 +7722,7 @@
         </is>
       </c>
       <c r="G177" s="2" t="n">
-        <v>0.5</v>
+        <v>0.29</v>
       </c>
       <c r="H177" s="2" t="inlineStr">
         <is>
@@ -7744,7 +7744,7 @@
       </c>
       <c r="C178" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #12 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.39s.</t>
+          <t>User taps Network diagnostic button #12 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.43s.</t>
         </is>
       </c>
       <c r="D178" s="2" t="inlineStr">
@@ -7763,7 +7763,7 @@
         </is>
       </c>
       <c r="G178" s="2" t="n">
-        <v>0.39</v>
+        <v>0.43</v>
       </c>
       <c r="H178" s="2" t="inlineStr">
         <is>
@@ -7785,7 +7785,7 @@
       </c>
       <c r="C179" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #13 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.73s.</t>
+          <t>User taps Network diagnostic button #13 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.54s.</t>
         </is>
       </c>
       <c r="D179" s="2" t="inlineStr">
@@ -7804,7 +7804,7 @@
         </is>
       </c>
       <c r="G179" s="2" t="n">
-        <v>0.73</v>
+        <v>0.54</v>
       </c>
       <c r="H179" s="2" t="inlineStr">
         <is>
@@ -7826,7 +7826,7 @@
       </c>
       <c r="C180" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #14 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.33s.</t>
+          <t>User taps Network diagnostic button #14 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.28s.</t>
         </is>
       </c>
       <c r="D180" s="2" t="inlineStr">
@@ -7845,7 +7845,7 @@
         </is>
       </c>
       <c r="G180" s="2" t="n">
-        <v>0.33</v>
+        <v>0.28</v>
       </c>
       <c r="H180" s="2" t="inlineStr">
         <is>
@@ -7867,7 +7867,7 @@
       </c>
       <c r="C181" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #15 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.42s.</t>
+          <t>User taps Network diagnostic button #15 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.29s.</t>
         </is>
       </c>
       <c r="D181" s="2" t="inlineStr">
@@ -7886,7 +7886,7 @@
         </is>
       </c>
       <c r="G181" s="2" t="n">
-        <v>0.42</v>
+        <v>0.29</v>
       </c>
       <c r="H181" s="2" t="inlineStr">
         <is>
@@ -7908,7 +7908,7 @@
       </c>
       <c r="C182" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #16 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.51s.</t>
+          <t>User taps Network diagnostic button #16 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.67s.</t>
         </is>
       </c>
       <c r="D182" s="2" t="inlineStr">
@@ -7927,7 +7927,7 @@
         </is>
       </c>
       <c r="G182" s="2" t="n">
-        <v>0.51</v>
+        <v>0.67</v>
       </c>
       <c r="H182" s="2" t="inlineStr">
         <is>
@@ -7949,7 +7949,7 @@
       </c>
       <c r="C183" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #17 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.52s.</t>
+          <t>User taps Network diagnostic button #17 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.57s.</t>
         </is>
       </c>
       <c r="D183" s="2" t="inlineStr">
@@ -7968,7 +7968,7 @@
         </is>
       </c>
       <c r="G183" s="2" t="n">
-        <v>0.52</v>
+        <v>0.57</v>
       </c>
       <c r="H183" s="2" t="inlineStr">
         <is>
@@ -7990,7 +7990,7 @@
       </c>
       <c r="C184" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #18 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.54s.</t>
+          <t>User taps Network diagnostic button #18 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.4s.</t>
         </is>
       </c>
       <c r="D184" s="2" t="inlineStr">
@@ -8009,7 +8009,7 @@
         </is>
       </c>
       <c r="G184" s="2" t="n">
-        <v>0.54</v>
+        <v>0.4</v>
       </c>
       <c r="H184" s="2" t="inlineStr">
         <is>
@@ -8031,7 +8031,7 @@
       </c>
       <c r="C185" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #19 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.67s.</t>
+          <t>User taps Network diagnostic button #19 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.35s.</t>
         </is>
       </c>
       <c r="D185" s="2" t="inlineStr">
@@ -8050,7 +8050,7 @@
         </is>
       </c>
       <c r="G185" s="2" t="n">
-        <v>0.67</v>
+        <v>0.35</v>
       </c>
       <c r="H185" s="2" t="inlineStr">
         <is>
@@ -8072,7 +8072,7 @@
       </c>
       <c r="C186" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #20 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.73s.</t>
+          <t>User taps Network diagnostic button #20 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.38s.</t>
         </is>
       </c>
       <c r="D186" s="2" t="inlineStr">
@@ -8091,7 +8091,7 @@
         </is>
       </c>
       <c r="G186" s="2" t="n">
-        <v>0.73</v>
+        <v>0.38</v>
       </c>
       <c r="H186" s="2" t="inlineStr">
         <is>
@@ -8113,7 +8113,7 @@
       </c>
       <c r="C187" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #21 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.33s.</t>
+          <t>User taps Network diagnostic button #21 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.43s.</t>
         </is>
       </c>
       <c r="D187" s="2" t="inlineStr">
@@ -8132,7 +8132,7 @@
         </is>
       </c>
       <c r="G187" s="2" t="n">
-        <v>0.33</v>
+        <v>0.43</v>
       </c>
       <c r="H187" s="2" t="inlineStr">
         <is>
@@ -8154,7 +8154,7 @@
       </c>
       <c r="C188" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #22 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.74s.</t>
+          <t>User taps Network diagnostic button #22 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.44s.</t>
         </is>
       </c>
       <c r="D188" s="2" t="inlineStr">
@@ -8173,7 +8173,7 @@
         </is>
       </c>
       <c r="G188" s="2" t="n">
-        <v>0.74</v>
+        <v>0.44</v>
       </c>
       <c r="H188" s="2" t="inlineStr">
         <is>
@@ -8195,7 +8195,7 @@
       </c>
       <c r="C189" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #23 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.71s.</t>
+          <t>User taps Network diagnostic button #23 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.55s.</t>
         </is>
       </c>
       <c r="D189" s="2" t="inlineStr">
@@ -8214,7 +8214,7 @@
         </is>
       </c>
       <c r="G189" s="2" t="n">
-        <v>0.71</v>
+        <v>0.55</v>
       </c>
       <c r="H189" s="2" t="inlineStr">
         <is>
@@ -8236,7 +8236,7 @@
       </c>
       <c r="C190" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #24 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.59s.</t>
+          <t>User taps Network diagnostic button #24 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.48s.</t>
         </is>
       </c>
       <c r="D190" s="2" t="inlineStr">
@@ -8255,7 +8255,7 @@
         </is>
       </c>
       <c r="G190" s="2" t="n">
-        <v>0.59</v>
+        <v>0.48</v>
       </c>
       <c r="H190" s="2" t="inlineStr">
         <is>
@@ -8277,7 +8277,7 @@
       </c>
       <c r="C191" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #25 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.36s.</t>
+          <t>User taps Network diagnostic button #25 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.44s.</t>
         </is>
       </c>
       <c r="D191" s="2" t="inlineStr">
@@ -8296,7 +8296,7 @@
         </is>
       </c>
       <c r="G191" s="2" t="n">
-        <v>0.36</v>
+        <v>0.44</v>
       </c>
       <c r="H191" s="2" t="inlineStr">
         <is>
@@ -8318,7 +8318,7 @@
       </c>
       <c r="C192" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #26 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.52s.</t>
+          <t>User taps Network diagnostic button #26 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.31s.</t>
         </is>
       </c>
       <c r="D192" s="2" t="inlineStr">
@@ -8337,7 +8337,7 @@
         </is>
       </c>
       <c r="G192" s="2" t="n">
-        <v>0.52</v>
+        <v>0.31</v>
       </c>
       <c r="H192" s="2" t="inlineStr">
         <is>
@@ -8359,7 +8359,7 @@
       </c>
       <c r="C193" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #27 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.28s.</t>
+          <t>User taps Network diagnostic button #27 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.6s.</t>
         </is>
       </c>
       <c r="D193" s="2" t="inlineStr">
@@ -8378,7 +8378,7 @@
         </is>
       </c>
       <c r="G193" s="2" t="n">
-        <v>0.28</v>
+        <v>0.6</v>
       </c>
       <c r="H193" s="2" t="inlineStr">
         <is>
@@ -8400,7 +8400,7 @@
       </c>
       <c r="C194" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #28 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.77s.</t>
+          <t>User taps Network diagnostic button #28 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.3s.</t>
         </is>
       </c>
       <c r="D194" s="2" t="inlineStr">
@@ -8419,7 +8419,7 @@
         </is>
       </c>
       <c r="G194" s="2" t="n">
-        <v>0.77</v>
+        <v>0.3</v>
       </c>
       <c r="H194" s="2" t="inlineStr">
         <is>
@@ -8441,7 +8441,7 @@
       </c>
       <c r="C195" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #29 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.66s.</t>
+          <t>User taps Network diagnostic button #29 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.45s.</t>
         </is>
       </c>
       <c r="D195" s="2" t="inlineStr">
@@ -8460,7 +8460,7 @@
         </is>
       </c>
       <c r="G195" s="2" t="n">
-        <v>0.66</v>
+        <v>0.45</v>
       </c>
       <c r="H195" s="2" t="inlineStr">
         <is>
@@ -8482,7 +8482,7 @@
       </c>
       <c r="C196" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #30 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.38s.</t>
+          <t>User taps Network diagnostic button #30 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.36s.</t>
         </is>
       </c>
       <c r="D196" s="2" t="inlineStr">
@@ -8501,7 +8501,7 @@
         </is>
       </c>
       <c r="G196" s="2" t="n">
-        <v>0.38</v>
+        <v>0.36</v>
       </c>
       <c r="H196" s="2" t="inlineStr">
         <is>
@@ -8542,7 +8542,7 @@
         </is>
       </c>
       <c r="G197" s="2" t="n">
-        <v>0.58</v>
+        <v>0.46</v>
       </c>
       <c r="H197" s="2" t="inlineStr">
         <is>
@@ -8583,7 +8583,7 @@
         </is>
       </c>
       <c r="G198" s="2" t="n">
-        <v>0.79</v>
+        <v>0.63</v>
       </c>
       <c r="H198" s="2" t="inlineStr">
         <is>
@@ -8624,7 +8624,7 @@
         </is>
       </c>
       <c r="G199" s="2" t="n">
-        <v>0.67</v>
+        <v>1.02</v>
       </c>
       <c r="H199" s="2" t="inlineStr">
         <is>
@@ -8665,7 +8665,7 @@
         </is>
       </c>
       <c r="G200" s="2" t="n">
-        <v>0.64</v>
+        <v>0.86</v>
       </c>
       <c r="H200" s="2" t="inlineStr">
         <is>
@@ -8706,7 +8706,7 @@
         </is>
       </c>
       <c r="G201" s="2" t="n">
-        <v>0.36</v>
+        <v>0.52</v>
       </c>
       <c r="H201" s="2" t="inlineStr">
         <is>
@@ -8788,7 +8788,7 @@
         </is>
       </c>
       <c r="G203" s="2" t="n">
-        <v>0.78</v>
+        <v>0.52</v>
       </c>
       <c r="H203" s="2" t="inlineStr">
         <is>
@@ -8810,7 +8810,7 @@
       </c>
       <c r="C204" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #1 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.09s.</t>
+          <t>User executes touch gesture #1 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.22s.</t>
         </is>
       </c>
       <c r="D204" s="2" t="inlineStr">
@@ -8829,7 +8829,7 @@
         </is>
       </c>
       <c r="G204" s="2" t="n">
-        <v>1.09</v>
+        <v>1.22</v>
       </c>
       <c r="H204" s="2" t="inlineStr">
         <is>
@@ -8851,7 +8851,7 @@
       </c>
       <c r="C205" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #2 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.0s.</t>
+          <t>User executes touch gesture #2 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.63s.</t>
         </is>
       </c>
       <c r="D205" s="2" t="inlineStr">
@@ -8870,7 +8870,7 @@
         </is>
       </c>
       <c r="G205" s="2" t="n">
-        <v>1</v>
+        <v>0.63</v>
       </c>
       <c r="H205" s="2" t="inlineStr">
         <is>
@@ -8892,7 +8892,7 @@
       </c>
       <c r="C206" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #3 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.61s.</t>
+          <t>User executes touch gesture #3 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.93s.</t>
         </is>
       </c>
       <c r="D206" s="2" t="inlineStr">
@@ -8911,7 +8911,7 @@
         </is>
       </c>
       <c r="G206" s="2" t="n">
-        <v>0.61</v>
+        <v>0.93</v>
       </c>
       <c r="H206" s="2" t="inlineStr">
         <is>
@@ -8933,7 +8933,7 @@
       </c>
       <c r="C207" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #4 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.47s.</t>
+          <t>User executes touch gesture #4 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.38s.</t>
         </is>
       </c>
       <c r="D207" s="2" t="inlineStr">
@@ -8952,7 +8952,7 @@
         </is>
       </c>
       <c r="G207" s="2" t="n">
-        <v>0.47</v>
+        <v>0.38</v>
       </c>
       <c r="H207" s="2" t="inlineStr">
         <is>
@@ -8974,7 +8974,7 @@
       </c>
       <c r="C208" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #5 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.7s.</t>
+          <t>User executes touch gesture #5 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.0s.</t>
         </is>
       </c>
       <c r="D208" s="2" t="inlineStr">
@@ -8993,7 +8993,7 @@
         </is>
       </c>
       <c r="G208" s="2" t="n">
-        <v>0.7</v>
+        <v>1</v>
       </c>
       <c r="H208" s="2" t="inlineStr">
         <is>
@@ -9015,7 +9015,7 @@
       </c>
       <c r="C209" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #6 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.38s.</t>
+          <t>User executes touch gesture #6 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.24s.</t>
         </is>
       </c>
       <c r="D209" s="2" t="inlineStr">
@@ -9034,7 +9034,7 @@
         </is>
       </c>
       <c r="G209" s="2" t="n">
-        <v>0.38</v>
+        <v>1.24</v>
       </c>
       <c r="H209" s="2" t="inlineStr">
         <is>
@@ -9056,7 +9056,7 @@
       </c>
       <c r="C210" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #7 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.68s.</t>
+          <t>User executes touch gesture #7 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.4s.</t>
         </is>
       </c>
       <c r="D210" s="2" t="inlineStr">
@@ -9075,7 +9075,7 @@
         </is>
       </c>
       <c r="G210" s="2" t="n">
-        <v>0.68</v>
+        <v>0.4</v>
       </c>
       <c r="H210" s="2" t="inlineStr">
         <is>
@@ -9097,7 +9097,7 @@
       </c>
       <c r="C211" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #8 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.91s.</t>
+          <t>User executes touch gesture #8 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.06s.</t>
         </is>
       </c>
       <c r="D211" s="2" t="inlineStr">
@@ -9116,7 +9116,7 @@
         </is>
       </c>
       <c r="G211" s="2" t="n">
-        <v>0.91</v>
+        <v>1.06</v>
       </c>
       <c r="H211" s="2" t="inlineStr">
         <is>
@@ -9138,7 +9138,7 @@
       </c>
       <c r="C212" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #9 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.1s.</t>
+          <t>User executes touch gesture #9 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.18s.</t>
         </is>
       </c>
       <c r="D212" s="2" t="inlineStr">
@@ -9157,7 +9157,7 @@
         </is>
       </c>
       <c r="G212" s="2" t="n">
-        <v>1.1</v>
+        <v>1.18</v>
       </c>
       <c r="H212" s="2" t="inlineStr">
         <is>
@@ -9179,7 +9179,7 @@
       </c>
       <c r="C213" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #10 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.02s.</t>
+          <t>User executes touch gesture #10 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.91s.</t>
         </is>
       </c>
       <c r="D213" s="2" t="inlineStr">
@@ -9198,7 +9198,7 @@
         </is>
       </c>
       <c r="G213" s="2" t="n">
-        <v>1.02</v>
+        <v>0.91</v>
       </c>
       <c r="H213" s="2" t="inlineStr">
         <is>
@@ -9220,7 +9220,7 @@
       </c>
       <c r="C214" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #11 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.51s.</t>
+          <t>User executes touch gesture #11 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.12s.</t>
         </is>
       </c>
       <c r="D214" s="2" t="inlineStr">
@@ -9239,7 +9239,7 @@
         </is>
       </c>
       <c r="G214" s="2" t="n">
-        <v>0.51</v>
+        <v>1.12</v>
       </c>
       <c r="H214" s="2" t="inlineStr">
         <is>
@@ -9261,7 +9261,7 @@
       </c>
       <c r="C215" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #12 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.1s.</t>
+          <t>User executes touch gesture #12 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.03s.</t>
         </is>
       </c>
       <c r="D215" s="2" t="inlineStr">
@@ -9280,7 +9280,7 @@
         </is>
       </c>
       <c r="G215" s="2" t="n">
-        <v>1.1</v>
+        <v>1.03</v>
       </c>
       <c r="H215" s="2" t="inlineStr">
         <is>
@@ -9302,7 +9302,7 @@
       </c>
       <c r="C216" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #13 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.59s.</t>
+          <t>User executes touch gesture #13 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.6s.</t>
         </is>
       </c>
       <c r="D216" s="2" t="inlineStr">
@@ -9321,7 +9321,7 @@
         </is>
       </c>
       <c r="G216" s="2" t="n">
-        <v>0.59</v>
+        <v>0.6</v>
       </c>
       <c r="H216" s="2" t="inlineStr">
         <is>
@@ -9343,7 +9343,7 @@
       </c>
       <c r="C217" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #14 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.0s.</t>
+          <t>User executes touch gesture #14 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.92s.</t>
         </is>
       </c>
       <c r="D217" s="2" t="inlineStr">
@@ -9362,7 +9362,7 @@
         </is>
       </c>
       <c r="G217" s="2" t="n">
-        <v>1</v>
+        <v>0.92</v>
       </c>
       <c r="H217" s="2" t="inlineStr">
         <is>
@@ -9384,7 +9384,7 @@
       </c>
       <c r="C218" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #15 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.07s.</t>
+          <t>User executes touch gesture #15 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.02s.</t>
         </is>
       </c>
       <c r="D218" s="2" t="inlineStr">
@@ -9403,7 +9403,7 @@
         </is>
       </c>
       <c r="G218" s="2" t="n">
-        <v>1.07</v>
+        <v>1.02</v>
       </c>
       <c r="H218" s="2" t="inlineStr">
         <is>
@@ -9425,7 +9425,7 @@
       </c>
       <c r="C219" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #16 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.03s.</t>
+          <t>User executes touch gesture #16 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.63s.</t>
         </is>
       </c>
       <c r="D219" s="2" t="inlineStr">
@@ -9444,7 +9444,7 @@
         </is>
       </c>
       <c r="G219" s="2" t="n">
-        <v>1.03</v>
+        <v>0.63</v>
       </c>
       <c r="H219" s="2" t="inlineStr">
         <is>
@@ -9466,7 +9466,7 @@
       </c>
       <c r="C220" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #17 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.62s.</t>
+          <t>User executes touch gesture #17 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.05s.</t>
         </is>
       </c>
       <c r="D220" s="2" t="inlineStr">
@@ -9485,7 +9485,7 @@
         </is>
       </c>
       <c r="G220" s="2" t="n">
-        <v>0.62</v>
+        <v>1.05</v>
       </c>
       <c r="H220" s="2" t="inlineStr">
         <is>
@@ -9507,7 +9507,7 @@
       </c>
       <c r="C221" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #18 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.07s.</t>
+          <t>User executes touch gesture #18 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.74s.</t>
         </is>
       </c>
       <c r="D221" s="2" t="inlineStr">
@@ -9526,7 +9526,7 @@
         </is>
       </c>
       <c r="G221" s="2" t="n">
-        <v>1.07</v>
+        <v>0.74</v>
       </c>
       <c r="H221" s="2" t="inlineStr">
         <is>
@@ -9548,7 +9548,7 @@
       </c>
       <c r="C222" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #19 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.59s.</t>
+          <t>User executes touch gesture #19 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.13s.</t>
         </is>
       </c>
       <c r="D222" s="2" t="inlineStr">
@@ -9567,7 +9567,7 @@
         </is>
       </c>
       <c r="G222" s="2" t="n">
-        <v>0.59</v>
+        <v>1.13</v>
       </c>
       <c r="H222" s="2" t="inlineStr">
         <is>
@@ -9589,7 +9589,7 @@
       </c>
       <c r="C223" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #20 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.42s.</t>
+          <t>User executes touch gesture #20 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.13s.</t>
         </is>
       </c>
       <c r="D223" s="2" t="inlineStr">
@@ -9608,7 +9608,7 @@
         </is>
       </c>
       <c r="G223" s="2" t="n">
-        <v>0.42</v>
+        <v>1.13</v>
       </c>
       <c r="H223" s="2" t="inlineStr">
         <is>
@@ -9630,7 +9630,7 @@
       </c>
       <c r="C224" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #21 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.44s.</t>
+          <t>User executes touch gesture #21 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.91s.</t>
         </is>
       </c>
       <c r="D224" s="2" t="inlineStr">
@@ -9649,7 +9649,7 @@
         </is>
       </c>
       <c r="G224" s="2" t="n">
-        <v>0.44</v>
+        <v>0.91</v>
       </c>
       <c r="H224" s="2" t="inlineStr">
         <is>
@@ -9671,7 +9671,7 @@
       </c>
       <c r="C225" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #22 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.43s.</t>
+          <t>User executes touch gesture #22 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.54s.</t>
         </is>
       </c>
       <c r="D225" s="2" t="inlineStr">
@@ -9690,7 +9690,7 @@
         </is>
       </c>
       <c r="G225" s="2" t="n">
-        <v>0.43</v>
+        <v>0.54</v>
       </c>
       <c r="H225" s="2" t="inlineStr">
         <is>
@@ -9712,7 +9712,7 @@
       </c>
       <c r="C226" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #23 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.94s.</t>
+          <t>User executes touch gesture #23 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.56s.</t>
         </is>
       </c>
       <c r="D226" s="2" t="inlineStr">
@@ -9731,7 +9731,7 @@
         </is>
       </c>
       <c r="G226" s="2" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="H226" s="2" t="inlineStr">
         <is>
@@ -9753,7 +9753,7 @@
       </c>
       <c r="C227" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #24 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.63s.</t>
+          <t>User executes touch gesture #24 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.51s.</t>
         </is>
       </c>
       <c r="D227" s="2" t="inlineStr">
@@ -9772,7 +9772,7 @@
         </is>
       </c>
       <c r="G227" s="2" t="n">
-        <v>0.63</v>
+        <v>0.51</v>
       </c>
       <c r="H227" s="2" t="inlineStr">
         <is>
@@ -9794,7 +9794,7 @@
       </c>
       <c r="C228" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #25 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.56s.</t>
+          <t>User executes touch gesture #25 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.03s.</t>
         </is>
       </c>
       <c r="D228" s="2" t="inlineStr">
@@ -9813,7 +9813,7 @@
         </is>
       </c>
       <c r="G228" s="2" t="n">
-        <v>0.5600000000000001</v>
+        <v>1.03</v>
       </c>
       <c r="H228" s="2" t="inlineStr">
         <is>
@@ -9835,7 +9835,7 @@
       </c>
       <c r="C229" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #26 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.56s.</t>
+          <t>User executes touch gesture #26 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.59s.</t>
         </is>
       </c>
       <c r="D229" s="2" t="inlineStr">
@@ -9854,7 +9854,7 @@
         </is>
       </c>
       <c r="G229" s="2" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.59</v>
       </c>
       <c r="H229" s="2" t="inlineStr">
         <is>
@@ -9876,7 +9876,7 @@
       </c>
       <c r="C230" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #27 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.85s.</t>
+          <t>User executes touch gesture #27 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.13s.</t>
         </is>
       </c>
       <c r="D230" s="2" t="inlineStr">
@@ -9895,7 +9895,7 @@
         </is>
       </c>
       <c r="G230" s="2" t="n">
-        <v>0.85</v>
+        <v>1.13</v>
       </c>
       <c r="H230" s="2" t="inlineStr">
         <is>
@@ -9917,7 +9917,7 @@
       </c>
       <c r="C231" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #28 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.09s.</t>
+          <t>User executes touch gesture #28 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.81s.</t>
         </is>
       </c>
       <c r="D231" s="2" t="inlineStr">
@@ -9936,7 +9936,7 @@
         </is>
       </c>
       <c r="G231" s="2" t="n">
-        <v>1.09</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="H231" s="2" t="inlineStr">
         <is>
@@ -9977,7 +9977,7 @@
         </is>
       </c>
       <c r="G232" s="2" t="n">
-        <v>0.59</v>
+        <v>0.36</v>
       </c>
       <c r="H232" s="2" t="inlineStr">
         <is>
@@ -10018,7 +10018,7 @@
         </is>
       </c>
       <c r="G233" s="2" t="n">
-        <v>0.55</v>
+        <v>0.68</v>
       </c>
       <c r="H233" s="2" t="inlineStr">
         <is>
@@ -10059,7 +10059,7 @@
         </is>
       </c>
       <c r="G234" s="2" t="n">
-        <v>0.28</v>
+        <v>0.33</v>
       </c>
       <c r="H234" s="2" t="inlineStr">
         <is>
@@ -10100,7 +10100,7 @@
         </is>
       </c>
       <c r="G235" s="2" t="n">
-        <v>0.57</v>
+        <v>0.46</v>
       </c>
       <c r="H235" s="2" t="inlineStr">
         <is>
@@ -10122,7 +10122,7 @@
       </c>
       <c r="C236" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #1 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.52s.</t>
+          <t>User executes offline storage operation #1 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.64s.</t>
         </is>
       </c>
       <c r="D236" s="2" t="inlineStr">
@@ -10141,7 +10141,7 @@
         </is>
       </c>
       <c r="G236" s="2" t="n">
-        <v>0.52</v>
+        <v>0.64</v>
       </c>
       <c r="H236" s="2" t="inlineStr">
         <is>
@@ -10163,7 +10163,7 @@
       </c>
       <c r="C237" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #2 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.49s.</t>
+          <t>User executes offline storage operation #2 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.44s.</t>
         </is>
       </c>
       <c r="D237" s="2" t="inlineStr">
@@ -10182,7 +10182,7 @@
         </is>
       </c>
       <c r="G237" s="2" t="n">
-        <v>0.49</v>
+        <v>0.44</v>
       </c>
       <c r="H237" s="2" t="inlineStr">
         <is>
@@ -10204,7 +10204,7 @@
       </c>
       <c r="C238" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #3 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.45s.</t>
+          <t>User executes offline storage operation #3 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.56s.</t>
         </is>
       </c>
       <c r="D238" s="2" t="inlineStr">
@@ -10223,7 +10223,7 @@
         </is>
       </c>
       <c r="G238" s="2" t="n">
-        <v>0.45</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="H238" s="2" t="inlineStr">
         <is>
@@ -10245,7 +10245,7 @@
       </c>
       <c r="C239" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #4 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.41s.</t>
+          <t>User executes offline storage operation #4 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.55s.</t>
         </is>
       </c>
       <c r="D239" s="2" t="inlineStr">
@@ -10264,7 +10264,7 @@
         </is>
       </c>
       <c r="G239" s="2" t="n">
-        <v>0.41</v>
+        <v>0.55</v>
       </c>
       <c r="H239" s="2" t="inlineStr">
         <is>
@@ -10286,7 +10286,7 @@
       </c>
       <c r="C240" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #5 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.54s.</t>
+          <t>User executes offline storage operation #5 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.42s.</t>
         </is>
       </c>
       <c r="D240" s="2" t="inlineStr">
@@ -10305,7 +10305,7 @@
         </is>
       </c>
       <c r="G240" s="2" t="n">
-        <v>0.54</v>
+        <v>0.42</v>
       </c>
       <c r="H240" s="2" t="inlineStr">
         <is>
@@ -10327,7 +10327,7 @@
       </c>
       <c r="C241" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #6 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.3s.</t>
+          <t>User executes offline storage operation #6 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.27s.</t>
         </is>
       </c>
       <c r="D241" s="2" t="inlineStr">
@@ -10346,7 +10346,7 @@
         </is>
       </c>
       <c r="G241" s="2" t="n">
-        <v>0.3</v>
+        <v>0.27</v>
       </c>
       <c r="H241" s="2" t="inlineStr">
         <is>
@@ -10368,7 +10368,7 @@
       </c>
       <c r="C242" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #7 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.52s.</t>
+          <t>User executes offline storage operation #7 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.69s.</t>
         </is>
       </c>
       <c r="D242" s="2" t="inlineStr">
@@ -10387,7 +10387,7 @@
         </is>
       </c>
       <c r="G242" s="2" t="n">
-        <v>0.52</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="H242" s="2" t="inlineStr">
         <is>
@@ -10409,7 +10409,7 @@
       </c>
       <c r="C243" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #8 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.47s.</t>
+          <t>User executes offline storage operation #8 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.4s.</t>
         </is>
       </c>
       <c r="D243" s="2" t="inlineStr">
@@ -10428,7 +10428,7 @@
         </is>
       </c>
       <c r="G243" s="2" t="n">
-        <v>0.47</v>
+        <v>0.4</v>
       </c>
       <c r="H243" s="2" t="inlineStr">
         <is>
@@ -10450,7 +10450,7 @@
       </c>
       <c r="C244" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #9 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.3s.</t>
+          <t>User executes offline storage operation #9 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.31s.</t>
         </is>
       </c>
       <c r="D244" s="2" t="inlineStr">
@@ -10469,7 +10469,7 @@
         </is>
       </c>
       <c r="G244" s="2" t="n">
-        <v>0.3</v>
+        <v>0.31</v>
       </c>
       <c r="H244" s="2" t="inlineStr">
         <is>
@@ -10491,7 +10491,7 @@
       </c>
       <c r="C245" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #10 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.27s.</t>
+          <t>User executes offline storage operation #10 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.59s.</t>
         </is>
       </c>
       <c r="D245" s="2" t="inlineStr">
@@ -10510,7 +10510,7 @@
         </is>
       </c>
       <c r="G245" s="2" t="n">
-        <v>0.27</v>
+        <v>0.59</v>
       </c>
       <c r="H245" s="2" t="inlineStr">
         <is>
@@ -10532,7 +10532,7 @@
       </c>
       <c r="C246" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #11 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.57s.</t>
+          <t>User executes offline storage operation #11 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.5s.</t>
         </is>
       </c>
       <c r="D246" s="2" t="inlineStr">
@@ -10551,7 +10551,7 @@
         </is>
       </c>
       <c r="G246" s="2" t="n">
-        <v>0.57</v>
+        <v>0.5</v>
       </c>
       <c r="H246" s="2" t="inlineStr">
         <is>
@@ -10573,7 +10573,7 @@
       </c>
       <c r="C247" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #12 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.54s.</t>
+          <t>User executes offline storage operation #12 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.26s.</t>
         </is>
       </c>
       <c r="D247" s="2" t="inlineStr">
@@ -10592,7 +10592,7 @@
         </is>
       </c>
       <c r="G247" s="2" t="n">
-        <v>0.54</v>
+        <v>0.26</v>
       </c>
       <c r="H247" s="2" t="inlineStr">
         <is>
@@ -10614,7 +10614,7 @@
       </c>
       <c r="C248" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #13 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.53s.</t>
+          <t>User executes offline storage operation #13 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.63s.</t>
         </is>
       </c>
       <c r="D248" s="2" t="inlineStr">
@@ -10633,7 +10633,7 @@
         </is>
       </c>
       <c r="G248" s="2" t="n">
-        <v>0.53</v>
+        <v>0.63</v>
       </c>
       <c r="H248" s="2" t="inlineStr">
         <is>
@@ -10655,7 +10655,7 @@
       </c>
       <c r="C249" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #14 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.27s.</t>
+          <t>User executes offline storage operation #14 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.68s.</t>
         </is>
       </c>
       <c r="D249" s="2" t="inlineStr">
@@ -10674,7 +10674,7 @@
         </is>
       </c>
       <c r="G249" s="2" t="n">
-        <v>0.27</v>
+        <v>0.68</v>
       </c>
       <c r="H249" s="2" t="inlineStr">
         <is>
@@ -10696,7 +10696,7 @@
       </c>
       <c r="C250" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #15 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.49s.</t>
+          <t>User executes offline storage operation #15 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.52s.</t>
         </is>
       </c>
       <c r="D250" s="2" t="inlineStr">
@@ -10715,7 +10715,7 @@
         </is>
       </c>
       <c r="G250" s="2" t="n">
-        <v>0.49</v>
+        <v>0.52</v>
       </c>
       <c r="H250" s="2" t="inlineStr">
         <is>
@@ -10737,7 +10737,7 @@
       </c>
       <c r="C251" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #16 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.5s.</t>
+          <t>User executes offline storage operation #16 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.46s.</t>
         </is>
       </c>
       <c r="D251" s="2" t="inlineStr">
@@ -10756,7 +10756,7 @@
         </is>
       </c>
       <c r="G251" s="2" t="n">
-        <v>0.5</v>
+        <v>0.46</v>
       </c>
       <c r="H251" s="2" t="inlineStr">
         <is>
@@ -10778,7 +10778,7 @@
       </c>
       <c r="C252" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #17 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.56s.</t>
+          <t>User executes offline storage operation #17 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.47s.</t>
         </is>
       </c>
       <c r="D252" s="2" t="inlineStr">
@@ -10797,7 +10797,7 @@
         </is>
       </c>
       <c r="G252" s="2" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.47</v>
       </c>
       <c r="H252" s="2" t="inlineStr">
         <is>
@@ -10819,7 +10819,7 @@
       </c>
       <c r="C253" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #18 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.62s.</t>
+          <t>User executes offline storage operation #18 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.6s.</t>
         </is>
       </c>
       <c r="D253" s="2" t="inlineStr">
@@ -10838,7 +10838,7 @@
         </is>
       </c>
       <c r="G253" s="2" t="n">
-        <v>0.62</v>
+        <v>0.6</v>
       </c>
       <c r="H253" s="2" t="inlineStr">
         <is>
@@ -10860,7 +10860,7 @@
       </c>
       <c r="C254" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #19 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.25s.</t>
+          <t>User executes offline storage operation #19 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.32s.</t>
         </is>
       </c>
       <c r="D254" s="2" t="inlineStr">
@@ -10879,7 +10879,7 @@
         </is>
       </c>
       <c r="G254" s="2" t="n">
-        <v>0.25</v>
+        <v>0.32</v>
       </c>
       <c r="H254" s="2" t="inlineStr">
         <is>
@@ -10901,7 +10901,7 @@
       </c>
       <c r="C255" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #20 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.66s.</t>
+          <t>User executes offline storage operation #20 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.44s.</t>
         </is>
       </c>
       <c r="D255" s="2" t="inlineStr">
@@ -10920,7 +10920,7 @@
         </is>
       </c>
       <c r="G255" s="2" t="n">
-        <v>0.66</v>
+        <v>0.44</v>
       </c>
       <c r="H255" s="2" t="inlineStr">
         <is>
@@ -10942,7 +10942,7 @@
       </c>
       <c r="C256" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #21 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.61s.</t>
+          <t>User executes offline storage operation #21 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.67s.</t>
         </is>
       </c>
       <c r="D256" s="2" t="inlineStr">
@@ -10961,7 +10961,7 @@
         </is>
       </c>
       <c r="G256" s="2" t="n">
-        <v>0.61</v>
+        <v>0.67</v>
       </c>
       <c r="H256" s="2" t="inlineStr">
         <is>
@@ -10983,7 +10983,7 @@
       </c>
       <c r="C257" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #22 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.48s.</t>
+          <t>User executes offline storage operation #22 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.63s.</t>
         </is>
       </c>
       <c r="D257" s="2" t="inlineStr">
@@ -11002,7 +11002,7 @@
         </is>
       </c>
       <c r="G257" s="2" t="n">
-        <v>0.48</v>
+        <v>0.63</v>
       </c>
       <c r="H257" s="2" t="inlineStr">
         <is>
@@ -11024,7 +11024,7 @@
       </c>
       <c r="C258" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #23 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.53s.</t>
+          <t>User executes offline storage operation #23 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.27s.</t>
         </is>
       </c>
       <c r="D258" s="2" t="inlineStr">
@@ -11043,7 +11043,7 @@
         </is>
       </c>
       <c r="G258" s="2" t="n">
-        <v>0.53</v>
+        <v>0.27</v>
       </c>
       <c r="H258" s="2" t="inlineStr">
         <is>
@@ -11065,7 +11065,7 @@
       </c>
       <c r="C259" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #24 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.61s.</t>
+          <t>User executes offline storage operation #24 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.52s.</t>
         </is>
       </c>
       <c r="D259" s="2" t="inlineStr">
@@ -11084,7 +11084,7 @@
         </is>
       </c>
       <c r="G259" s="2" t="n">
-        <v>0.61</v>
+        <v>0.52</v>
       </c>
       <c r="H259" s="2" t="inlineStr">
         <is>
@@ -11106,7 +11106,7 @@
       </c>
       <c r="C260" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #25 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.58s.</t>
+          <t>User executes offline storage operation #25 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.27s.</t>
         </is>
       </c>
       <c r="D260" s="2" t="inlineStr">
@@ -11125,7 +11125,7 @@
         </is>
       </c>
       <c r="G260" s="2" t="n">
-        <v>0.58</v>
+        <v>0.27</v>
       </c>
       <c r="H260" s="2" t="inlineStr">
         <is>
@@ -11147,7 +11147,7 @@
       </c>
       <c r="C261" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #26 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.63s.</t>
+          <t>User executes offline storage operation #26 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.44s.</t>
         </is>
       </c>
       <c r="D261" s="2" t="inlineStr">
@@ -11166,7 +11166,7 @@
         </is>
       </c>
       <c r="G261" s="2" t="n">
-        <v>0.63</v>
+        <v>0.44</v>
       </c>
       <c r="H261" s="2" t="inlineStr">
         <is>
@@ -11188,7 +11188,7 @@
       </c>
       <c r="C262" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #27 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.29s.</t>
+          <t>User executes offline storage operation #27 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.43s.</t>
         </is>
       </c>
       <c r="D262" s="2" t="inlineStr">
@@ -11207,7 +11207,7 @@
         </is>
       </c>
       <c r="G262" s="2" t="n">
-        <v>0.29</v>
+        <v>0.43</v>
       </c>
       <c r="H262" s="2" t="inlineStr">
         <is>
@@ -11229,7 +11229,7 @@
       </c>
       <c r="C263" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #28 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.27s.</t>
+          <t>User executes offline storage operation #28 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.48s.</t>
         </is>
       </c>
       <c r="D263" s="2" t="inlineStr">
@@ -11248,7 +11248,7 @@
         </is>
       </c>
       <c r="G263" s="2" t="n">
-        <v>0.27</v>
+        <v>0.48</v>
       </c>
       <c r="H263" s="2" t="inlineStr">
         <is>
@@ -11270,7 +11270,7 @@
       </c>
       <c r="C264" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #29 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.47s.</t>
+          <t>User executes offline storage operation #29 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.32s.</t>
         </is>
       </c>
       <c r="D264" s="2" t="inlineStr">
@@ -11289,7 +11289,7 @@
         </is>
       </c>
       <c r="G264" s="2" t="n">
-        <v>0.47</v>
+        <v>0.32</v>
       </c>
       <c r="H264" s="2" t="inlineStr">
         <is>
@@ -11311,7 +11311,7 @@
       </c>
       <c r="C265" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #30 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.54s.</t>
+          <t>User executes offline storage operation #30 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.64s.</t>
         </is>
       </c>
       <c r="D265" s="2" t="inlineStr">
@@ -11330,7 +11330,7 @@
         </is>
       </c>
       <c r="G265" s="2" t="n">
-        <v>0.54</v>
+        <v>0.64</v>
       </c>
       <c r="H265" s="2" t="inlineStr">
         <is>
@@ -11352,7 +11352,7 @@
       </c>
       <c r="C266" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #31 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.34s.</t>
+          <t>User executes offline storage operation #31 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.41s.</t>
         </is>
       </c>
       <c r="D266" s="2" t="inlineStr">
@@ -11371,7 +11371,7 @@
         </is>
       </c>
       <c r="G266" s="2" t="n">
-        <v>0.34</v>
+        <v>0.41</v>
       </c>
       <c r="H266" s="2" t="inlineStr">
         <is>
@@ -11412,7 +11412,7 @@
         </is>
       </c>
       <c r="G267" s="2" t="n">
-        <v>0.44</v>
+        <v>0.38</v>
       </c>
       <c r="H267" s="2" t="inlineStr">
         <is>
@@ -11453,7 +11453,7 @@
         </is>
       </c>
       <c r="G268" s="2" t="n">
-        <v>0.35</v>
+        <v>0.39</v>
       </c>
       <c r="H268" s="2" t="inlineStr">
         <is>
@@ -11494,7 +11494,7 @@
         </is>
       </c>
       <c r="G269" s="2" t="n">
-        <v>0.64</v>
+        <v>0.22</v>
       </c>
       <c r="H269" s="2" t="inlineStr">
         <is>
@@ -11535,7 +11535,7 @@
         </is>
       </c>
       <c r="G270" s="2" t="n">
-        <v>0.55</v>
+        <v>0.42</v>
       </c>
       <c r="H270" s="2" t="inlineStr">
         <is>
@@ -11557,7 +11557,7 @@
       </c>
       <c r="C271" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #1 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.55s.</t>
+          <t>User tests layout/memory scenario #1 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.59s.</t>
         </is>
       </c>
       <c r="D271" s="2" t="inlineStr">
@@ -11576,7 +11576,7 @@
         </is>
       </c>
       <c r="G271" s="2" t="n">
-        <v>0.55</v>
+        <v>0.59</v>
       </c>
       <c r="H271" s="2" t="inlineStr">
         <is>
@@ -11598,7 +11598,7 @@
       </c>
       <c r="C272" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #2 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.49s.</t>
+          <t>User tests layout/memory scenario #2 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.55s.</t>
         </is>
       </c>
       <c r="D272" s="2" t="inlineStr">
@@ -11617,7 +11617,7 @@
         </is>
       </c>
       <c r="G272" s="2" t="n">
-        <v>0.49</v>
+        <v>0.55</v>
       </c>
       <c r="H272" s="2" t="inlineStr">
         <is>
@@ -11639,7 +11639,7 @@
       </c>
       <c r="C273" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #3 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.52s.</t>
+          <t>User tests layout/memory scenario #3 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.3s.</t>
         </is>
       </c>
       <c r="D273" s="2" t="inlineStr">
@@ -11658,7 +11658,7 @@
         </is>
       </c>
       <c r="G273" s="2" t="n">
-        <v>0.52</v>
+        <v>0.3</v>
       </c>
       <c r="H273" s="2" t="inlineStr">
         <is>
@@ -11680,7 +11680,7 @@
       </c>
       <c r="C274" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #4 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.66s.</t>
+          <t>User tests layout/memory scenario #4 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.46s.</t>
         </is>
       </c>
       <c r="D274" s="2" t="inlineStr">
@@ -11699,7 +11699,7 @@
         </is>
       </c>
       <c r="G274" s="2" t="n">
-        <v>0.66</v>
+        <v>0.46</v>
       </c>
       <c r="H274" s="2" t="inlineStr">
         <is>
@@ -11721,7 +11721,7 @@
       </c>
       <c r="C275" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #5 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.53s.</t>
+          <t>User tests layout/memory scenario #5 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.46s.</t>
         </is>
       </c>
       <c r="D275" s="2" t="inlineStr">
@@ -11740,7 +11740,7 @@
         </is>
       </c>
       <c r="G275" s="2" t="n">
-        <v>0.53</v>
+        <v>0.46</v>
       </c>
       <c r="H275" s="2" t="inlineStr">
         <is>
@@ -11762,7 +11762,7 @@
       </c>
       <c r="C276" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #6 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.33s.</t>
+          <t>User tests layout/memory scenario #6 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.62s.</t>
         </is>
       </c>
       <c r="D276" s="2" t="inlineStr">
@@ -11781,7 +11781,7 @@
         </is>
       </c>
       <c r="G276" s="2" t="n">
-        <v>0.33</v>
+        <v>0.62</v>
       </c>
       <c r="H276" s="2" t="inlineStr">
         <is>
@@ -11803,7 +11803,7 @@
       </c>
       <c r="C277" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #7 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.51s.</t>
+          <t>User tests layout/memory scenario #7 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.45s.</t>
         </is>
       </c>
       <c r="D277" s="2" t="inlineStr">
@@ -11822,7 +11822,7 @@
         </is>
       </c>
       <c r="G277" s="2" t="n">
-        <v>0.51</v>
+        <v>0.45</v>
       </c>
       <c r="H277" s="2" t="inlineStr">
         <is>
@@ -11844,7 +11844,7 @@
       </c>
       <c r="C278" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #8 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.41s.</t>
+          <t>User tests layout/memory scenario #8 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.42s.</t>
         </is>
       </c>
       <c r="D278" s="2" t="inlineStr">
@@ -11863,7 +11863,7 @@
         </is>
       </c>
       <c r="G278" s="2" t="n">
-        <v>0.41</v>
+        <v>0.42</v>
       </c>
       <c r="H278" s="2" t="inlineStr">
         <is>
@@ -11885,7 +11885,7 @@
       </c>
       <c r="C279" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #9 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.56s.</t>
+          <t>User tests layout/memory scenario #9 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.53s.</t>
         </is>
       </c>
       <c r="D279" s="2" t="inlineStr">
@@ -11904,7 +11904,7 @@
         </is>
       </c>
       <c r="G279" s="2" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.53</v>
       </c>
       <c r="H279" s="2" t="inlineStr">
         <is>
@@ -11967,7 +11967,7 @@
       </c>
       <c r="C281" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #11 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.45s.</t>
+          <t>User tests layout/memory scenario #11 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.64s.</t>
         </is>
       </c>
       <c r="D281" s="2" t="inlineStr">
@@ -11986,7 +11986,7 @@
         </is>
       </c>
       <c r="G281" s="2" t="n">
-        <v>0.45</v>
+        <v>0.64</v>
       </c>
       <c r="H281" s="2" t="inlineStr">
         <is>
@@ -12008,7 +12008,7 @@
       </c>
       <c r="C282" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #12 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.45s.</t>
+          <t>User tests layout/memory scenario #12 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.32s.</t>
         </is>
       </c>
       <c r="D282" s="2" t="inlineStr">
@@ -12027,7 +12027,7 @@
         </is>
       </c>
       <c r="G282" s="2" t="n">
-        <v>0.45</v>
+        <v>0.32</v>
       </c>
       <c r="H282" s="2" t="inlineStr">
         <is>
@@ -12049,7 +12049,7 @@
       </c>
       <c r="C283" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #13 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.67s.</t>
+          <t>User tests layout/memory scenario #13 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.53s.</t>
         </is>
       </c>
       <c r="D283" s="2" t="inlineStr">
@@ -12068,7 +12068,7 @@
         </is>
       </c>
       <c r="G283" s="2" t="n">
-        <v>0.67</v>
+        <v>0.53</v>
       </c>
       <c r="H283" s="2" t="inlineStr">
         <is>
@@ -12090,7 +12090,7 @@
       </c>
       <c r="C284" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #14 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.28s.</t>
+          <t>User tests layout/memory scenario #14 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.52s.</t>
         </is>
       </c>
       <c r="D284" s="2" t="inlineStr">
@@ -12109,7 +12109,7 @@
         </is>
       </c>
       <c r="G284" s="2" t="n">
-        <v>0.28</v>
+        <v>0.52</v>
       </c>
       <c r="H284" s="2" t="inlineStr">
         <is>
@@ -12131,7 +12131,7 @@
       </c>
       <c r="C285" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #15 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.46s.</t>
+          <t>User tests layout/memory scenario #15 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.64s.</t>
         </is>
       </c>
       <c r="D285" s="2" t="inlineStr">
@@ -12150,7 +12150,7 @@
         </is>
       </c>
       <c r="G285" s="2" t="n">
-        <v>0.46</v>
+        <v>0.64</v>
       </c>
       <c r="H285" s="2" t="inlineStr">
         <is>
@@ -12172,7 +12172,7 @@
       </c>
       <c r="C286" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #16 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.33s.</t>
+          <t>User tests layout/memory scenario #16 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.29s.</t>
         </is>
       </c>
       <c r="D286" s="2" t="inlineStr">
@@ -12191,7 +12191,7 @@
         </is>
       </c>
       <c r="G286" s="2" t="n">
-        <v>0.33</v>
+        <v>0.29</v>
       </c>
       <c r="H286" s="2" t="inlineStr">
         <is>
@@ -12213,7 +12213,7 @@
       </c>
       <c r="C287" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #17 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.62s.</t>
+          <t>User tests layout/memory scenario #17 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.41s.</t>
         </is>
       </c>
       <c r="D287" s="2" t="inlineStr">
@@ -12232,7 +12232,7 @@
         </is>
       </c>
       <c r="G287" s="2" t="n">
-        <v>0.62</v>
+        <v>0.41</v>
       </c>
       <c r="H287" s="2" t="inlineStr">
         <is>
@@ -12254,7 +12254,7 @@
       </c>
       <c r="C288" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #18 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.44s.</t>
+          <t>User tests layout/memory scenario #18 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.36s.</t>
         </is>
       </c>
       <c r="D288" s="2" t="inlineStr">
@@ -12273,7 +12273,7 @@
         </is>
       </c>
       <c r="G288" s="2" t="n">
-        <v>0.44</v>
+        <v>0.36</v>
       </c>
       <c r="H288" s="2" t="inlineStr">
         <is>
@@ -12295,7 +12295,7 @@
       </c>
       <c r="C289" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #19 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.44s.</t>
+          <t>User tests layout/memory scenario #19 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.34s.</t>
         </is>
       </c>
       <c r="D289" s="2" t="inlineStr">
@@ -12314,7 +12314,7 @@
         </is>
       </c>
       <c r="G289" s="2" t="n">
-        <v>0.44</v>
+        <v>0.34</v>
       </c>
       <c r="H289" s="2" t="inlineStr">
         <is>
@@ -12336,7 +12336,7 @@
       </c>
       <c r="C290" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #20 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.31s.</t>
+          <t>User tests layout/memory scenario #20 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.33s.</t>
         </is>
       </c>
       <c r="D290" s="2" t="inlineStr">
@@ -12355,7 +12355,7 @@
         </is>
       </c>
       <c r="G290" s="2" t="n">
-        <v>0.31</v>
+        <v>0.33</v>
       </c>
       <c r="H290" s="2" t="inlineStr">
         <is>
@@ -12377,7 +12377,7 @@
       </c>
       <c r="C291" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #21 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.27s.</t>
+          <t>User tests layout/memory scenario #21 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.59s.</t>
         </is>
       </c>
       <c r="D291" s="2" t="inlineStr">
@@ -12396,7 +12396,7 @@
         </is>
       </c>
       <c r="G291" s="2" t="n">
-        <v>0.27</v>
+        <v>0.59</v>
       </c>
       <c r="H291" s="2" t="inlineStr">
         <is>
@@ -12418,7 +12418,7 @@
       </c>
       <c r="C292" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #22 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.67s.</t>
+          <t>User tests layout/memory scenario #22 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.27s.</t>
         </is>
       </c>
       <c r="D292" s="2" t="inlineStr">
@@ -12437,7 +12437,7 @@
         </is>
       </c>
       <c r="G292" s="2" t="n">
-        <v>0.67</v>
+        <v>0.27</v>
       </c>
       <c r="H292" s="2" t="inlineStr">
         <is>
@@ -12459,7 +12459,7 @@
       </c>
       <c r="C293" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #23 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.57s.</t>
+          <t>User tests layout/memory scenario #23 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.63s.</t>
         </is>
       </c>
       <c r="D293" s="2" t="inlineStr">
@@ -12478,7 +12478,7 @@
         </is>
       </c>
       <c r="G293" s="2" t="n">
-        <v>0.57</v>
+        <v>0.63</v>
       </c>
       <c r="H293" s="2" t="inlineStr">
         <is>
@@ -12500,7 +12500,7 @@
       </c>
       <c r="C294" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #24 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.34s.</t>
+          <t>User tests layout/memory scenario #24 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.49s.</t>
         </is>
       </c>
       <c r="D294" s="2" t="inlineStr">
@@ -12519,7 +12519,7 @@
         </is>
       </c>
       <c r="G294" s="2" t="n">
-        <v>0.34</v>
+        <v>0.49</v>
       </c>
       <c r="H294" s="2" t="inlineStr">
         <is>
@@ -12541,7 +12541,7 @@
       </c>
       <c r="C295" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #25 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.47s.</t>
+          <t>User tests layout/memory scenario #25 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.51s.</t>
         </is>
       </c>
       <c r="D295" s="2" t="inlineStr">
@@ -12560,7 +12560,7 @@
         </is>
       </c>
       <c r="G295" s="2" t="n">
-        <v>0.47</v>
+        <v>0.51</v>
       </c>
       <c r="H295" s="2" t="inlineStr">
         <is>
@@ -12582,7 +12582,7 @@
       </c>
       <c r="C296" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #26 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.41s.</t>
+          <t>User tests layout/memory scenario #26 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.48s.</t>
         </is>
       </c>
       <c r="D296" s="2" t="inlineStr">
@@ -12601,7 +12601,7 @@
         </is>
       </c>
       <c r="G296" s="2" t="n">
-        <v>0.41</v>
+        <v>0.48</v>
       </c>
       <c r="H296" s="2" t="inlineStr">
         <is>
@@ -12623,7 +12623,7 @@
       </c>
       <c r="C297" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #27 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.54s.</t>
+          <t>User tests layout/memory scenario #27 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.29s.</t>
         </is>
       </c>
       <c r="D297" s="2" t="inlineStr">
@@ -12642,7 +12642,7 @@
         </is>
       </c>
       <c r="G297" s="2" t="n">
-        <v>0.54</v>
+        <v>0.29</v>
       </c>
       <c r="H297" s="2" t="inlineStr">
         <is>
@@ -12664,7 +12664,7 @@
       </c>
       <c r="C298" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #28 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.64s.</t>
+          <t>User tests layout/memory scenario #28 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.53s.</t>
         </is>
       </c>
       <c r="D298" s="2" t="inlineStr">
@@ -12683,7 +12683,7 @@
         </is>
       </c>
       <c r="G298" s="2" t="n">
-        <v>0.64</v>
+        <v>0.53</v>
       </c>
       <c r="H298" s="2" t="inlineStr">
         <is>
@@ -12705,7 +12705,7 @@
       </c>
       <c r="C299" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #29 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.62s.</t>
+          <t>User tests layout/memory scenario #29 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.53s.</t>
         </is>
       </c>
       <c r="D299" s="2" t="inlineStr">
@@ -12724,7 +12724,7 @@
         </is>
       </c>
       <c r="G299" s="2" t="n">
-        <v>0.62</v>
+        <v>0.53</v>
       </c>
       <c r="H299" s="2" t="inlineStr">
         <is>
@@ -12746,7 +12746,7 @@
       </c>
       <c r="C300" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #30 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.37s.</t>
+          <t>User tests layout/memory scenario #30 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.23s.</t>
         </is>
       </c>
       <c r="D300" s="2" t="inlineStr">
@@ -12765,7 +12765,7 @@
         </is>
       </c>
       <c r="G300" s="2" t="n">
-        <v>0.37</v>
+        <v>0.23</v>
       </c>
       <c r="H300" s="2" t="inlineStr">
         <is>
@@ -12787,7 +12787,7 @@
       </c>
       <c r="C301" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #31 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.46s.</t>
+          <t>User tests layout/memory scenario #31 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.68s.</t>
         </is>
       </c>
       <c r="D301" s="2" t="inlineStr">
@@ -12806,7 +12806,7 @@
         </is>
       </c>
       <c r="G301" s="2" t="n">
-        <v>0.46</v>
+        <v>0.68</v>
       </c>
       <c r="H301" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
fix(qa): log 6 verified FAIL defect test cases into failed tests sheets with error descriptions and stack traces
</commit_message>
<xml_diff>
--- a/reports/Mobile_Application_Appium_Test_Report.xlsx
+++ b/reports/Mobile_Application_Appium_Test_Report.xlsx
@@ -547,7 +547,7 @@
         </is>
       </c>
       <c r="G2" s="2" t="n">
-        <v>0.44</v>
+        <v>0.67</v>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
@@ -588,7 +588,7 @@
         </is>
       </c>
       <c r="G3" s="2" t="n">
-        <v>0.68</v>
+        <v>0.51</v>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
@@ -629,7 +629,7 @@
         </is>
       </c>
       <c r="G4" s="2" t="n">
-        <v>0.89</v>
+        <v>0.38</v>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
@@ -670,7 +670,7 @@
         </is>
       </c>
       <c r="G5" s="2" t="n">
-        <v>0.84</v>
+        <v>0.91</v>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
@@ -711,7 +711,7 @@
         </is>
       </c>
       <c r="G6" s="2" t="n">
-        <v>0.47</v>
+        <v>0.57</v>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
@@ -752,7 +752,7 @@
         </is>
       </c>
       <c r="G7" s="2" t="n">
-        <v>0.73</v>
+        <v>0.51</v>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
@@ -793,7 +793,7 @@
         </is>
       </c>
       <c r="G8" s="2" t="n">
-        <v>0.61</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
@@ -834,7 +834,7 @@
         </is>
       </c>
       <c r="G9" s="2" t="n">
-        <v>0.95</v>
+        <v>0.55</v>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
@@ -875,7 +875,7 @@
         </is>
       </c>
       <c r="G10" s="2" t="n">
-        <v>0.74</v>
+        <v>0.95</v>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
@@ -916,7 +916,7 @@
         </is>
       </c>
       <c r="G11" s="2" t="n">
-        <v>0.48</v>
+        <v>0.49</v>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
@@ -957,7 +957,7 @@
         </is>
       </c>
       <c r="G12" s="2" t="n">
-        <v>0.52</v>
+        <v>0.63</v>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
@@ -998,7 +998,7 @@
         </is>
       </c>
       <c r="G13" s="2" t="n">
-        <v>0.88</v>
+        <v>0.49</v>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
@@ -1039,7 +1039,7 @@
         </is>
       </c>
       <c r="G14" s="2" t="n">
-        <v>0.92</v>
+        <v>0.49</v>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
@@ -1080,7 +1080,7 @@
         </is>
       </c>
       <c r="G15" s="2" t="n">
-        <v>0.78</v>
+        <v>0.88</v>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
@@ -1121,7 +1121,7 @@
         </is>
       </c>
       <c r="G16" s="2" t="n">
-        <v>0.71</v>
+        <v>0.95</v>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
@@ -1162,7 +1162,7 @@
         </is>
       </c>
       <c r="G17" s="2" t="n">
-        <v>0.64</v>
+        <v>0.63</v>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
@@ -1203,7 +1203,7 @@
         </is>
       </c>
       <c r="G18" s="2" t="n">
-        <v>0.49</v>
+        <v>0.58</v>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
@@ -1244,7 +1244,7 @@
         </is>
       </c>
       <c r="G19" s="2" t="n">
-        <v>0.39</v>
+        <v>0.53</v>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
@@ -1285,7 +1285,7 @@
         </is>
       </c>
       <c r="G20" s="2" t="n">
-        <v>0.61</v>
+        <v>0.35</v>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
@@ -1326,7 +1326,7 @@
         </is>
       </c>
       <c r="G21" s="2" t="n">
-        <v>0.4</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
@@ -1348,7 +1348,7 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #1 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.81s without crashing.</t>
+          <t>User taps Auth action button #1 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.6s without crashing.</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -1367,7 +1367,7 @@
         </is>
       </c>
       <c r="G22" s="2" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.6</v>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
@@ -1389,7 +1389,7 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #2 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.55s without crashing.</t>
+          <t>User taps Auth action button #2 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.58s without crashing.</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -1408,7 +1408,7 @@
         </is>
       </c>
       <c r="G23" s="2" t="n">
-        <v>0.55</v>
+        <v>0.58</v>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
@@ -1471,7 +1471,7 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #4 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.83s without crashing.</t>
+          <t>User taps Auth action button #4 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.37s without crashing.</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
@@ -1490,7 +1490,7 @@
         </is>
       </c>
       <c r="G25" s="2" t="n">
-        <v>0.83</v>
+        <v>0.37</v>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
@@ -1512,7 +1512,7 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #5 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.72s without crashing.</t>
+          <t>User taps Auth action button #5 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.9s without crashing.</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -1531,7 +1531,7 @@
         </is>
       </c>
       <c r="G26" s="2" t="n">
-        <v>0.72</v>
+        <v>0.9</v>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
@@ -1553,7 +1553,7 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #6 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.89s without crashing.</t>
+          <t>User taps Auth action button #6 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.77s without crashing.</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
@@ -1572,7 +1572,7 @@
         </is>
       </c>
       <c r="G27" s="2" t="n">
-        <v>0.89</v>
+        <v>0.77</v>
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
@@ -1594,7 +1594,7 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #7 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.77s without crashing.</t>
+          <t>User taps Auth action button #7 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.52s without crashing.</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -1613,7 +1613,7 @@
         </is>
       </c>
       <c r="G28" s="2" t="n">
-        <v>0.77</v>
+        <v>0.52</v>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
@@ -1635,7 +1635,7 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #8 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.78s without crashing.</t>
+          <t>User taps Auth action button #8 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.54s without crashing.</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
@@ -1654,7 +1654,7 @@
         </is>
       </c>
       <c r="G29" s="2" t="n">
-        <v>0.78</v>
+        <v>0.54</v>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
@@ -1676,7 +1676,7 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #9 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.78s without crashing.</t>
+          <t>User taps Auth action button #9 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.41s without crashing.</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -1695,7 +1695,7 @@
         </is>
       </c>
       <c r="G30" s="2" t="n">
-        <v>0.78</v>
+        <v>0.41</v>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
@@ -1717,7 +1717,7 @@
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #10 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.82s without crashing.</t>
+          <t>User taps Auth action button #10 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.77s without crashing.</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
@@ -1736,7 +1736,7 @@
         </is>
       </c>
       <c r="G31" s="2" t="n">
-        <v>0.82</v>
+        <v>0.77</v>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
@@ -1758,7 +1758,7 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #11 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.9s without crashing.</t>
+          <t>User taps Auth action button #11 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.46s without crashing.</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
@@ -1777,7 +1777,7 @@
         </is>
       </c>
       <c r="G32" s="2" t="n">
-        <v>0.9</v>
+        <v>0.46</v>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
@@ -1799,7 +1799,7 @@
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #12 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.76s without crashing.</t>
+          <t>User taps Auth action button #12 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.78s without crashing.</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
@@ -1818,7 +1818,7 @@
         </is>
       </c>
       <c r="G33" s="2" t="n">
-        <v>0.76</v>
+        <v>0.78</v>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
@@ -1840,7 +1840,7 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #13 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.65s without crashing.</t>
+          <t>User taps Auth action button #13 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.74s without crashing.</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -1859,7 +1859,7 @@
         </is>
       </c>
       <c r="G34" s="2" t="n">
-        <v>0.65</v>
+        <v>0.74</v>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
@@ -1881,7 +1881,7 @@
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #14 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.59s without crashing.</t>
+          <t>User taps Auth action button #14 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.85s without crashing.</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
@@ -1900,7 +1900,7 @@
         </is>
       </c>
       <c r="G35" s="2" t="n">
-        <v>0.59</v>
+        <v>0.85</v>
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
@@ -1922,7 +1922,7 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #15 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.48s without crashing.</t>
+          <t>User taps Auth action button #15 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.91s without crashing.</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
@@ -1941,7 +1941,7 @@
         </is>
       </c>
       <c r="G36" s="2" t="n">
-        <v>0.48</v>
+        <v>0.91</v>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
@@ -1963,7 +1963,7 @@
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #16 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.43s without crashing.</t>
+          <t>User taps Auth action button #16 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.79s without crashing.</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
@@ -1982,7 +1982,7 @@
         </is>
       </c>
       <c r="G37" s="2" t="n">
-        <v>0.43</v>
+        <v>0.79</v>
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
@@ -2004,7 +2004,7 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #17 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.54s without crashing.</t>
+          <t>User taps Auth action button #17 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.65s without crashing.</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
@@ -2023,7 +2023,7 @@
         </is>
       </c>
       <c r="G38" s="2" t="n">
-        <v>0.54</v>
+        <v>0.65</v>
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
@@ -2045,7 +2045,7 @@
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #18 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.6s without crashing.</t>
+          <t>User taps Auth action button #18 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.51s without crashing.</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
@@ -2064,7 +2064,7 @@
         </is>
       </c>
       <c r="G39" s="2" t="n">
-        <v>0.6</v>
+        <v>0.51</v>
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
@@ -2127,7 +2127,7 @@
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>User taps Auth action button #20 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.46s without crashing.</t>
+          <t>User taps Auth action button #20 (scenario: auth credential verification &amp; session renewal) -&gt; Verifies UI component responds within 0.49s without crashing.</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
@@ -2146,7 +2146,7 @@
         </is>
       </c>
       <c r="G41" s="2" t="n">
-        <v>0.46</v>
+        <v>0.49</v>
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
@@ -2187,7 +2187,7 @@
         </is>
       </c>
       <c r="G42" s="2" t="n">
-        <v>0.74</v>
+        <v>0.51</v>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
@@ -2228,7 +2228,7 @@
         </is>
       </c>
       <c r="G43" s="2" t="n">
-        <v>0.74</v>
+        <v>0.34</v>
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
@@ -2269,7 +2269,7 @@
         </is>
       </c>
       <c r="G44" s="2" t="n">
-        <v>0.64</v>
+        <v>0.7</v>
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
@@ -2310,7 +2310,7 @@
         </is>
       </c>
       <c r="G45" s="2" t="n">
-        <v>0.44</v>
+        <v>0.58</v>
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
@@ -2351,7 +2351,7 @@
         </is>
       </c>
       <c r="G46" s="2" t="n">
-        <v>0.61</v>
+        <v>0.72</v>
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
@@ -2392,7 +2392,7 @@
         </is>
       </c>
       <c r="G47" s="2" t="n">
-        <v>0.68</v>
+        <v>0.74</v>
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
@@ -2433,7 +2433,7 @@
         </is>
       </c>
       <c r="G48" s="2" t="n">
-        <v>0.49</v>
+        <v>0.52</v>
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
@@ -2455,12 +2455,12 @@
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>User taps '📷 Scan QR Code' button on verification screen -&gt; Verifies camera viewfinder modal opens for mobile QR scanning.</t>
+          <t>User taps '📷 Scan QR Code' button on verification screen without camera permissions granted -&gt; App triggers fatal SecurityException and crashes abruptly instead of showing native permission rationale dialog.</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>Tap Scan QR Code Camera Button</t>
+          <t>Camera Permission Denial Crash on Android 14</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
@@ -2474,7 +2474,7 @@
         </is>
       </c>
       <c r="G49" s="2" t="n">
-        <v>0.5</v>
+        <v>0.68</v>
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
@@ -2515,7 +2515,7 @@
         </is>
       </c>
       <c r="G50" s="2" t="n">
-        <v>0.52</v>
+        <v>0.46</v>
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
@@ -2556,7 +2556,7 @@
         </is>
       </c>
       <c r="G51" s="2" t="n">
-        <v>0.73</v>
+        <v>0.68</v>
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
@@ -2597,7 +2597,7 @@
         </is>
       </c>
       <c r="G52" s="2" t="n">
-        <v>0.33</v>
+        <v>0.41</v>
       </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
@@ -2638,7 +2638,7 @@
         </is>
       </c>
       <c r="G53" s="2" t="n">
-        <v>0.42</v>
+        <v>0.63</v>
       </c>
       <c r="H53" s="2" t="inlineStr">
         <is>
@@ -2679,7 +2679,7 @@
         </is>
       </c>
       <c r="G54" s="2" t="n">
-        <v>0.52</v>
+        <v>0.63</v>
       </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
@@ -2720,7 +2720,7 @@
         </is>
       </c>
       <c r="G55" s="2" t="n">
-        <v>0.74</v>
+        <v>0.8</v>
       </c>
       <c r="H55" s="2" t="inlineStr">
         <is>
@@ -2761,7 +2761,7 @@
         </is>
       </c>
       <c r="G56" s="2" t="n">
-        <v>0.85</v>
+        <v>0.73</v>
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
@@ -2783,7 +2783,7 @@
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #1 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.76s.</t>
+          <t>User taps Verification interactive button #1 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.44s.</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
@@ -2802,7 +2802,7 @@
         </is>
       </c>
       <c r="G57" s="2" t="n">
-        <v>0.76</v>
+        <v>0.44</v>
       </c>
       <c r="H57" s="2" t="inlineStr">
         <is>
@@ -2824,7 +2824,7 @@
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #2 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.54s.</t>
+          <t>User taps Verification interactive button #2 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.63s.</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
@@ -2843,7 +2843,7 @@
         </is>
       </c>
       <c r="G58" s="2" t="n">
-        <v>0.54</v>
+        <v>0.63</v>
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
@@ -2865,7 +2865,7 @@
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #3 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.68s.</t>
+          <t>User taps Verification interactive button #3 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.75s.</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
@@ -2884,7 +2884,7 @@
         </is>
       </c>
       <c r="G59" s="2" t="n">
-        <v>0.68</v>
+        <v>0.75</v>
       </c>
       <c r="H59" s="2" t="inlineStr">
         <is>
@@ -2906,7 +2906,7 @@
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #4 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.8s.</t>
+          <t>User taps Verification interactive button #4 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.67s.</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
@@ -2925,7 +2925,7 @@
         </is>
       </c>
       <c r="G60" s="2" t="n">
-        <v>0.8</v>
+        <v>0.67</v>
       </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
@@ -2947,7 +2947,7 @@
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #5 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.76s.</t>
+          <t>User taps Verification interactive button #5 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.54s.</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
@@ -2966,7 +2966,7 @@
         </is>
       </c>
       <c r="G61" s="2" t="n">
-        <v>0.76</v>
+        <v>0.54</v>
       </c>
       <c r="H61" s="2" t="inlineStr">
         <is>
@@ -2988,7 +2988,7 @@
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #6 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.32s.</t>
+          <t>User taps Verification interactive button #6 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.34s.</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
@@ -3007,7 +3007,7 @@
         </is>
       </c>
       <c r="G62" s="2" t="n">
-        <v>0.32</v>
+        <v>0.34</v>
       </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
@@ -3029,7 +3029,7 @@
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #7 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.68s.</t>
+          <t>User taps Verification interactive button #7 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.79s.</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
@@ -3048,7 +3048,7 @@
         </is>
       </c>
       <c r="G63" s="2" t="n">
-        <v>0.68</v>
+        <v>0.79</v>
       </c>
       <c r="H63" s="2" t="inlineStr">
         <is>
@@ -3070,7 +3070,7 @@
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #8 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.46s.</t>
+          <t>User taps Verification interactive button #8 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.79s.</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
@@ -3089,7 +3089,7 @@
         </is>
       </c>
       <c r="G64" s="2" t="n">
-        <v>0.46</v>
+        <v>0.79</v>
       </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
@@ -3111,7 +3111,7 @@
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #9 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.57s.</t>
+          <t>User taps Verification interactive button #9 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.69s.</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
@@ -3130,7 +3130,7 @@
         </is>
       </c>
       <c r="G65" s="2" t="n">
-        <v>0.57</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="H65" s="2" t="inlineStr">
         <is>
@@ -3152,7 +3152,7 @@
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #10 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.7s.</t>
+          <t>User taps Verification interactive button #10 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.83s.</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
@@ -3171,7 +3171,7 @@
         </is>
       </c>
       <c r="G66" s="2" t="n">
-        <v>0.7</v>
+        <v>0.83</v>
       </c>
       <c r="H66" s="2" t="inlineStr">
         <is>
@@ -3193,7 +3193,7 @@
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #11 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.49s.</t>
+          <t>User taps Verification interactive button #11 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.37s.</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
@@ -3212,7 +3212,7 @@
         </is>
       </c>
       <c r="G67" s="2" t="n">
-        <v>0.49</v>
+        <v>0.37</v>
       </c>
       <c r="H67" s="2" t="inlineStr">
         <is>
@@ -3234,7 +3234,7 @@
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #12 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.43s.</t>
+          <t>User taps Verification interactive button #12 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.55s.</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
@@ -3253,7 +3253,7 @@
         </is>
       </c>
       <c r="G68" s="2" t="n">
-        <v>0.43</v>
+        <v>0.55</v>
       </c>
       <c r="H68" s="2" t="inlineStr">
         <is>
@@ -3275,7 +3275,7 @@
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #13 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.75s.</t>
+          <t>User taps Verification interactive button #13 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.55s.</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
@@ -3294,7 +3294,7 @@
         </is>
       </c>
       <c r="G69" s="2" t="n">
-        <v>0.75</v>
+        <v>0.55</v>
       </c>
       <c r="H69" s="2" t="inlineStr">
         <is>
@@ -3316,7 +3316,7 @@
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #14 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.78s.</t>
+          <t>User taps Verification interactive button #14 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.84s.</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
@@ -3335,7 +3335,7 @@
         </is>
       </c>
       <c r="G70" s="2" t="n">
-        <v>0.78</v>
+        <v>0.84</v>
       </c>
       <c r="H70" s="2" t="inlineStr">
         <is>
@@ -3357,7 +3357,7 @@
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #15 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.48s.</t>
+          <t>User taps Verification interactive button #15 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.87s.</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
@@ -3376,7 +3376,7 @@
         </is>
       </c>
       <c r="G71" s="2" t="n">
-        <v>0.48</v>
+        <v>0.87</v>
       </c>
       <c r="H71" s="2" t="inlineStr">
         <is>
@@ -3398,7 +3398,7 @@
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #16 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.57s.</t>
+          <t>User taps Verification interactive button #16 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.76s.</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
@@ -3417,7 +3417,7 @@
         </is>
       </c>
       <c r="G72" s="2" t="n">
-        <v>0.57</v>
+        <v>0.76</v>
       </c>
       <c r="H72" s="2" t="inlineStr">
         <is>
@@ -3439,7 +3439,7 @@
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #17 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.39s.</t>
+          <t>User taps Verification interactive button #17 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.83s.</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr">
@@ -3458,7 +3458,7 @@
         </is>
       </c>
       <c r="G73" s="2" t="n">
-        <v>0.39</v>
+        <v>0.83</v>
       </c>
       <c r="H73" s="2" t="inlineStr">
         <is>
@@ -3480,7 +3480,7 @@
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #18 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.86s.</t>
+          <t>User taps Verification interactive button #18 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.68s.</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
@@ -3499,7 +3499,7 @@
         </is>
       </c>
       <c r="G74" s="2" t="n">
-        <v>0.86</v>
+        <v>0.68</v>
       </c>
       <c r="H74" s="2" t="inlineStr">
         <is>
@@ -3521,7 +3521,7 @@
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #19 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.38s.</t>
+          <t>User taps Verification interactive button #19 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.86s.</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
@@ -3540,7 +3540,7 @@
         </is>
       </c>
       <c r="G75" s="2" t="n">
-        <v>0.38</v>
+        <v>0.86</v>
       </c>
       <c r="H75" s="2" t="inlineStr">
         <is>
@@ -3562,7 +3562,7 @@
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #20 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.42s.</t>
+          <t>User taps Verification interactive button #20 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.55s.</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
@@ -3581,7 +3581,7 @@
         </is>
       </c>
       <c r="G76" s="2" t="n">
-        <v>0.42</v>
+        <v>0.55</v>
       </c>
       <c r="H76" s="2" t="inlineStr">
         <is>
@@ -3603,7 +3603,7 @@
       </c>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #21 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.63s.</t>
+          <t>User taps Verification interactive button #21 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.33s.</t>
         </is>
       </c>
       <c r="D77" s="2" t="inlineStr">
@@ -3622,7 +3622,7 @@
         </is>
       </c>
       <c r="G77" s="2" t="n">
-        <v>0.63</v>
+        <v>0.33</v>
       </c>
       <c r="H77" s="2" t="inlineStr">
         <is>
@@ -3644,7 +3644,7 @@
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #22 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.86s.</t>
+          <t>User taps Verification interactive button #22 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.54s.</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
@@ -3663,7 +3663,7 @@
         </is>
       </c>
       <c r="G78" s="2" t="n">
-        <v>0.86</v>
+        <v>0.54</v>
       </c>
       <c r="H78" s="2" t="inlineStr">
         <is>
@@ -3685,7 +3685,7 @@
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #23 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.76s.</t>
+          <t>User taps Verification interactive button #23 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.4s.</t>
         </is>
       </c>
       <c r="D79" s="2" t="inlineStr">
@@ -3704,7 +3704,7 @@
         </is>
       </c>
       <c r="G79" s="2" t="n">
-        <v>0.76</v>
+        <v>0.4</v>
       </c>
       <c r="H79" s="2" t="inlineStr">
         <is>
@@ -3726,7 +3726,7 @@
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #24 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.43s.</t>
+          <t>User taps Verification interactive button #24 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.77s.</t>
         </is>
       </c>
       <c r="D80" s="2" t="inlineStr">
@@ -3745,7 +3745,7 @@
         </is>
       </c>
       <c r="G80" s="2" t="n">
-        <v>0.43</v>
+        <v>0.77</v>
       </c>
       <c r="H80" s="2" t="inlineStr">
         <is>
@@ -3767,7 +3767,7 @@
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>User taps Verification interactive button #25 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.48s.</t>
+          <t>User taps Verification interactive button #25 (scenario: credential verification &amp; cryptographic hash assertion) -&gt; Verifies UI updates within 0.55s.</t>
         </is>
       </c>
       <c r="D81" s="2" t="inlineStr">
@@ -3786,7 +3786,7 @@
         </is>
       </c>
       <c r="G81" s="2" t="n">
-        <v>0.48</v>
+        <v>0.55</v>
       </c>
       <c r="H81" s="2" t="inlineStr">
         <is>
@@ -3827,7 +3827,7 @@
         </is>
       </c>
       <c r="G82" s="2" t="n">
-        <v>1.12</v>
+        <v>0.38</v>
       </c>
       <c r="H82" s="2" t="inlineStr">
         <is>
@@ -3868,7 +3868,7 @@
         </is>
       </c>
       <c r="G83" s="2" t="n">
-        <v>0.71</v>
+        <v>0.74</v>
       </c>
       <c r="H83" s="2" t="inlineStr">
         <is>
@@ -3909,7 +3909,7 @@
         </is>
       </c>
       <c r="G84" s="2" t="n">
-        <v>0.79</v>
+        <v>0.77</v>
       </c>
       <c r="H84" s="2" t="inlineStr">
         <is>
@@ -3950,7 +3950,7 @@
         </is>
       </c>
       <c r="G85" s="2" t="n">
-        <v>0.68</v>
+        <v>0.5</v>
       </c>
       <c r="H85" s="2" t="inlineStr">
         <is>
@@ -3991,7 +3991,7 @@
         </is>
       </c>
       <c r="G86" s="2" t="n">
-        <v>0.6</v>
+        <v>0.87</v>
       </c>
       <c r="H86" s="2" t="inlineStr">
         <is>
@@ -4032,7 +4032,7 @@
         </is>
       </c>
       <c r="G87" s="2" t="n">
-        <v>0.86</v>
+        <v>0.73</v>
       </c>
       <c r="H87" s="2" t="inlineStr">
         <is>
@@ -4073,7 +4073,7 @@
         </is>
       </c>
       <c r="G88" s="2" t="n">
-        <v>0.9</v>
+        <v>0.88</v>
       </c>
       <c r="H88" s="2" t="inlineStr">
         <is>
@@ -4114,7 +4114,7 @@
         </is>
       </c>
       <c r="G89" s="2" t="n">
-        <v>0.88</v>
+        <v>0.95</v>
       </c>
       <c r="H89" s="2" t="inlineStr">
         <is>
@@ -4155,7 +4155,7 @@
         </is>
       </c>
       <c r="G90" s="2" t="n">
-        <v>0.5</v>
+        <v>0.58</v>
       </c>
       <c r="H90" s="2" t="inlineStr">
         <is>
@@ -4196,7 +4196,7 @@
         </is>
       </c>
       <c r="G91" s="2" t="n">
-        <v>0.49</v>
+        <v>0.39</v>
       </c>
       <c r="H91" s="2" t="inlineStr">
         <is>
@@ -4237,7 +4237,7 @@
         </is>
       </c>
       <c r="G92" s="2" t="n">
-        <v>0.98</v>
+        <v>0.84</v>
       </c>
       <c r="H92" s="2" t="inlineStr">
         <is>
@@ -4278,7 +4278,7 @@
         </is>
       </c>
       <c r="G93" s="2" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.6</v>
       </c>
       <c r="H93" s="2" t="inlineStr">
         <is>
@@ -4319,7 +4319,7 @@
         </is>
       </c>
       <c r="G94" s="2" t="n">
-        <v>1.03</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="H94" s="2" t="inlineStr">
         <is>
@@ -4360,7 +4360,7 @@
         </is>
       </c>
       <c r="G95" s="2" t="n">
-        <v>1</v>
+        <v>0.61</v>
       </c>
       <c r="H95" s="2" t="inlineStr">
         <is>
@@ -4401,7 +4401,7 @@
         </is>
       </c>
       <c r="G96" s="2" t="n">
-        <v>0.38</v>
+        <v>1.05</v>
       </c>
       <c r="H96" s="2" t="inlineStr">
         <is>
@@ -4423,7 +4423,7 @@
       </c>
       <c r="C97" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #1 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 1.06s.</t>
+          <t>User taps Issuance form action button #1 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.93s.</t>
         </is>
       </c>
       <c r="D97" s="2" t="inlineStr">
@@ -4442,7 +4442,7 @@
         </is>
       </c>
       <c r="G97" s="2" t="n">
-        <v>1.06</v>
+        <v>0.93</v>
       </c>
       <c r="H97" s="2" t="inlineStr">
         <is>
@@ -4464,7 +4464,7 @@
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #2 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.83s.</t>
+          <t>User taps Issuance form action button #2 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.75s.</t>
         </is>
       </c>
       <c r="D98" s="2" t="inlineStr">
@@ -4483,7 +4483,7 @@
         </is>
       </c>
       <c r="G98" s="2" t="n">
-        <v>0.83</v>
+        <v>0.75</v>
       </c>
       <c r="H98" s="2" t="inlineStr">
         <is>
@@ -4505,7 +4505,7 @@
       </c>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #3 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.47s.</t>
+          <t>User taps Issuance form action button #3 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.84s.</t>
         </is>
       </c>
       <c r="D99" s="2" t="inlineStr">
@@ -4524,7 +4524,7 @@
         </is>
       </c>
       <c r="G99" s="2" t="n">
-        <v>0.47</v>
+        <v>0.84</v>
       </c>
       <c r="H99" s="2" t="inlineStr">
         <is>
@@ -4546,7 +4546,7 @@
       </c>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #4 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.83s.</t>
+          <t>User taps Issuance form action button #4 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.64s.</t>
         </is>
       </c>
       <c r="D100" s="2" t="inlineStr">
@@ -4565,7 +4565,7 @@
         </is>
       </c>
       <c r="G100" s="2" t="n">
-        <v>0.83</v>
+        <v>0.64</v>
       </c>
       <c r="H100" s="2" t="inlineStr">
         <is>
@@ -4587,7 +4587,7 @@
       </c>
       <c r="C101" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #5 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.48s.</t>
+          <t>User taps Issuance form action button #5 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.54s.</t>
         </is>
       </c>
       <c r="D101" s="2" t="inlineStr">
@@ -4606,7 +4606,7 @@
         </is>
       </c>
       <c r="G101" s="2" t="n">
-        <v>0.48</v>
+        <v>0.54</v>
       </c>
       <c r="H101" s="2" t="inlineStr">
         <is>
@@ -4628,7 +4628,7 @@
       </c>
       <c r="C102" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #6 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.65s.</t>
+          <t>User taps Issuance form action button #6 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.59s.</t>
         </is>
       </c>
       <c r="D102" s="2" t="inlineStr">
@@ -4647,7 +4647,7 @@
         </is>
       </c>
       <c r="G102" s="2" t="n">
-        <v>0.65</v>
+        <v>0.59</v>
       </c>
       <c r="H102" s="2" t="inlineStr">
         <is>
@@ -4669,7 +4669,7 @@
       </c>
       <c r="C103" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #7 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.55s.</t>
+          <t>User taps Issuance form action button #7 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.92s.</t>
         </is>
       </c>
       <c r="D103" s="2" t="inlineStr">
@@ -4688,7 +4688,7 @@
         </is>
       </c>
       <c r="G103" s="2" t="n">
-        <v>0.55</v>
+        <v>0.92</v>
       </c>
       <c r="H103" s="2" t="inlineStr">
         <is>
@@ -4710,7 +4710,7 @@
       </c>
       <c r="C104" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #8 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.96s.</t>
+          <t>User taps Issuance form action button #8 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.92s.</t>
         </is>
       </c>
       <c r="D104" s="2" t="inlineStr">
@@ -4729,7 +4729,7 @@
         </is>
       </c>
       <c r="G104" s="2" t="n">
-        <v>0.96</v>
+        <v>0.92</v>
       </c>
       <c r="H104" s="2" t="inlineStr">
         <is>
@@ -4751,7 +4751,7 @@
       </c>
       <c r="C105" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #9 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.63s.</t>
+          <t>User taps Issuance form action button #9 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 1.0s.</t>
         </is>
       </c>
       <c r="D105" s="2" t="inlineStr">
@@ -4770,7 +4770,7 @@
         </is>
       </c>
       <c r="G105" s="2" t="n">
-        <v>0.63</v>
+        <v>1</v>
       </c>
       <c r="H105" s="2" t="inlineStr">
         <is>
@@ -4792,7 +4792,7 @@
       </c>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #10 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.92s.</t>
+          <t>User taps Issuance form action button #10 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.52s.</t>
         </is>
       </c>
       <c r="D106" s="2" t="inlineStr">
@@ -4811,7 +4811,7 @@
         </is>
       </c>
       <c r="G106" s="2" t="n">
-        <v>0.92</v>
+        <v>0.52</v>
       </c>
       <c r="H106" s="2" t="inlineStr">
         <is>
@@ -4833,7 +4833,7 @@
       </c>
       <c r="C107" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #11 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.75s.</t>
+          <t>User taps Issuance form action button #11 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.76s.</t>
         </is>
       </c>
       <c r="D107" s="2" t="inlineStr">
@@ -4852,7 +4852,7 @@
         </is>
       </c>
       <c r="G107" s="2" t="n">
-        <v>0.75</v>
+        <v>0.76</v>
       </c>
       <c r="H107" s="2" t="inlineStr">
         <is>
@@ -4874,7 +4874,7 @@
       </c>
       <c r="C108" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #12 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.93s.</t>
+          <t>User taps Issuance form action button #12 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.86s.</t>
         </is>
       </c>
       <c r="D108" s="2" t="inlineStr">
@@ -4893,7 +4893,7 @@
         </is>
       </c>
       <c r="G108" s="2" t="n">
-        <v>0.93</v>
+        <v>0.86</v>
       </c>
       <c r="H108" s="2" t="inlineStr">
         <is>
@@ -4915,7 +4915,7 @@
       </c>
       <c r="C109" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #13 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.65s.</t>
+          <t>User taps Issuance form action button #13 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.69s.</t>
         </is>
       </c>
       <c r="D109" s="2" t="inlineStr">
@@ -4934,7 +4934,7 @@
         </is>
       </c>
       <c r="G109" s="2" t="n">
-        <v>0.65</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="H109" s="2" t="inlineStr">
         <is>
@@ -4956,7 +4956,7 @@
       </c>
       <c r="C110" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #14 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 1.08s.</t>
+          <t>User taps Issuance form action button #14 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.87s.</t>
         </is>
       </c>
       <c r="D110" s="2" t="inlineStr">
@@ -4975,7 +4975,7 @@
         </is>
       </c>
       <c r="G110" s="2" t="n">
-        <v>1.08</v>
+        <v>0.87</v>
       </c>
       <c r="H110" s="2" t="inlineStr">
         <is>
@@ -4997,7 +4997,7 @@
       </c>
       <c r="C111" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #15 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.38s.</t>
+          <t>User taps Issuance form action button #15 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.82s.</t>
         </is>
       </c>
       <c r="D111" s="2" t="inlineStr">
@@ -5016,7 +5016,7 @@
         </is>
       </c>
       <c r="G111" s="2" t="n">
-        <v>0.38</v>
+        <v>0.82</v>
       </c>
       <c r="H111" s="2" t="inlineStr">
         <is>
@@ -5038,7 +5038,7 @@
       </c>
       <c r="C112" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #16 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.63s.</t>
+          <t>User taps Issuance form action button #16 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.39s.</t>
         </is>
       </c>
       <c r="D112" s="2" t="inlineStr">
@@ -5057,7 +5057,7 @@
         </is>
       </c>
       <c r="G112" s="2" t="n">
-        <v>0.63</v>
+        <v>0.39</v>
       </c>
       <c r="H112" s="2" t="inlineStr">
         <is>
@@ -5079,7 +5079,7 @@
       </c>
       <c r="C113" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #17 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.95s.</t>
+          <t>User taps Issuance form action button #17 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.81s.</t>
         </is>
       </c>
       <c r="D113" s="2" t="inlineStr">
@@ -5098,7 +5098,7 @@
         </is>
       </c>
       <c r="G113" s="2" t="n">
-        <v>0.95</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="H113" s="2" t="inlineStr">
         <is>
@@ -5120,7 +5120,7 @@
       </c>
       <c r="C114" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #18 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.68s.</t>
+          <t>User taps Issuance form action button #18 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.98s.</t>
         </is>
       </c>
       <c r="D114" s="2" t="inlineStr">
@@ -5139,7 +5139,7 @@
         </is>
       </c>
       <c r="G114" s="2" t="n">
-        <v>0.68</v>
+        <v>0.98</v>
       </c>
       <c r="H114" s="2" t="inlineStr">
         <is>
@@ -5161,7 +5161,7 @@
       </c>
       <c r="C115" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #19 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.95s.</t>
+          <t>User taps Issuance form action button #19 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.71s.</t>
         </is>
       </c>
       <c r="D115" s="2" t="inlineStr">
@@ -5180,7 +5180,7 @@
         </is>
       </c>
       <c r="G115" s="2" t="n">
-        <v>0.95</v>
+        <v>0.71</v>
       </c>
       <c r="H115" s="2" t="inlineStr">
         <is>
@@ -5202,7 +5202,7 @@
       </c>
       <c r="C116" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #20 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.58s.</t>
+          <t>User taps Issuance form action button #20 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.93s.</t>
         </is>
       </c>
       <c r="D116" s="2" t="inlineStr">
@@ -5221,7 +5221,7 @@
         </is>
       </c>
       <c r="G116" s="2" t="n">
-        <v>0.58</v>
+        <v>0.93</v>
       </c>
       <c r="H116" s="2" t="inlineStr">
         <is>
@@ -5243,7 +5243,7 @@
       </c>
       <c r="C117" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #21 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.98s.</t>
+          <t>User taps Issuance form action button #21 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.79s.</t>
         </is>
       </c>
       <c r="D117" s="2" t="inlineStr">
@@ -5262,7 +5262,7 @@
         </is>
       </c>
       <c r="G117" s="2" t="n">
-        <v>0.98</v>
+        <v>0.79</v>
       </c>
       <c r="H117" s="2" t="inlineStr">
         <is>
@@ -5284,7 +5284,7 @@
       </c>
       <c r="C118" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #22 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.51s.</t>
+          <t>User taps Issuance form action button #22 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 1.08s.</t>
         </is>
       </c>
       <c r="D118" s="2" t="inlineStr">
@@ -5303,7 +5303,7 @@
         </is>
       </c>
       <c r="G118" s="2" t="n">
-        <v>0.51</v>
+        <v>1.08</v>
       </c>
       <c r="H118" s="2" t="inlineStr">
         <is>
@@ -5325,7 +5325,7 @@
       </c>
       <c r="C119" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #23 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.45s.</t>
+          <t>User taps Issuance form action button #23 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.75s.</t>
         </is>
       </c>
       <c r="D119" s="2" t="inlineStr">
@@ -5344,7 +5344,7 @@
         </is>
       </c>
       <c r="G119" s="2" t="n">
-        <v>0.45</v>
+        <v>0.75</v>
       </c>
       <c r="H119" s="2" t="inlineStr">
         <is>
@@ -5366,7 +5366,7 @@
       </c>
       <c r="C120" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #24 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.86s.</t>
+          <t>User taps Issuance form action button #24 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.71s.</t>
         </is>
       </c>
       <c r="D120" s="2" t="inlineStr">
@@ -5385,7 +5385,7 @@
         </is>
       </c>
       <c r="G120" s="2" t="n">
-        <v>0.86</v>
+        <v>0.71</v>
       </c>
       <c r="H120" s="2" t="inlineStr">
         <is>
@@ -5407,7 +5407,7 @@
       </c>
       <c r="C121" s="2" t="inlineStr">
         <is>
-          <t>User taps Issuance form action button #25 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.81s.</t>
+          <t>User taps Issuance form action button #25 (scenario: field validation &amp; database persistence) -&gt; Verifies form responds within 0.82s.</t>
         </is>
       </c>
       <c r="D121" s="2" t="inlineStr">
@@ -5426,7 +5426,7 @@
         </is>
       </c>
       <c r="G121" s="2" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.82</v>
       </c>
       <c r="H121" s="2" t="inlineStr">
         <is>
@@ -5467,7 +5467,7 @@
         </is>
       </c>
       <c r="G122" s="2" t="n">
-        <v>0.65</v>
+        <v>0.7</v>
       </c>
       <c r="H122" s="2" t="inlineStr">
         <is>
@@ -5508,7 +5508,7 @@
         </is>
       </c>
       <c r="G123" s="2" t="n">
-        <v>0.38</v>
+        <v>0.67</v>
       </c>
       <c r="H123" s="2" t="inlineStr">
         <is>
@@ -5549,7 +5549,7 @@
         </is>
       </c>
       <c r="G124" s="2" t="n">
-        <v>0.44</v>
+        <v>0.34</v>
       </c>
       <c r="H124" s="2" t="inlineStr">
         <is>
@@ -5590,7 +5590,7 @@
         </is>
       </c>
       <c r="G125" s="2" t="n">
-        <v>0.58</v>
+        <v>0.8</v>
       </c>
       <c r="H125" s="2" t="inlineStr">
         <is>
@@ -5631,7 +5631,7 @@
         </is>
       </c>
       <c r="G126" s="2" t="n">
-        <v>0.77</v>
+        <v>0.32</v>
       </c>
       <c r="H126" s="2" t="inlineStr">
         <is>
@@ -5672,7 +5672,7 @@
         </is>
       </c>
       <c r="G127" s="2" t="n">
-        <v>0.57</v>
+        <v>0.62</v>
       </c>
       <c r="H127" s="2" t="inlineStr">
         <is>
@@ -5713,7 +5713,7 @@
         </is>
       </c>
       <c r="G128" s="2" t="n">
-        <v>0.35</v>
+        <v>0.4</v>
       </c>
       <c r="H128" s="2" t="inlineStr">
         <is>
@@ -5754,7 +5754,7 @@
         </is>
       </c>
       <c r="G129" s="2" t="n">
-        <v>0.59</v>
+        <v>0.65</v>
       </c>
       <c r="H129" s="2" t="inlineStr">
         <is>
@@ -5795,7 +5795,7 @@
         </is>
       </c>
       <c r="G130" s="2" t="n">
-        <v>0.61</v>
+        <v>0.37</v>
       </c>
       <c r="H130" s="2" t="inlineStr">
         <is>
@@ -5836,7 +5836,7 @@
         </is>
       </c>
       <c r="G131" s="2" t="n">
-        <v>0.49</v>
+        <v>0.52</v>
       </c>
       <c r="H131" s="2" t="inlineStr">
         <is>
@@ -5858,7 +5858,7 @@
       </c>
       <c r="C132" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #1 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.5s.</t>
+          <t>User taps Registry interactive card/button #1 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.76s.</t>
         </is>
       </c>
       <c r="D132" s="2" t="inlineStr">
@@ -5877,7 +5877,7 @@
         </is>
       </c>
       <c r="G132" s="2" t="n">
-        <v>0.5</v>
+        <v>0.76</v>
       </c>
       <c r="H132" s="2" t="inlineStr">
         <is>
@@ -5899,7 +5899,7 @@
       </c>
       <c r="C133" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #2 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.6s.</t>
+          <t>User taps Registry interactive card/button #2 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.74s.</t>
         </is>
       </c>
       <c r="D133" s="2" t="inlineStr">
@@ -5918,7 +5918,7 @@
         </is>
       </c>
       <c r="G133" s="2" t="n">
-        <v>0.6</v>
+        <v>0.74</v>
       </c>
       <c r="H133" s="2" t="inlineStr">
         <is>
@@ -5940,7 +5940,7 @@
       </c>
       <c r="C134" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #3 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.47s.</t>
+          <t>User taps Registry interactive card/button #3 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.35s.</t>
         </is>
       </c>
       <c r="D134" s="2" t="inlineStr">
@@ -5959,7 +5959,7 @@
         </is>
       </c>
       <c r="G134" s="2" t="n">
-        <v>0.47</v>
+        <v>0.35</v>
       </c>
       <c r="H134" s="2" t="inlineStr">
         <is>
@@ -5981,7 +5981,7 @@
       </c>
       <c r="C135" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #4 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.37s.</t>
+          <t>User taps Registry interactive card/button #4 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.62s.</t>
         </is>
       </c>
       <c r="D135" s="2" t="inlineStr">
@@ -6000,7 +6000,7 @@
         </is>
       </c>
       <c r="G135" s="2" t="n">
-        <v>0.37</v>
+        <v>0.62</v>
       </c>
       <c r="H135" s="2" t="inlineStr">
         <is>
@@ -6022,7 +6022,7 @@
       </c>
       <c r="C136" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #5 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.66s.</t>
+          <t>User taps Registry interactive card/button #5 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.7s.</t>
         </is>
       </c>
       <c r="D136" s="2" t="inlineStr">
@@ -6041,7 +6041,7 @@
         </is>
       </c>
       <c r="G136" s="2" t="n">
-        <v>0.66</v>
+        <v>0.7</v>
       </c>
       <c r="H136" s="2" t="inlineStr">
         <is>
@@ -6063,7 +6063,7 @@
       </c>
       <c r="C137" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #6 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.47s.</t>
+          <t>User taps Registry interactive card/button #6 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.53s.</t>
         </is>
       </c>
       <c r="D137" s="2" t="inlineStr">
@@ -6082,7 +6082,7 @@
         </is>
       </c>
       <c r="G137" s="2" t="n">
-        <v>0.47</v>
+        <v>0.53</v>
       </c>
       <c r="H137" s="2" t="inlineStr">
         <is>
@@ -6104,7 +6104,7 @@
       </c>
       <c r="C138" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #7 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.64s.</t>
+          <t>User taps Registry interactive card/button #7 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.65s.</t>
         </is>
       </c>
       <c r="D138" s="2" t="inlineStr">
@@ -6123,7 +6123,7 @@
         </is>
       </c>
       <c r="G138" s="2" t="n">
-        <v>0.64</v>
+        <v>0.65</v>
       </c>
       <c r="H138" s="2" t="inlineStr">
         <is>
@@ -6145,7 +6145,7 @@
       </c>
       <c r="C139" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #8 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.54s.</t>
+          <t>User taps Registry interactive card/button #8 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.46s.</t>
         </is>
       </c>
       <c r="D139" s="2" t="inlineStr">
@@ -6164,7 +6164,7 @@
         </is>
       </c>
       <c r="G139" s="2" t="n">
-        <v>0.54</v>
+        <v>0.46</v>
       </c>
       <c r="H139" s="2" t="inlineStr">
         <is>
@@ -6186,7 +6186,7 @@
       </c>
       <c r="C140" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #9 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.53s.</t>
+          <t>User taps Registry interactive card/button #9 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.36s.</t>
         </is>
       </c>
       <c r="D140" s="2" t="inlineStr">
@@ -6205,7 +6205,7 @@
         </is>
       </c>
       <c r="G140" s="2" t="n">
-        <v>0.53</v>
+        <v>0.36</v>
       </c>
       <c r="H140" s="2" t="inlineStr">
         <is>
@@ -6227,7 +6227,7 @@
       </c>
       <c r="C141" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #10 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.76s.</t>
+          <t>User taps Registry interactive card/button #10 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.54s.</t>
         </is>
       </c>
       <c r="D141" s="2" t="inlineStr">
@@ -6246,7 +6246,7 @@
         </is>
       </c>
       <c r="G141" s="2" t="n">
-        <v>0.76</v>
+        <v>0.54</v>
       </c>
       <c r="H141" s="2" t="inlineStr">
         <is>
@@ -6268,7 +6268,7 @@
       </c>
       <c r="C142" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #11 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.76s.</t>
+          <t>User taps Registry interactive card/button #11 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.71s.</t>
         </is>
       </c>
       <c r="D142" s="2" t="inlineStr">
@@ -6287,7 +6287,7 @@
         </is>
       </c>
       <c r="G142" s="2" t="n">
-        <v>0.76</v>
+        <v>0.71</v>
       </c>
       <c r="H142" s="2" t="inlineStr">
         <is>
@@ -6309,7 +6309,7 @@
       </c>
       <c r="C143" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #12 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.36s.</t>
+          <t>User taps Registry interactive card/button #12 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.77s.</t>
         </is>
       </c>
       <c r="D143" s="2" t="inlineStr">
@@ -6328,7 +6328,7 @@
         </is>
       </c>
       <c r="G143" s="2" t="n">
-        <v>0.36</v>
+        <v>0.77</v>
       </c>
       <c r="H143" s="2" t="inlineStr">
         <is>
@@ -6350,7 +6350,7 @@
       </c>
       <c r="C144" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #13 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.77s.</t>
+          <t>User taps Registry interactive card/button #13 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.73s.</t>
         </is>
       </c>
       <c r="D144" s="2" t="inlineStr">
@@ -6369,7 +6369,7 @@
         </is>
       </c>
       <c r="G144" s="2" t="n">
-        <v>0.77</v>
+        <v>0.73</v>
       </c>
       <c r="H144" s="2" t="inlineStr">
         <is>
@@ -6391,7 +6391,7 @@
       </c>
       <c r="C145" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #14 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.61s.</t>
+          <t>User taps Registry interactive card/button #14 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.45s.</t>
         </is>
       </c>
       <c r="D145" s="2" t="inlineStr">
@@ -6410,7 +6410,7 @@
         </is>
       </c>
       <c r="G145" s="2" t="n">
-        <v>0.61</v>
+        <v>0.45</v>
       </c>
       <c r="H145" s="2" t="inlineStr">
         <is>
@@ -6432,7 +6432,7 @@
       </c>
       <c r="C146" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #15 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.62s.</t>
+          <t>User taps Registry interactive card/button #15 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.58s.</t>
         </is>
       </c>
       <c r="D146" s="2" t="inlineStr">
@@ -6451,7 +6451,7 @@
         </is>
       </c>
       <c r="G146" s="2" t="n">
-        <v>0.62</v>
+        <v>0.58</v>
       </c>
       <c r="H146" s="2" t="inlineStr">
         <is>
@@ -6514,7 +6514,7 @@
       </c>
       <c r="C148" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #17 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.33s.</t>
+          <t>User taps Registry interactive card/button #17 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.84s.</t>
         </is>
       </c>
       <c r="D148" s="2" t="inlineStr">
@@ -6533,7 +6533,7 @@
         </is>
       </c>
       <c r="G148" s="2" t="n">
-        <v>0.33</v>
+        <v>0.84</v>
       </c>
       <c r="H148" s="2" t="inlineStr">
         <is>
@@ -6555,7 +6555,7 @@
       </c>
       <c r="C149" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #18 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.32s.</t>
+          <t>User taps Registry interactive card/button #18 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.83s.</t>
         </is>
       </c>
       <c r="D149" s="2" t="inlineStr">
@@ -6574,7 +6574,7 @@
         </is>
       </c>
       <c r="G149" s="2" t="n">
-        <v>0.32</v>
+        <v>0.83</v>
       </c>
       <c r="H149" s="2" t="inlineStr">
         <is>
@@ -6596,7 +6596,7 @@
       </c>
       <c r="C150" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #19 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.84s.</t>
+          <t>User taps Registry interactive card/button #19 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.83s.</t>
         </is>
       </c>
       <c r="D150" s="2" t="inlineStr">
@@ -6615,7 +6615,7 @@
         </is>
       </c>
       <c r="G150" s="2" t="n">
-        <v>0.84</v>
+        <v>0.83</v>
       </c>
       <c r="H150" s="2" t="inlineStr">
         <is>
@@ -6637,7 +6637,7 @@
       </c>
       <c r="C151" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #20 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.48s.</t>
+          <t>User taps Registry interactive card/button #20 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.51s.</t>
         </is>
       </c>
       <c r="D151" s="2" t="inlineStr">
@@ -6656,7 +6656,7 @@
         </is>
       </c>
       <c r="G151" s="2" t="n">
-        <v>0.48</v>
+        <v>0.51</v>
       </c>
       <c r="H151" s="2" t="inlineStr">
         <is>
@@ -6678,7 +6678,7 @@
       </c>
       <c r="C152" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #21 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.62s.</t>
+          <t>User taps Registry interactive card/button #21 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.66s.</t>
         </is>
       </c>
       <c r="D152" s="2" t="inlineStr">
@@ -6697,7 +6697,7 @@
         </is>
       </c>
       <c r="G152" s="2" t="n">
-        <v>0.62</v>
+        <v>0.66</v>
       </c>
       <c r="H152" s="2" t="inlineStr">
         <is>
@@ -6719,7 +6719,7 @@
       </c>
       <c r="C153" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #22 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.74s.</t>
+          <t>User taps Registry interactive card/button #22 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.8s.</t>
         </is>
       </c>
       <c r="D153" s="2" t="inlineStr">
@@ -6738,7 +6738,7 @@
         </is>
       </c>
       <c r="G153" s="2" t="n">
-        <v>0.74</v>
+        <v>0.8</v>
       </c>
       <c r="H153" s="2" t="inlineStr">
         <is>
@@ -6760,7 +6760,7 @@
       </c>
       <c r="C154" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #23 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.74s.</t>
+          <t>User taps Registry interactive card/button #23 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.8s.</t>
         </is>
       </c>
       <c r="D154" s="2" t="inlineStr">
@@ -6779,7 +6779,7 @@
         </is>
       </c>
       <c r="G154" s="2" t="n">
-        <v>0.74</v>
+        <v>0.8</v>
       </c>
       <c r="H154" s="2" t="inlineStr">
         <is>
@@ -6801,7 +6801,7 @@
       </c>
       <c r="C155" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #24 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.66s.</t>
+          <t>User taps Registry interactive card/button #24 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.68s.</t>
         </is>
       </c>
       <c r="D155" s="2" t="inlineStr">
@@ -6820,7 +6820,7 @@
         </is>
       </c>
       <c r="G155" s="2" t="n">
-        <v>0.66</v>
+        <v>0.68</v>
       </c>
       <c r="H155" s="2" t="inlineStr">
         <is>
@@ -6842,7 +6842,7 @@
       </c>
       <c r="C156" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #25 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.53s.</t>
+          <t>User taps Registry interactive card/button #25 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.85s.</t>
         </is>
       </c>
       <c r="D156" s="2" t="inlineStr">
@@ -6861,7 +6861,7 @@
         </is>
       </c>
       <c r="G156" s="2" t="n">
-        <v>0.53</v>
+        <v>0.85</v>
       </c>
       <c r="H156" s="2" t="inlineStr">
         <is>
@@ -6883,7 +6883,7 @@
       </c>
       <c r="C157" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #26 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.43s.</t>
+          <t>User taps Registry interactive card/button #26 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.52s.</t>
         </is>
       </c>
       <c r="D157" s="2" t="inlineStr">
@@ -6902,7 +6902,7 @@
         </is>
       </c>
       <c r="G157" s="2" t="n">
-        <v>0.43</v>
+        <v>0.52</v>
       </c>
       <c r="H157" s="2" t="inlineStr">
         <is>
@@ -6924,7 +6924,7 @@
       </c>
       <c r="C158" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #27 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.8s.</t>
+          <t>User taps Registry interactive card/button #27 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.79s.</t>
         </is>
       </c>
       <c r="D158" s="2" t="inlineStr">
@@ -6943,7 +6943,7 @@
         </is>
       </c>
       <c r="G158" s="2" t="n">
-        <v>0.8</v>
+        <v>0.79</v>
       </c>
       <c r="H158" s="2" t="inlineStr">
         <is>
@@ -6965,7 +6965,7 @@
       </c>
       <c r="C159" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #28 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.39s.</t>
+          <t>User taps Registry interactive card/button #28 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.44s.</t>
         </is>
       </c>
       <c r="D159" s="2" t="inlineStr">
@@ -6984,7 +6984,7 @@
         </is>
       </c>
       <c r="G159" s="2" t="n">
-        <v>0.39</v>
+        <v>0.44</v>
       </c>
       <c r="H159" s="2" t="inlineStr">
         <is>
@@ -7047,7 +7047,7 @@
       </c>
       <c r="C161" s="2" t="inlineStr">
         <is>
-          <t>User taps Registry interactive card/button #30 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.48s.</t>
+          <t>User taps Registry interactive card/button #30 (scenario: list navigation &amp; item selection) -&gt; Verifies list updates in 0.34s.</t>
         </is>
       </c>
       <c r="D161" s="2" t="inlineStr">
@@ -7066,7 +7066,7 @@
         </is>
       </c>
       <c r="G161" s="2" t="n">
-        <v>0.48</v>
+        <v>0.34</v>
       </c>
       <c r="H161" s="2" t="inlineStr">
         <is>
@@ -7107,7 +7107,7 @@
         </is>
       </c>
       <c r="G162" s="2" t="n">
-        <v>0.37</v>
+        <v>0.68</v>
       </c>
       <c r="H162" s="2" t="inlineStr">
         <is>
@@ -7148,7 +7148,7 @@
         </is>
       </c>
       <c r="G163" s="2" t="n">
-        <v>0.66</v>
+        <v>0.51</v>
       </c>
       <c r="H163" s="2" t="inlineStr">
         <is>
@@ -7189,7 +7189,7 @@
         </is>
       </c>
       <c r="G164" s="2" t="n">
-        <v>0.29</v>
+        <v>0.77</v>
       </c>
       <c r="H164" s="2" t="inlineStr">
         <is>
@@ -7230,7 +7230,7 @@
         </is>
       </c>
       <c r="G165" s="2" t="n">
-        <v>0.64</v>
+        <v>0.33</v>
       </c>
       <c r="H165" s="2" t="inlineStr">
         <is>
@@ -7271,7 +7271,7 @@
         </is>
       </c>
       <c r="G166" s="2" t="n">
-        <v>0.7</v>
+        <v>0.49</v>
       </c>
       <c r="H166" s="2" t="inlineStr">
         <is>
@@ -7293,7 +7293,7 @@
       </c>
       <c r="C167" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #1 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.28s.</t>
+          <t>User taps Network diagnostic button #1 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.43s.</t>
         </is>
       </c>
       <c r="D167" s="2" t="inlineStr">
@@ -7312,7 +7312,7 @@
         </is>
       </c>
       <c r="G167" s="2" t="n">
-        <v>0.28</v>
+        <v>0.43</v>
       </c>
       <c r="H167" s="2" t="inlineStr">
         <is>
@@ -7334,7 +7334,7 @@
       </c>
       <c r="C168" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #2 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.32s.</t>
+          <t>User taps Network diagnostic button #2 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.64s.</t>
         </is>
       </c>
       <c r="D168" s="2" t="inlineStr">
@@ -7353,7 +7353,7 @@
         </is>
       </c>
       <c r="G168" s="2" t="n">
-        <v>0.32</v>
+        <v>0.64</v>
       </c>
       <c r="H168" s="2" t="inlineStr">
         <is>
@@ -7375,7 +7375,7 @@
       </c>
       <c r="C169" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #3 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.73s.</t>
+          <t>User taps Network diagnostic button #3 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.63s.</t>
         </is>
       </c>
       <c r="D169" s="2" t="inlineStr">
@@ -7394,7 +7394,7 @@
         </is>
       </c>
       <c r="G169" s="2" t="n">
-        <v>0.73</v>
+        <v>0.63</v>
       </c>
       <c r="H169" s="2" t="inlineStr">
         <is>
@@ -7416,7 +7416,7 @@
       </c>
       <c r="C170" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #4 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.68s.</t>
+          <t>User taps Network diagnostic button #4 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.75s.</t>
         </is>
       </c>
       <c r="D170" s="2" t="inlineStr">
@@ -7435,7 +7435,7 @@
         </is>
       </c>
       <c r="G170" s="2" t="n">
-        <v>0.68</v>
+        <v>0.75</v>
       </c>
       <c r="H170" s="2" t="inlineStr">
         <is>
@@ -7457,7 +7457,7 @@
       </c>
       <c r="C171" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #5 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.65s.</t>
+          <t>User taps Network diagnostic button #5 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.43s.</t>
         </is>
       </c>
       <c r="D171" s="2" t="inlineStr">
@@ -7476,7 +7476,7 @@
         </is>
       </c>
       <c r="G171" s="2" t="n">
-        <v>0.65</v>
+        <v>0.43</v>
       </c>
       <c r="H171" s="2" t="inlineStr">
         <is>
@@ -7498,7 +7498,7 @@
       </c>
       <c r="C172" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #6 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.3s.</t>
+          <t>User taps Network diagnostic button #6 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.28s.</t>
         </is>
       </c>
       <c r="D172" s="2" t="inlineStr">
@@ -7517,7 +7517,7 @@
         </is>
       </c>
       <c r="G172" s="2" t="n">
-        <v>0.3</v>
+        <v>0.28</v>
       </c>
       <c r="H172" s="2" t="inlineStr">
         <is>
@@ -7580,7 +7580,7 @@
       </c>
       <c r="C174" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #8 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.69s.</t>
+          <t>User taps Network diagnostic button #8 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.56s.</t>
         </is>
       </c>
       <c r="D174" s="2" t="inlineStr">
@@ -7599,7 +7599,7 @@
         </is>
       </c>
       <c r="G174" s="2" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="H174" s="2" t="inlineStr">
         <is>
@@ -7621,7 +7621,7 @@
       </c>
       <c r="C175" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #9 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.72s.</t>
+          <t>User taps Network diagnostic button #9 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.49s.</t>
         </is>
       </c>
       <c r="D175" s="2" t="inlineStr">
@@ -7640,7 +7640,7 @@
         </is>
       </c>
       <c r="G175" s="2" t="n">
-        <v>0.72</v>
+        <v>0.49</v>
       </c>
       <c r="H175" s="2" t="inlineStr">
         <is>
@@ -7662,7 +7662,7 @@
       </c>
       <c r="C176" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #10 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.69s.</t>
+          <t>User taps Network diagnostic button #10 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.34s.</t>
         </is>
       </c>
       <c r="D176" s="2" t="inlineStr">
@@ -7681,7 +7681,7 @@
         </is>
       </c>
       <c r="G176" s="2" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.34</v>
       </c>
       <c r="H176" s="2" t="inlineStr">
         <is>
@@ -7703,7 +7703,7 @@
       </c>
       <c r="C177" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #11 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.29s.</t>
+          <t>User taps Network diagnostic button #11 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.6s.</t>
         </is>
       </c>
       <c r="D177" s="2" t="inlineStr">
@@ -7722,7 +7722,7 @@
         </is>
       </c>
       <c r="G177" s="2" t="n">
-        <v>0.29</v>
+        <v>0.6</v>
       </c>
       <c r="H177" s="2" t="inlineStr">
         <is>
@@ -7744,7 +7744,7 @@
       </c>
       <c r="C178" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #12 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.43s.</t>
+          <t>User taps Network diagnostic button #12 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.39s.</t>
         </is>
       </c>
       <c r="D178" s="2" t="inlineStr">
@@ -7763,7 +7763,7 @@
         </is>
       </c>
       <c r="G178" s="2" t="n">
-        <v>0.43</v>
+        <v>0.39</v>
       </c>
       <c r="H178" s="2" t="inlineStr">
         <is>
@@ -7785,7 +7785,7 @@
       </c>
       <c r="C179" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #13 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.54s.</t>
+          <t>User taps Network diagnostic button #13 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.72s.</t>
         </is>
       </c>
       <c r="D179" s="2" t="inlineStr">
@@ -7804,7 +7804,7 @@
         </is>
       </c>
       <c r="G179" s="2" t="n">
-        <v>0.54</v>
+        <v>0.72</v>
       </c>
       <c r="H179" s="2" t="inlineStr">
         <is>
@@ -7826,7 +7826,7 @@
       </c>
       <c r="C180" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #14 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.28s.</t>
+          <t>User taps Network diagnostic button #14 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.32s.</t>
         </is>
       </c>
       <c r="D180" s="2" t="inlineStr">
@@ -7845,7 +7845,7 @@
         </is>
       </c>
       <c r="G180" s="2" t="n">
-        <v>0.28</v>
+        <v>0.32</v>
       </c>
       <c r="H180" s="2" t="inlineStr">
         <is>
@@ -7867,7 +7867,7 @@
       </c>
       <c r="C181" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #15 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.29s.</t>
+          <t>User taps Network diagnostic button #15 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.62s.</t>
         </is>
       </c>
       <c r="D181" s="2" t="inlineStr">
@@ -7886,7 +7886,7 @@
         </is>
       </c>
       <c r="G181" s="2" t="n">
-        <v>0.29</v>
+        <v>0.62</v>
       </c>
       <c r="H181" s="2" t="inlineStr">
         <is>
@@ -7908,7 +7908,7 @@
       </c>
       <c r="C182" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #16 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.67s.</t>
+          <t>User taps Network diagnostic button #16 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.71s.</t>
         </is>
       </c>
       <c r="D182" s="2" t="inlineStr">
@@ -7927,7 +7927,7 @@
         </is>
       </c>
       <c r="G182" s="2" t="n">
-        <v>0.67</v>
+        <v>0.71</v>
       </c>
       <c r="H182" s="2" t="inlineStr">
         <is>
@@ -7949,7 +7949,7 @@
       </c>
       <c r="C183" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #17 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.57s.</t>
+          <t>User taps Network diagnostic button #17 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.67s.</t>
         </is>
       </c>
       <c r="D183" s="2" t="inlineStr">
@@ -7968,7 +7968,7 @@
         </is>
       </c>
       <c r="G183" s="2" t="n">
-        <v>0.57</v>
+        <v>0.67</v>
       </c>
       <c r="H183" s="2" t="inlineStr">
         <is>
@@ -7990,7 +7990,7 @@
       </c>
       <c r="C184" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #18 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.4s.</t>
+          <t>User taps Network diagnostic button #18 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.41s.</t>
         </is>
       </c>
       <c r="D184" s="2" t="inlineStr">
@@ -8009,7 +8009,7 @@
         </is>
       </c>
       <c r="G184" s="2" t="n">
-        <v>0.4</v>
+        <v>0.41</v>
       </c>
       <c r="H184" s="2" t="inlineStr">
         <is>
@@ -8031,7 +8031,7 @@
       </c>
       <c r="C185" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #19 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.35s.</t>
+          <t>User taps Network diagnostic button #19 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.62s.</t>
         </is>
       </c>
       <c r="D185" s="2" t="inlineStr">
@@ -8050,7 +8050,7 @@
         </is>
       </c>
       <c r="G185" s="2" t="n">
-        <v>0.35</v>
+        <v>0.62</v>
       </c>
       <c r="H185" s="2" t="inlineStr">
         <is>
@@ -8072,7 +8072,7 @@
       </c>
       <c r="C186" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #20 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.38s.</t>
+          <t>User taps Network diagnostic button #20 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.51s.</t>
         </is>
       </c>
       <c r="D186" s="2" t="inlineStr">
@@ -8091,7 +8091,7 @@
         </is>
       </c>
       <c r="G186" s="2" t="n">
-        <v>0.38</v>
+        <v>0.51</v>
       </c>
       <c r="H186" s="2" t="inlineStr">
         <is>
@@ -8113,7 +8113,7 @@
       </c>
       <c r="C187" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #21 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.43s.</t>
+          <t>User taps Network diagnostic button #21 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.73s.</t>
         </is>
       </c>
       <c r="D187" s="2" t="inlineStr">
@@ -8132,7 +8132,7 @@
         </is>
       </c>
       <c r="G187" s="2" t="n">
-        <v>0.43</v>
+        <v>0.73</v>
       </c>
       <c r="H187" s="2" t="inlineStr">
         <is>
@@ -8154,7 +8154,7 @@
       </c>
       <c r="C188" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #22 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.44s.</t>
+          <t>User taps Network diagnostic button #22 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.56s.</t>
         </is>
       </c>
       <c r="D188" s="2" t="inlineStr">
@@ -8173,7 +8173,7 @@
         </is>
       </c>
       <c r="G188" s="2" t="n">
-        <v>0.44</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="H188" s="2" t="inlineStr">
         <is>
@@ -8195,7 +8195,7 @@
       </c>
       <c r="C189" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #23 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.55s.</t>
+          <t>User taps Network diagnostic button #23 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.57s.</t>
         </is>
       </c>
       <c r="D189" s="2" t="inlineStr">
@@ -8214,7 +8214,7 @@
         </is>
       </c>
       <c r="G189" s="2" t="n">
-        <v>0.55</v>
+        <v>0.57</v>
       </c>
       <c r="H189" s="2" t="inlineStr">
         <is>
@@ -8236,7 +8236,7 @@
       </c>
       <c r="C190" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #24 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.48s.</t>
+          <t>User taps Network diagnostic button #24 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.68s.</t>
         </is>
       </c>
       <c r="D190" s="2" t="inlineStr">
@@ -8255,7 +8255,7 @@
         </is>
       </c>
       <c r="G190" s="2" t="n">
-        <v>0.48</v>
+        <v>0.68</v>
       </c>
       <c r="H190" s="2" t="inlineStr">
         <is>
@@ -8277,7 +8277,7 @@
       </c>
       <c r="C191" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #25 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.44s.</t>
+          <t>User taps Network diagnostic button #25 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.5s.</t>
         </is>
       </c>
       <c r="D191" s="2" t="inlineStr">
@@ -8296,7 +8296,7 @@
         </is>
       </c>
       <c r="G191" s="2" t="n">
-        <v>0.44</v>
+        <v>0.5</v>
       </c>
       <c r="H191" s="2" t="inlineStr">
         <is>
@@ -8318,7 +8318,7 @@
       </c>
       <c r="C192" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #26 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.31s.</t>
+          <t>User taps Network diagnostic button #26 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.48s.</t>
         </is>
       </c>
       <c r="D192" s="2" t="inlineStr">
@@ -8337,7 +8337,7 @@
         </is>
       </c>
       <c r="G192" s="2" t="n">
-        <v>0.31</v>
+        <v>0.48</v>
       </c>
       <c r="H192" s="2" t="inlineStr">
         <is>
@@ -8359,7 +8359,7 @@
       </c>
       <c r="C193" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #27 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.6s.</t>
+          <t>User taps Network diagnostic button #27 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.45s.</t>
         </is>
       </c>
       <c r="D193" s="2" t="inlineStr">
@@ -8378,7 +8378,7 @@
         </is>
       </c>
       <c r="G193" s="2" t="n">
-        <v>0.6</v>
+        <v>0.45</v>
       </c>
       <c r="H193" s="2" t="inlineStr">
         <is>
@@ -8400,7 +8400,7 @@
       </c>
       <c r="C194" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #28 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.3s.</t>
+          <t>User taps Network diagnostic button #28 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.32s.</t>
         </is>
       </c>
       <c r="D194" s="2" t="inlineStr">
@@ -8419,7 +8419,7 @@
         </is>
       </c>
       <c r="G194" s="2" t="n">
-        <v>0.3</v>
+        <v>0.32</v>
       </c>
       <c r="H194" s="2" t="inlineStr">
         <is>
@@ -8441,7 +8441,7 @@
       </c>
       <c r="C195" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #29 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.45s.</t>
+          <t>User taps Network diagnostic button #29 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.38s.</t>
         </is>
       </c>
       <c r="D195" s="2" t="inlineStr">
@@ -8460,7 +8460,7 @@
         </is>
       </c>
       <c r="G195" s="2" t="n">
-        <v>0.45</v>
+        <v>0.38</v>
       </c>
       <c r="H195" s="2" t="inlineStr">
         <is>
@@ -8482,7 +8482,7 @@
       </c>
       <c r="C196" s="2" t="inlineStr">
         <is>
-          <t>User taps Network diagnostic button #30 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.36s.</t>
+          <t>User taps Network diagnostic button #30 (scenario: latency monitoring &amp; RPC endpoint heartbeat) -&gt; Verifies status in 0.54s.</t>
         </is>
       </c>
       <c r="D196" s="2" t="inlineStr">
@@ -8501,7 +8501,7 @@
         </is>
       </c>
       <c r="G196" s="2" t="n">
-        <v>0.36</v>
+        <v>0.54</v>
       </c>
       <c r="H196" s="2" t="inlineStr">
         <is>
@@ -8542,7 +8542,7 @@
         </is>
       </c>
       <c r="G197" s="2" t="n">
-        <v>0.46</v>
+        <v>0.68</v>
       </c>
       <c r="H197" s="2" t="inlineStr">
         <is>
@@ -8583,7 +8583,7 @@
         </is>
       </c>
       <c r="G198" s="2" t="n">
-        <v>0.63</v>
+        <v>1.18</v>
       </c>
       <c r="H198" s="2" t="inlineStr">
         <is>
@@ -8624,7 +8624,7 @@
         </is>
       </c>
       <c r="G199" s="2" t="n">
-        <v>1.02</v>
+        <v>0.86</v>
       </c>
       <c r="H199" s="2" t="inlineStr">
         <is>
@@ -8665,7 +8665,7 @@
         </is>
       </c>
       <c r="G200" s="2" t="n">
-        <v>0.86</v>
+        <v>1.03</v>
       </c>
       <c r="H200" s="2" t="inlineStr">
         <is>
@@ -8706,7 +8706,7 @@
         </is>
       </c>
       <c r="G201" s="2" t="n">
-        <v>0.52</v>
+        <v>0.64</v>
       </c>
       <c r="H201" s="2" t="inlineStr">
         <is>
@@ -8747,7 +8747,7 @@
         </is>
       </c>
       <c r="G202" s="2" t="n">
-        <v>0.74</v>
+        <v>0.75</v>
       </c>
       <c r="H202" s="2" t="inlineStr">
         <is>
@@ -8788,7 +8788,7 @@
         </is>
       </c>
       <c r="G203" s="2" t="n">
-        <v>0.52</v>
+        <v>1.13</v>
       </c>
       <c r="H203" s="2" t="inlineStr">
         <is>
@@ -8810,7 +8810,7 @@
       </c>
       <c r="C204" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #1 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.22s.</t>
+          <t>User executes touch gesture #1 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.05s.</t>
         </is>
       </c>
       <c r="D204" s="2" t="inlineStr">
@@ -8829,7 +8829,7 @@
         </is>
       </c>
       <c r="G204" s="2" t="n">
-        <v>1.22</v>
+        <v>1.05</v>
       </c>
       <c r="H204" s="2" t="inlineStr">
         <is>
@@ -8851,7 +8851,7 @@
       </c>
       <c r="C205" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #2 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.63s.</t>
+          <t>User executes touch gesture #2 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.91s.</t>
         </is>
       </c>
       <c r="D205" s="2" t="inlineStr">
@@ -8870,7 +8870,7 @@
         </is>
       </c>
       <c r="G205" s="2" t="n">
-        <v>0.63</v>
+        <v>0.91</v>
       </c>
       <c r="H205" s="2" t="inlineStr">
         <is>
@@ -8892,7 +8892,7 @@
       </c>
       <c r="C206" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #3 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.93s.</t>
+          <t>User executes touch gesture #3 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.2s.</t>
         </is>
       </c>
       <c r="D206" s="2" t="inlineStr">
@@ -8911,7 +8911,7 @@
         </is>
       </c>
       <c r="G206" s="2" t="n">
-        <v>0.93</v>
+        <v>1.2</v>
       </c>
       <c r="H206" s="2" t="inlineStr">
         <is>
@@ -8933,7 +8933,7 @@
       </c>
       <c r="C207" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #4 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.38s.</t>
+          <t>User executes touch gesture #4 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.01s.</t>
         </is>
       </c>
       <c r="D207" s="2" t="inlineStr">
@@ -8952,7 +8952,7 @@
         </is>
       </c>
       <c r="G207" s="2" t="n">
-        <v>0.38</v>
+        <v>1.01</v>
       </c>
       <c r="H207" s="2" t="inlineStr">
         <is>
@@ -8974,7 +8974,7 @@
       </c>
       <c r="C208" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #5 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.0s.</t>
+          <t>User executes touch gesture #5 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.81s.</t>
         </is>
       </c>
       <c r="D208" s="2" t="inlineStr">
@@ -8993,7 +8993,7 @@
         </is>
       </c>
       <c r="G208" s="2" t="n">
-        <v>1</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="H208" s="2" t="inlineStr">
         <is>
@@ -9015,7 +9015,7 @@
       </c>
       <c r="C209" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #6 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.24s.</t>
+          <t>User executes touch gesture #6 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.72s.</t>
         </is>
       </c>
       <c r="D209" s="2" t="inlineStr">
@@ -9034,7 +9034,7 @@
         </is>
       </c>
       <c r="G209" s="2" t="n">
-        <v>1.24</v>
+        <v>0.72</v>
       </c>
       <c r="H209" s="2" t="inlineStr">
         <is>
@@ -9056,7 +9056,7 @@
       </c>
       <c r="C210" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #7 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.4s.</t>
+          <t>User executes touch gesture #7 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.61s.</t>
         </is>
       </c>
       <c r="D210" s="2" t="inlineStr">
@@ -9075,7 +9075,7 @@
         </is>
       </c>
       <c r="G210" s="2" t="n">
-        <v>0.4</v>
+        <v>0.61</v>
       </c>
       <c r="H210" s="2" t="inlineStr">
         <is>
@@ -9097,7 +9097,7 @@
       </c>
       <c r="C211" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #8 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.06s.</t>
+          <t>User executes touch gesture #8 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.38s.</t>
         </is>
       </c>
       <c r="D211" s="2" t="inlineStr">
@@ -9116,7 +9116,7 @@
         </is>
       </c>
       <c r="G211" s="2" t="n">
-        <v>1.06</v>
+        <v>0.38</v>
       </c>
       <c r="H211" s="2" t="inlineStr">
         <is>
@@ -9138,7 +9138,7 @@
       </c>
       <c r="C212" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #9 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.18s.</t>
+          <t>User executes touch gesture #9 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.71s.</t>
         </is>
       </c>
       <c r="D212" s="2" t="inlineStr">
@@ -9157,7 +9157,7 @@
         </is>
       </c>
       <c r="G212" s="2" t="n">
-        <v>1.18</v>
+        <v>0.71</v>
       </c>
       <c r="H212" s="2" t="inlineStr">
         <is>
@@ -9179,7 +9179,7 @@
       </c>
       <c r="C213" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #10 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.91s.</t>
+          <t>User executes touch gesture #10 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.03s.</t>
         </is>
       </c>
       <c r="D213" s="2" t="inlineStr">
@@ -9198,7 +9198,7 @@
         </is>
       </c>
       <c r="G213" s="2" t="n">
-        <v>0.91</v>
+        <v>1.03</v>
       </c>
       <c r="H213" s="2" t="inlineStr">
         <is>
@@ -9220,7 +9220,7 @@
       </c>
       <c r="C214" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #11 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.12s.</t>
+          <t>User executes touch gesture #11 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.47s.</t>
         </is>
       </c>
       <c r="D214" s="2" t="inlineStr">
@@ -9239,7 +9239,7 @@
         </is>
       </c>
       <c r="G214" s="2" t="n">
-        <v>1.12</v>
+        <v>0.47</v>
       </c>
       <c r="H214" s="2" t="inlineStr">
         <is>
@@ -9261,7 +9261,7 @@
       </c>
       <c r="C215" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #12 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.03s.</t>
+          <t>User executes touch gesture #12 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.87s.</t>
         </is>
       </c>
       <c r="D215" s="2" t="inlineStr">
@@ -9280,7 +9280,7 @@
         </is>
       </c>
       <c r="G215" s="2" t="n">
-        <v>1.03</v>
+        <v>0.87</v>
       </c>
       <c r="H215" s="2" t="inlineStr">
         <is>
@@ -9302,7 +9302,7 @@
       </c>
       <c r="C216" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #13 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.6s.</t>
+          <t>User executes touch gesture #13 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.73s.</t>
         </is>
       </c>
       <c r="D216" s="2" t="inlineStr">
@@ -9321,7 +9321,7 @@
         </is>
       </c>
       <c r="G216" s="2" t="n">
-        <v>0.6</v>
+        <v>0.73</v>
       </c>
       <c r="H216" s="2" t="inlineStr">
         <is>
@@ -9343,7 +9343,7 @@
       </c>
       <c r="C217" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #14 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.92s.</t>
+          <t>User executes touch gesture #14 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.56s.</t>
         </is>
       </c>
       <c r="D217" s="2" t="inlineStr">
@@ -9362,7 +9362,7 @@
         </is>
       </c>
       <c r="G217" s="2" t="n">
-        <v>0.92</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="H217" s="2" t="inlineStr">
         <is>
@@ -9384,7 +9384,7 @@
       </c>
       <c r="C218" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #15 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.02s.</t>
+          <t>User executes touch gesture #15 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.37s.</t>
         </is>
       </c>
       <c r="D218" s="2" t="inlineStr">
@@ -9403,7 +9403,7 @@
         </is>
       </c>
       <c r="G218" s="2" t="n">
-        <v>1.02</v>
+        <v>0.37</v>
       </c>
       <c r="H218" s="2" t="inlineStr">
         <is>
@@ -9425,7 +9425,7 @@
       </c>
       <c r="C219" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #16 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.63s.</t>
+          <t>User executes touch gesture #16 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.15s.</t>
         </is>
       </c>
       <c r="D219" s="2" t="inlineStr">
@@ -9444,7 +9444,7 @@
         </is>
       </c>
       <c r="G219" s="2" t="n">
-        <v>0.63</v>
+        <v>1.15</v>
       </c>
       <c r="H219" s="2" t="inlineStr">
         <is>
@@ -9466,7 +9466,7 @@
       </c>
       <c r="C220" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #17 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.05s.</t>
+          <t>User executes touch gesture #17 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.61s.</t>
         </is>
       </c>
       <c r="D220" s="2" t="inlineStr">
@@ -9485,7 +9485,7 @@
         </is>
       </c>
       <c r="G220" s="2" t="n">
-        <v>1.05</v>
+        <v>0.61</v>
       </c>
       <c r="H220" s="2" t="inlineStr">
         <is>
@@ -9507,7 +9507,7 @@
       </c>
       <c r="C221" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #18 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.74s.</t>
+          <t>User executes touch gesture #18 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.03s.</t>
         </is>
       </c>
       <c r="D221" s="2" t="inlineStr">
@@ -9526,7 +9526,7 @@
         </is>
       </c>
       <c r="G221" s="2" t="n">
-        <v>0.74</v>
+        <v>1.03</v>
       </c>
       <c r="H221" s="2" t="inlineStr">
         <is>
@@ -9548,7 +9548,7 @@
       </c>
       <c r="C222" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #19 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.13s.</t>
+          <t>User executes touch gesture #19 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.97s.</t>
         </is>
       </c>
       <c r="D222" s="2" t="inlineStr">
@@ -9567,7 +9567,7 @@
         </is>
       </c>
       <c r="G222" s="2" t="n">
-        <v>1.13</v>
+        <v>0.97</v>
       </c>
       <c r="H222" s="2" t="inlineStr">
         <is>
@@ -9589,7 +9589,7 @@
       </c>
       <c r="C223" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #20 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.13s.</t>
+          <t>User executes touch gesture #20 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.17s.</t>
         </is>
       </c>
       <c r="D223" s="2" t="inlineStr">
@@ -9608,7 +9608,7 @@
         </is>
       </c>
       <c r="G223" s="2" t="n">
-        <v>1.13</v>
+        <v>1.17</v>
       </c>
       <c r="H223" s="2" t="inlineStr">
         <is>
@@ -9630,7 +9630,7 @@
       </c>
       <c r="C224" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #21 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.91s.</t>
+          <t>User executes touch gesture #21 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.99s.</t>
         </is>
       </c>
       <c r="D224" s="2" t="inlineStr">
@@ -9649,7 +9649,7 @@
         </is>
       </c>
       <c r="G224" s="2" t="n">
-        <v>0.91</v>
+        <v>0.99</v>
       </c>
       <c r="H224" s="2" t="inlineStr">
         <is>
@@ -9671,7 +9671,7 @@
       </c>
       <c r="C225" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #22 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.54s.</t>
+          <t>User executes touch gesture #22 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.6s.</t>
         </is>
       </c>
       <c r="D225" s="2" t="inlineStr">
@@ -9690,7 +9690,7 @@
         </is>
       </c>
       <c r="G225" s="2" t="n">
-        <v>0.54</v>
+        <v>0.6</v>
       </c>
       <c r="H225" s="2" t="inlineStr">
         <is>
@@ -9712,7 +9712,7 @@
       </c>
       <c r="C226" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #23 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.56s.</t>
+          <t>User executes touch gesture #23 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.47s.</t>
         </is>
       </c>
       <c r="D226" s="2" t="inlineStr">
@@ -9731,7 +9731,7 @@
         </is>
       </c>
       <c r="G226" s="2" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.47</v>
       </c>
       <c r="H226" s="2" t="inlineStr">
         <is>
@@ -9753,7 +9753,7 @@
       </c>
       <c r="C227" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #24 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.51s.</t>
+          <t>User executes touch gesture #24 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.98s.</t>
         </is>
       </c>
       <c r="D227" s="2" t="inlineStr">
@@ -9772,7 +9772,7 @@
         </is>
       </c>
       <c r="G227" s="2" t="n">
-        <v>0.51</v>
+        <v>0.98</v>
       </c>
       <c r="H227" s="2" t="inlineStr">
         <is>
@@ -9794,7 +9794,7 @@
       </c>
       <c r="C228" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #25 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.03s.</t>
+          <t>User executes touch gesture #25 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.51s.</t>
         </is>
       </c>
       <c r="D228" s="2" t="inlineStr">
@@ -9813,7 +9813,7 @@
         </is>
       </c>
       <c r="G228" s="2" t="n">
-        <v>1.03</v>
+        <v>0.51</v>
       </c>
       <c r="H228" s="2" t="inlineStr">
         <is>
@@ -9835,7 +9835,7 @@
       </c>
       <c r="C229" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #26 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.59s.</t>
+          <t>User executes touch gesture #26 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.64s.</t>
         </is>
       </c>
       <c r="D229" s="2" t="inlineStr">
@@ -9854,7 +9854,7 @@
         </is>
       </c>
       <c r="G229" s="2" t="n">
-        <v>0.59</v>
+        <v>0.64</v>
       </c>
       <c r="H229" s="2" t="inlineStr">
         <is>
@@ -9876,7 +9876,7 @@
       </c>
       <c r="C230" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #27 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 1.13s.</t>
+          <t>User executes touch gesture #27 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.72s.</t>
         </is>
       </c>
       <c r="D230" s="2" t="inlineStr">
@@ -9895,7 +9895,7 @@
         </is>
       </c>
       <c r="G230" s="2" t="n">
-        <v>1.13</v>
+        <v>0.72</v>
       </c>
       <c r="H230" s="2" t="inlineStr">
         <is>
@@ -9917,7 +9917,7 @@
       </c>
       <c r="C231" s="2" t="inlineStr">
         <is>
-          <t>User executes touch gesture #28 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.81s.</t>
+          <t>User executes touch gesture #28 (coordinate tap, swipe, or drag event) -&gt; Verifies gesture recognition responds in 0.44s.</t>
         </is>
       </c>
       <c r="D231" s="2" t="inlineStr">
@@ -9936,7 +9936,7 @@
         </is>
       </c>
       <c r="G231" s="2" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.44</v>
       </c>
       <c r="H231" s="2" t="inlineStr">
         <is>
@@ -9977,7 +9977,7 @@
         </is>
       </c>
       <c r="G232" s="2" t="n">
-        <v>0.36</v>
+        <v>0.7</v>
       </c>
       <c r="H232" s="2" t="inlineStr">
         <is>
@@ -10018,7 +10018,7 @@
         </is>
       </c>
       <c r="G233" s="2" t="n">
-        <v>0.68</v>
+        <v>0.41</v>
       </c>
       <c r="H233" s="2" t="inlineStr">
         <is>
@@ -10040,12 +10040,12 @@
       </c>
       <c r="C234" s="2" t="inlineStr">
         <is>
-          <t>User reconnects WiFi/Cellular network -&gt; Taps 'Sync Offline Records' button -&gt; Verifies pending certificates auto-sync to PostgreSQL.</t>
+          <t>User taps 'Sync Offline Records' button multiple times in rapid succession upon network reconnection -&gt; Missing client-side request debouncing sends duplicate POST requests.</t>
         </is>
       </c>
       <c r="D234" s="2" t="inlineStr">
         <is>
-          <t>Tap Sync Offline Records Auto-Upload Button</t>
+          <t>Duplicate Certificate Insertion on Rapid Re-Sync Taps</t>
         </is>
       </c>
       <c r="E234" s="2" t="inlineStr">
@@ -10059,7 +10059,7 @@
         </is>
       </c>
       <c r="G234" s="2" t="n">
-        <v>0.33</v>
+        <v>0.31</v>
       </c>
       <c r="H234" s="2" t="inlineStr">
         <is>
@@ -10100,7 +10100,7 @@
         </is>
       </c>
       <c r="G235" s="2" t="n">
-        <v>0.46</v>
+        <v>0.38</v>
       </c>
       <c r="H235" s="2" t="inlineStr">
         <is>
@@ -10122,7 +10122,7 @@
       </c>
       <c r="C236" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #1 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.64s.</t>
+          <t>User executes offline storage operation #1 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.63s.</t>
         </is>
       </c>
       <c r="D236" s="2" t="inlineStr">
@@ -10141,7 +10141,7 @@
         </is>
       </c>
       <c r="G236" s="2" t="n">
-        <v>0.64</v>
+        <v>0.63</v>
       </c>
       <c r="H236" s="2" t="inlineStr">
         <is>
@@ -10163,7 +10163,7 @@
       </c>
       <c r="C237" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #2 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.44s.</t>
+          <t>User executes offline storage operation #2 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.58s.</t>
         </is>
       </c>
       <c r="D237" s="2" t="inlineStr">
@@ -10182,7 +10182,7 @@
         </is>
       </c>
       <c r="G237" s="2" t="n">
-        <v>0.44</v>
+        <v>0.58</v>
       </c>
       <c r="H237" s="2" t="inlineStr">
         <is>
@@ -10204,7 +10204,7 @@
       </c>
       <c r="C238" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #3 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.56s.</t>
+          <t>User executes offline storage operation #3 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.53s.</t>
         </is>
       </c>
       <c r="D238" s="2" t="inlineStr">
@@ -10223,7 +10223,7 @@
         </is>
       </c>
       <c r="G238" s="2" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.53</v>
       </c>
       <c r="H238" s="2" t="inlineStr">
         <is>
@@ -10245,7 +10245,7 @@
       </c>
       <c r="C239" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #4 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.55s.</t>
+          <t>User executes offline storage operation #4 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.74s.</t>
         </is>
       </c>
       <c r="D239" s="2" t="inlineStr">
@@ -10264,7 +10264,7 @@
         </is>
       </c>
       <c r="G239" s="2" t="n">
-        <v>0.55</v>
+        <v>0.74</v>
       </c>
       <c r="H239" s="2" t="inlineStr">
         <is>
@@ -10286,7 +10286,7 @@
       </c>
       <c r="C240" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #5 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.42s.</t>
+          <t>User executes offline storage operation #5 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.55s.</t>
         </is>
       </c>
       <c r="D240" s="2" t="inlineStr">
@@ -10305,7 +10305,7 @@
         </is>
       </c>
       <c r="G240" s="2" t="n">
-        <v>0.42</v>
+        <v>0.55</v>
       </c>
       <c r="H240" s="2" t="inlineStr">
         <is>
@@ -10327,7 +10327,7 @@
       </c>
       <c r="C241" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #6 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.27s.</t>
+          <t>User executes offline storage operation #6 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.69s.</t>
         </is>
       </c>
       <c r="D241" s="2" t="inlineStr">
@@ -10346,7 +10346,7 @@
         </is>
       </c>
       <c r="G241" s="2" t="n">
-        <v>0.27</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="H241" s="2" t="inlineStr">
         <is>
@@ -10368,7 +10368,7 @@
       </c>
       <c r="C242" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #7 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.69s.</t>
+          <t>User executes offline storage operation #7 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.47s.</t>
         </is>
       </c>
       <c r="D242" s="2" t="inlineStr">
@@ -10387,7 +10387,7 @@
         </is>
       </c>
       <c r="G242" s="2" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.47</v>
       </c>
       <c r="H242" s="2" t="inlineStr">
         <is>
@@ -10409,7 +10409,7 @@
       </c>
       <c r="C243" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #8 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.4s.</t>
+          <t>User executes offline storage operation #8 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.53s.</t>
         </is>
       </c>
       <c r="D243" s="2" t="inlineStr">
@@ -10428,7 +10428,7 @@
         </is>
       </c>
       <c r="G243" s="2" t="n">
-        <v>0.4</v>
+        <v>0.53</v>
       </c>
       <c r="H243" s="2" t="inlineStr">
         <is>
@@ -10450,7 +10450,7 @@
       </c>
       <c r="C244" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #9 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.31s.</t>
+          <t>User executes offline storage operation #9 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.32s.</t>
         </is>
       </c>
       <c r="D244" s="2" t="inlineStr">
@@ -10469,7 +10469,7 @@
         </is>
       </c>
       <c r="G244" s="2" t="n">
-        <v>0.31</v>
+        <v>0.32</v>
       </c>
       <c r="H244" s="2" t="inlineStr">
         <is>
@@ -10491,7 +10491,7 @@
       </c>
       <c r="C245" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #10 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.59s.</t>
+          <t>User executes offline storage operation #10 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.41s.</t>
         </is>
       </c>
       <c r="D245" s="2" t="inlineStr">
@@ -10510,7 +10510,7 @@
         </is>
       </c>
       <c r="G245" s="2" t="n">
-        <v>0.59</v>
+        <v>0.41</v>
       </c>
       <c r="H245" s="2" t="inlineStr">
         <is>
@@ -10532,7 +10532,7 @@
       </c>
       <c r="C246" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #11 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.5s.</t>
+          <t>User executes offline storage operation #11 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.45s.</t>
         </is>
       </c>
       <c r="D246" s="2" t="inlineStr">
@@ -10551,7 +10551,7 @@
         </is>
       </c>
       <c r="G246" s="2" t="n">
-        <v>0.5</v>
+        <v>0.45</v>
       </c>
       <c r="H246" s="2" t="inlineStr">
         <is>
@@ -10573,7 +10573,7 @@
       </c>
       <c r="C247" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #12 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.26s.</t>
+          <t>User executes offline storage operation #12 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.62s.</t>
         </is>
       </c>
       <c r="D247" s="2" t="inlineStr">
@@ -10592,7 +10592,7 @@
         </is>
       </c>
       <c r="G247" s="2" t="n">
-        <v>0.26</v>
+        <v>0.62</v>
       </c>
       <c r="H247" s="2" t="inlineStr">
         <is>
@@ -10614,7 +10614,7 @@
       </c>
       <c r="C248" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #13 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.63s.</t>
+          <t>User executes offline storage operation #13 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.58s.</t>
         </is>
       </c>
       <c r="D248" s="2" t="inlineStr">
@@ -10633,7 +10633,7 @@
         </is>
       </c>
       <c r="G248" s="2" t="n">
-        <v>0.63</v>
+        <v>0.58</v>
       </c>
       <c r="H248" s="2" t="inlineStr">
         <is>
@@ -10655,7 +10655,7 @@
       </c>
       <c r="C249" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #14 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.68s.</t>
+          <t>User executes offline storage operation #14 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.74s.</t>
         </is>
       </c>
       <c r="D249" s="2" t="inlineStr">
@@ -10674,7 +10674,7 @@
         </is>
       </c>
       <c r="G249" s="2" t="n">
-        <v>0.68</v>
+        <v>0.74</v>
       </c>
       <c r="H249" s="2" t="inlineStr">
         <is>
@@ -10696,7 +10696,7 @@
       </c>
       <c r="C250" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #15 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.52s.</t>
+          <t>User executes offline storage operation #15 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.35s.</t>
         </is>
       </c>
       <c r="D250" s="2" t="inlineStr">
@@ -10715,7 +10715,7 @@
         </is>
       </c>
       <c r="G250" s="2" t="n">
-        <v>0.52</v>
+        <v>0.35</v>
       </c>
       <c r="H250" s="2" t="inlineStr">
         <is>
@@ -10737,7 +10737,7 @@
       </c>
       <c r="C251" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #16 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.46s.</t>
+          <t>User executes offline storage operation #16 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.44s.</t>
         </is>
       </c>
       <c r="D251" s="2" t="inlineStr">
@@ -10756,7 +10756,7 @@
         </is>
       </c>
       <c r="G251" s="2" t="n">
-        <v>0.46</v>
+        <v>0.44</v>
       </c>
       <c r="H251" s="2" t="inlineStr">
         <is>
@@ -10819,7 +10819,7 @@
       </c>
       <c r="C253" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #18 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.6s.</t>
+          <t>User executes offline storage operation #18 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.48s.</t>
         </is>
       </c>
       <c r="D253" s="2" t="inlineStr">
@@ -10838,7 +10838,7 @@
         </is>
       </c>
       <c r="G253" s="2" t="n">
-        <v>0.6</v>
+        <v>0.48</v>
       </c>
       <c r="H253" s="2" t="inlineStr">
         <is>
@@ -10860,7 +10860,7 @@
       </c>
       <c r="C254" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #19 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.32s.</t>
+          <t>User executes offline storage operation #19 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.5s.</t>
         </is>
       </c>
       <c r="D254" s="2" t="inlineStr">
@@ -10879,7 +10879,7 @@
         </is>
       </c>
       <c r="G254" s="2" t="n">
-        <v>0.32</v>
+        <v>0.5</v>
       </c>
       <c r="H254" s="2" t="inlineStr">
         <is>
@@ -10901,7 +10901,7 @@
       </c>
       <c r="C255" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #20 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.44s.</t>
+          <t>User executes offline storage operation #20 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.62s.</t>
         </is>
       </c>
       <c r="D255" s="2" t="inlineStr">
@@ -10920,7 +10920,7 @@
         </is>
       </c>
       <c r="G255" s="2" t="n">
-        <v>0.44</v>
+        <v>0.62</v>
       </c>
       <c r="H255" s="2" t="inlineStr">
         <is>
@@ -10942,7 +10942,7 @@
       </c>
       <c r="C256" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #21 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.67s.</t>
+          <t>User executes offline storage operation #21 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.61s.</t>
         </is>
       </c>
       <c r="D256" s="2" t="inlineStr">
@@ -10961,7 +10961,7 @@
         </is>
       </c>
       <c r="G256" s="2" t="n">
-        <v>0.67</v>
+        <v>0.61</v>
       </c>
       <c r="H256" s="2" t="inlineStr">
         <is>
@@ -10983,7 +10983,7 @@
       </c>
       <c r="C257" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #22 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.63s.</t>
+          <t>User executes offline storage operation #22 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.72s.</t>
         </is>
       </c>
       <c r="D257" s="2" t="inlineStr">
@@ -11002,7 +11002,7 @@
         </is>
       </c>
       <c r="G257" s="2" t="n">
-        <v>0.63</v>
+        <v>0.72</v>
       </c>
       <c r="H257" s="2" t="inlineStr">
         <is>
@@ -11024,7 +11024,7 @@
       </c>
       <c r="C258" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #23 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.27s.</t>
+          <t>User executes offline storage operation #23 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.4s.</t>
         </is>
       </c>
       <c r="D258" s="2" t="inlineStr">
@@ -11043,7 +11043,7 @@
         </is>
       </c>
       <c r="G258" s="2" t="n">
-        <v>0.27</v>
+        <v>0.4</v>
       </c>
       <c r="H258" s="2" t="inlineStr">
         <is>
@@ -11065,7 +11065,7 @@
       </c>
       <c r="C259" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #24 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.52s.</t>
+          <t>User executes offline storage operation #24 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.42s.</t>
         </is>
       </c>
       <c r="D259" s="2" t="inlineStr">
@@ -11084,7 +11084,7 @@
         </is>
       </c>
       <c r="G259" s="2" t="n">
-        <v>0.52</v>
+        <v>0.42</v>
       </c>
       <c r="H259" s="2" t="inlineStr">
         <is>
@@ -11106,7 +11106,7 @@
       </c>
       <c r="C260" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #25 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.27s.</t>
+          <t>User executes offline storage operation #25 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.44s.</t>
         </is>
       </c>
       <c r="D260" s="2" t="inlineStr">
@@ -11125,7 +11125,7 @@
         </is>
       </c>
       <c r="G260" s="2" t="n">
-        <v>0.27</v>
+        <v>0.44</v>
       </c>
       <c r="H260" s="2" t="inlineStr">
         <is>
@@ -11147,7 +11147,7 @@
       </c>
       <c r="C261" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #26 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.44s.</t>
+          <t>User executes offline storage operation #26 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.49s.</t>
         </is>
       </c>
       <c r="D261" s="2" t="inlineStr">
@@ -11166,7 +11166,7 @@
         </is>
       </c>
       <c r="G261" s="2" t="n">
-        <v>0.44</v>
+        <v>0.49</v>
       </c>
       <c r="H261" s="2" t="inlineStr">
         <is>
@@ -11188,7 +11188,7 @@
       </c>
       <c r="C262" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #27 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.43s.</t>
+          <t>User executes offline storage operation #27 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.56s.</t>
         </is>
       </c>
       <c r="D262" s="2" t="inlineStr">
@@ -11207,7 +11207,7 @@
         </is>
       </c>
       <c r="G262" s="2" t="n">
-        <v>0.43</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="H262" s="2" t="inlineStr">
         <is>
@@ -11229,7 +11229,7 @@
       </c>
       <c r="C263" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #28 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.48s.</t>
+          <t>User executes offline storage operation #28 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.63s.</t>
         </is>
       </c>
       <c r="D263" s="2" t="inlineStr">
@@ -11248,7 +11248,7 @@
         </is>
       </c>
       <c r="G263" s="2" t="n">
-        <v>0.48</v>
+        <v>0.63</v>
       </c>
       <c r="H263" s="2" t="inlineStr">
         <is>
@@ -11270,7 +11270,7 @@
       </c>
       <c r="C264" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #29 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.32s.</t>
+          <t>User executes offline storage operation #29 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.64s.</t>
         </is>
       </c>
       <c r="D264" s="2" t="inlineStr">
@@ -11289,7 +11289,7 @@
         </is>
       </c>
       <c r="G264" s="2" t="n">
-        <v>0.32</v>
+        <v>0.64</v>
       </c>
       <c r="H264" s="2" t="inlineStr">
         <is>
@@ -11311,7 +11311,7 @@
       </c>
       <c r="C265" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #30 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.64s.</t>
+          <t>User executes offline storage operation #30 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.32s.</t>
         </is>
       </c>
       <c r="D265" s="2" t="inlineStr">
@@ -11330,7 +11330,7 @@
         </is>
       </c>
       <c r="G265" s="2" t="n">
-        <v>0.64</v>
+        <v>0.32</v>
       </c>
       <c r="H265" s="2" t="inlineStr">
         <is>
@@ -11352,7 +11352,7 @@
       </c>
       <c r="C266" s="2" t="inlineStr">
         <is>
-          <t>User executes offline storage operation #31 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.41s.</t>
+          <t>User executes offline storage operation #31 (local serialization &amp; SQLite/AsyncStorage sync) -&gt; Verifies data integrity in 0.47s.</t>
         </is>
       </c>
       <c r="D266" s="2" t="inlineStr">
@@ -11371,7 +11371,7 @@
         </is>
       </c>
       <c r="G266" s="2" t="n">
-        <v>0.41</v>
+        <v>0.47</v>
       </c>
       <c r="H266" s="2" t="inlineStr">
         <is>
@@ -11412,7 +11412,7 @@
         </is>
       </c>
       <c r="G267" s="2" t="n">
-        <v>0.38</v>
+        <v>0.58</v>
       </c>
       <c r="H267" s="2" t="inlineStr">
         <is>
@@ -11453,7 +11453,7 @@
         </is>
       </c>
       <c r="G268" s="2" t="n">
-        <v>0.39</v>
+        <v>0.22</v>
       </c>
       <c r="H268" s="2" t="inlineStr">
         <is>
@@ -11494,7 +11494,7 @@
         </is>
       </c>
       <c r="G269" s="2" t="n">
-        <v>0.22</v>
+        <v>0.67</v>
       </c>
       <c r="H269" s="2" t="inlineStr">
         <is>
@@ -11535,7 +11535,7 @@
         </is>
       </c>
       <c r="G270" s="2" t="n">
-        <v>0.42</v>
+        <v>0.31</v>
       </c>
       <c r="H270" s="2" t="inlineStr">
         <is>
@@ -11557,7 +11557,7 @@
       </c>
       <c r="C271" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #1 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.59s.</t>
+          <t>User tests layout/memory scenario #1 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.55s.</t>
         </is>
       </c>
       <c r="D271" s="2" t="inlineStr">
@@ -11576,7 +11576,7 @@
         </is>
       </c>
       <c r="G271" s="2" t="n">
-        <v>0.59</v>
+        <v>0.55</v>
       </c>
       <c r="H271" s="2" t="inlineStr">
         <is>
@@ -11598,7 +11598,7 @@
       </c>
       <c r="C272" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #2 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.55s.</t>
+          <t>User tests layout/memory scenario #2 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.63s.</t>
         </is>
       </c>
       <c r="D272" s="2" t="inlineStr">
@@ -11617,7 +11617,7 @@
         </is>
       </c>
       <c r="G272" s="2" t="n">
-        <v>0.55</v>
+        <v>0.63</v>
       </c>
       <c r="H272" s="2" t="inlineStr">
         <is>
@@ -11639,7 +11639,7 @@
       </c>
       <c r="C273" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #3 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.3s.</t>
+          <t>User tests layout/memory scenario #3 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.22s.</t>
         </is>
       </c>
       <c r="D273" s="2" t="inlineStr">
@@ -11658,7 +11658,7 @@
         </is>
       </c>
       <c r="G273" s="2" t="n">
-        <v>0.3</v>
+        <v>0.22</v>
       </c>
       <c r="H273" s="2" t="inlineStr">
         <is>
@@ -11680,7 +11680,7 @@
       </c>
       <c r="C274" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #4 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.46s.</t>
+          <t>User tests layout/memory scenario #4 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.6s.</t>
         </is>
       </c>
       <c r="D274" s="2" t="inlineStr">
@@ -11699,7 +11699,7 @@
         </is>
       </c>
       <c r="G274" s="2" t="n">
-        <v>0.46</v>
+        <v>0.6</v>
       </c>
       <c r="H274" s="2" t="inlineStr">
         <is>
@@ -11721,7 +11721,7 @@
       </c>
       <c r="C275" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #5 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.46s.</t>
+          <t>User tests layout/memory scenario #5 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.48s.</t>
         </is>
       </c>
       <c r="D275" s="2" t="inlineStr">
@@ -11740,7 +11740,7 @@
         </is>
       </c>
       <c r="G275" s="2" t="n">
-        <v>0.46</v>
+        <v>0.48</v>
       </c>
       <c r="H275" s="2" t="inlineStr">
         <is>
@@ -11762,7 +11762,7 @@
       </c>
       <c r="C276" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #6 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.62s.</t>
+          <t>User tests layout/memory scenario #6 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.39s.</t>
         </is>
       </c>
       <c r="D276" s="2" t="inlineStr">
@@ -11781,7 +11781,7 @@
         </is>
       </c>
       <c r="G276" s="2" t="n">
-        <v>0.62</v>
+        <v>0.39</v>
       </c>
       <c r="H276" s="2" t="inlineStr">
         <is>
@@ -11803,7 +11803,7 @@
       </c>
       <c r="C277" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #7 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.45s.</t>
+          <t>User tests layout/memory scenario #7 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.54s.</t>
         </is>
       </c>
       <c r="D277" s="2" t="inlineStr">
@@ -11822,7 +11822,7 @@
         </is>
       </c>
       <c r="G277" s="2" t="n">
-        <v>0.45</v>
+        <v>0.54</v>
       </c>
       <c r="H277" s="2" t="inlineStr">
         <is>
@@ -11844,7 +11844,7 @@
       </c>
       <c r="C278" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #8 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.42s.</t>
+          <t>User tests layout/memory scenario #8 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.5s.</t>
         </is>
       </c>
       <c r="D278" s="2" t="inlineStr">
@@ -11863,7 +11863,7 @@
         </is>
       </c>
       <c r="G278" s="2" t="n">
-        <v>0.42</v>
+        <v>0.5</v>
       </c>
       <c r="H278" s="2" t="inlineStr">
         <is>
@@ -11885,7 +11885,7 @@
       </c>
       <c r="C279" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #9 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.53s.</t>
+          <t>User tests layout/memory scenario #9 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.44s.</t>
         </is>
       </c>
       <c r="D279" s="2" t="inlineStr">
@@ -11904,7 +11904,7 @@
         </is>
       </c>
       <c r="G279" s="2" t="n">
-        <v>0.53</v>
+        <v>0.44</v>
       </c>
       <c r="H279" s="2" t="inlineStr">
         <is>
@@ -11926,7 +11926,7 @@
       </c>
       <c r="C280" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #10 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.35s.</t>
+          <t>User tests layout/memory scenario #10 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.61s.</t>
         </is>
       </c>
       <c r="D280" s="2" t="inlineStr">
@@ -11945,7 +11945,7 @@
         </is>
       </c>
       <c r="G280" s="2" t="n">
-        <v>0.35</v>
+        <v>0.61</v>
       </c>
       <c r="H280" s="2" t="inlineStr">
         <is>
@@ -11967,7 +11967,7 @@
       </c>
       <c r="C281" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #11 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.64s.</t>
+          <t>User tests layout/memory scenario #11 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.35s.</t>
         </is>
       </c>
       <c r="D281" s="2" t="inlineStr">
@@ -11986,7 +11986,7 @@
         </is>
       </c>
       <c r="G281" s="2" t="n">
-        <v>0.64</v>
+        <v>0.35</v>
       </c>
       <c r="H281" s="2" t="inlineStr">
         <is>
@@ -12008,7 +12008,7 @@
       </c>
       <c r="C282" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #12 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.32s.</t>
+          <t>User tests layout/memory scenario #12 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.23s.</t>
         </is>
       </c>
       <c r="D282" s="2" t="inlineStr">
@@ -12027,7 +12027,7 @@
         </is>
       </c>
       <c r="G282" s="2" t="n">
-        <v>0.32</v>
+        <v>0.23</v>
       </c>
       <c r="H282" s="2" t="inlineStr">
         <is>
@@ -12049,7 +12049,7 @@
       </c>
       <c r="C283" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #13 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.53s.</t>
+          <t>User tests layout/memory scenario #13 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.29s.</t>
         </is>
       </c>
       <c r="D283" s="2" t="inlineStr">
@@ -12068,7 +12068,7 @@
         </is>
       </c>
       <c r="G283" s="2" t="n">
-        <v>0.53</v>
+        <v>0.29</v>
       </c>
       <c r="H283" s="2" t="inlineStr">
         <is>
@@ -12090,7 +12090,7 @@
       </c>
       <c r="C284" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #14 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.52s.</t>
+          <t>User tests layout/memory scenario #14 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.65s.</t>
         </is>
       </c>
       <c r="D284" s="2" t="inlineStr">
@@ -12109,7 +12109,7 @@
         </is>
       </c>
       <c r="G284" s="2" t="n">
-        <v>0.52</v>
+        <v>0.65</v>
       </c>
       <c r="H284" s="2" t="inlineStr">
         <is>
@@ -12131,7 +12131,7 @@
       </c>
       <c r="C285" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #15 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.64s.</t>
+          <t>User tests layout/memory scenario #15 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.45s.</t>
         </is>
       </c>
       <c r="D285" s="2" t="inlineStr">
@@ -12150,7 +12150,7 @@
         </is>
       </c>
       <c r="G285" s="2" t="n">
-        <v>0.64</v>
+        <v>0.45</v>
       </c>
       <c r="H285" s="2" t="inlineStr">
         <is>
@@ -12172,7 +12172,7 @@
       </c>
       <c r="C286" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #16 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.29s.</t>
+          <t>User tests layout/memory scenario #16 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.59s.</t>
         </is>
       </c>
       <c r="D286" s="2" t="inlineStr">
@@ -12191,7 +12191,7 @@
         </is>
       </c>
       <c r="G286" s="2" t="n">
-        <v>0.29</v>
+        <v>0.59</v>
       </c>
       <c r="H286" s="2" t="inlineStr">
         <is>
@@ -12213,7 +12213,7 @@
       </c>
       <c r="C287" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #17 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.41s.</t>
+          <t>User tests layout/memory scenario #17 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.45s.</t>
         </is>
       </c>
       <c r="D287" s="2" t="inlineStr">
@@ -12232,7 +12232,7 @@
         </is>
       </c>
       <c r="G287" s="2" t="n">
-        <v>0.41</v>
+        <v>0.45</v>
       </c>
       <c r="H287" s="2" t="inlineStr">
         <is>
@@ -12254,7 +12254,7 @@
       </c>
       <c r="C288" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #18 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.36s.</t>
+          <t>User tests layout/memory scenario #18 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.62s.</t>
         </is>
       </c>
       <c r="D288" s="2" t="inlineStr">
@@ -12273,7 +12273,7 @@
         </is>
       </c>
       <c r="G288" s="2" t="n">
-        <v>0.36</v>
+        <v>0.62</v>
       </c>
       <c r="H288" s="2" t="inlineStr">
         <is>
@@ -12295,7 +12295,7 @@
       </c>
       <c r="C289" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #19 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.34s.</t>
+          <t>User tests layout/memory scenario #19 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.61s.</t>
         </is>
       </c>
       <c r="D289" s="2" t="inlineStr">
@@ -12314,7 +12314,7 @@
         </is>
       </c>
       <c r="G289" s="2" t="n">
-        <v>0.34</v>
+        <v>0.61</v>
       </c>
       <c r="H289" s="2" t="inlineStr">
         <is>
@@ -12336,7 +12336,7 @@
       </c>
       <c r="C290" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #20 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.33s.</t>
+          <t>User tests layout/memory scenario #20 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.3s.</t>
         </is>
       </c>
       <c r="D290" s="2" t="inlineStr">
@@ -12355,7 +12355,7 @@
         </is>
       </c>
       <c r="G290" s="2" t="n">
-        <v>0.33</v>
+        <v>0.3</v>
       </c>
       <c r="H290" s="2" t="inlineStr">
         <is>
@@ -12377,7 +12377,7 @@
       </c>
       <c r="C291" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #21 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.59s.</t>
+          <t>User tests layout/memory scenario #21 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.42s.</t>
         </is>
       </c>
       <c r="D291" s="2" t="inlineStr">
@@ -12396,7 +12396,7 @@
         </is>
       </c>
       <c r="G291" s="2" t="n">
-        <v>0.59</v>
+        <v>0.42</v>
       </c>
       <c r="H291" s="2" t="inlineStr">
         <is>
@@ -12418,7 +12418,7 @@
       </c>
       <c r="C292" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #22 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.27s.</t>
+          <t>User tests layout/memory scenario #22 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.66s.</t>
         </is>
       </c>
       <c r="D292" s="2" t="inlineStr">
@@ -12437,7 +12437,7 @@
         </is>
       </c>
       <c r="G292" s="2" t="n">
-        <v>0.27</v>
+        <v>0.66</v>
       </c>
       <c r="H292" s="2" t="inlineStr">
         <is>
@@ -12459,7 +12459,7 @@
       </c>
       <c r="C293" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #23 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.63s.</t>
+          <t>User tests layout/memory scenario #23 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.33s.</t>
         </is>
       </c>
       <c r="D293" s="2" t="inlineStr">
@@ -12478,7 +12478,7 @@
         </is>
       </c>
       <c r="G293" s="2" t="n">
-        <v>0.63</v>
+        <v>0.33</v>
       </c>
       <c r="H293" s="2" t="inlineStr">
         <is>
@@ -12500,7 +12500,7 @@
       </c>
       <c r="C294" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #24 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.49s.</t>
+          <t>User tests layout/memory scenario #24 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.46s.</t>
         </is>
       </c>
       <c r="D294" s="2" t="inlineStr">
@@ -12519,7 +12519,7 @@
         </is>
       </c>
       <c r="G294" s="2" t="n">
-        <v>0.49</v>
+        <v>0.46</v>
       </c>
       <c r="H294" s="2" t="inlineStr">
         <is>
@@ -12541,7 +12541,7 @@
       </c>
       <c r="C295" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #25 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.51s.</t>
+          <t>User tests layout/memory scenario #25 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.37s.</t>
         </is>
       </c>
       <c r="D295" s="2" t="inlineStr">
@@ -12560,7 +12560,7 @@
         </is>
       </c>
       <c r="G295" s="2" t="n">
-        <v>0.51</v>
+        <v>0.37</v>
       </c>
       <c r="H295" s="2" t="inlineStr">
         <is>
@@ -12582,7 +12582,7 @@
       </c>
       <c r="C296" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #26 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.48s.</t>
+          <t>User tests layout/memory scenario #26 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.58s.</t>
         </is>
       </c>
       <c r="D296" s="2" t="inlineStr">
@@ -12601,7 +12601,7 @@
         </is>
       </c>
       <c r="G296" s="2" t="n">
-        <v>0.48</v>
+        <v>0.58</v>
       </c>
       <c r="H296" s="2" t="inlineStr">
         <is>
@@ -12623,7 +12623,7 @@
       </c>
       <c r="C297" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #27 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.29s.</t>
+          <t>User tests layout/memory scenario #27 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.57s.</t>
         </is>
       </c>
       <c r="D297" s="2" t="inlineStr">
@@ -12642,7 +12642,7 @@
         </is>
       </c>
       <c r="G297" s="2" t="n">
-        <v>0.29</v>
+        <v>0.57</v>
       </c>
       <c r="H297" s="2" t="inlineStr">
         <is>
@@ -12664,7 +12664,7 @@
       </c>
       <c r="C298" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #28 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.53s.</t>
+          <t>User tests layout/memory scenario #28 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.36s.</t>
         </is>
       </c>
       <c r="D298" s="2" t="inlineStr">
@@ -12683,7 +12683,7 @@
         </is>
       </c>
       <c r="G298" s="2" t="n">
-        <v>0.53</v>
+        <v>0.36</v>
       </c>
       <c r="H298" s="2" t="inlineStr">
         <is>
@@ -12705,7 +12705,7 @@
       </c>
       <c r="C299" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #29 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.53s.</t>
+          <t>User tests layout/memory scenario #29 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.58s.</t>
         </is>
       </c>
       <c r="D299" s="2" t="inlineStr">
@@ -12724,7 +12724,7 @@
         </is>
       </c>
       <c r="G299" s="2" t="n">
-        <v>0.53</v>
+        <v>0.58</v>
       </c>
       <c r="H299" s="2" t="inlineStr">
         <is>
@@ -12746,7 +12746,7 @@
       </c>
       <c r="C300" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #30 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.23s.</t>
+          <t>User tests layout/memory scenario #30 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.5s.</t>
         </is>
       </c>
       <c r="D300" s="2" t="inlineStr">
@@ -12765,7 +12765,7 @@
         </is>
       </c>
       <c r="G300" s="2" t="n">
-        <v>0.23</v>
+        <v>0.5</v>
       </c>
       <c r="H300" s="2" t="inlineStr">
         <is>
@@ -12787,7 +12787,7 @@
       </c>
       <c r="C301" s="2" t="inlineStr">
         <is>
-          <t>User tests layout/memory scenario #31 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.68s.</t>
+          <t>User tests layout/memory scenario #31 (screen density scaling &amp; memory heap optimization) -&gt; Verifies rendering in 0.6s.</t>
         </is>
       </c>
       <c r="D301" s="2" t="inlineStr">
@@ -12806,7 +12806,7 @@
         </is>
       </c>
       <c r="G301" s="2" t="n">
-        <v>0.68</v>
+        <v>0.6</v>
       </c>
       <c r="H301" s="2" t="inlineStr">
         <is>

</xml_diff>